<commit_message>
chore: stocktwits data 2026-06-02 20:29 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D687"/>
+  <dimension ref="A1:D787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15564,6 +15564,2206 @@
       <c r="D687" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B688" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C688" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X Saylor must be selling BTC and buying MSTR stock right now. That might explain their divergence.</t>
+        </is>
+      </c>
+      <c r="D688" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B689" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C689" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X</t>
+        </is>
+      </c>
+      <c r="D689" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B690" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C690" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X told you all this was a scam</t>
+        </is>
+      </c>
+      <c r="D690" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B691" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C691" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X Where the fuck the buyers go?</t>
+        </is>
+      </c>
+      <c r="D691" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B692" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C692" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X 👇🩸👍✊</t>
+        </is>
+      </c>
+      <c r="D692" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B693" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C693" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X</t>
+        </is>
+      </c>
+      <c r="D693" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B694" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C694" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X biggest scam in human history. PERIOD</t>
+        </is>
+      </c>
+      <c r="D694" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B695" s="2" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C695" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X 32? 🤣🤣🤣🤣 out of his 900k stash? holy shit better go 100x short 🤣🤣 fucking imbeciles</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B696" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C696" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X 3000 eoy.</t>
+        </is>
+      </c>
+      <c r="D696" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B697" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C697" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X Below $71K . Here we go.</t>
+        </is>
+      </c>
+      <c r="D697" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B698" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C698" s="2" t="inlineStr">
+        <is>
+          <t>$BB only a matter of time before $tslA signs an agreement and 25/25 OEM manufacturers are in the pocket.</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B699" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C699" s="3" t="inlineStr">
+        <is>
+          <t>$BB this is fire!!!</t>
+        </is>
+      </c>
+      <c r="D699" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B700" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C700" s="2" t="inlineStr">
+        <is>
+          <t>$BB Are those Naked Shorts - Fake Shares boiling over, bahaha!!!!! Who will be holding the bag of Fake Shares? Short Headwinds!</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B701" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="inlineStr">
+        <is>
+          <t>$BB short squeeze coming very soon hold and keep buying.  Lets squeeze them short bitches 🤪</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B702" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>$BB</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B703" s="4" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C703" s="4" t="inlineStr">
+        <is>
+          <t>$BB  this is honestly the best argument this guy can come up with lmao</t>
+        </is>
+      </c>
+      <c r="D703" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B704" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>$BB $BB The real question isn’t “am I selling?” The real question is, am I adding every day and averaging UP like fear and I are not on speaking terms?</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B705" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>$BB invest!  earning is on June 25! this will keep continuing to go higher!</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B706" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C706" s="3" t="inlineStr">
+        <is>
+          <t>$BB   Is this actually squeezing? What’s the short interest on this?  Or is this just undervalued?</t>
+        </is>
+      </c>
+      <c r="D706" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B707" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C707" s="3" t="inlineStr">
+        <is>
+          <t>@rogerR000 They have been friends since April... Friends stick together until the correlation breaks.. If its good for $BB it should be good for $NOK as well. Enjoy the ride.</t>
+        </is>
+      </c>
+      <c r="D707" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B708" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C708" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ f*** now i feel dumb trading this</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B709" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B710" s="3" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C710" s="3" t="inlineStr">
+        <is>
+          <t>$INFQ go baby jump</t>
+        </is>
+      </c>
+      <c r="D710" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B711" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B712" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C712" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ literally 🚀 boosted the last 26 minutes before closing and broke the $19.75 barrier. The secret is out. Lets go!</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B713" s="3" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C713" s="3" t="inlineStr">
+        <is>
+          <t>$INFQ Lamborghini mercy</t>
+        </is>
+      </c>
+      <c r="D713" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B714" s="3" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C714" s="3" t="inlineStr">
+        <is>
+          <t>$INFQ #3 trending</t>
+        </is>
+      </c>
+      <c r="D714" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B715" s="3" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C715" s="3" t="inlineStr">
+        <is>
+          <t>$INFQ I remember the idiots from yesterday and I see more today</t>
+        </is>
+      </c>
+      <c r="D715" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B716" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ wanted to take a screenshot but can’t curse it like that</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B717" s="3" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C717" s="3" t="inlineStr">
+        <is>
+          <t>$INFQ Not  even out of the gate yet.🤔😎</t>
+        </is>
+      </c>
+      <c r="D717" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B718" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C718" s="3" t="inlineStr">
+        <is>
+          <t>$PANW I’m getting ready for all the “BLOODBATH BY 6:30 AM” “BAG HOLDERS GETTING WRECKED HERE”</t>
+        </is>
+      </c>
+      <c r="D718" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B719" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C719" s="3" t="inlineStr">
+        <is>
+          <t>$PANW earnings don’t justify gap up. Imo</t>
+        </is>
+      </c>
+      <c r="D719" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B720" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>$PANW I Love you PANW!!!</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B721" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C721" s="3" t="inlineStr">
+        <is>
+          <t>$PANW feeling heavy here no long</t>
+        </is>
+      </c>
+      <c r="D721" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B722" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C722" s="2" t="inlineStr">
+        <is>
+          <t>$PANW</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B723" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C723" s="3" t="inlineStr">
+        <is>
+          <t>$PANW released its third-quarter 2026 results. https://www.rapidticker.com/news/panw-sec-filing-8-k-43effd</t>
+        </is>
+      </c>
+      <c r="D723" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B724" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C724" s="2" t="inlineStr">
+        <is>
+          <t>$PANW hoping this doesn’t crash and burn during the call</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B725" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C725" s="3" t="inlineStr">
+        <is>
+          <t>$PANW   Feels like the market just need a beat of any sort-   Traders wanted to moon PANW.  This is ridiculous- but congrats.  63% gain in month leading up and add 11% more AH today.  Unreal.  Hate me - but next week the market crashes.  Mark my word  Wall Street is greedy manipu</t>
+        </is>
+      </c>
+      <c r="D725" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B726" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C726" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Palo Alto Networks pops 12% on earnings beat, rosy guidance https://www.cnbc.com/2026/06/02/palo-alto-networks-panw-q3-earnings-2026.html?__source=iosappshare%7Ccom.stocktwits.StockTwits.STShareExtension</t>
+        </is>
+      </c>
+      <c r="D726" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B727" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C727" s="3" t="inlineStr">
+        <is>
+          <t>$PANW my giant chub is AI related lol</t>
+        </is>
+      </c>
+      <c r="D727" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B728" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C728" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR hahaha they sold 32 btc comical. This company is stupid bullish. And I love it. Going to be worth so so much in the future</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B729" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C729" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X $FBTC $GBTC $IBIT $MSTR   Maybe fat finger but he indeed sold 32 BTC  And the market already went crazy. Crypto is really a joke. We see even more dips this summer.   Loaded up on MSTR puts</t>
+        </is>
+      </c>
+      <c r="D729" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B730" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C730" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR they sell $32 bitty what the heck, a lot of family to feed?  Sell this outdated outfit and buy $PURR</t>
+        </is>
+      </c>
+      <c r="D730" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B731" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C731" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X $ETH.X $MSTR If Saylor put the bottom in to add to the max FUD campaign thats been going on by selling a meager 32 bitcoin that would honestly be a hilarious bear trap.</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B732" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C732" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR yeah, this is going down..</t>
+        </is>
+      </c>
+      <c r="D732" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B733" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C733" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR just added another layer to the Bitcoin treasury story, and the tape is getting more interesting than the headlines     Selling 32 BTC for $2.5M while simultaneously raising $128.3M via share issuance shows they’re still actively managing liquidity, not passively holding. W</t>
+        </is>
+      </c>
+      <c r="D733" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B734" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C734" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR how is this above 150? are they loading up for reversal or are they proping to liquidate long positions and build short positions? only time will tell.... $BTC.X</t>
+        </is>
+      </c>
+      <c r="D734" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B735" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C735" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR give me 160</t>
+        </is>
+      </c>
+      <c r="D735" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B736" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C736" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $DJT just absolute fraud being perpetuated by banks here trying to liquidate saylor and scare retail out of a life free of debt to them  $MSTR   criminal</t>
+        </is>
+      </c>
+      <c r="D736" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B737" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C737" s="2" t="inlineStr">
+        <is>
+          <t>$HIVE $CLSK $MSTR $ASST You cant Shake me out mr market. Im deep in Green 🤝</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B738" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C738" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR $ETH.X $ASST $BMNR New Coinbase trading floor</t>
+        </is>
+      </c>
+      <c r="D738" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B739" s="2" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C739" s="2" t="inlineStr">
+        <is>
+          <t>$HYPE.X $PURR $BTC.X $ETH.X   Goldman Sachs invested into hyperliquid</t>
+        </is>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B740" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C740" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X don’t mind me just selling all my eth for a tax loss then immediately repurchasing.</t>
+        </is>
+      </c>
+      <c r="D740" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B741" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C741" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X Sub 1900 soon.</t>
+        </is>
+      </c>
+      <c r="D741" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B742" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C742" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X we are cooked and nobody is coming to help</t>
+        </is>
+      </c>
+      <c r="D742" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B743" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C743" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X oof</t>
+        </is>
+      </c>
+      <c r="D743" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B744" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C744" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X I&amp;#39;m pretty sure I remember him making predictions like this for Bitcoin 5 years ago.  That turned out well.</t>
+        </is>
+      </c>
+      <c r="D744" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B745" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C745" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X Payments are automatic and made in USDC, which is real money—no tricks or scams, and no staking required.</t>
+        </is>
+      </c>
+      <c r="D745" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B746" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C746" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X drops below 67K its lowest level in nearly 2 months.    $ETH.X drops below 1.9K its lowest level in 3 months.    About 1.35B in long positions liquidated over the last 24 hours.    All this while the US stock market hits yet another all time high.    Crypto and equities di</t>
+        </is>
+      </c>
+      <c r="D746" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B747" s="2" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C747" s="2" t="inlineStr">
+        <is>
+          <t>$ETH.X genuinely think it&amp;#39;s a big green day tomorrow</t>
+        </is>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B748" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C748" s="4" t="inlineStr">
+        <is>
+          <t>One of the largest equity capital raises in tech history $GOOGL  $GOOG</t>
+        </is>
+      </c>
+      <c r="D748" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B749" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C749" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL Destroy it.</t>
+        </is>
+      </c>
+      <c r="D749" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B750" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C750" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL 351 offer magnet</t>
+        </is>
+      </c>
+      <c r="D750" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B751" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C751" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL ppl freaking out on 2% drop in AH with this crazy run until now</t>
+        </is>
+      </c>
+      <c r="D751" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B752" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C752" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL very interesting reaction IMO. Telling of more to come?</t>
+        </is>
+      </c>
+      <c r="D752" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B753" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C753" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL Fair value is $ 122</t>
+        </is>
+      </c>
+      <c r="D753" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B754" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C754" s="3" t="inlineStr">
+        <is>
+          <t>$BRK.X $GOOGL</t>
+        </is>
+      </c>
+      <c r="D754" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B755" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C755" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL   If this report is true, it&amp;#39;s a pretty wild development.    Google potentially raising $80B to accelerate growth while $BRK.X steps in with a $10B investment?     Not gonna lie, that&amp;#39;s not the kind of headline I expected to see today.    The interesting part isn&amp;#</t>
+        </is>
+      </c>
+      <c r="D755" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B756" s="2" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C756" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY  $GOOG $GOOGL Alphabet has to be inntalks with Galaxy for their Helios Data Center capacity   https://finance.yahoo.com/sectors/technology/articles/alphabet-plans-80-billion-raise-213043536.html</t>
+        </is>
+      </c>
+      <c r="D756" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B757" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C757" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL the irony is that people predicted this ai overspend would be needed well over a year ago — but yet the stock ran up over 200% instead on ai hype alone… now the chicken is coming home to roost… last earnings beat was due to their anthropic investment mark to market, exclud</t>
+        </is>
+      </c>
+      <c r="D757" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B758" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C758" s="2" t="inlineStr">
+        <is>
+          <t>$NBIS $ASTC $TE $SPCE $KEEL   #TopWatches #WW</t>
+        </is>
+      </c>
+      <c r="D758" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B759" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C759" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B760" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C760" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D760" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B761" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C761" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL 6.5 coming</t>
+        </is>
+      </c>
+      <c r="D761" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B762" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C762" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL deal announcement soon looks like it. Big boys know something</t>
+        </is>
+      </c>
+      <c r="D762" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B763" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C763" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL I have a strong feeling a deal will be announced in one of these days AH. Maybe even today who knows 🤷‍♂️</t>
+        </is>
+      </c>
+      <c r="D763" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B764" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C764" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL Congrats on this milestone!  What an achievement!</t>
+        </is>
+      </c>
+      <c r="D764" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B765" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C765" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL  love it 😍!!!!!!</t>
+        </is>
+      </c>
+      <c r="D765" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B766" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C766" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL Just keeps ripping!</t>
+        </is>
+      </c>
+      <c r="D766" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B767" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C767" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL Higher than you ever imagined!</t>
+        </is>
+      </c>
+      <c r="D767" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B768" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C768" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB what even is the bear case here?</t>
+        </is>
+      </c>
+      <c r="D768" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B769" s="3" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C769" s="3" t="inlineStr">
+        <is>
+          <t>$GTLB POS shouldn’t have played options here. The IV was crazy</t>
+        </is>
+      </c>
+      <c r="D769" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B770" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C770" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB why are bears yapping 😂😂💀</t>
+        </is>
+      </c>
+      <c r="D770" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B771" s="4" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C771" s="4" t="inlineStr">
+        <is>
+          <t>$GTLB</t>
+        </is>
+      </c>
+      <c r="D771" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B772" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C772" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB potential with Antrophic btw - will shoot up this year</t>
+        </is>
+      </c>
+      <c r="D772" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B773" s="4" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C773" s="4" t="inlineStr">
+        <is>
+          <t>$GTLB   Easy red soon not seeing any potential here.</t>
+        </is>
+      </c>
+      <c r="D773" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B774" s="4" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C774" s="4" t="inlineStr">
+        <is>
+          <t>$GTLB Why buy now??!! When you could buy next week at 28$…</t>
+        </is>
+      </c>
+      <c r="D774" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B775" s="3" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C775" s="3" t="inlineStr">
+        <is>
+          <t>$GTLB Raised FY27 guidance is what we need to jump, and commentary that AI products are becoming a meaningful revenue contributor.  If they deliver, we can expect 20% up.</t>
+        </is>
+      </c>
+      <c r="D775" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B776" s="3" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C776" s="3" t="inlineStr">
+        <is>
+          <t>$GTLB Picked up $102,000 here</t>
+        </is>
+      </c>
+      <c r="D776" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B777" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C777" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB please give us another green dildo 🙏</t>
+        </is>
+      </c>
+      <c r="D777" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B778" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C778" s="3" t="inlineStr">
+        <is>
+          <t>$SOXX is big boss Jen Sen having any other Trillion dollar talking any other forum. Have him few more forums to move this 700 in a week.</t>
+        </is>
+      </c>
+      <c r="D778" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B779" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C779" s="3" t="inlineStr">
+        <is>
+          <t>$SOXX keep buying</t>
+        </is>
+      </c>
+      <c r="D779" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B780" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C780" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS $SOXX Losses (so far). SOXS avg at 14 and SOXX short average at 458</t>
+        </is>
+      </c>
+      <c r="D780" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B781" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C781" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ $SPY $SOXX $SOXL $NBIS   As much as people hate the scam you have to participate in the scam. Imagine being handed a money cheat code and throwing it in the trash.</t>
+        </is>
+      </c>
+      <c r="D781" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B782" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C782" s="3" t="inlineStr">
+        <is>
+          <t>$SOXX  $QQQ Pure Mania</t>
+        </is>
+      </c>
+      <c r="D782" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B783" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C783" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ $SOXL $SOXS $SOXX $SPY</t>
+        </is>
+      </c>
+      <c r="D783" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B784" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C784" s="3" t="inlineStr">
+        <is>
+          <t>$SOXX retail frenzy here!   A/D has not made a new high since May 8th 2026. Price is 15% higher.</t>
+        </is>
+      </c>
+      <c r="D784" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B785" s="4" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C785" s="4" t="inlineStr">
+        <is>
+          <t>$SOXX this is stupid. multiples expansion. cool i get it. just another name for treasury pushing money into markets.</t>
+        </is>
+      </c>
+      <c r="D785" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B786" s="2" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C786" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO if this goes wrong, it could be the start of massive profit taking in semis. People are getting so confident buying everything blindly everyday. $SOXL $SOXS $SOXX</t>
+        </is>
+      </c>
+      <c r="D786" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+      <c r="B787" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C787" s="3" t="inlineStr">
+        <is>
+          <t>$SOXL $SOXX got lucky last night from Jesen&amp;#39;s casual talk - Lets see if there is another game tonight or tomorrow $SOXS</t>
+        </is>
+      </c>
+      <c r="D787" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -15578,7 +17778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15640,7 +17840,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -15650,24 +17850,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:29 UTC</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
@@ -15691,97 +17891,97 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-02 20:29 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-02 20:29 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:29 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -15793,41 +17993,41 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -15837,19 +18037,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -16144,6 +18344,108 @@
       <c r="C33" t="inlineStr">
         <is>
           <t>2026-06-01 22:07 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:29 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-02 20:35 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Raw Messages" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ticker Frequency" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FinViz Data" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D787"/>
+  <dimension ref="A1:D863"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17762,6 +17763,1678 @@
         </is>
       </c>
       <c r="D787" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B788" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C788" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X can’t catch a bid today</t>
+        </is>
+      </c>
+      <c r="D788" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B789" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C789" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X People are selling. So should you.</t>
+        </is>
+      </c>
+      <c r="D789" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B790" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C790" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X</t>
+        </is>
+      </c>
+      <c r="D790" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B791" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C791" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X</t>
+        </is>
+      </c>
+      <c r="D791" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B792" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C792" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X Bitcoin dead. AI stocks flying again. Market green. Bitcoin trash. Every day red.</t>
+        </is>
+      </c>
+      <c r="D792" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B793" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C793" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X I would love to see this at $65,000 again</t>
+        </is>
+      </c>
+      <c r="D793" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B794" s="2" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C794" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X .....    Iran knows Trumps approval is in the toilet,  that&amp;#39;s why they are now cancelling negotiations  ...  Both sides are playing games with the Markets.     .......</t>
+        </is>
+      </c>
+      <c r="D794" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B795" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C795" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X just wait until it goes down to $20000 and buy a lot then . For now this thing is a burning pile of garbage that is exit liquidity for the billionaires just like you said</t>
+        </is>
+      </c>
+      <c r="D795" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B796" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C796" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X</t>
+        </is>
+      </c>
+      <c r="D796" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B797" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C797" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X not one cares about this garbage any more.   Money is going back to the Stock market and with the lift on Day Trading restrictions millions o people will go back to trade .   Sorry fake coins $ETH.X $XRP.X $TRUMP.X $NDAQ</t>
+        </is>
+      </c>
+      <c r="D797" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B798" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C798" s="2" t="inlineStr">
+        <is>
+          <t>$BB when 80% of your account is in BB and wondering if you’re under allocated.</t>
+        </is>
+      </c>
+      <c r="D798" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B799" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C799" s="3" t="inlineStr">
+        <is>
+          <t>$BB</t>
+        </is>
+      </c>
+      <c r="D799" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B800" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C800" s="2" t="inlineStr">
+        <is>
+          <t>$BB feeling so sad and happy at same time...  Sad because i saw the first jumps around 4,50 and thought i was too late and seeing this every week scares me to jump in...    But so Happy seeing shorts being squeezed like little lemons 😂</t>
+        </is>
+      </c>
+      <c r="D800" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B801" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C801" s="2" t="inlineStr">
+        <is>
+          <t>$BB what the hell was revealed today behind closed doors? QNX2000</t>
+        </is>
+      </c>
+      <c r="D801" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B802" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C802" s="2" t="inlineStr">
+        <is>
+          <t>$BB Thanks for your money shorties ! Good night !</t>
+        </is>
+      </c>
+      <c r="D802" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B803" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C803" s="2" t="inlineStr">
+        <is>
+          <t>$BB if WSB gets a hold of this...</t>
+        </is>
+      </c>
+      <c r="D803" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B804" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C804" s="3" t="inlineStr">
+        <is>
+          <t>$BB everytime I look back this thing is higher!!!</t>
+        </is>
+      </c>
+      <c r="D804" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B805" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C805" s="2" t="inlineStr">
+        <is>
+          <t>$BB Squeezing</t>
+        </is>
+      </c>
+      <c r="D805" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B806" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C806" s="2" t="inlineStr">
+        <is>
+          <t>$BB $AMD $ONDS</t>
+        </is>
+      </c>
+      <c r="D806" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B807" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C807" s="2" t="inlineStr">
+        <is>
+          <t>$BB i just realized something veery scary...  I dont have enough shares.</t>
+        </is>
+      </c>
+      <c r="D807" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B808" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C808" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ +25%</t>
+        </is>
+      </c>
+      <c r="D808" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B809" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C809" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ The only time in my life I perfectly called a bottom.</t>
+        </is>
+      </c>
+      <c r="D809" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B810" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C810" s="2" t="inlineStr">
+        <is>
+          <t>$PANW  I missed this move.</t>
+        </is>
+      </c>
+      <c r="D810" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B811" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C811" s="2" t="inlineStr">
+        <is>
+          <t>$PANW 😉 if anthropic is right is accurate the this will be the first trillion dollar market cap cybersecurity company together with $CRWD . Remember i said this first.</t>
+        </is>
+      </c>
+      <c r="D811" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B812" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C812" s="3" t="inlineStr">
+        <is>
+          <t>$PANW They just need to say AI AI AI and stock will be $350 pronto</t>
+        </is>
+      </c>
+      <c r="D812" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B813" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C813" s="2" t="inlineStr">
+        <is>
+          <t>$PANW   And after the Earnings Call- take your profits to $ZS   ZSCALER- pulled back too far on its weak guidance but revenue and EPS beats…..  Nice way to get another 10% on your Palo gains.😉</t>
+        </is>
+      </c>
+      <c r="D813" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B814" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C814" s="2" t="inlineStr">
+        <is>
+          <t>$PANW i wouldnt rule out 500 eoy</t>
+        </is>
+      </c>
+      <c r="D814" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B815" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C815" s="3" t="inlineStr">
+        <is>
+          <t>$PANW I bought at the top 😬😬😬😬😬😬😬</t>
+        </is>
+      </c>
+      <c r="D815" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B816" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C816" s="3" t="inlineStr">
+        <is>
+          <t>$PANW reported  Billings for Q3. http://www.estimize.com/intro/panw?chart=historical&amp;amp;metric_name=billings&amp;amp;utm_content=PANW&amp;amp;utm_medium=metri</t>
+        </is>
+      </c>
+      <c r="D816" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B817" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C817" s="2" t="inlineStr">
+        <is>
+          <t>$PANW BUY, reach 350 soon and 400 in an year $PANW then will be in steady phase, 2 years target 500. Cybersecurity is MUST.</t>
+        </is>
+      </c>
+      <c r="D817" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B818" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C818" s="3" t="inlineStr">
+        <is>
+          <t>$PANW released fiscal Q3 2026 results with $3.0 billion revenue, up 31% YoY, and 60% ARR growth. https://www.rapidticker.com/news/panw-palo-alto-networks-reports-fiscal-a97278</t>
+        </is>
+      </c>
+      <c r="D818" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B819" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C819" s="3" t="inlineStr">
+        <is>
+          <t>$PANW $2 billion quarterly revenue and market cap heading to $300 Billion    Very Very cheap, load up !!!</t>
+        </is>
+      </c>
+      <c r="D819" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B820" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C820" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR patience bears. This is way high VS BTC PA. MSTR sitting IMO about 5% high. Seems something is either brewing behind the curtain.. this should take a 💩 soon if BTC can&amp;#39;t make a big push back into the 72.5k range(based on MSTR at 152-ish).</t>
+        </is>
+      </c>
+      <c r="D820" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B821" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C821" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X what happens when $MSTR and $BLK starts selling even more, no bids</t>
+        </is>
+      </c>
+      <c r="D821" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B822" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C822" s="2" t="inlineStr">
+        <is>
+          <t>$ASST  well reddit is calling $MSTR a ponzi again must be market bottom 😂🍻</t>
+        </is>
+      </c>
+      <c r="D822" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B823" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C823" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR sold 32 BTC had to be a joke</t>
+        </is>
+      </c>
+      <c r="D823" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B824" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C824" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR no i bought my puts at 148</t>
+        </is>
+      </c>
+      <c r="D824" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B825" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C825" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR small 150strike put position for this week started at 152.</t>
+        </is>
+      </c>
+      <c r="D825" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B826" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C826" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR triple down on puts</t>
+        </is>
+      </c>
+      <c r="D826" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B827" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C827" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR surprised this isn’t down 50% today</t>
+        </is>
+      </c>
+      <c r="D827" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B828" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C828" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR if a company who said they would never sell btc is selling btc, why are you still holding it 😂</t>
+        </is>
+      </c>
+      <c r="D828" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B829" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C829" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR Wow, Iran is literally castrating Trump.</t>
+        </is>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B830" s="2" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C830" s="2" t="inlineStr">
+        <is>
+          <t>$ETH.X looking like bottom boys</t>
+        </is>
+      </c>
+      <c r="D830" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B831" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C831" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X bad for the mental health for sure</t>
+        </is>
+      </c>
+      <c r="D831" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B832" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C832" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR $ETH.X $BMNR $SOL.X  If you are still hodling this dogsh*t this should come in handy:</t>
+        </is>
+      </c>
+      <c r="D832" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B833" s="2" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C833" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X $DJT $ETH.X $PEPE.X</t>
+        </is>
+      </c>
+      <c r="D833" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B834" s="2" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C834" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X $ETH.X $DJT $PEPE.X   I trigger dummies. 😆🫡🇺🇸</t>
+        </is>
+      </c>
+      <c r="D834" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B835" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C835" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR $ETH.X $SOL.X $ASST The crypto trading desk:</t>
+        </is>
+      </c>
+      <c r="D835" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B836" s="4" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C836" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X $SOL.X $ETH.X $XRP.X   Easy money being made shorting this 🙌🤑</t>
+        </is>
+      </c>
+      <c r="D836" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B837" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C837" s="3" t="inlineStr">
+        <is>
+          <t>Dumb retail will sell $GOOG $GOOGL And chase  300+ PE chips.  Smart money will be on the side of $BRK.B AND BUY IT ALL THE WAY PAST 400.</t>
+        </is>
+      </c>
+      <c r="D837" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B838" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C838" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL   Expecting Quantom Computing news relatively soon out of Google.   Thinking this could be part of the funding rounds.</t>
+        </is>
+      </c>
+      <c r="D838" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B839" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C839" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL imagine being on a stock app and not knowing this is the fastest growing cloud company on earth. 60% growth last q. #1 search. Top LLM. #1 streamer. #1 quantum. #1 robotaxi. #1 TPU chip. And backed by the greatest investor of all time $BRK.B</t>
+        </is>
+      </c>
+      <c r="D839" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B840" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C840" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL dump this and let’s buy below Berkshire’s price</t>
+        </is>
+      </c>
+      <c r="D840" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B841" s="2" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C841" s="2" t="inlineStr">
+        <is>
+          <t>$GOOGL $GOOG Has always been about long term growth.  More compute equals more money.  Everntually, everyone will be using AI for everything.  Gotta trust the process.  I’d rather invest in Google than a GM that can’t ever make big bets bc they have to please the current sharehol</t>
+        </is>
+      </c>
+      <c r="D841" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B842" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C842" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT classic msft.,, dumps on someone else’s news but never ever goes up with them, $GOOGL makes an offering and msft tanks…lmao…literally gave back 4% of gains in one trading day</t>
+        </is>
+      </c>
+      <c r="D842" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B843" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C843" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL the whole market will be in deep red tomorrow mark my words</t>
+        </is>
+      </c>
+      <c r="D843" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B844" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C844" s="4" t="inlineStr">
+        <is>
+          <t>$NVDA  revenue drop probability starting to bubble. $GOOGL</t>
+        </is>
+      </c>
+      <c r="D844" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B845" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C845" s="4" t="inlineStr">
+        <is>
+          <t>$NVDA $GOOGL doing the market dirty.</t>
+        </is>
+      </c>
+      <c r="D845" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B846" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C846" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL why is this down AH?</t>
+        </is>
+      </c>
+      <c r="D846" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B847" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C847" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D847" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B848" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C848" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL I wish I bought more lol.</t>
+        </is>
+      </c>
+      <c r="D848" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B849" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C849" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL $7.X before a deal is announced? Imagine when a deal is announced, not 1, not 2 but 3 deals!</t>
+        </is>
+      </c>
+      <c r="D849" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B850" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C850" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D850" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B851" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C851" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL what color lambo</t>
+        </is>
+      </c>
+      <c r="D851" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B852" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C852" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL yey im no longer a bag holder and in the profits another 5 month hold for long term tax deduction 10k strong 💪🏼</t>
+        </is>
+      </c>
+      <c r="D852" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B853" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C853" s="2" t="inlineStr">
+        <is>
+          <t>$APLD $KEEL $HIVE $AGPU</t>
+        </is>
+      </c>
+      <c r="D853" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B854" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C854" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D854" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B855" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C855" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL LFG 🚀</t>
+        </is>
+      </c>
+      <c r="D855" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B856" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C856" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL Remember everyone, anything can happen , don’t get attached and move accordingly   Remember what your goal was</t>
+        </is>
+      </c>
+      <c r="D856" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B857" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C857" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB bears finding a reason to hate on something because no one likes them lol</t>
+        </is>
+      </c>
+      <c r="D857" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B858" s="3" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C858" s="3" t="inlineStr">
+        <is>
+          <t>$GTLB   Solid great ER.  It should go HIGHER..35&amp;#39; or higher tomorrow and beyond.</t>
+        </is>
+      </c>
+      <c r="D858" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B859" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C859" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB then sell lol</t>
+        </is>
+      </c>
+      <c r="D859" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B860" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C860" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB Already bagholding 🥹</t>
+        </is>
+      </c>
+      <c r="D860" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B861" s="4" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C861" s="4" t="inlineStr">
+        <is>
+          <t>$GTLB   Wait for CC to start then this will dive .</t>
+        </is>
+      </c>
+      <c r="D861" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B862" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C862" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS this chart is long out by year count, but doesn&amp;#39;t this look ridiculous? The $SOXX index is probably worth much more than the spx500 if you take the semi companies out of the spx500. Sure $SOXL can go higher and $SOXS lower, but the law of large numbers should mute these</t>
+        </is>
+      </c>
+      <c r="D862" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B863" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C863" s="3" t="inlineStr">
+        <is>
+          <t>$SPY from this point on, I will be updating the $SOXX -&amp;gt; $SOXL $SOXS conversion chart each time we hit a new high.  Now SOXX is up nearly 100% in 2 months, making any specific time semis rallied in the dot com boom look like child&amp;#39;s play.  Even most of the Mag7 sold off; $</t>
+        </is>
+      </c>
+      <c r="D863" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -17845,12 +19518,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
@@ -17874,85 +19547,85 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>45</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>38</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
@@ -18061,46 +19734,46 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -18112,143 +19785,143 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:34 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -18258,14 +19931,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -18275,14 +19948,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -18292,14 +19965,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -18309,14 +19982,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -18326,14 +19999,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -18343,14 +20016,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -18360,14 +20033,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -18377,14 +20050,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -18394,14 +20067,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -18411,14 +20084,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -18428,26 +20101,236 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-02 20:29 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-06-01 22:07 UTC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SYMBOL</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PRICE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CHANGE_PCT</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>VOLUME</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>REL_VOLUME</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MARKET_CAP</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>SECTOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>SOXX</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2026-06-02 20:29 UTC</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-02 20:40 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D863"/>
+  <dimension ref="A1:D935"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -19435,6 +19435,1590 @@
         </is>
       </c>
       <c r="D863" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B864" s="2" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C864" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X   bears i the last 30 days doing to us</t>
+        </is>
+      </c>
+      <c r="D864" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B865" s="4" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C865" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X HURTS TO SEE SHIP IS SINKING AND BACKING TO 40K AND OUR MONEY SLOWLY BURNING</t>
+        </is>
+      </c>
+      <c r="D865" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B866" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C866" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X at least we can have fun with GIFs. LOL!</t>
+        </is>
+      </c>
+      <c r="D866" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B867" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C867" s="3" t="inlineStr">
+        <is>
+          <t>$SPY payday drinks $BTC.X</t>
+        </is>
+      </c>
+      <c r="D867" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B868" s="2" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C868" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY actually green even with $BTC.X falling like a rock</t>
+        </is>
+      </c>
+      <c r="D868" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B869" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C869" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X Saylor is a fucking scam artist, but he&amp;#39;s not the reason for this drop. The peace &amp;quot;deal&amp;quot; that pumped this garbage by 2k in minutes just expired, it would&amp;#39;ve been at or below this level days ago if not for Trump and Axios bullshitting lol</t>
+        </is>
+      </c>
+      <c r="D869" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B870" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C870" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X   62K next hopium support.</t>
+        </is>
+      </c>
+      <c r="D870" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B871" s="2" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C871" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X $ETH.X $MSTR If Saylor put the bottom in to add to the max FUD campaign thats been going on by selling a meager 32 bitcoin that would honestly be a hilarious bear trap.</t>
+        </is>
+      </c>
+      <c r="D871" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B872" s="2" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C872" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X Looking at the technicals on a 200MA the support should be somewhere around 68k based on the Oct. 7th, May 15th peaks and Feb. 5th trough. If 68k doesn&amp;#39;t hold we maybe in for a ride lower back down to test the 60k floor</t>
+        </is>
+      </c>
+      <c r="D872" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B873" s="3" t="inlineStr">
+        <is>
+          <t>BTC.X</t>
+        </is>
+      </c>
+      <c r="C873" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X</t>
+        </is>
+      </c>
+      <c r="D873" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B874" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C874" s="2" t="inlineStr">
+        <is>
+          <t>$BB too many damn posts to read them all, i gave up. Glad to have been duying this from 6.50 in one fund, closed one position with a incompetent ceo to max out here. Making money back already. QNX is the future!</t>
+        </is>
+      </c>
+      <c r="D874" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B875" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C875" s="2" t="inlineStr">
+        <is>
+          <t>$BB Winner Winner Chicken Dinner</t>
+        </is>
+      </c>
+      <c r="D875" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B876" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C876" s="2" t="inlineStr">
+        <is>
+          <t>$BB when 100% of your account is in BB It feels nice fellas.</t>
+        </is>
+      </c>
+      <c r="D876" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B877" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C877" s="3" t="inlineStr">
+        <is>
+          <t>$BB could it touch 50 EOY</t>
+        </is>
+      </c>
+      <c r="D877" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B878" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C878" s="3" t="inlineStr">
+        <is>
+          <t>$BB a good old fashioned HODL!</t>
+        </is>
+      </c>
+      <c r="D878" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B879" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C879" s="3" t="inlineStr">
+        <is>
+          <t>$BB bizmac you good?</t>
+        </is>
+      </c>
+      <c r="D879" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B880" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C880" s="3" t="inlineStr">
+        <is>
+          <t>$BB $NOK</t>
+        </is>
+      </c>
+      <c r="D880" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B881" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C881" s="3" t="inlineStr">
+        <is>
+          <t>$BB I would love to know what the big guys know this is incredible for not really any major news directly from bb</t>
+        </is>
+      </c>
+      <c r="D881" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B882" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C882" s="2" t="inlineStr">
+        <is>
+          <t>$BB Shorts feeling the heat!</t>
+        </is>
+      </c>
+      <c r="D882" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B883" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C883" s="2" t="inlineStr">
+        <is>
+          <t>$BB  Let‘s get ready for new highs!</t>
+        </is>
+      </c>
+      <c r="D883" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B884" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C884" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ Catching up to IONQ. We will get there. This is the leader.</t>
+        </is>
+      </c>
+      <c r="D884" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B885" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C885" s="2" t="inlineStr">
+        <is>
+          <t>$INFQ +130%, nice</t>
+        </is>
+      </c>
+      <c r="D885" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B886" s="2" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C886" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$INFQ Still half the valuation of Rigetti and 1/6 the valuation of IONQ.  Will be 1/3 the valuation of Quantunuum.  I expect it will eventually eclipse all.  Best value even after our big run.  Sells are drying up.  Shorts are shitting their pants.  The longer you wait, the more </t>
+        </is>
+      </c>
+      <c r="D886" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B887" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C887" s="2" t="inlineStr">
+        <is>
+          <t>$PANW alright, I never post anything like this, but after a decade of trading stock I put $1K into a Robinhood account solely to play around with options. To say it has gone well would be an understatement. Closed everything but $10K worth of lottery plays that I was willing to l</t>
+        </is>
+      </c>
+      <c r="D887" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B888" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C888" s="3" t="inlineStr">
+        <is>
+          <t>$PANW $CRWD Sooooo AI isn&amp;#39;t killing software?</t>
+        </is>
+      </c>
+      <c r="D888" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B889" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C889" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Up from 200 just 20 days ago.  Insiders drove it up, now they cash out.  Game is rigged, someone always knows.  The move had already been made.  baked in.</t>
+        </is>
+      </c>
+      <c r="D889" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B890" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C890" s="3" t="inlineStr">
+        <is>
+          <t>$PANW is this what everyone in vongress bought?</t>
+        </is>
+      </c>
+      <c r="D890" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B891" s="4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C891" s="4" t="inlineStr">
+        <is>
+          <t>$PANW beautiful short at $337</t>
+        </is>
+      </c>
+      <c r="D891" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B892" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C892" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Nothing burger move just like MDB to kill the options. Then will make the move the day after.</t>
+        </is>
+      </c>
+      <c r="D892" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B893" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C893" s="2" t="inlineStr">
+        <is>
+          <t>$PANW Almost sad I trimmed about 20% of my position lol    Completely assinine idea a few months ago that AI was going to negate the use for these companies instead of increasing the need for them.    Like long hold.</t>
+        </is>
+      </c>
+      <c r="D893" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B894" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C894" s="3" t="inlineStr">
+        <is>
+          <t>$PANW  No no no, AI is pulling back.  Just tell them the truth</t>
+        </is>
+      </c>
+      <c r="D894" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B895" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C895" s="3" t="inlineStr">
+        <is>
+          <t>$PANW crushed it</t>
+        </is>
+      </c>
+      <c r="D895" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B896" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C896" s="3" t="inlineStr">
+        <is>
+          <t>$PANW whyyyy i get outtttttt fcckkkkk</t>
+        </is>
+      </c>
+      <c r="D896" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B897" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C897" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR UPGRADES COMING IN HOT!!!!!!!!   BUY BUY BUY!!!!!!!!!!!!!!</t>
+        </is>
+      </c>
+      <c r="D897" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B898" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C898" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR 99</t>
+        </is>
+      </c>
+      <c r="D898" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B899" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C899" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR stocktwits post on x.</t>
+        </is>
+      </c>
+      <c r="D899" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B900" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C900" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR buy high sell low. $BTC.X 30k soon</t>
+        </is>
+      </c>
+      <c r="D900" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B901" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C901" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR HAHAHAHAHA RUBBISH FROM THE VILLAGE IDIOT  BACK INTO YOUR CAVE TROLL</t>
+        </is>
+      </c>
+      <c r="D901" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B902" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C902" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR $COIN doing incredible compare to Coinbase. Can’t wait to buy more if we get another 4-5% dip anytime this week</t>
+        </is>
+      </c>
+      <c r="D902" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B903" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C903" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR holding on</t>
+        </is>
+      </c>
+      <c r="D903" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B904" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C904" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR WOWZA SHORTY TAKIN IT UP THE A!!!!!! HAHAHAHAHAH @MisterTim2020 @TopWaterSniper</t>
+        </is>
+      </c>
+      <c r="D904" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B905" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C905" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X guys the stock market just made its 45th new all time high of the past few months this morning. U are bagholding something with ZERO upcoming catalysts and MANY looming doom catalysts. your biggest pumper is signaling that he is going to sell the hell out of this in perpet</t>
+        </is>
+      </c>
+      <c r="D905" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B906" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C906" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X Saylor should be the new ceo of bricks and minifigs   He has stolen from old people even more than their current ceo $MSTR</t>
+        </is>
+      </c>
+      <c r="D906" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B907" s="4" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C907" s="4" t="inlineStr">
+        <is>
+          <t>dinner service got ugly: btc lost $70K and finished near $67.2K.    $70,669 is the repair ticket now. overnight watch is funding. $BTC.X $ETH.X $SOL.X</t>
+        </is>
+      </c>
+      <c r="D907" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B908" s="3" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C908" s="3" t="inlineStr">
+        <is>
+          <t>$ETH.X cool I bought 2 yesterday my timing sucks</t>
+        </is>
+      </c>
+      <c r="D908" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B909" s="2" t="inlineStr">
+        <is>
+          <t>ETH.X</t>
+        </is>
+      </c>
+      <c r="C909" s="2" t="inlineStr">
+        <is>
+          <t>$PEPE.X I added more.   $ETH.X $BTC.X $DJT</t>
+        </is>
+      </c>
+      <c r="D909" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B910" s="2" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C910" s="2" t="inlineStr">
+        <is>
+          <t>$GOOGL Berkshire putting the floor at 350 on google now. More money means there going to dominate this AI/Quantum race even harder .</t>
+        </is>
+      </c>
+      <c r="D910" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B911" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C911" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL Abel seems to think Google will be the long term AI winner. Is he right? That’s not how it’s worked in the past.</t>
+        </is>
+      </c>
+      <c r="D911" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B912" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C912" s="4" t="inlineStr">
+        <is>
+          <t>$SPY $META $GOOGL $MSFT $AMZN Market top. Piggies will be cooked.</t>
+        </is>
+      </c>
+      <c r="D912" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B913" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C913" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL and $BRK.B = 🤝 . Bullish or bearish in your opinion?</t>
+        </is>
+      </c>
+      <c r="D913" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B914" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C914" s="3" t="inlineStr">
+        <is>
+          <t>$SPY $GOOGL $GOOG $BRK.B OK so who pulled the okey-doke on poor Abel? This definitely isn’t the logic of Warren. $10 billion worth of discounted shares at $351.91? Not much of a deal there￼￼</t>
+        </is>
+      </c>
+      <c r="D914" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B915" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C915" s="3" t="inlineStr">
+        <is>
+          <t>$POET JUST IN: GOOGLE $GOOGL JUST ANNOUNCED AN $80 BILLION CAPITAL RAISE TO BUILD AI INFRASTRUCTURE  https://x.com/i/status/2061550400046809587</t>
+        </is>
+      </c>
+      <c r="D915" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B916" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C916" s="3" t="inlineStr">
+        <is>
+          <t>$BRK.A gives $10B check to $GOOGL   $GOOG $BRK.B</t>
+        </is>
+      </c>
+      <c r="D916" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B917" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C917" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL private placement...are they restricted shares they can&amp;#39;t sell?</t>
+        </is>
+      </c>
+      <c r="D917" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B918" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C918" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT on time $AAPL $TSLA $META $GOOGL</t>
+        </is>
+      </c>
+      <c r="D918" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B919" s="2" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C919" s="2" t="inlineStr">
+        <is>
+          <t>$GOOGL Actually bullish news. Berkshire doesn&amp;#39;t flip shares, they invest for long term value.    There&amp;#39;s only one reason Google does this: they need this much cash immediately to fulfill strategic business objectives.    Yes it might dip to 350 but thats not guaranteed no</t>
+        </is>
+      </c>
+      <c r="D919" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B920" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C920" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D920" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B921" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C921" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D921" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B922" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C922" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL Can I get a....fckn yeah baby!</t>
+        </is>
+      </c>
+      <c r="D922" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B923" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C923" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D923" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B924" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C924" s="2" t="inlineStr">
+        <is>
+          <t>$VIVO is the next $KEEL $APLD $NBIS except it’s got a 2.3M float and 3.6M shares short… 153% SI/FF - announcing the finalization of their tier 1 tenant by June 30th. Expecting a parabolic move</t>
+        </is>
+      </c>
+      <c r="D924" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B925" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C925" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL no need to panic if you’re holding KEEL. Nothing can stop that green candle 🤑🤑🤑</t>
+        </is>
+      </c>
+      <c r="D925" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B926" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C926" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL $CLSK $BB the only three leaps I’m holding until January 2027 expiry ima be rich</t>
+        </is>
+      </c>
+      <c r="D926" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B927" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C927" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL higher!!!!</t>
+        </is>
+      </c>
+      <c r="D927" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B928" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C928" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL when do we think infrastructure deal is coming</t>
+        </is>
+      </c>
+      <c r="D928" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B929" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C929" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL on tsx most active list</t>
+        </is>
+      </c>
+      <c r="D929" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B930" s="3" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C930" s="3" t="inlineStr">
+        <is>
+          <t>$GTLB +6.44% AH off the 31.82 close, sitting up at 33.87. these vertical AH moves can fade fast and this one&amp;#39;s already up 53% on the month so it&amp;#39;s stretched. waiting for a base before I trust it. who else is watching the reopen?</t>
+        </is>
+      </c>
+      <c r="D930" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B931" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C931" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB lets see how high we can get 🔥</t>
+        </is>
+      </c>
+      <c r="D931" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B932" s="2" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C932" s="2" t="inlineStr">
+        <is>
+          <t>$GTLB need to go over $35 to run</t>
+        </is>
+      </c>
+      <c r="D932" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B933" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C933" s="3" t="inlineStr">
+        <is>
+          <t>$SOXX blah blah blah, we rip!!!   This ain&amp;#39;t 1999 bro, semis are the FUTURE!!!</t>
+        </is>
+      </c>
+      <c r="D933" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B934" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C934" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS $SOXX $SOXL $SPY $QQQ     The retail FOMO crowd is not nervous at all right now about the historic 78% over-extension of the Semiconductor index from the 200 day moving average; they are experiencing absolute dopamine euphoria.     Because the momentum has been so fast sinc</t>
+        </is>
+      </c>
+      <c r="D934" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B935" s="3" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C935" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS its not a matter of IF $SOXX will fall back to earth but WHEN? That is the question of all questions</t>
+        </is>
+      </c>
+      <c r="D935" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -19479,41 +21063,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19523,92 +21107,92 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-01 21:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>55</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
@@ -19632,63 +21216,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -19700,41 +21284,41 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -19744,14 +21328,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -19761,82 +21345,82 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -19853,7 +21437,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -19863,24 +21447,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
@@ -19892,12 +21476,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
@@ -19909,12 +21493,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
@@ -20133,7 +21717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20332,6 +21916,306 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>10.32</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>6.17%</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>49,397,951</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>6.05B</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>19.87</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>12.32%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>31,290,757</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2.89</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>4.34B</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>297.18</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>-1.10%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>17,896,065</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>242.50B</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>136.08</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-9.15%</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>30,534,080</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>47.69B</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>361.85</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-3.86%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>47,633,403</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4364.33B</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>6.14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>45,869,486</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3.71B</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>31.82</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>-5.83%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>23,326,197</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3.65</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>5.37B</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-02 20:40 UTC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>605.02</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>5.79%</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>7,319,401</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 00:31 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D935"/>
+  <dimension ref="A1:D1035"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -21019,6 +21019,2206 @@
         </is>
       </c>
       <c r="D935" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B936" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C936" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL I mean…. Like I said, NOBODY is better than me🥳  Link in bio to join the BEST discord ever✔️</t>
+        </is>
+      </c>
+      <c r="D936" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B937" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C937" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL i have a feeling they keeping this up so hedge funds can close their 320 calls</t>
+        </is>
+      </c>
+      <c r="D937" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B938" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C938" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL pinned below $320</t>
+        </is>
+      </c>
+      <c r="D938" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B939" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C939" s="3" t="inlineStr">
+        <is>
+          <t>$TE If you liked the price action on the common stock, you would have really liked the Warrants today.  They were in a neck and neck battle with my $MRVL stock to see which would win the 50% gain race today.</t>
+        </is>
+      </c>
+      <c r="D939" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B940" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C940" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL Seriously you have to be some kind of imbecile to short this. This isn&amp;#39;t some f&amp;#39;ng Bio..company that got approval for a fart drug.</t>
+        </is>
+      </c>
+      <c r="D940" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B941" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C941" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL  lol</t>
+        </is>
+      </c>
+      <c r="D941" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B942" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C942" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL when 1k? Lol</t>
+        </is>
+      </c>
+      <c r="D942" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B943" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C943" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL oh the shorts are getting slaughtered. Fuck em</t>
+        </is>
+      </c>
+      <c r="D943" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B944" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C944" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL shorts</t>
+        </is>
+      </c>
+      <c r="D944" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B945" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C945" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL Sleep well shorts ....</t>
+        </is>
+      </c>
+      <c r="D945" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B946" s="4" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C946" s="4" t="inlineStr">
+        <is>
+          <t>$IBIT bitcoin is not oversold on the longer-term:  daily weekly monthly pay attention to those and do not get caught up on the shoulder term time frames.  $QQQ $NVDA $SPY $MU</t>
+        </is>
+      </c>
+      <c r="D946" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B947" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C947" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ Stay strong my brothers. Don&amp;#39;t let them scare you on closing your short position especially if your put option is until Dec 2026.  You will gain it back during the summer. Will definitely go below 700.</t>
+        </is>
+      </c>
+      <c r="D947" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B948" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C948" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ it&amp;#39;s a liquidity grab for the bears - AGAIN!!! We got another 10% up minimum just watch</t>
+        </is>
+      </c>
+      <c r="D948" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B949" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C949" s="3" t="inlineStr">
+        <is>
+          <t>$DIA $QQQ $SPY glad you are bullish now</t>
+        </is>
+      </c>
+      <c r="D949" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B950" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C950" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ hats off to the marketmakers for manipulating this so easily</t>
+        </is>
+      </c>
+      <c r="D950" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B951" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C951" s="3" t="inlineStr">
+        <is>
+          <t>they&amp;#39;re not able to refund that cash, that cash being reinvested in the market currently and thats exactly whats holding certain stocks up 🚬  $SPY $QQQ $BTC.X $USO</t>
+        </is>
+      </c>
+      <c r="D951" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B952" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C952" s="3" t="inlineStr">
+        <is>
+          <t>$DIA $QQQ $SPY Don’t overthink it.  Buy puts when the market opens. Big boys want a clean exit at the top.</t>
+        </is>
+      </c>
+      <c r="D952" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B953" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C953" s="3" t="inlineStr">
+        <is>
+          <t>$SPY $QQQ cant wait for another peace deal tomorrow!</t>
+        </is>
+      </c>
+      <c r="D953" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B954" s="4" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C954" s="4" t="inlineStr">
+        <is>
+          <t>$QQQ $DIA $SPY REPORTS OF US ATTACKING IRAN LIKE AN HOUR AGO, MARKET THAT IS UP 40% ALREADY DOESNT REACT. WHAT THE FUCK IS THIS MARKET.</t>
+        </is>
+      </c>
+      <c r="D954" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B955" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C955" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ $SPY he did go full force in Lebanon already</t>
+        </is>
+      </c>
+      <c r="D955" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B956" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C956" s="3" t="inlineStr">
+        <is>
+          <t>$SPY crude is up 8% markets flat. lol I remember a time when we&amp;#39;d be down 1-2%. Wild strength.</t>
+        </is>
+      </c>
+      <c r="D956" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B957" s="2" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C957" s="2" t="inlineStr">
+        <is>
+          <t>$SPY ok so…. Lets go? Took calls</t>
+        </is>
+      </c>
+      <c r="D957" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B958" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C958" s="3" t="inlineStr">
+        <is>
+          <t>$SPY oil going berserk and this keeps getting saved. I&amp;#39;m sick of c🔯ncer so so so much</t>
+        </is>
+      </c>
+      <c r="D958" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B959" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C959" s="3" t="inlineStr">
+        <is>
+          <t>$SPY crazy bears bragging about a buck 🤔😂ain’t nobody making money today looks like a boring day 😴😂</t>
+        </is>
+      </c>
+      <c r="D959" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B960" s="4" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C960" s="4" t="inlineStr">
+        <is>
+          <t>$SPY major indices doesn’t move on two key straits being closed… waiting for the fat pedo retard to compose a fake tweet</t>
+        </is>
+      </c>
+      <c r="D960" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B961" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C961" s="3" t="inlineStr">
+        <is>
+          <t>$SPY https://x.com/HalfwayPost/status/2061297843948912839?s=20</t>
+        </is>
+      </c>
+      <c r="D961" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B962" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C962" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ $SPY $XBI $IBB.   Paradigm shift for cancer treatment moving along nicely</t>
+        </is>
+      </c>
+      <c r="D962" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B963" s="2" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C963" s="2" t="inlineStr">
+        <is>
+          <t>$SPY green eod?</t>
+        </is>
+      </c>
+      <c r="D963" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B964" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C964" s="3" t="inlineStr">
+        <is>
+          <t>$INOD $QQQ $SPY the market isn’t ignoring it, the government is just injecting trillions to offset any selling.</t>
+        </is>
+      </c>
+      <c r="D964" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B965" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C965" s="3" t="inlineStr">
+        <is>
+          <t>$SPY seen this before I’m not missing out on this bs</t>
+        </is>
+      </c>
+      <c r="D965" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B966" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C966" s="2" t="inlineStr">
+        <is>
+          <t>$CLSK 💎🤲  $MSTR $SPY $XXI $BTC.X</t>
+        </is>
+      </c>
+      <c r="D966" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B967" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C967" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR guys what&amp;#39;s your bull thesis now?</t>
+        </is>
+      </c>
+      <c r="D967" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B968" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C968" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR $BTC.X wen $IBM is mooning that is working on quantum compute then Houston we got a problem.</t>
+        </is>
+      </c>
+      <c r="D968" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B969" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C969" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR $STRD $STRC $BTC.X</t>
+        </is>
+      </c>
+      <c r="D969" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B970" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C970" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR just that squeaky voice pervert conditioning his sheeple.</t>
+        </is>
+      </c>
+      <c r="D970" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B971" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C971" s="3" t="inlineStr">
+        <is>
+          <t>$10K invested one year ago across high beta defense, AI, and nuclear names would’ve produced very mixed outcomes depending on positioning and timing    $BBAI → $13,600 steady defense AI grind higher with volatility  $OKLO → $13,100 early nuclear narrative still highly speculative</t>
+        </is>
+      </c>
+      <c r="D971" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B972" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C972" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR 🚀🚀🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D972" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B973" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C973" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR  https://www.cnbc.com/2026/06/01/strategy-shares-fall-after-selling-2point5-million-in-bitcoin-its-first-sale-since-2022.html</t>
+        </is>
+      </c>
+      <c r="D973" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B974" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C974" s="3" t="inlineStr">
+        <is>
+          <t>$STRC in last two weeks, $BTC.X down 15%. $MSTR down 20% and STRC down 0.25%. This is what Saylor said would happen during Bitcoin down trends.   If you want leveraged Bitcoin and love rollercoasters buy MSTR. A bit less risk/reward, buy BTC. Considerably less risk, buy STRC. Str</t>
+        </is>
+      </c>
+      <c r="D974" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B975" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C975" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR $BTC.X sells 2.5M??? Something doesnt feel right about this. This is a nasdaq listed company were talking. Thats a retail amount.</t>
+        </is>
+      </c>
+      <c r="D975" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B976" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C976" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Over  priced even before this move.   The news is mediocre and they already added 1/3 of market cap in value in last 20 days.  Insiders win!</t>
+        </is>
+      </c>
+      <c r="D976" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B977" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C977" s="3" t="inlineStr">
+        <is>
+          <t>$PANW now 316</t>
+        </is>
+      </c>
+      <c r="D977" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B978" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C978" s="2" t="inlineStr">
+        <is>
+          <t>$PANW PANW reported excellent numbers and guidance BUT....still remains  extremely overvalued with  forward PE multiple of ......85x  full year guidance of $3.78      In comparison, Sentinel One (S) currently trades for only......50x forward EPS guidance of  $0.35       With a fe</t>
+        </is>
+      </c>
+      <c r="D978" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B979" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C979" s="3" t="inlineStr">
+        <is>
+          <t>$PANW $FRSH will go up</t>
+        </is>
+      </c>
+      <c r="D979" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B980" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C980" s="3" t="inlineStr">
+        <is>
+          <t>$S oh wow, $PANW beating expectations significantly doesn’t bode well for us that couldn’t even meet expectations.  $CRWD probably going to destroy their earnings.   The MMs always know I guess. Shocking this management team can’t sign an extra contract or two from someone who ca</t>
+        </is>
+      </c>
+      <c r="D980" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B981" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C981" s="3" t="inlineStr">
+        <is>
+          <t>$PANW hmm 339 high and now 321, interesting</t>
+        </is>
+      </c>
+      <c r="D981" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B982" s="4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C982" s="4" t="inlineStr">
+        <is>
+          <t>$PANW somehow feel that there is more downward pressure here…traders want to lock in profits and move on. Will not be surprised if it ends up red.</t>
+        </is>
+      </c>
+      <c r="D982" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B983" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C983" s="3" t="inlineStr">
+        <is>
+          <t>$PANW bag is getting heavy</t>
+        </is>
+      </c>
+      <c r="D983" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B984" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C984" s="3" t="inlineStr">
+        <is>
+          <t>$ULTA $PANW  similar no weeklies but 2, cubie teaches</t>
+        </is>
+      </c>
+      <c r="D984" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B985" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C985" s="3" t="inlineStr">
+        <is>
+          <t>$PANW - it will open red tomorrow..$FTNT</t>
+        </is>
+      </c>
+      <c r="D985" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B986" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C986" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO do we see 480 tomorrow?</t>
+        </is>
+      </c>
+      <c r="D986" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B987" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C987" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO H&amp;amp;S first  now bull flag forming</t>
+        </is>
+      </c>
+      <c r="D987" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B988" s="4" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C988" s="4" t="inlineStr">
+        <is>
+          <t>$AVGO Can not sustain the hype long!</t>
+        </is>
+      </c>
+      <c r="D988" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B989" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C989" s="3" t="inlineStr">
+        <is>
+          <t>AI watchlist for the next 1–5 years is less about hype names and more about infrastructure layers that actually scale compute    $AVGO core AI networking + custom silicon backbone of data center expansion  $ALAB emerging AI infrastructure hardware play, high beta but strong narra</t>
+        </is>
+      </c>
+      <c r="D989" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B990" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C990" s="3" t="inlineStr">
+        <is>
+          <t>Friday closed with a monster $6M in calls hitting $AVGO right at the bell.    Big block, right in the money. Someone clearly has intel .    Funny how it always shows up after the fact,market loves to whisper before it screams. Keep your eyes peeled; setups like this rarely go unn</t>
+        </is>
+      </c>
+      <c r="D990" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B991" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C991" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO if this hits $600+ by eow I will quit my job.</t>
+        </is>
+      </c>
+      <c r="D991" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B992" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C992" s="3" t="inlineStr">
+        <is>
+          <t>$SPY google money going into $HPE $AVGO $NOK $DELL .. all hardware companies. Next will be nvda ... Every dip on nvda is a buying opportunity IMO</t>
+        </is>
+      </c>
+      <c r="D992" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B993" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C993" s="2" t="inlineStr">
+        <is>
+          <t>$HPE $AVGO Wednesday is going to be wild likely $5-7 eps</t>
+        </is>
+      </c>
+      <c r="D993" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B994" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C994" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO 10 fold since I bought at $47 for my retirement account. Holding strong $1,000 next. Make it 20 fold!</t>
+        </is>
+      </c>
+      <c r="D994" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B995" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C995" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO Wednesday is gonna be nutty</t>
+        </is>
+      </c>
+      <c r="D995" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B996" s="3" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C996" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS afraid of widow maker.  Is there a 2x and 1x inverse soxx etf?</t>
+        </is>
+      </c>
+      <c r="D996" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B997" s="3" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C997" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS ok i&amp;#39;ll hit you up in 2500</t>
+        </is>
+      </c>
+      <c r="D997" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B998" s="3" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C998" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS when a large cap semiconductor company runs over 40% because someone said it could be the next trillion dollar company that is the exact definition of market overexuberance… Eventually a reckoning will happen, eventually the markets will have to pay attention to the interes</t>
+        </is>
+      </c>
+      <c r="D998" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B999" s="2" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C999" s="2" t="inlineStr">
+        <is>
+          <t>$SOXS Hopium and FOMO are finite! The world is on fire lol reality will set one day</t>
+        </is>
+      </c>
+      <c r="D999" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1000" s="2" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C1000" s="2" t="inlineStr">
+        <is>
+          <t>$SOXS Buying more and more!!</t>
+        </is>
+      </c>
+      <c r="D1000" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1001" s="3" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C1001" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS got in at 5 but ready for 4</t>
+        </is>
+      </c>
+      <c r="D1001" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1002" s="3" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C1002" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS why this trending so it can creat more bagholders 😁 Ill take a bit to hedge some here soon soon</t>
+        </is>
+      </c>
+      <c r="D1002" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1003" s="2" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C1003" s="2" t="inlineStr">
+        <is>
+          <t>$SOXS &amp;quot;Feeling&amp;quot; a big jump here in the making. Fumes are now driving markets that a word from this or that can add hundreds of billions to valuations instantly. That talent used to be Elon&amp;#39;s but now anyone can do it. Fucked* indeed.</t>
+        </is>
+      </c>
+      <c r="D1003" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1004" s="3" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C1004" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS sell off resume ?</t>
+        </is>
+      </c>
+      <c r="D1004" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1005" s="2" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C1005" s="2" t="inlineStr">
+        <is>
+          <t>$SOXS  I have figured it out!! It really is over. NVDA really is Sky Net and Jensen is the terminator.  AI has taken over and is buying everything AI related regardless of the value. We are doomed!!!</t>
+        </is>
+      </c>
+      <c r="D1005" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1006" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1006" s="2" t="inlineStr">
+        <is>
+          <t>$NOK $BB a golden opportunity to invest in my opinion</t>
+        </is>
+      </c>
+      <c r="D1006" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1007" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1007" s="2" t="inlineStr">
+        <is>
+          <t>$BB What a ride!!  Keep er cookin&amp;#39;!!</t>
+        </is>
+      </c>
+      <c r="D1007" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1008" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1008" s="2" t="inlineStr">
+        <is>
+          <t>$BB goddamn my call positions starting to look like the option chain 😂</t>
+        </is>
+      </c>
+      <c r="D1008" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1009" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1009" s="3" t="inlineStr">
+        <is>
+          <t>$BB “QNX, AI, Security...  QNX, AI, Security.. are you guys not getting it?!”      inspired by that black berry mufi..</t>
+        </is>
+      </c>
+      <c r="D1009" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1010" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1010" s="2" t="inlineStr">
+        <is>
+          <t>$BB $AMC $NOK $GME - BANG is back, but this time without $GME and $AMC so it seems 🤷‍♂️🚀🚀🚀🚀🚀💎💎💎💎💎</t>
+        </is>
+      </c>
+      <c r="D1010" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1011" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1011" s="3" t="inlineStr">
+        <is>
+          <t>$BB damn guess I was better off buying BB leaps than $NOK still up significantly but damn haha</t>
+        </is>
+      </c>
+      <c r="D1011" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1012" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1012" s="2" t="inlineStr">
+        <is>
+          <t>$BB up over 80% all time lil bro.</t>
+        </is>
+      </c>
+      <c r="D1012" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1013" s="4" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1013" s="4" t="inlineStr">
+        <is>
+          <t>@Bay2La2000 u should feel lucky that am opening ur eyes to reality mate instead of following dreams,,, imagine u bought $BB couple of weeks ago u would have made better profit that staying months waiting for this shitty stock :)</t>
+        </is>
+      </c>
+      <c r="D1013" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1014" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1014" s="3" t="inlineStr">
+        <is>
+          <t>@Itchytelivision from $BB holders to Cramer</t>
+        </is>
+      </c>
+      <c r="D1014" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1015" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1015" s="3" t="inlineStr">
+        <is>
+          <t>$BB Keep on trending BB, we love it!!!!! $20 this week.</t>
+        </is>
+      </c>
+      <c r="D1015" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1016" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1016" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT nice!  I  like  dips!  Load more!</t>
+        </is>
+      </c>
+      <c r="D1016" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1017" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1017" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Up a whopping $2 on the day. Nice AH DUMP.</t>
+        </is>
+      </c>
+      <c r="D1017" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1018" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1018" s="3" t="inlineStr">
+        <is>
+          <t>2026 Price Targets — Updated    $ZETA→ $32+    $OSCR → $30+    $NBIS→ $300+    $NOW→ $170+    $MSFT→ $520+    The largest gains are typically achieved by holding the right stocks longer than the market.</t>
+        </is>
+      </c>
+      <c r="D1018" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1019" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1019" s="3" t="inlineStr">
+        <is>
+          <t>⚖ 𝐓𝐡𝐞 𝐍𝐞𝐱𝐭 𝐂𝐡𝐚𝐩𝐭𝐞𝐫 𝐎𝐟 𝐐𝐮𝐚𝐧𝐭    🧭 The old model: $300-500K quant seat at a fund. Pay was good. Trade-off was your time, your IP, your direction.    📜 What&amp;#39;s changing:  ▪ AI compressing junior quant roles — tools that needed teams now need oversight  ▪ Modeling tasks that justi</t>
+        </is>
+      </c>
+      <c r="D1019" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1020" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1020" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT Bears are going to get trapped, and the market will shake out the weak hands before the next leg higher.</t>
+        </is>
+      </c>
+      <c r="D1020" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1021" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1021" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT $470 tomorrow</t>
+        </is>
+      </c>
+      <c r="D1021" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1022" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1022" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT $NVDA  Both are mid and long term winners. In this exercise, You can only choose one for this argument, we all know owning both to some degree the right move. Can only choose one: which has bigger upside move next 90 days?</t>
+        </is>
+      </c>
+      <c r="D1022" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1023" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1023" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT bring it back down to $435 so I can reload</t>
+        </is>
+      </c>
+      <c r="D1023" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1024" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1024" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT well confrence tomorrow!! See what happens .   How to watch the Microsoft Build 2026 keynote with Satya Nadella live - Tech https://share.google/787B8KKOAdE6UKX5x</t>
+        </is>
+      </c>
+      <c r="D1024" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1025" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1025" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT and it’s over</t>
+        </is>
+      </c>
+      <c r="D1025" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1026" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1026" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR I’m not greedy, 10% gain would be fine this this round 😊</t>
+        </is>
+      </c>
+      <c r="D1026" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1027" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1027" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR picked up 4000 cheap ones today</t>
+        </is>
+      </c>
+      <c r="D1027" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1028" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1028" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR it’s good old fashioned shakedown! Nobody can predict the outcome of this! Dang . be careful catching falling knife.</t>
+        </is>
+      </c>
+      <c r="D1028" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1029" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1029" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR All the opportunity cost within a decade. You could probably retire, but you were in crypto. Somehow this is bullish?</t>
+        </is>
+      </c>
+      <c r="D1029" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1030" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1030" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR MNAv increasing by the day.   The market trusts Tom to figure this out.</t>
+        </is>
+      </c>
+      <c r="D1030" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1031" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1031" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR 250k per ether 🤦🏻‍♂️</t>
+        </is>
+      </c>
+      <c r="D1031" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1032" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1032" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR $28 by the end of this month 👍</t>
+        </is>
+      </c>
+      <c r="D1032" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1033" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1033" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR alchemy within this month ?! That will be awesome !</t>
+        </is>
+      </c>
+      <c r="D1033" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1034" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1034" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR sorry guys. I thought $16 was the bottom. Looks like we might see much lower. Hold strong. Sell CCs. Do what you must!</t>
+        </is>
+      </c>
+      <c r="D1034" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1035" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1035" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR people pulling from crypto to chase these monster %10-%40 gains on multibillion dollar companies. All these pumps are insane. The market will correct soon and money will come bacj to crypto. Long term bullish but we may see much worse drop upcoming.</t>
+        </is>
+      </c>
+      <c r="D1035" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -21035,7 +23235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21114,29 +23314,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>58</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>55</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -21148,7 +23348,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -21158,24 +23358,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
@@ -21199,75 +23399,75 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -21277,19 +23477,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -21301,12 +23501,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -21318,24 +23518,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -21345,14 +23545,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -21362,19 +23562,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -21386,46 +23586,46 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -21437,29 +23637,29 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -21471,75 +23671,75 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -21556,7 +23756,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -21573,7 +23773,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -21590,7 +23790,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -21607,7 +23807,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -21617,14 +23817,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -21641,7 +23841,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -21658,7 +23858,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -21668,14 +23868,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -21692,7 +23892,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -21702,7 +23902,75 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
@@ -21717,14 +23985,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
@@ -22216,6 +24484,374 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>290.79</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>32.52%</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>103,396,690</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>3.78</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>254.38B</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>746.16</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.46%</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>29,290,504</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.56</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>759.57</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.14%</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>30,728,402</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.44</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>136.08</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>-9.15%</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>30,791,916</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>47.69B</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>297.18</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-1.10%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>18,592,763</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>242.50B</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>481.57</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>4.70%</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>37,297,822</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2280.07B</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SOXS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5.17</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>-17.41%</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>455,574,483</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2.74</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>10.32</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>6.17%</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>49,600,528</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>6.05B</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>441.31</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>-4.17%</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>36,634,724</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>3278.24B</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>17.97</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>-4.67%</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>46,757,785</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>10.24B</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 00:59 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1035"/>
+  <dimension ref="A1:D1098"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23219,6 +23219,1392 @@
         </is>
       </c>
       <c r="D1035" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1036" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1036" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL charging</t>
+        </is>
+      </c>
+      <c r="D1036" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1037" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1037" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL Will easily hit $350 overnight, get in while you still can</t>
+        </is>
+      </c>
+      <c r="D1037" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1038" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1038" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT  stupid loser that why told u dump 467!!    I got small call today ;  but dont like it all!!    $Googl $MU $MRVL call way better!     Remind me not touch msft next time till 400-410!</t>
+        </is>
+      </c>
+      <c r="D1038" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1039" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1039" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL bad news is now with this run there is only 80% upside for the year left here. Guess we barely outperform $qqQ .....</t>
+        </is>
+      </c>
+      <c r="D1039" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1040" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1040" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL wonder what happened to this trigger finger guy that said don&amp;#39;t buy 🚀🚀</t>
+        </is>
+      </c>
+      <c r="D1040" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1041" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1041" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL  there’s an unusual amount of support beneath this.</t>
+        </is>
+      </c>
+      <c r="D1041" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1042" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1042" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL Max pain for this week signal where it can get a magnet to and where it is near a fair valuation, guess where it is? More than 118$ below. That is a huge premium that bulls pay now</t>
+        </is>
+      </c>
+      <c r="D1042" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1043" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1043" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL will hit $350 overnight.</t>
+        </is>
+      </c>
+      <c r="D1043" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1044" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1044" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL if you short this, there is a reason why you are broke</t>
+        </is>
+      </c>
+      <c r="D1044" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1045" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1045" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL stressed for a year about this at 50 billion and in a few months it’s 200 billion.   investing is stupid   thank god</t>
+        </is>
+      </c>
+      <c r="D1045" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1046" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1046" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR</t>
+        </is>
+      </c>
+      <c r="D1046" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1047" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1047" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR $BMNR never forget these fraud pumpers</t>
+        </is>
+      </c>
+      <c r="D1047" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1048" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1048" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR $BTC.X I have literally made more money on this in one week than most will see in a lifetime. Not done yet. In and out as precise as I can but no one can time the market. This however has been fairly predictable.</t>
+        </is>
+      </c>
+      <c r="D1048" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1049" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1049" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR this is going to be an ugly week here if something doesn&amp;#39;t change fast for BTC.</t>
+        </is>
+      </c>
+      <c r="D1049" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1050" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1050" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR Yearn Finance https://yearn.fi Yearn Finance 33 billion market cap takes (YFI) OVER 1 MILLION DOLLARS. Yearn Finance (YFI) is a foundational DeFi yield aggregator. Often dubbed a &amp;quot;sleeping giant&amp;quot; due to its rarity—only 36,666 tokens exist—and its historical $95,00</t>
+        </is>
+      </c>
+      <c r="D1050" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1051" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1051" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR trimmed 50% at 149.60</t>
+        </is>
+      </c>
+      <c r="D1051" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1052" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1052" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR just look at $UVXY if you are wondering where this is headed to. lol</t>
+        </is>
+      </c>
+      <c r="D1052" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1053" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1053" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR bitcoin tanking and MSTR holding ground. Right shoulder for an inverse H/S pattern might be brewing</t>
+        </is>
+      </c>
+      <c r="D1053" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1054" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1054" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR</t>
+        </is>
+      </c>
+      <c r="D1054" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1055" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1055" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR Premium Heatmap &amp;amp; Key Strikes    Last: $150.81    Critical Resistance Levels:    $151.94 ($147.1M) | $157.16 ($133.3M) | $158.19 ($241.2M)    Decisive Support Points:    $146.44 ($120.9M)    For the most up-to-date market insights, visit our profile for additional ticke</t>
+        </is>
+      </c>
+      <c r="D1055" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1056" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1056" s="3" t="inlineStr">
+        <is>
+          <t>$PANW this gone fly i so sad that i sold before ER</t>
+        </is>
+      </c>
+      <c r="D1056" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1057" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1057" s="2" t="inlineStr">
+        <is>
+          <t>$PANW Bears are worried, some Bulls are worried. Just goes to show this was lotto for most people. The one who actually did their research before purchase are seating legs crossed and smiling to the bank. Can’t wait for the open to cash my first tranche of these checks!!! 🥂🤟🏾</t>
+        </is>
+      </c>
+      <c r="D1057" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1058" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1058" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Nancy never loses, sold half at 100%+ from Nancy’s buy area loll</t>
+        </is>
+      </c>
+      <c r="D1058" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1059" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1059" s="2" t="inlineStr">
+        <is>
+          <t>$PANW Sold half at 330. Now mm will be like Fuck your calls, fuck your puts.</t>
+        </is>
+      </c>
+      <c r="D1059" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1060" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1060" s="3" t="inlineStr">
+        <is>
+          <t>$PANW did they have their conference call yet? High of 339 and down to 319 already. Is it going to tank? lol</t>
+        </is>
+      </c>
+      <c r="D1060" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1061" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1061" s="3" t="inlineStr">
+        <is>
+          <t>$PANW why is it tanking?</t>
+        </is>
+      </c>
+      <c r="D1061" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1062" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1062" s="3" t="inlineStr">
+        <is>
+          <t>$PANW     Did they not say AI enough times?    Why is it dropping?</t>
+        </is>
+      </c>
+      <c r="D1062" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1063" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1063" s="3" t="inlineStr">
+        <is>
+          <t>@Jeremymartin007 @simon58 @judgeyoung2 @jenbunn @EBE_day @ribbey @TraderRapp @Godreal1 @tonyctl @zuby34  $panw and fml should&amp;#39;ve just shorted $CRWD 805-$809 😑</t>
+        </is>
+      </c>
+      <c r="D1063" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1064" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1064" s="2" t="inlineStr">
+        <is>
+          <t>$PANW   cybersecurity will be as critical a data center component as chips, memory, and servers.  holding my shares here.  though i see the nice AH spike selling off...  if $CRWD can hit $800 today, this should surely see $400 in due course.</t>
+        </is>
+      </c>
+      <c r="D1064" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1065" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1065" s="3" t="inlineStr">
+        <is>
+          <t>$PANW   Now we talking........    go flat buddy.</t>
+        </is>
+      </c>
+      <c r="D1065" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1066" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1066" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO 🤡  avgo is primed!</t>
+        </is>
+      </c>
+      <c r="D1066" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1067" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1067" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO boring !</t>
+        </is>
+      </c>
+      <c r="D1067" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1068" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1068" s="3" t="inlineStr">
+        <is>
+          <t>Even Google leaning into equity dilution to fund AI capex tells you how capital-intensive this phase of the cycle has become. An $80B war chest isn’t just expansion, it’s a full commitment to staying in the AI infrastructure arms race.    Near term, you can absolutely argue press</t>
+        </is>
+      </c>
+      <c r="D1068" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1069" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1069" s="2" t="inlineStr">
+        <is>
+          <t>$NVDA $227-230+ coming   $QQQ $SPY $AVGO $MU</t>
+        </is>
+      </c>
+      <c r="D1069" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1070" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1070" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO get in on $VEEV before earnings same time as avgo.</t>
+        </is>
+      </c>
+      <c r="D1070" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1071" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1071" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic Files S-1 Opening The IPO Floodgates, Analyst Says  $GOOGL $GOOG $AMZN $AVGO   https://www.benzinga.com/analyst-stock-ratings/analyst-color/26/06/52927424/anthropic-files-s-1-opening-the-ipo-floodgates-analyst-says</t>
+        </is>
+      </c>
+      <c r="D1071" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1072" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1072" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX $AVGO In fall for now!</t>
+        </is>
+      </c>
+      <c r="D1072" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1073" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1073" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO This isnt going to $500 over night is it?</t>
+        </is>
+      </c>
+      <c r="D1073" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1074" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1074" s="3" t="inlineStr">
+        <is>
+          <t>$GOOG $GOOGL MONEY GOING STRAIGHT INTO $AVGO‼️‼️  https://stocktwits.com/news-articles/markets/equity/alphabet-80b-fundraise-berkshire-hathaway-invests-10b-artificial-intelligence/cZ0WEfvRevi</t>
+        </is>
+      </c>
+      <c r="D1074" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1075" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1075" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO goog raising 80b from Berkshire for AI spend!  Avgo 550 incoming</t>
+        </is>
+      </c>
+      <c r="D1075" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1076" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1076" s="3" t="inlineStr">
+        <is>
+          <t>$BB I like the stock !</t>
+        </is>
+      </c>
+      <c r="D1076" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1077" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1077" s="3" t="inlineStr">
+        <is>
+          <t>$BB i ented at 9.50  and we are near already 11 ! God damn!</t>
+        </is>
+      </c>
+      <c r="D1077" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1078" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1078" s="2" t="inlineStr">
+        <is>
+          <t>$BB DO NOT YIELD. DO NOT RETREAT. NEVER STOP. ALWAYS ATTACK.   TO $100!!!!!!</t>
+        </is>
+      </c>
+      <c r="D1078" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1079" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1079" s="2" t="inlineStr">
+        <is>
+          <t>$BB i missed the call this morning from the baird conference. Can&amp;#39;t find anything online. Will someone give me the rundown? Thanks</t>
+        </is>
+      </c>
+      <c r="D1079" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1080" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1080" s="3" t="inlineStr">
+        <is>
+          <t>$BB good job son, go get me a beer</t>
+        </is>
+      </c>
+      <c r="D1080" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1081" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1081" s="3" t="inlineStr">
+        <is>
+          <t>$BB still down 42% in my retirement account. I cannot wait to get my money back and then some. Lots of some.</t>
+        </is>
+      </c>
+      <c r="D1081" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1082" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1082" s="3" t="inlineStr">
+        <is>
+          <t>$BB I’m telling you $BB looks like $PLTR before it mooned. Look at the charts.</t>
+        </is>
+      </c>
+      <c r="D1082" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1083" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1083" s="2" t="inlineStr">
+        <is>
+          <t>$BB</t>
+        </is>
+      </c>
+      <c r="D1083" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1084" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1084" s="3" t="inlineStr">
+        <is>
+          <t>$BB $BB.TSX  Backlog exploding??</t>
+        </is>
+      </c>
+      <c r="D1084" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1085" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1085" s="3" t="inlineStr">
+        <is>
+          <t>$BB https://stockhouse.com/companies/bullboard?symbol=bb&amp;amp;postid=37016099</t>
+        </is>
+      </c>
+      <c r="D1085" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1086" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1086" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT on time $AAPL $TSLA $META $GOOGL</t>
+        </is>
+      </c>
+      <c r="D1086" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1087" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1087" s="4" t="inlineStr">
+        <is>
+          <t>$MSFT you’re  a idiot or just blind buying off pure euphoria. Get your head out of your ass you’ll get rich from both sides not one side hopium pumps.. that’s don’t give a fuk about your calls 😂😂🔻 $TSLA $QQQ $META $SPY</t>
+        </is>
+      </c>
+      <c r="D1087" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1088" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1088" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Hello darkness my old friend</t>
+        </is>
+      </c>
+      <c r="D1088" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1089" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1089" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT lol time to jump in I guess</t>
+        </is>
+      </c>
+      <c r="D1089" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1090" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1090" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT this always tanks down hard after pump. Hardly seen consistently pumping.</t>
+        </is>
+      </c>
+      <c r="D1090" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1091" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1091" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT MAG7 must tank tomorrow including all index. Let’s go.</t>
+        </is>
+      </c>
+      <c r="D1091" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1092" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1092" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT this will be under 400 by Friday…look at the way it’s dumping…lmao…on google news ffsk. Didn’t even go up a penny when google was running (dumped harder actually) and now dunking as hard as google on offering news 🤣…you can’t make this up….lose lose no matter what the marke</t>
+        </is>
+      </c>
+      <c r="D1092" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1093" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1093" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT it’s dumping because Google is raising money? What happens when msft wants to raise?</t>
+        </is>
+      </c>
+      <c r="D1093" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1094" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1094" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT</t>
+        </is>
+      </c>
+      <c r="D1094" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1095" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1095" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT lol what now? Haha ahh fawk- never fails - just let it run</t>
+        </is>
+      </c>
+      <c r="D1095" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1096" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1096" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR $ETH.X   https://decrypt.co/369803/bitcoin-sinks-time-ethereum-outperform-standard-chartered  Well said</t>
+        </is>
+      </c>
+      <c r="D1096" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1097" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1097" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR $ETH.X   My Journey, bag holding.</t>
+        </is>
+      </c>
+      <c r="D1097" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1098" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1098" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR back in. At a certain point price does matter and we are at bottom resistance. Everything else is so expensive in this market.</t>
+        </is>
+      </c>
+      <c r="D1098" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -23280,51 +24666,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>68</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 21:58 UTC</t>
         </is>
       </c>
     </row>
@@ -23382,41 +24768,41 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -23426,65 +24812,65 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>36</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -23494,19 +24880,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -23518,12 +24904,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -23535,24 +24921,24 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -23562,14 +24948,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -23579,14 +24965,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -23596,7 +24982,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
@@ -23620,24 +25006,24 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -23647,48 +25033,48 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -23705,24 +25091,24 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -23739,41 +25125,41 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -23790,7 +25176,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -23807,7 +25193,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -23824,7 +25210,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -23834,14 +25220,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -23851,14 +25237,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -23875,7 +25261,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -23885,14 +25271,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -23902,14 +25288,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -23919,14 +25305,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -23936,14 +25322,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -23960,7 +25346,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -23985,7 +25371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24852,6 +26238,272 @@
       </c>
       <c r="H27" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>290.79</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>32.52%</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>103,396,690</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>3.78</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>254.38B</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>136.08</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>-9.15%</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>30,791,916</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>47.69B</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>297.18</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>-1.10%</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>18,592,763</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>242.50B</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>481.57</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>4.70%</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>37,297,822</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2280.07B</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>10.32</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>6.17%</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>49,600,528</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>6.05B</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>441.31</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>-4.17%</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>36,634,724</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>3278.24B</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>17.97</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>-4.67%</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>46,757,785</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>10.24B</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 01:04 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1098"/>
+  <dimension ref="A1:D1188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24607,6 +24607,1986 @@
       <c r="D1098" s="3" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1099" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1099" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL We all know this is a bubble now, so now it is musical chairs until the bulltards will realize its fair value is 50% lower based on their own projections in a DCF</t>
+        </is>
+      </c>
+      <c r="D1099" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1100" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1100" s="2" t="inlineStr">
+        <is>
+          <t>$PATH $SPY $CRM $MRVL $BTC.X     PATH  is  10-20X …at  least  $110  company…they  have  contracts  with  bigger  software  companies  for  implementation  of  AI  agents  invluding  new pure  AI  companies…Path has  the  infrastructure,  the  customers  (80% of  FORTUNE  500 comp</t>
+        </is>
+      </c>
+      <c r="D1100" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1101" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1101" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL can u take me higherrrrr</t>
+        </is>
+      </c>
+      <c r="D1101" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1102" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1102" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL read that info tab folks!! Good god we in the thick of it now!! Bottleneck constrained means prices soar for our products across many of these segments if not all!!  https://www.stocktwits.com/symbol/MRVL?utm_source=ios_app&amp;amp;utm_medium=symbol_share&amp;amp;utm_campaign=symbo</t>
+        </is>
+      </c>
+      <c r="D1102" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1103" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1103" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN $MRVL 👇…</t>
+        </is>
+      </c>
+      <c r="D1103" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1104" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1104" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL 44% pop or 100 billion dollar market cap increase because Jensen said the stock will quintuple.  Sure it may get there but does it mean literally tomorrow?  Didn&amp;#39;t Victoria Secret go up 47% after they talked about AI lingerie?</t>
+        </is>
+      </c>
+      <c r="D1104" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1105" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1105" s="3" t="inlineStr">
+        <is>
+          <t>$SPY $QQQ $MRVL   $NVDA  lovely gap up this morning. Will rebuy 🔐📨</t>
+        </is>
+      </c>
+      <c r="D1105" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1106" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1106" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL will it re-test 330 tonight?</t>
+        </is>
+      </c>
+      <c r="D1106" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1107" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1107" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL Likely  see a few analyst upgrades tomorrow morning.</t>
+        </is>
+      </c>
+      <c r="D1107" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1108" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1108" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL up 40% just because  Jensen said so ??? Big ass bubble</t>
+        </is>
+      </c>
+      <c r="D1108" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1109" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1109" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR  sincerely I’m very surprised: one week ago he has bought a lot and now he’s selling? When he said he would never sell. Where is this information from?</t>
+        </is>
+      </c>
+      <c r="D1109" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1110" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1110" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR The only thing mstr invented is the dilution machine and  all the s holders wil pay the price.   Haaaaaaaa.</t>
+        </is>
+      </c>
+      <c r="D1110" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1111" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1111" s="2" t="inlineStr">
+        <is>
+          <t>@XORAA oh ya, I saw that also!  Picked up a few of $MSTR  today as well!!</t>
+        </is>
+      </c>
+      <c r="D1111" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1112" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1112" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR</t>
+        </is>
+      </c>
+      <c r="D1112" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1113" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1113" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR after all he tried a strategy and it worked so far he sold at around $73K a  coin and now he can buy back at $70K and u keep calling this dude not smart</t>
+        </is>
+      </c>
+      <c r="D1113" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1114" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1114" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR</t>
+        </is>
+      </c>
+      <c r="D1114" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1115" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1115" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR LOL THIS LOSER PROBABLY MADE $5 SHORTING MSTR FROM 160 TO 155 AND NOW SHE THINKS SHE CAN MAKE LOTS OF MONEY.  PROBABLY THE DUMBEST PERSON ON THIS APP</t>
+        </is>
+      </c>
+      <c r="D1115" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1116" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1116" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR looks like long term bulls are selling covereds again. Lmao</t>
+        </is>
+      </c>
+      <c r="D1116" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1117" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1117" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR   SAYLOR SHOULD BUY MORE!!!! GOOD DEAL ON BTC TODAY!!!!!!</t>
+        </is>
+      </c>
+      <c r="D1117" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1118" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1118" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR this guy buys high sells low</t>
+        </is>
+      </c>
+      <c r="D1118" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1119" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1119" s="3" t="inlineStr">
+        <is>
+          <t>$PANW not holding gains very well. Smh. Earnings call is a snooze fest.</t>
+        </is>
+      </c>
+      <c r="D1119" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1120" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1120" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Need to see below 300 by tomorrow morning</t>
+        </is>
+      </c>
+      <c r="D1120" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1121" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1121" s="3" t="inlineStr">
+        <is>
+          <t>$PANW   How do we feel about this CEO?</t>
+        </is>
+      </c>
+      <c r="D1121" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1122" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1122" s="3" t="inlineStr">
+        <is>
+          <t>$CRWD up another 80 pts since and $30 more AH bc $PANW   crowdstrike better be massively good tomorrow,  just saying again😏</t>
+        </is>
+      </c>
+      <c r="D1122" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1123" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1123" s="2" t="inlineStr">
+        <is>
+          <t>$PANW</t>
+        </is>
+      </c>
+      <c r="D1123" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1124" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1124" s="2" t="inlineStr">
+        <is>
+          <t>$PANW heatmap changed. Dealer with double bolt 330 still there. With new king at 350 which is possible. Lets stack</t>
+        </is>
+      </c>
+      <c r="D1124" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1125" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1125" s="2" t="inlineStr">
+        <is>
+          <t>$NOW   $CRWD  earnings this week are going to send this. IGV still pumping  $PANW had an obvious beat  The run continues</t>
+        </is>
+      </c>
+      <c r="D1125" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1126" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1126" s="3" t="inlineStr">
+        <is>
+          <t>$PANW beat expectations with strong growth, boosted outlook, and rising AI security demand, sending shares sharply higher. https://notreload.xyz/panw-surges-after-q3-earnings-beat-raised-guidance/</t>
+        </is>
+      </c>
+      <c r="D1126" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1127" s="4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1127" s="4" t="inlineStr">
+        <is>
+          <t>$PANW the numbers wasn’t good. They have acquired all these companies over the years  and barley getting by with these numbers 🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸🩸</t>
+        </is>
+      </c>
+      <c r="D1127" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1128" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1128" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Look at the chart.  Insiders had already bought it.  1/3 of market cap added in last 20 days.  Now they&amp;#39;re selling it to you</t>
+        </is>
+      </c>
+      <c r="D1128" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1129" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1129" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO bought on Dec with the intent of selling when it gained $100, but it just blew past that. I guess $560 is my next target price.</t>
+        </is>
+      </c>
+      <c r="D1129" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1130" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1130" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO sold my covered call for $475. 😅 looking like a terrible call this week.</t>
+        </is>
+      </c>
+      <c r="D1130" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1131" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1131" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO Earnings in couple days…. 🤞🤞🤞</t>
+        </is>
+      </c>
+      <c r="D1131" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1132" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1132" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO Puts make sense here</t>
+        </is>
+      </c>
+      <c r="D1132" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1133" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1133" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1133" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1134" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1134" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO   https://www.youtube.com/watch?v=LJ0I0s-6Nqo    $500 Tonight!... not tomorrow... not after breakfast NOW!!</t>
+        </is>
+      </c>
+      <c r="D1134" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1135" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1135" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO Easy money</t>
+        </is>
+      </c>
+      <c r="D1135" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1136" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1136" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO $500. tomorrow?</t>
+        </is>
+      </c>
+      <c r="D1136" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1137" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1137" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO where are the haters? Usually they start showing up on the Monday of earnings. Cherrypicking facts, drawing cute lines on charts or posting plain old &amp;quot;this will tank&amp;quot; posts.  Did they get washed out over last 3 months or just biding their time?</t>
+        </is>
+      </c>
+      <c r="D1137" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1138" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1138" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $MU $NVDA $QQQ $SPY</t>
+        </is>
+      </c>
+      <c r="D1138" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1139" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1139" s="3" t="inlineStr">
+        <is>
+          <t>$BB sick that i sold almost half my calls today, but grateful that i diamond hands the rest. Can’t teade perfectly. if this bombs at open LOAD TF UP. buy shares or long calls to mitigate risk. EOW calls printing for me rn.</t>
+        </is>
+      </c>
+      <c r="D1139" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1140" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1140" s="2" t="inlineStr">
+        <is>
+          <t>$BB  Something is cooking at BB!!!! FINALLY, Big Investors realize BB is AI! 💰💰💰💰💰 💎💎💎💎💎</t>
+        </is>
+      </c>
+      <c r="D1140" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1141" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1141" s="2" t="inlineStr">
+        <is>
+          <t>$AMD $BB $ONDS Everyday I&amp;#39;m shuffling!</t>
+        </is>
+      </c>
+      <c r="D1141" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1142" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1142" s="2" t="inlineStr">
+        <is>
+          <t>@Onmyapeshiz $BB They deliver these on custom order if you ask nicely !</t>
+        </is>
+      </c>
+      <c r="D1142" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1143" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1143" s="3" t="inlineStr">
+        <is>
+          <t>$BB I’m sorry…did I stutter???</t>
+        </is>
+      </c>
+      <c r="D1143" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1144" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1144" s="3" t="inlineStr">
+        <is>
+          <t>$BB  this one is quietly making believers</t>
+        </is>
+      </c>
+      <c r="D1144" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1145" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1145" s="2" t="inlineStr">
+        <is>
+          <t>$BB hold on G force incoming on this rocket.....</t>
+        </is>
+      </c>
+      <c r="D1145" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1146" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1146" s="2" t="inlineStr">
+        <is>
+          <t>$BB didnt you ask?  lol.  Looking like a goof ball.  go play outside.  Men are making money.</t>
+        </is>
+      </c>
+      <c r="D1146" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1147" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1147" s="2" t="inlineStr">
+        <is>
+          <t>@Thamb19 You know what-- I take back what I said, you are a true holder of $BB and I apologize for my previous tone 🤝    Good luck to you man, I truly hope $BB and $NOK keep climing together to the Moon 🚀🌙    I&amp;#39;ll look deeper into $BB as well, must be a legit turnaround story</t>
+        </is>
+      </c>
+      <c r="D1147" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1148" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1148" s="2" t="inlineStr">
+        <is>
+          <t>$BB  #1 again 👏🏽😈🦾</t>
+        </is>
+      </c>
+      <c r="D1148" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1149" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1149" s="3" t="inlineStr">
+        <is>
+          <t>$IBM $NOW $MSFT opposite of last night HYPE....</t>
+        </is>
+      </c>
+      <c r="D1149" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1150" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1150" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT So, great day until it dipped below $460.  Once it confirms 460+ it flys back above 500.  AI Revenue realized, future is BRIGHT ☀️🌞🕶️</t>
+        </is>
+      </c>
+      <c r="D1150" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1151" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1151" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT massive dilution coming.  Building datacenters its very, very expensive.  $NVDA $AMD Party continues.</t>
+        </is>
+      </c>
+      <c r="D1151" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1152" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1152" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT what happened?</t>
+        </is>
+      </c>
+      <c r="D1152" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1153" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1153" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT fucking google .. like they don’t have the money</t>
+        </is>
+      </c>
+      <c r="D1153" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1154" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1154" s="4" t="inlineStr">
+        <is>
+          <t>$SPY $META $GOOGL $MSFT $AMZN Market top. Piggies will be cooked.</t>
+        </is>
+      </c>
+      <c r="D1154" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1155" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1155" s="2" t="inlineStr">
+        <is>
+          <t>$RZLV we&amp;#39;re in the same room as $NVDA and $MSFT this week!!</t>
+        </is>
+      </c>
+      <c r="D1155" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1156" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1156" s="4" t="inlineStr">
+        <is>
+          <t>$MSFT we going  to $433 tomorrow? Looks like it wants to revisit it’s previous resistance</t>
+        </is>
+      </c>
+      <c r="D1156" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1157" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1157" s="3" t="inlineStr">
+        <is>
+          <t>$IGV $MSFT $PLTR $QQQ $SPY</t>
+        </is>
+      </c>
+      <c r="D1157" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1158" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1158" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT shake out after hours</t>
+        </is>
+      </c>
+      <c r="D1158" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1159" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1159" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL $352 this week</t>
+        </is>
+      </c>
+      <c r="D1159" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1160" s="4" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1160" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL $GOOG $SPY $QQQ   ABSOLUTE INSANITY.  YOU KNOW THAT THIS AI BUBBLE HAS BECOME SO BIG WHEN A BLUE CHIP STOCK LIKE GOOGLE IS DILUTING Shareholders.  Horrible situation.</t>
+        </is>
+      </c>
+      <c r="D1160" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1161" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1161" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic Files S-1 Opening The IPO Floodgates, Analyst Says  $GOOGL $GOOG $AMZN $AVGO   https://www.benzinga.com/analyst-stock-ratings/analyst-color/26/06/52927424/anthropic-files-s-1-opening-the-ipo-floodgates-analyst-says</t>
+        </is>
+      </c>
+      <c r="D1161" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1162" s="2" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1162" s="2" t="inlineStr">
+        <is>
+          <t>$GOOGL owns 14% of Anthropic 👀</t>
+        </is>
+      </c>
+      <c r="D1162" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1163" s="2" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1163" s="2" t="inlineStr">
+        <is>
+          <t>$GOOGL There’s apatite  for risk</t>
+        </is>
+      </c>
+      <c r="D1163" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1164" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1164" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL $GOOG between this and the mosquitoes i might have to sell my shares 💩</t>
+        </is>
+      </c>
+      <c r="D1164" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1165" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1165" s="3" t="inlineStr">
+        <is>
+          <t>$GOOG $GOOGL MONEY GOING STRAIGHT INTO $AVGO‼️‼️  https://stocktwits.com/news-articles/markets/equity/alphabet-80b-fundraise-berkshire-hathaway-invests-10b-artificial-intelligence/cZ0WEfvRevi</t>
+        </is>
+      </c>
+      <c r="D1165" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1166" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1166" s="3" t="inlineStr">
+        <is>
+          <t>$META $GOOG $GOOGL one company diluting shareholders and one cutting jobs and not diluting to make way for spending. We are not the same.. :)</t>
+        </is>
+      </c>
+      <c r="D1166" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1167" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1167" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL Hmm why is google doing an offering, when they have more money than they know what to do with?</t>
+        </is>
+      </c>
+      <c r="D1167" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1168" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C1168" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL so Berkshire investing $10B in goggle. I wouldn’t be surprised if they do the same thing to the rest of MAGs except TSLA.</t>
+        </is>
+      </c>
+      <c r="D1168" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1169" s="2" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1169" s="2" t="inlineStr">
+        <is>
+          <t>$PUSA I&amp;#39;ve been lucky enough in Life to never have to pay for $PUSA but this $PUSA I  would empty the bank vault for!!!!</t>
+        </is>
+      </c>
+      <c r="D1169" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1170" s="3" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1170" s="3" t="inlineStr">
+        <is>
+          <t>$PUSA This is a must watch! Powerus President Brett Velicovich   https://www.foxbusiness.com/video/6397352601112</t>
+        </is>
+      </c>
+      <c r="D1170" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1171" s="3" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1171" s="3" t="inlineStr">
+        <is>
+          <t>$PUSA who’s getting pusa tomorrow lol</t>
+        </is>
+      </c>
+      <c r="D1171" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1172" s="2" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1172" s="2" t="inlineStr">
+        <is>
+          <t>$PUSA Every time one of these smaller stocks rallies recently they do an offering. Hope it isn&amp;#39;t one here, its killed momentum on a bunch of other stocks that were in this price range the last few weeks. But, solid day today</t>
+        </is>
+      </c>
+      <c r="D1172" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1173" s="2" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1173" s="2" t="inlineStr">
+        <is>
+          <t>$PUSA I am really shocked this isn’t getting more attention. Some pretty heavy hitters in the suite levels.</t>
+        </is>
+      </c>
+      <c r="D1173" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1174" s="3" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1174" s="3" t="inlineStr">
+        <is>
+          <t>$PUSA  there’s a noticeable lack of urgency from sellers.</t>
+        </is>
+      </c>
+      <c r="D1174" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1175" s="2" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1175" s="2" t="inlineStr">
+        <is>
+          <t>$PUSA no stopping this one!!</t>
+        </is>
+      </c>
+      <c r="D1175" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1176" s="3" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1176" s="3" t="inlineStr">
+        <is>
+          <t>$PUSA I believe we will reach $8-9 this week and 10 in the next few weeks.</t>
+        </is>
+      </c>
+      <c r="D1176" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1177" s="3" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1177" s="3" t="inlineStr">
+        <is>
+          <t>$SPY $PUSA $VELO $SMR $KSS</t>
+        </is>
+      </c>
+      <c r="D1177" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1178" s="3" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C1178" s="3" t="inlineStr">
+        <is>
+          <t>$PUSA</t>
+        </is>
+      </c>
+      <c r="D1178" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1179" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1179" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN  In February - Amazon&amp;#39;s $8 billion Anthropic investment balloons to $61 billion. On a lot more....</t>
+        </is>
+      </c>
+      <c r="D1179" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1180" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1180" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN like I said, $300 eoy</t>
+        </is>
+      </c>
+      <c r="D1180" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1181" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1181" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN 200,000 contracts of the jan 2027 275c traded  wow</t>
+        </is>
+      </c>
+      <c r="D1181" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1182" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1182" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN $190</t>
+        </is>
+      </c>
+      <c r="D1182" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1183" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1183" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN What’s going on here? What happened?</t>
+        </is>
+      </c>
+      <c r="D1183" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1184" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1184" s="3" t="inlineStr">
+        <is>
+          <t>$META one day of retail buying due to subscription news and they drop the price over $80 billion the next day. Cute. Fucking scumbags. $QQQ $AMZN $NVDA $MSFT</t>
+        </is>
+      </c>
+      <c r="D1184" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1185" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1185" s="3" t="inlineStr">
+        <is>
+          <t>I added some $GOOGL in my roth today. Looking to add some more $AMZN soon too.</t>
+        </is>
+      </c>
+      <c r="D1185" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1186" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1186" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN $META Amazon is up 20% ytd   We’re down 10% ytd   And yet we were still much redder than Amazon</t>
+        </is>
+      </c>
+      <c r="D1186" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1187" s="2" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1187" s="2" t="inlineStr">
+        <is>
+          <t>$META there is no news. $AMZN was also down a crap load. That&amp;#39;s why the call options barely moved.</t>
+        </is>
+      </c>
+      <c r="D1187" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1188" s="2" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1188" s="2" t="inlineStr">
+        <is>
+          <t>$SPY $META $GOOG $AMZN I chose the perfect trio today for holding calls🤦🏽‍♂️🤦🏽‍♂️🤦🏽‍♂️</t>
+        </is>
+      </c>
+      <c r="D1188" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
         </is>
       </c>
     </row>
@@ -24621,7 +26601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24649,34 +26629,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
@@ -24700,75 +26680,75 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 21:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -24778,14 +26758,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -24795,7 +26775,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
@@ -24807,12 +26787,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
@@ -24824,70 +26804,70 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>46</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -24897,19 +26877,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -24921,12 +26901,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -24938,24 +26918,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -24965,14 +26945,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -24982,14 +26962,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -24999,14 +26979,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -25016,7 +26996,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
@@ -25357,6 +27337,23 @@
       <c r="C43" t="inlineStr">
         <is>
           <t>2026-06-03 00:30 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
@@ -25371,7 +27368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -26504,6 +28501,426 @@
       </c>
       <c r="H34" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>290.79</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>32.52%</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>103,396,690</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>3.78</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>254.38B</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>136.08</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>-9.15%</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>30,791,916</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>47.69B</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>297.18</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>-1.10%</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>18,592,763</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>242.50B</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NDX, S&amp;P 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>481.57</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>4.70%</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>37,297,822</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2280.07B</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NDX, S&amp;P 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>10.32</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>6.17%</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>49,600,528</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>6.05B</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>441.31</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>-4.17%</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>36,634,724</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>3278.24B</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>DJIA, NDX, S&amp;P 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>17.97</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>-4.67%</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>46,757,785</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>10.24B</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>361.85</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>-3.86%</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>47,663,192</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>4364.33B</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NDX, S&amp;P 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>6.40</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>33.89%</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>5,972,215</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>3.28</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>138.27M</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>256.52</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>-1.81%</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>41,377,419</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2759.41B</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>DJIA, NDX, S&amp;P 500</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 01:22 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1188"/>
+  <dimension ref="A1:D1288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -26585,6 +26585,2206 @@
         </is>
       </c>
       <c r="D1188" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1189" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1189" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL bro I was trading MU hard for years, and the last trade I got in at $83 and out at $156…….FUCK!! $8300 too 100k, what could have beeen fuck!! Let’s see what MRVL can do!! 5x still to 1T market cap like Jensen says</t>
+        </is>
+      </c>
+      <c r="D1189" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1190" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1190" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL $MRVL $MSFT $MU I bought the calls when it was between 410-420. Thought I will sell when we touch 500. Now I am rethinking. This is a weird price action when they are announcing new things.</t>
+        </is>
+      </c>
+      <c r="D1190" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1191" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1191" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $DELL $MRVL $SOXS $SPY even if true a bubble now compared to a bubble then I imagine could be exponentially bigger than before</t>
+        </is>
+      </c>
+      <c r="D1191" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1192" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1192" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL Jensen aka NVDA had a big interest in MRVL  stock b 4 he open his mouth sea spewed a &amp;quot;trillion&amp;quot; --the earnings were not great but I doubt any 1 on this board read them--the stock was 222 a week ago and after earnings it fell to under 190 and made a small bounce --</t>
+        </is>
+      </c>
+      <c r="D1192" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1193" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1193" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$BTC.X $CRM $MRVL $PATH $SPY  Have 2300 shares PATH baby!! I agree 100% I have $30-$40 before year end but that could really be higher if traction fully takes off quickly. First profitable quarter in company history with 10,800+ clients. PATH stands to gain so much market cap in </t>
+        </is>
+      </c>
+      <c r="D1193" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1194" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1194" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL Seriously though, I don&amp;#39;t know what the f*** I&amp;#39;m doing. I thought I was a GeneAss for about a week after selling MU at 137$ ...lol</t>
+        </is>
+      </c>
+      <c r="D1194" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1195" s="4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1195" s="4" t="inlineStr">
+        <is>
+          <t>$MRVL the 9 EMA sits at 218$. Yeah this has to pullback</t>
+        </is>
+      </c>
+      <c r="D1195" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1196" s="4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1196" s="4" t="inlineStr">
+        <is>
+          <t>$MRVL almost 15 of the high. The sell off begins</t>
+        </is>
+      </c>
+      <c r="D1196" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1197" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1197" s="3" t="inlineStr">
+        <is>
+          <t>$SOXS during dotcom bubble, you could buy any dotcom and up and away everyday. Isn’t that basically what is happening today with AI stocks.  Just buy each and every one of them.  They say it’s not even comparable to dotcom. You will bank hard. $AVGO $MRVL $DELL $SPY</t>
+        </is>
+      </c>
+      <c r="D1197" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1198" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1198" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO Will not relent until the % gain either before or after earnings here is more than $MRVL 44% gain.. There must be justice.</t>
+        </is>
+      </c>
+      <c r="D1198" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1199" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1199" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO The Overnight clowns will try to bring it down over night so they can get in.</t>
+        </is>
+      </c>
+      <c r="D1199" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1200" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1200" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO holy crap. I literally bought the $500 calls today for one penny. I hope this goes parabolic after earnings just like DELL. It would be the trade of a lifetime</t>
+        </is>
+      </c>
+      <c r="D1200" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1201" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1201" s="3" t="inlineStr">
+        <is>
+          <t>A busy after-hours session with several key developments:    1.$HPE surged about 30% after beating earnings expectations and raising FY26 guidance.  2. $GOOGL announced plans to raise $80B to support its AI infrastructure expansion.  3. $HOOD saw an insider purchase worth roughly</t>
+        </is>
+      </c>
+      <c r="D1201" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1202" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1202" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO   This was a gimme. Only holding shares.    ER this week</t>
+        </is>
+      </c>
+      <c r="D1202" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1203" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1203" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO it looks like sympathy but it&amp;#39;s real deal Holyfield...</t>
+        </is>
+      </c>
+      <c r="D1203" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1204" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1204" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO anymore of those God candles ?</t>
+        </is>
+      </c>
+      <c r="D1204" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1205" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1205" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO if you’re trading earnings , $VEEV is the better buy with way more upside.</t>
+        </is>
+      </c>
+      <c r="D1205" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1206" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1206" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1206" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1207" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1207" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO but before earnings? Can be a face ripper like Dell and HP recently</t>
+        </is>
+      </c>
+      <c r="D1207" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1208" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1208" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO sitting near 52w highs into earnings, analysts bumping targets ahead of the print. last time a name set up this clean before results it gapped one way and never looked back. anyone playing the report or waiting for the reaction?  live tape + filings here: https://tapeboard.</t>
+        </is>
+      </c>
+      <c r="D1208" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1209" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1209" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT oversold - overreaction-google is gay- they have the money</t>
+        </is>
+      </c>
+      <c r="D1209" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1210" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1210" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT what tanked this AH</t>
+        </is>
+      </c>
+      <c r="D1210" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1211" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1211" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Massive upside tomorrow is coming $500 🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D1211" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1212" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1212" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Lots of Sell calls at the end of day. Will retest 420 area. Good luck to all</t>
+        </is>
+      </c>
+      <c r="D1212" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1213" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1213" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT damn, I&amp;#39;m not surprised. Always loosing its gains....</t>
+        </is>
+      </c>
+      <c r="D1213" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1214" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1214" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ could be the AI peak here.  Right Now.  Hyperscalers in trouble.  Damned if you do and dammed if you don’t.  $GOOG $META $MSFT 🤡🥵😜😛🤷🏻‍♂️🤑🤡😂🥵😜🤡😉</t>
+        </is>
+      </c>
+      <c r="D1214" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1215" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1215" s="3" t="inlineStr">
+        <is>
+          <t>$CRM $MSFT $NOW this was 265 when year started but its a bull trap I Like that! You like that??? 🤣</t>
+        </is>
+      </c>
+      <c r="D1215" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1216" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1216" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT this was over 471 premarket? Just now seeing that holy fuck good gawd almighty!!!</t>
+        </is>
+      </c>
+      <c r="D1216" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1217" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1217" s="3" t="inlineStr">
+        <is>
+          <t>$AMD $MSFT $NVDA not to mention the localized regulatory issues</t>
+        </is>
+      </c>
+      <c r="D1217" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1218" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1218" s="4" t="inlineStr">
+        <is>
+          <t>$MSFT $420 is on the table this week. Massive dilution coming. Capex is out of control.</t>
+        </is>
+      </c>
+      <c r="D1218" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1219" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1219" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR retrace  back to $130 it seems</t>
+        </is>
+      </c>
+      <c r="D1219" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1220" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1220" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR Sell reiterated. Now they&amp;#39;re selling her very asset longs want to get so they can pay dividends on preferred ahead of common shareholders  Fair value sun $100</t>
+        </is>
+      </c>
+      <c r="D1220" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1221" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1221" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR ....PREP&amp;amp;WATCH!!</t>
+        </is>
+      </c>
+      <c r="D1221" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1222" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1222" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR should be at $140 … how is it not tracking bitcoin ????</t>
+        </is>
+      </c>
+      <c r="D1222" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1223" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1223" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $ETH.X $MSTR it’s not real. There’s zero fundamental evidence for it anymore. Supply and demand from halving cycles is what drove it. Now it’s immaterial.  Michael Saylor, the ultimate perma bull that’s told people to sell organs before their bitcoin sold some of his bitco</t>
+        </is>
+      </c>
+      <c r="D1223" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1224" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1224" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR I think the board has figured out who that is. 😉</t>
+        </is>
+      </c>
+      <c r="D1224" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1225" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1225" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR waiting for $69,420....then I&amp;#39;M ALL IN</t>
+        </is>
+      </c>
+      <c r="D1225" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1226" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1226" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR This will make people very angry if it triples this summer</t>
+        </is>
+      </c>
+      <c r="D1226" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1227" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1227" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR looking for a buy signal?</t>
+        </is>
+      </c>
+      <c r="D1227" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1228" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1228" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR 6 years into his &amp;quot;journey&amp;quot; and his holdings are negative and now he needs to start dumping to fund his ponzis.     oops</t>
+        </is>
+      </c>
+      <c r="D1228" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1229" s="2" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1229" s="2" t="inlineStr">
+        <is>
+          <t>$NOK This is the next runner. Jenson is going to talk about them.</t>
+        </is>
+      </c>
+      <c r="D1229" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1230" s="3" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1230" s="3" t="inlineStr">
+        <is>
+          <t>$NOK  the chart is starting to attract more attention.</t>
+        </is>
+      </c>
+      <c r="D1230" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1231" s="3" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1231" s="3" t="inlineStr">
+        <is>
+          <t>$BB don’t forget to add $NOK guys</t>
+        </is>
+      </c>
+      <c r="D1231" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1232" s="3" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1232" s="3" t="inlineStr">
+        <is>
+          <t>$NOK +75K in OTM calls. Can bet I ain&amp;#39;t selling</t>
+        </is>
+      </c>
+      <c r="D1232" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1233" s="2" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1233" s="2" t="inlineStr">
+        <is>
+          <t>$NOK</t>
+        </is>
+      </c>
+      <c r="D1233" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1234" s="2" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1234" s="2" t="inlineStr">
+        <is>
+          <t>$NOK my largest position by far and I still feel like I didnt buy enough</t>
+        </is>
+      </c>
+      <c r="D1234" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1235" s="3" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1235" s="3" t="inlineStr">
+        <is>
+          <t>$NOK $30+ coming</t>
+        </is>
+      </c>
+      <c r="D1235" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1236" s="4" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1236" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X  before it goes to Zero sell and buy $NOK</t>
+        </is>
+      </c>
+      <c r="D1236" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1237" s="3" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1237" s="3" t="inlineStr">
+        <is>
+          <t>$NOK nok who&amp;#39;s there</t>
+        </is>
+      </c>
+      <c r="D1237" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1238" s="3" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C1238" s="3" t="inlineStr">
+        <is>
+          <t>$NOK they holding it at 17.20</t>
+        </is>
+      </c>
+      <c r="D1238" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1239" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1239" s="3" t="inlineStr">
+        <is>
+          <t>$PANW losing most of its AH gains.  PANW has been denied entry into the AI circle jerk club.  Sorry no 30% pop for you $PANW bulls.</t>
+        </is>
+      </c>
+      <c r="D1239" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1240" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1240" s="3" t="inlineStr">
+        <is>
+          <t>$PANW  Dust in the wind</t>
+        </is>
+      </c>
+      <c r="D1240" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1241" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1241" s="3" t="inlineStr">
+        <is>
+          <t>$PANW panties dropping 📉</t>
+        </is>
+      </c>
+      <c r="D1241" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1242" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1242" s="3" t="inlineStr">
+        <is>
+          <t>$PANW timber</t>
+        </is>
+      </c>
+      <c r="D1242" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1243" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1243" s="3" t="inlineStr">
+        <is>
+          <t>$PANW oh woah they ganked it sooo hard</t>
+        </is>
+      </c>
+      <c r="D1243" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1244" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1244" s="2" t="inlineStr">
+        <is>
+          <t>$PANW   earnings drop after the close today.    Consensus: $2.94B revenue (+27.7% YoY), $0.79 EPS (-23.0% YoY).    We sold a cash-secured put for a $515 credit, with IV spiked into the event.    Base case: capture ~90% of premium fast as vol collapses post-print.    Strike at 260</t>
+        </is>
+      </c>
+      <c r="D1244" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1245" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1245" s="2" t="inlineStr">
+        <is>
+          <t>$PANW be patient, with more upgrades, we will fly tomorrow</t>
+        </is>
+      </c>
+      <c r="D1245" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1246" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1246" s="3" t="inlineStr">
+        <is>
+          <t>$PANW +5.66% AH off the 297.18 close, pushing 312 near the highs. up 75% on the month already so this run&amp;#39;s been relentless, these vertical moves can cool fast once the chase crowd shows up. nothing on my feed behind the pop yet. anyone got a catalyst?  the level i&amp;#39;m watc</t>
+        </is>
+      </c>
+      <c r="D1246" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1247" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1247" s="3" t="inlineStr">
+        <is>
+          <t>$PANW why are we dropping</t>
+        </is>
+      </c>
+      <c r="D1247" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1248" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1248" s="2" t="inlineStr">
+        <is>
+          <t>$PANW mythos has increased importance of this company more then ever</t>
+        </is>
+      </c>
+      <c r="D1248" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1249" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1249" s="2" t="inlineStr">
+        <is>
+          <t>$BB 🍺</t>
+        </is>
+      </c>
+      <c r="D1249" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1250" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1250" s="2" t="inlineStr">
+        <is>
+          <t>$BB market loves these legacy comeback stories</t>
+        </is>
+      </c>
+      <c r="D1250" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1251" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1251" s="3" t="inlineStr">
+        <is>
+          <t>$BB we going kite .its good.i don&amp;#39;t have any DD but we go to $12...15  and 20 evantualy</t>
+        </is>
+      </c>
+      <c r="D1251" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1252" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1252" s="3" t="inlineStr">
+        <is>
+          <t>$BB holy shit my Bb might  be coming back from grave in my Ira from 2021</t>
+        </is>
+      </c>
+      <c r="D1252" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1253" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1253" s="2" t="inlineStr">
+        <is>
+          <t>$BB this is going $11+ AH. Smoking hot.</t>
+        </is>
+      </c>
+      <c r="D1253" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1254" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1254" s="2" t="inlineStr">
+        <is>
+          <t>$BB</t>
+        </is>
+      </c>
+      <c r="D1254" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1255" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1255" s="3" t="inlineStr">
+        <is>
+          <t>$BB Está lista para explotar para arriba!</t>
+        </is>
+      </c>
+      <c r="D1255" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1256" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1256" s="3" t="inlineStr">
+        <is>
+          <t>$BB I&amp;#39;ve never thought about this type of comeback 😧 I&amp;#39;m still holding the rest half 🤭</t>
+        </is>
+      </c>
+      <c r="D1256" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1257" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1257" s="3" t="inlineStr">
+        <is>
+          <t>$BB What&amp;#39;s The News?</t>
+        </is>
+      </c>
+      <c r="D1257" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1258" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1258" s="2" t="inlineStr">
+        <is>
+          <t>$BB It&amp;#39;s been amazing, guys—what a ride my best trade by far! 🚀 I&amp;#39;ve always felt this thing was headed to $12–$14 and beyond, but the wife said no more living down by the river in a cardboard box while I wait for the next leg up. 😆 So I had to lock in all gains and stay m</t>
+        </is>
+      </c>
+      <c r="D1258" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1259" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1259" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX wtf happened? No position here</t>
+        </is>
+      </c>
+      <c r="D1259" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1260" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1260" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX entyvio had the same malignancy profile. I had no position before data but bought the dip.</t>
+        </is>
+      </c>
+      <c r="D1260" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1261" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1261" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX  between this and prax bad day for data.</t>
+        </is>
+      </c>
+      <c r="D1261" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1262" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1262" s="2" t="inlineStr">
+        <is>
+          <t>$ABVX overreaction is insane!</t>
+        </is>
+      </c>
+      <c r="D1262" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1263" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1263" s="2" t="inlineStr">
+        <is>
+          <t>$ABVX cancer news is a hit piece, they want retail out.</t>
+        </is>
+      </c>
+      <c r="D1263" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1264" s="4" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1264" s="4" t="inlineStr">
+        <is>
+          <t>$ABVX OFFERING SOON</t>
+        </is>
+      </c>
+      <c r="D1264" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1265" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1265" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX looks like I picked the wrong day to quit smoking meth</t>
+        </is>
+      </c>
+      <c r="D1265" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1266" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1266" s="2" t="inlineStr">
+        <is>
+          <t>$ABVX everything under 120 is a steal</t>
+        </is>
+      </c>
+      <c r="D1266" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1267" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1267" s="2" t="inlineStr">
+        <is>
+          <t>$ABVX tomorrow 130 imo</t>
+        </is>
+      </c>
+      <c r="D1267" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1268" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1268" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX GLP-1 class showing reduction in cancer risk. Unlike this trash. Shouldve invested in VKTX</t>
+        </is>
+      </c>
+      <c r="D1268" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1269" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1269" s="3" t="inlineStr">
+        <is>
+          <t>$RUM rumble becoming a major ai cloud player $SPCE</t>
+        </is>
+      </c>
+      <c r="D1269" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1270" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1270" s="2" t="inlineStr">
+        <is>
+          <t>$RUM Looking good. 9.20 support held like a champ.    WAR is calling for a sniper entry. Let&amp;#39;s see how this unfolds..    ━━━━━━  ⚔️ SNIPER BOT  ━━━━━━  ✅ Ideal Entry Zone: 9.56 – 9.59  ⛔ Reject Trigger: Breakdown under 9.54  📉 Stop Loss: 9.54 (VWAP – 1x ATR)  📏 Tick Gap: tick</t>
+        </is>
+      </c>
+      <c r="D1270" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1271" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1271" s="2" t="inlineStr">
+        <is>
+          <t>$RUM FOMO IS HERE, burn the shorts</t>
+        </is>
+      </c>
+      <c r="D1271" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1272" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1272" s="3" t="inlineStr">
+        <is>
+          <t>$RUM 10$ soon</t>
+        </is>
+      </c>
+      <c r="D1272" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1273" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1273" s="3" t="inlineStr">
+        <is>
+          <t>$RUM she wants to rip</t>
+        </is>
+      </c>
+      <c r="D1273" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1274" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1274" s="2" t="inlineStr">
+        <is>
+          <t>$RUM Trending #2 !!!!!</t>
+        </is>
+      </c>
+      <c r="D1274" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1275" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1275" s="3" t="inlineStr">
+        <is>
+          <t>$RUM buy and hold</t>
+        </is>
+      </c>
+      <c r="D1275" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1276" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1276" s="3" t="inlineStr">
+        <is>
+          <t>$RUM push it</t>
+        </is>
+      </c>
+      <c r="D1276" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1277" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1277" s="3" t="inlineStr">
+        <is>
+          <t>$RUM THE NEXT MOVE IS OBVIOUS    CHRIS PAVLOVSKI ALREADY:  CLOSED THE TETHER DEAL  PULLED OFF THE NORTHERN DATA ACQUISITION  BROUGHT IN AN INTEL-VET CFO TO RUN THE AI INFRA NUMBERS    THE NEXT STEP ISN’T PROVING HE CAN EXECUTE  IT’S PUTTING BIG THIRD-PARTY NAMES ON STAGE WITH HIM</t>
+        </is>
+      </c>
+      <c r="D1277" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1278" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1278" s="2" t="inlineStr">
+        <is>
+          <t>$RUM This could honestly be the meme stock of 2026, but the funny thing is it isn&amp;#39;t a meme with their business pivot</t>
+        </is>
+      </c>
+      <c r="D1278" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1279" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1279" s="3" t="inlineStr">
+        <is>
+          <t>$BB $GME</t>
+        </is>
+      </c>
+      <c r="D1279" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1280" s="2" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1280" s="2" t="inlineStr">
+        <is>
+          <t>$BB is the new $GME</t>
+        </is>
+      </c>
+      <c r="D1280" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1281" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1281" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR maybe $GME Cohen makes an offer to buy $MSTR and can fund $STRC dividends selling used Madden 21’s. He seems bored.</t>
+        </is>
+      </c>
+      <c r="D1281" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1282" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1282" s="3" t="inlineStr">
+        <is>
+          <t>$GME gotta think surprise earnings disclosure is related to left conviction. That boy will throw everyone under the bus to cut time., and if you are complicit you aren’t gonna keep making shady moves. 👏🏽👏🏽👏🏽👏🏽 timing is everything RC 🫡</t>
+        </is>
+      </c>
+      <c r="D1282" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1283" s="2" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1283" s="2" t="inlineStr">
+        <is>
+          <t>$GME you love to see it.</t>
+        </is>
+      </c>
+      <c r="D1283" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1284" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1284" s="3" t="inlineStr">
+        <is>
+          <t>$GME oh shit here we go!</t>
+        </is>
+      </c>
+      <c r="D1284" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1285" s="2" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1285" s="2" t="inlineStr">
+        <is>
+          <t>$GME  Andrew left is singing like a bird trying to avoid hard time. Is Kenny g worried?</t>
+        </is>
+      </c>
+      <c r="D1285" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1286" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1286" s="3" t="inlineStr">
+        <is>
+          <t>$EBAY $GME  Ebay like - no thanks Cohen.</t>
+        </is>
+      </c>
+      <c r="D1286" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1287" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1287" s="3" t="inlineStr">
+        <is>
+          <t>$GME   THE BAGGIES ARE REALLY OUT TONIGHT! 😆🤣😆🫠</t>
+        </is>
+      </c>
+      <c r="D1287" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+      <c r="B1288" s="2" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="C1288" s="2" t="inlineStr">
+        <is>
+          <t>$GME</t>
+        </is>
+      </c>
+      <c r="D1288" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
@@ -26601,7 +28801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26634,12 +28834,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
@@ -26663,63 +28863,63 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -26731,7 +28931,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -26741,31 +28941,31 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-01 21:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>56</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -26775,14 +28975,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -26792,19 +28992,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -26821,58 +29021,58 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>34</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -26884,7 +29084,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -26894,7 +29094,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
@@ -26986,7 +29186,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -26996,31 +29196,31 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -27030,48 +29230,48 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -27088,24 +29288,24 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -27122,41 +29322,41 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -27173,7 +29373,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -27190,7 +29390,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -27207,7 +29407,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -27224,7 +29424,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -27234,14 +29434,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -27258,7 +29458,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -27275,7 +29475,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -27285,14 +29485,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -27354,6 +29554,40 @@
       <c r="C44" t="inlineStr">
         <is>
           <t>2026-06-03 01:03 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
@@ -27368,7 +29602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -27417,70 +29651,122 @@
           <t>MARKET_CAP</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>SECTOR</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>290.79</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>32.52%</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>103,396,690</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>3.78</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>254.38B</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INFQ</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>481.57</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4.70%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>37,297,822</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2280.07B</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>441.31</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-4.17%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>36,634,724</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3278.24B</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -27488,1436 +29774,251 @@
           <t>MSTR</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>136.08</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-9.15%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>30,791,916</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>47.69B</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GOOGL</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>16.85</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3.69%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>129,860,545</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1.38</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>94.24B</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KEEL</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>297.18</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-1.10%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>18,592,763</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>242.50B</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GTLB</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>10.32</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>6.17%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>49,600,528</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6.05B</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-02 20:34 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SOXX</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>72.50</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-44.10%</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>16,033,983</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>14.40</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>5.78B</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.32</t>
+          <t>8.97</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>6.17%</t>
+          <t>-6.27%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>49,397,951</t>
+          <t>2,271,408</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>6.05B</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>3.91B</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>19.87</t>
+          <t>20.92</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.32%</t>
+          <t>-2.06%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>31,290,757</t>
+          <t>4,638,527</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>0.63</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4.34B</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-06-02 20:40 UTC</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>297.18</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>-1.10%</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>17,896,065</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2.22</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>242.50B</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06-02 20:40 UTC</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>MSTR</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>136.08</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>-9.15%</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>30,534,080</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>47.69B</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-06-02 20:40 UTC</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>GOOGL</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>361.85</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>-3.86%</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>47,633,403</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>4364.33B</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-06-02 20:40 UTC</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>KEEL</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>6.14</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>0.66%</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>45,869,486</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>3.71B</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-02 20:40 UTC</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>GTLB</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>31.82</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>-5.83%</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>23,326,197</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>3.65</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>5.37B</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-02 20:40 UTC</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SOXX</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>605.02</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>5.79%</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>7,319,401</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0.94</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>290.79</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>32.52%</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>103,396,690</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>3.78</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>254.38B</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>746.16</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>0.46%</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>29,290,504</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>0.56</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>759.57</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>0.14%</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>30,728,402</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>0.44</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>MSTR</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>136.08</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>-9.15%</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>30,791,916</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>47.69B</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>297.18</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>-1.10%</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>18,592,763</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>242.50B</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>481.57</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>4.70%</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>37,297,822</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>1.56</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2280.07B</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>SOXS</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>5.17</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>-17.41%</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>455,574,483</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>2.74</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>10.32</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>6.17%</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>49,600,528</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>2.51</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>6.05B</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>441.31</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>-4.17%</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>36,634,724</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>1.06</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>3278.24B</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:30 UTC</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>BMNR</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>17.97</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>-4.67%</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>46,757,785</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>10.24B</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:59 UTC</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>290.79</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>32.52%</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>103,396,690</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>3.78</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>254.38B</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:59 UTC</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>MSTR</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>136.08</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>-9.15%</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>30,791,916</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>47.69B</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:59 UTC</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>297.18</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>-1.10%</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>18,592,763</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>242.50B</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:59 UTC</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>481.57</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>4.70%</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>37,297,822</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>1.56</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>2280.07B</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:59 UTC</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>10.32</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>6.17%</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>49,600,528</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2.51</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>6.05B</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:59 UTC</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>441.31</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>-4.17%</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>36,634,724</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>1.06</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>3278.24B</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:59 UTC</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>BMNR</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>17.97</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>-4.67%</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>46,757,785</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>10.24B</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>290.79</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>32.52%</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>103,396,690</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>3.78</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>254.38B</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>MSTR</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>136.08</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>-9.15%</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>30,791,916</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>47.69B</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>297.18</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>-1.10%</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>18,592,763</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>242.50B</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>NDX, S&amp;P 500</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>481.57</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>4.70%</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>37,297,822</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>1.56</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2280.07B</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>NDX, S&amp;P 500</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>10.32</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>6.17%</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>49,600,528</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>2.51</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>6.05B</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>441.31</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>-4.17%</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>36,634,724</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>1.06</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>3278.24B</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>DJIA, NDX, S&amp;P 500</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>BMNR</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>17.97</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>-4.67%</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>46,757,785</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>10.24B</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>GOOGL</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>361.85</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>-3.86%</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>47,663,192</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>4364.33B</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>NDX, S&amp;P 500</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>PUSA</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>6.40</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>33.89%</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>5,972,215</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>3.28</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>138.27M</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2026-06-03 01:03 UTC</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>AMZN</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>256.52</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>-1.81%</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>41,377,419</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>0.92</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2759.41B</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>DJIA, NDX, S&amp;P 500</t>
+          <t>9.39B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 15:27 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1288"/>
+  <dimension ref="A1:D1388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -28785,6 +28785,2206 @@
         </is>
       </c>
       <c r="D1288" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1289" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1289" s="2" t="inlineStr">
+        <is>
+          <t>$BB so I guess tomorrow we’ll be in the 11-11.50 range?</t>
+        </is>
+      </c>
+      <c r="D1289" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1290" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1290" s="2" t="inlineStr">
+        <is>
+          <t>$BB $BB.TSX  Whatever they revealed behind closed doors, we didn’t need the memo😉 We’ve been here, still long, and very much unbothered, just patience and more shares</t>
+        </is>
+      </c>
+      <c r="D1290" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1291" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1291" s="2" t="inlineStr">
+        <is>
+          <t>$BB $GME  📈 🚀</t>
+        </is>
+      </c>
+      <c r="D1291" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1292" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1292" s="2" t="inlineStr">
+        <is>
+          <t>$BB After Hours up $0.40 on 2M volume. 😁</t>
+        </is>
+      </c>
+      <c r="D1292" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1293" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1293" s="2" t="inlineStr">
+        <is>
+          <t>$BB now the name will be marked with the legacy of euphoria, new, and overly advanced product, linked to the  Once derogatory ‘phone’ connotation.</t>
+        </is>
+      </c>
+      <c r="D1293" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1294" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1294" s="2" t="inlineStr">
+        <is>
+          <t>$BB Btw, in few days the PDT rule will be removed, that means more FOMO and volume overall on the markets 😏</t>
+        </is>
+      </c>
+      <c r="D1294" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1295" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1295" s="2" t="inlineStr">
+        <is>
+          <t>$BB hey bizmac, you wanna join the bull side instead? We’re really nice. And you could make a shit ton of money too.   Never mind. Keep shorting. That helps us more, for now. ☺️</t>
+        </is>
+      </c>
+      <c r="D1295" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1296" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1296" s="2" t="inlineStr">
+        <is>
+          <t>$BB   Tmrw 12  this physicsl AI with security is next $NVDA and $MU</t>
+        </is>
+      </c>
+      <c r="D1296" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1297" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1297" s="2" t="inlineStr">
+        <is>
+          <t>$BB  This stock market cap is 6 billion. For an AI stock, this is VERY LOW! Bears, cover quickly as BB will ROCKET UP to HIGH WEALTH!!! 🚀🚀🚀🚀🚀 💰💰💰💰💰</t>
+        </is>
+      </c>
+      <c r="D1297" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1298" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1298" s="3" t="inlineStr">
+        <is>
+          <t>$BB = AI LFG!!!!</t>
+        </is>
+      </c>
+      <c r="D1298" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1299" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1299" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO given they are pumping this into earnings, I would load puts come Thursday morning. The smells like an $NVDA earnings trap 🪤</t>
+        </is>
+      </c>
+      <c r="D1299" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1300" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1300" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO 500 incoming told yaa!!</t>
+        </is>
+      </c>
+      <c r="D1300" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1301" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1301" s="3" t="inlineStr">
+        <is>
+          <t>$SPY oil will go down and spy will go down with it .. your mind will be blown. $AAPL $MSFT $AVGO</t>
+        </is>
+      </c>
+      <c r="D1301" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1302" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1302" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO This can pull an AMD type of move...$600 after earnings...</t>
+        </is>
+      </c>
+      <c r="D1302" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1303" s="4" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1303" s="4" t="inlineStr">
+        <is>
+          <t>$AVGO ran up to much classic beat and raise and drop . All options premiums wiped out</t>
+        </is>
+      </c>
+      <c r="D1303" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1304" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1304" s="3" t="inlineStr">
+        <is>
+          <t>Overnight market moves:    $CRDO slipped over 11% despite beating all earnings estimates—a reminder that strong results don’t always translate to positive price action when expectations are high.    $HPE jumped 27% after posting Q2 revenue well above estimates and raising full-ye</t>
+        </is>
+      </c>
+      <c r="D1304" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1305" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1305" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO still holding it, and has more than covered the lag of any of the others… and some more   🚀</t>
+        </is>
+      </c>
+      <c r="D1305" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1306" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1306" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO only thing holding up my portfolio today babyyyyy</t>
+        </is>
+      </c>
+      <c r="D1306" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1307" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1307" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO there it is, hope you banked</t>
+        </is>
+      </c>
+      <c r="D1307" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1308" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1308" s="3" t="inlineStr">
+        <is>
+          <t>$SPY one day your going to wake up and be like shit I&amp;#39;m old now. I&amp;#39;m turning 40 in November, all my 30s went to concentrating on gaining wealth in the market by compounding shares of quality assets. I played options lightly but always focused on stacking shares and taking</t>
+        </is>
+      </c>
+      <c r="D1308" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1309" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1309" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL trend</t>
+        </is>
+      </c>
+      <c r="D1309" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1310" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1310" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D1310" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1311" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1311" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL could see $7 today</t>
+        </is>
+      </c>
+      <c r="D1311" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1312" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1312" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D1312" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1313" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1313" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL KEEL me some of that cash.</t>
+        </is>
+      </c>
+      <c r="D1313" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1314" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1314" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL we are going above and beyond!!!!20$ this year!!!🔥🔥🔥</t>
+        </is>
+      </c>
+      <c r="D1314" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1315" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1315" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL yes BABYYYYYY!</t>
+        </is>
+      </c>
+      <c r="D1315" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1316" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1316" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL Time to make $6 our new support</t>
+        </is>
+      </c>
+      <c r="D1316" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1317" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1317" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL  Amazing and Bullish !!</t>
+        </is>
+      </c>
+      <c r="D1317" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1318" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1318" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL 66666666666666666</t>
+        </is>
+      </c>
+      <c r="D1318" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1319" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1319" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL Mind you it was 195$ yesterday after already big move, you are buying the bags of insiders just like you will buy the bags of Musk on his IPO like a bozo</t>
+        </is>
+      </c>
+      <c r="D1319" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1320" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1320" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL   lol what a rip</t>
+        </is>
+      </c>
+      <c r="D1320" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1321" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1321" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL  Can we open with $350+ tomorrow?</t>
+        </is>
+      </c>
+      <c r="D1321" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1322" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1322" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL undervalued at 200B now with today’s move!! Yeah all in is what most are doing!! Follow the money</t>
+        </is>
+      </c>
+      <c r="D1322" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1323" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1323" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL any chance this tests AH ath??</t>
+        </is>
+      </c>
+      <c r="D1323" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1324" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1324" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL  +255% WE DID IT AGAIN!! 🙃 ✨️  NEXT STOP $555</t>
+        </is>
+      </c>
+      <c r="D1324" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1325" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1325" s="3" t="inlineStr">
+        <is>
+          <t>$SPY $QQQ $MRVL i get AI and all but you can’t tell me the market is not getting bubbly when a CEO pumps a stock 40% in a day!  40%!!!</t>
+        </is>
+      </c>
+      <c r="D1325" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1326" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1326" s="2" t="inlineStr">
+        <is>
+          <t>$QMCO I have a good feeling this one will be a big winner! Mature company with good leadership experience, in the AI data center business $DELL $MRVL $NVDA</t>
+        </is>
+      </c>
+      <c r="D1326" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1327" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1327" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL minimum 1x</t>
+        </is>
+      </c>
+      <c r="D1327" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1328" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1328" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL If Marvell Technology (NASDAQ: MRVL) reached a $1 trillion market capitalization, its stock price would be approximately $1,143.12 per share, based on current outstanding shares.</t>
+        </is>
+      </c>
+      <c r="D1328" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1329" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1329" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN Keep away from your keyboard and stop trading with Rivian.  If you love Rivian EV as much as I do, stay invested with your intention and hold strong with your vision.  This is an easy $25 before 4th of July.</t>
+        </is>
+      </c>
+      <c r="D1329" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1330" s="4" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1330" s="4" t="inlineStr">
+        <is>
+          <t>Watching $RIVN at this $18ISH level for another consecutive rejection. RSI getting overextended with this recent rally, exceeding 71 on the daily timeframe.</t>
+        </is>
+      </c>
+      <c r="D1330" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1331" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1331" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN Yep, and VW purchased shares are in the black too  Latest Share Purchase: In late April, VW purchased 62.9 million newly issued Rivian shares at $15.90 per share, totaling $1 billion</t>
+        </is>
+      </c>
+      <c r="D1331" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1332" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1332" s="2" t="inlineStr">
+        <is>
+          <t>Anyone else miss the old meme 2021 days when $RIVN $BULL $AMC $GME squeezed nuts?      Look at MLEC right now. MLEC is breaking out with 600k shares float.      Will another short get eliminated on MLEC like in the old 2021 days?!!</t>
+        </is>
+      </c>
+      <c r="D1332" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1333" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1333" s="2" t="inlineStr">
+        <is>
+          <t>$GRML Greenland Mines Signs Definitive Agreement to Acquire the Sarfartoq Neodymium-Praseodymium Rare Earths Project in Greenland https://finance.yahoo.com/sectors/energy/articles/greenland-mines-signs-definitive-agreement-123000225.html       $AVGO $RIVN $QQQ</t>
+        </is>
+      </c>
+      <c r="D1333" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1334" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1334" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN looks like we blowing past the 12-month PT of $17.88. Going to the higher PT of $25</t>
+        </is>
+      </c>
+      <c r="D1334" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1335" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1335" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN</t>
+        </is>
+      </c>
+      <c r="D1335" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1336" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1336" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN https://www.linkedin.com/posts/marinamhoffmann_rivian-r2-excitement-continues-brooke-crothers-activity-7467175624026279937-i6B3</t>
+        </is>
+      </c>
+      <c r="D1336" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1337" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1337" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN it’s getting soooo juicy up in here!!! 🤤</t>
+        </is>
+      </c>
+      <c r="D1337" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1338" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1338" s="3" t="inlineStr">
+        <is>
+          <t>$NCLH $RIVN Both those insider buys are now very much in profit. (and haven&amp;#39;t sold yet)    It pays to keep an eye on large trades like these by insiders or Hedge Funds. They KNOW.</t>
+        </is>
+      </c>
+      <c r="D1338" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1339" s="2" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1339" s="2" t="inlineStr">
+        <is>
+          <t>$GRML Greenland Mines Signs Definitive Agreement to Acquire the Sarfartoq Neodymium-Praseodymium Rare Earths Project in Greenland https://finance.yahoo.com/sectors/energy/articles/greenland-mines-signs-definitive-agreement-123000225.html         $MSFT $DRTS $SPY</t>
+        </is>
+      </c>
+      <c r="D1339" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1340" s="2" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1340" s="2" t="inlineStr">
+        <is>
+          <t>$DRTS back to 11 pls</t>
+        </is>
+      </c>
+      <c r="D1340" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1341" s="3" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1341" s="3" t="inlineStr">
+        <is>
+          <t>$DRTS new HOD coming</t>
+        </is>
+      </c>
+      <c r="D1341" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1342" s="3" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1342" s="3" t="inlineStr">
+        <is>
+          <t>$NVTS $FABC $DRTS ***</t>
+        </is>
+      </c>
+      <c r="D1342" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1343" s="2" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1343" s="2" t="inlineStr">
+        <is>
+          <t>@JohnStocksNY @FMazur That $DRTS CEO is a smart man</t>
+        </is>
+      </c>
+      <c r="D1343" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1344" s="2" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1344" s="2" t="inlineStr">
+        <is>
+          <t>@FMazur $DRTS 💪🙏</t>
+        </is>
+      </c>
+      <c r="D1344" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1345" s="2" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1345" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$DRTS There&amp;#39;s never a lack of excitement around this stock. One day, there&amp;#39;s extending the lives of PDAC Pancreatic cancer patients. The next day, they&amp;#39;re doing global commercial deals for prostate cancer.  The next day they&amp;#39;re getting two complete responses, out </t>
+        </is>
+      </c>
+      <c r="D1345" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1346" s="3" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1346" s="3" t="inlineStr">
+        <is>
+          <t>@OnlyGB $DRTS annual cash burn rate is approximately from$19 million to $22 million. The investment of $20 million covers one year not just one quarter.</t>
+        </is>
+      </c>
+      <c r="D1346" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1347" s="2" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1347" s="2" t="inlineStr">
+        <is>
+          <t>@topstockalerts Yes! $DRTS</t>
+        </is>
+      </c>
+      <c r="D1347" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1348" s="2" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="C1348" s="2" t="inlineStr">
+        <is>
+          <t>@OnlyGB I&amp;#39;m not so smart cause I didn&amp;#39;t buy enough 🤣. $DRTS</t>
+        </is>
+      </c>
+      <c r="D1348" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1349" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1349" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT just gave back the entire day’s gains in after hours, and that kind of reversal always gets attention.    What looked like steady accumulation during the session turned into a full round-trip once liquidity thinned out, which is pretty typical for mega caps when positioning</t>
+        </is>
+      </c>
+      <c r="D1349" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1350" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1350" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT   If google are selling share...what does that have to do with MS?  And why is it impacting us more that google?</t>
+        </is>
+      </c>
+      <c r="D1350" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1351" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1351" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT i guess its dilution risk.</t>
+        </is>
+      </c>
+      <c r="D1351" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1352" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1352" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT at these the gap is filled. Onwards and upwards</t>
+        </is>
+      </c>
+      <c r="D1352" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1353" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1353" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT poopy time!</t>
+        </is>
+      </c>
+      <c r="D1353" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1354" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1354" s="4" t="inlineStr">
+        <is>
+          <t>$MSFT   SHAREHOLDER DILUTION COMiNG.  Sell first ask questions later.  Look at $GOOG</t>
+        </is>
+      </c>
+      <c r="D1354" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1355" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1355" s="3" t="inlineStr">
+        <is>
+          <t>$PLTR OS is replacing $MSFT at $DELL $SPY $NVDA on the CHIPS!!!    https://www.dell.com/en-us/blog/dell-and-palantir-introduce-an-on-premises-ai-operating-system/</t>
+        </is>
+      </c>
+      <c r="D1355" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1356" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1356" s="3" t="inlineStr">
+        <is>
+          <t>$CRDO may be stay like this manipulated for 3.5 weeks just like they did to $MSFT</t>
+        </is>
+      </c>
+      <c r="D1356" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1357" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1357" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT would absolutely adore a retest to $435!!</t>
+        </is>
+      </c>
+      <c r="D1357" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1358" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1358" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT  👀   https://stocktwits.com/news-articles/markets/equity/microsoft-ai-models-in-windows-nvidia-rtx-spark-laptops-build-2026/cZ0gzPNRev2</t>
+        </is>
+      </c>
+      <c r="D1358" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1359" s="4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1359" s="4" t="inlineStr">
+        <is>
+          <t>$PANW AI told me to short this</t>
+        </is>
+      </c>
+      <c r="D1359" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1360" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1360" s="3" t="inlineStr">
+        <is>
+          <t>$PANW not good enough</t>
+        </is>
+      </c>
+      <c r="D1360" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1361" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1361" s="3" t="inlineStr">
+        <is>
+          <t>$PANW uh oh, spaghetti os</t>
+        </is>
+      </c>
+      <c r="D1361" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1362" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1362" s="3" t="inlineStr">
+        <is>
+          <t>$S Yeah $PANW smoked us on a much larger base</t>
+        </is>
+      </c>
+      <c r="D1362" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1363" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1363" s="3" t="inlineStr">
+        <is>
+          <t>$PANW well the stocked doubled they were expected to crush it they needed Dell Numbers</t>
+        </is>
+      </c>
+      <c r="D1363" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1364" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1364" s="2" t="inlineStr">
+        <is>
+          <t>$SNOW There&amp;#39;s going to be a RALLY tomorrow, the LIKES of which have never been seen by human eyes on the Planet Earth. $IBM $ULTA $PANW $SNOW $IBM #ThankYouForYourMuthaFukkinAttentionToThisMuthaFukkinMatter</t>
+        </is>
+      </c>
+      <c r="D1364" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1365" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1365" s="3" t="inlineStr">
+        <is>
+          <t>$PANW gonna see profit taking?</t>
+        </is>
+      </c>
+      <c r="D1365" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1366" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1366" s="3" t="inlineStr">
+        <is>
+          <t>$PANW why are we dropping</t>
+        </is>
+      </c>
+      <c r="D1366" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1367" s="4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1367" s="4" t="inlineStr">
+        <is>
+          <t>$PANW fucken knew it. Unfortunately this will be deep in the red tomorrow. From +10% to at least -6% if we’re lucky tomorrow. Well there goes 70k down the drain</t>
+        </is>
+      </c>
+      <c r="D1367" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1368" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1368" s="3" t="inlineStr">
+        <is>
+          <t>$PANW - told you all this will crash after this ridiculous move and lackluster guidance as algos are expecting  strong beats and guidances….might close below 270 tomorrow…$FTNT will close below 140 tomorrow…imo</t>
+        </is>
+      </c>
+      <c r="D1368" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1369" s="4" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1369" s="4" t="inlineStr">
+        <is>
+          <t>$AMZN oh wow so $GOOG is diluting. Very bearish for the hyperscaler complex.</t>
+        </is>
+      </c>
+      <c r="D1369" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1370" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1370" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN https://www.zerohedge.com/technology/spacex-ipo-update-new-filing-reveals-friends-family-share-allocation-anthropic-ai-deal</t>
+        </is>
+      </c>
+      <c r="D1370" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1371" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1371" s="3" t="inlineStr">
+        <is>
+          <t>@ribbey @Jeremymartin007 @simon58 @judgeyoung2 @jenbunn @cubie @EBE_day @Godreal1 @TraderRapp @tonyctl $META  😨😳 $AMZN</t>
+        </is>
+      </c>
+      <c r="D1371" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1372" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1372" s="3" t="inlineStr">
+        <is>
+          <t>$GOOG called it last week. Hyperscaler will need to dilute to fund capex. $META $AMZN Will be next</t>
+        </is>
+      </c>
+      <c r="D1372" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1373" s="2" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1373" s="2" t="inlineStr">
+        <is>
+          <t>$AMZN I will add more tomorrow if it’s dropping more</t>
+        </is>
+      </c>
+      <c r="D1373" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1374" s="2" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1374" s="2" t="inlineStr">
+        <is>
+          <t>$SPY hyperscalers getting sold to oblivion in ah.... Man this is rough. $GOOG $AMZN $MSFT $META</t>
+        </is>
+      </c>
+      <c r="D1374" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1375" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1375" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN omg what is happening here in AH, wtffff</t>
+        </is>
+      </c>
+      <c r="D1375" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1376" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1376" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN     Dropping hard AH here along with $MSFT     both dragging down $SPY</t>
+        </is>
+      </c>
+      <c r="D1376" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1377" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1377" s="3" t="inlineStr">
+        <is>
+          <t>@RunirStockWlerts Why $AMZN is not here?</t>
+        </is>
+      </c>
+      <c r="D1377" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1378" s="4" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1378" s="4" t="inlineStr">
+        <is>
+          <t>$AMZN not working</t>
+        </is>
+      </c>
+      <c r="D1378" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1379" s="4" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1379" s="4" t="inlineStr">
+        <is>
+          <t>$NFLX  They can come way down after they go way up...</t>
+        </is>
+      </c>
+      <c r="D1379" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1380" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1380" s="3" t="inlineStr">
+        <is>
+          <t>$CMG $NFLX</t>
+        </is>
+      </c>
+      <c r="D1380" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1381" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1381" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX look at this chart, only sellers</t>
+        </is>
+      </c>
+      <c r="D1381" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1382" s="4" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1382" s="4" t="inlineStr">
+        <is>
+          <t>$NFLX $BTC.X $DIS$MSTR  THESE ARE NOT AI, BUY POOOTS!!!</t>
+        </is>
+      </c>
+      <c r="D1382" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1383" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1383" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX $100 is a pipe dream now</t>
+        </is>
+      </c>
+      <c r="D1383" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1384" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1384" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX added another 25 calls to my position today. WITH TIME!</t>
+        </is>
+      </c>
+      <c r="D1384" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1385" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1385" s="2" t="inlineStr">
+        <is>
+          <t>$NFLX would be great if netflix can now use their 31 billion usd fund left for stock buyback now</t>
+        </is>
+      </c>
+      <c r="D1385" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1386" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1386" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX this supposed to be a hedge against red market 🤔</t>
+        </is>
+      </c>
+      <c r="D1386" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1387" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1387" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX pretty incredible there’s been no investigation or lawsuit into the criminal business practice of this company flat out lying about buy backs</t>
+        </is>
+      </c>
+      <c r="D1387" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+      <c r="B1388" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1388" s="2" t="inlineStr">
+        <is>
+          <t>$NFLX gimmie!</t>
+        </is>
+      </c>
+      <c r="D1388" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
@@ -28801,7 +31001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28846,41 +31046,41 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -28890,7 +31090,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
@@ -28914,51 +31114,51 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 21:58 UTC</t>
         </is>
       </c>
     </row>
@@ -28970,53 +31170,53 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -29026,7 +31226,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
@@ -29038,12 +31238,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -29588,6 +31788,57 @@
       <c r="C46" t="inlineStr">
         <is>
           <t>2026-06-02 21:21 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>DRTS</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -29602,7 +31853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -29643,56 +31894,106 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>AVG_VOLUME</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>REL_VOLUME</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>MARKET_CAP</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>BETA</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SECTOR</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>INDUSTRY</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>290.79</t>
+          <t>10.69</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>32.52%</t>
+          <t>3.54%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>103,396,690</t>
+          <t>44,287,617</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3.78</t>
+          <t>20.57M</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>254.38B</t>
+          <t>7.27</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>6.26B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>93.17</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -29702,323 +32003,548 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>481.57</t>
+          <t>487.97</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>1.33%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>37,297,822</t>
+          <t>14,053,254</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>24.17M</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2280.07B</t>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2310.38B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>76.01</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>441.31</t>
+          <t>6.30</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-4.17%</t>
+          <t>2.69%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>36,634,724</t>
+          <t>21,811,967</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>34.62M</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3278.24B</t>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3.81B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>83.85</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>136.08</t>
+          <t>306.98</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-9.15%</t>
+          <t>5.57%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>30,791,916</t>
+          <t>61,694,318</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>28.91M</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>47.69B</t>
+          <t>7.15</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>268.55B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>87.28</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>RIVN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>16.85</t>
+          <t>17.93</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.70%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>129,860,545</t>
+          <t>23,382,726</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>29.00M</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>94.24B</t>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>22.60B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>72.15</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>297.18</t>
+          <t>10.53</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-1.10%</t>
+          <t>17.96%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>18,592,763</t>
+          <t>1,370,089</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.30</t>
+          <t>566.17K</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>242.50B</t>
+          <t>8.11</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>927.07M</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>56.98</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.32</t>
+          <t>426.50</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>6.17%</t>
+          <t>-3.36%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>49,600,528</t>
+          <t>14,021,404</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>34.62M</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6.05B</t>
+          <t>1.36</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>3168.24B</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>52.22</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>72.50</t>
+          <t>282.17</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-44.10%</t>
+          <t>-5.05%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>16,033,983</t>
+          <t>6,994,189</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.40</t>
+          <t>8.27M</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5.78B</t>
+          <t>2.83</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>230.25B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>70.63</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8.97</t>
+          <t>250.64</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-6.27%</t>
+          <t>-2.29%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2,271,408</t>
+          <t>15,734,373</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>44.96M</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3.91B</t>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2696.16B</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>39.83</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Internet Retail</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>20.92</t>
+          <t>81.73</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-2.06%</t>
+          <t>-1.92%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4,638,527</t>
+          <t>11,587,811</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.63</t>
+          <t>38.82M</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>9.39B</t>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>344.14B</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>27.61</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 15:36 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1388"/>
+  <dimension ref="A1:D1471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30987,6 +30987,1832 @@
       <c r="D1388" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1389" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1389" s="2" t="inlineStr">
+        <is>
+          <t>$BB i bought in exactly 5 years ago today. Hit my breakeven today. Wild!!</t>
+        </is>
+      </c>
+      <c r="D1389" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1390" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1390" s="2" t="inlineStr">
+        <is>
+          <t>$BB With all due respect, please do not put $GME and $BB in the same post as comparables.... BB is the real deal, not a meme.</t>
+        </is>
+      </c>
+      <c r="D1390" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1391" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1391" s="2" t="inlineStr">
+        <is>
+          <t>$BB gonna buy 10 kg of blackberries when this hits 50$</t>
+        </is>
+      </c>
+      <c r="D1391" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1392" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1392" s="2" t="inlineStr">
+        <is>
+          <t>$BB</t>
+        </is>
+      </c>
+      <c r="D1392" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1393" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1393" s="3" t="inlineStr">
+        <is>
+          <t>$BB</t>
+        </is>
+      </c>
+      <c r="D1393" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1394" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1394" s="3" t="inlineStr">
+        <is>
+          <t>$GME I&amp;#39;m really gladwe&amp;#39;re holding onto all this money. Just wish we would do something with it. Look at $BB. I&amp;#39;m holding that one as well. They&amp;#39;ve completely reinvented themselves. It&amp;#39;d be nice to see something like that here.</t>
+        </is>
+      </c>
+      <c r="D1394" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1395" s="3" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1395" s="3" t="inlineStr">
+        <is>
+          <t>$BB</t>
+        </is>
+      </c>
+      <c r="D1395" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1396" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1396" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$BB When someone asks where is BB heading next?  $25. This VWAP from the beginning of the stock marked the top of the MEME run but it may only serve as a pause this time... We will DEFINITELY pay respect to this VWAP. 100%    I do feel we will go way higher over time... But over </t>
+        </is>
+      </c>
+      <c r="D1396" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1397" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1397" s="2" t="inlineStr">
+        <is>
+          <t>$BB WTFFF LOLL.. It&amp;#39;s literally $25K gains daily at this point Holy shit</t>
+        </is>
+      </c>
+      <c r="D1397" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1398" s="2" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C1398" s="2" t="inlineStr">
+        <is>
+          <t>$BB     Bulls right now....    12+++ (please make me raise the target soon) 😂</t>
+        </is>
+      </c>
+      <c r="D1398" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1399" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1399" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO $INTC $MRVL $NVDA $QCOM</t>
+        </is>
+      </c>
+      <c r="D1399" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1400" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1400" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL $NVDA $QCOM $AVGO $INTC   https://www.stocktwits.com/symbol/MRVL/companycall</t>
+        </is>
+      </c>
+      <c r="D1400" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1401" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1401" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO is 3% AH on the day $SPY is down…. Imagine what happens when $SPY is back up green….  $1000 printing on this. $QQQ</t>
+        </is>
+      </c>
+      <c r="D1401" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1402" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1402" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1402" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1403" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1403" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO  🗣</t>
+        </is>
+      </c>
+      <c r="D1403" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1404" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1404" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1404" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1405" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1405" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO over $500 after earnings</t>
+        </is>
+      </c>
+      <c r="D1405" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1406" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1406" s="3" t="inlineStr">
+        <is>
+          <t>$NVDA and $AVGO continue to show a constructive technical picture:  • Roughly 6-month base formation  • Confirmed breakout  • Successful retest of the breakout zone  The price structure remains strong, with both stocks continuing to display characteristics of established market l</t>
+        </is>
+      </c>
+      <c r="D1406" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1407" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1407" s="3" t="inlineStr">
+        <is>
+          <t>The biggest opportunity in AI may not be finding the fastest-moving stock, but identifying the companies that consistently execute.  Key names on my radar:    $NVDA — AI compute leader  $MSFT — Enterprise AI monetization  $AVGO — Networking and custom silicon  $AMD — Expanding AI</t>
+        </is>
+      </c>
+      <c r="D1407" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1408" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1408" s="2" t="inlineStr">
+        <is>
+          <t>$NVDA B/O Rally Continuation Coming  240.00’s  $AVGO ER AMC 6/2/2026  $QQQ $SPY $SMH</t>
+        </is>
+      </c>
+      <c r="D1408" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1409" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1409" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL waited for 5 years. now lets ride the bullet train........</t>
+        </is>
+      </c>
+      <c r="D1409" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1410" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1410" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL. LG 🚀</t>
+        </is>
+      </c>
+      <c r="D1410" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1411" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1411" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL trending #3, lets get this to 6.25</t>
+        </is>
+      </c>
+      <c r="D1411" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1412" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1412" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL Stop and think for a second over 6$ and they still haven&amp;#39;t announced any of the 3 deals this is now entering 20$ potential in the year with those deals.  Leopold def knows what&amp;#39;s coming shorts and penny flippers hit the road!! 🚀 🚀</t>
+        </is>
+      </c>
+      <c r="D1412" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1413" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1413" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL if Ben is smart, he should announce a deal soon.</t>
+        </is>
+      </c>
+      <c r="D1413" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1414" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1414" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL c&amp;#39;mon Ben, drop it already</t>
+        </is>
+      </c>
+      <c r="D1414" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1415" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1415" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL Contract soon 📰</t>
+        </is>
+      </c>
+      <c r="D1415" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1416" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1416" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL who got shaken off this morning ?</t>
+        </is>
+      </c>
+      <c r="D1416" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1417" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1417" s="3" t="inlineStr">
+        <is>
+          <t>$TE red to green   $KEEL new highs, swing in tact  $BTDR $20S on deck imo</t>
+        </is>
+      </c>
+      <c r="D1417" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1418" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1418" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL $7.00</t>
+        </is>
+      </c>
+      <c r="D1418" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1419" s="4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1419" s="4" t="inlineStr">
+        <is>
+          <t>$MRVL   $800 by tommorow afternoon? That would be MARVELOUS wouldn’t it</t>
+        </is>
+      </c>
+      <c r="D1419" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1420" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1420" s="3" t="inlineStr">
+        <is>
+          <t>$AMBA $AVGO $MRVL $OSS $TSLA  Fah-king bangers</t>
+        </is>
+      </c>
+      <c r="D1420" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1421" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1421" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL an offering is coming---NVDA madean  investment in MRVL around 150--MRVL needed money to expand even though their products are great--u have to have big $ to get bigger and buy a manufacturing plant---NVDA made the investment to get their products--whether it turns out is a</t>
+        </is>
+      </c>
+      <c r="D1421" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1422" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1422" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL This is what you are fomo buying? Really? They ain&amp;#39;t no Nvidia or Micron, not even AMD</t>
+        </is>
+      </c>
+      <c r="D1422" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1423" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1423" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL yes 420 tomorrow, could squeeze to 800 by afternoon.</t>
+        </is>
+      </c>
+      <c r="D1423" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1424" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1424" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL march to 500</t>
+        </is>
+      </c>
+      <c r="D1424" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1425" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1425" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $DELL $MRVL $SOXS $SPY counter argument is you had hundreds of dotcoms going from 50m to 500m. Is that the same as 30-40 companies of 25b going to 200b+ market cap companies?  Soxx went from 4T to 15T market cap.  Which is the bigger bubble even if they are making money?</t>
+        </is>
+      </c>
+      <c r="D1425" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1426" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1426" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL I purchased $150 of fractional shares today so the inside traders can lick my bag I don’t go full retard on moves like this, but I do like to take a tiny piece of the pie.</t>
+        </is>
+      </c>
+      <c r="D1426" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1427" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1427" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL finally caught a nice move here sold everything at 329</t>
+        </is>
+      </c>
+      <c r="D1427" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1428" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1428" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL   😊😊😊😊😊😊😊😊😊😊😊 This is my time traveler proof   👇👇👇👇👇👇👇👇👇👇👇  $NVDA $AMD $IONQ  I told u at $63</t>
+        </is>
+      </c>
+      <c r="D1428" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1429" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1429" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN gawd damn fade again</t>
+        </is>
+      </c>
+      <c r="D1429" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1430" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1430" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN and $NIO trending with MLEC</t>
+        </is>
+      </c>
+      <c r="D1430" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1431" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1431" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN Not too shabby for a down market day  Shows just how strong Rivian is going forward :)</t>
+        </is>
+      </c>
+      <c r="D1431" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1432" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1432" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT LOL...People people...you sell the news when you get the news.  The Microsoft event is tomorrow...</t>
+        </is>
+      </c>
+      <c r="D1432" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1433" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1433" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT looking forward to buying more</t>
+        </is>
+      </c>
+      <c r="D1433" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1434" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1434" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL $META $MSFT $AMZN mega rich companies with hundreds of billions of profits are laying off people and raising cash issuing new shares and  debt 💸! We are living in a fking crazy ugly 🤮 world !!</t>
+        </is>
+      </c>
+      <c r="D1434" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1435" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1435" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT I&amp;#39;m out. Looks like the run is over.</t>
+        </is>
+      </c>
+      <c r="D1435" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1436" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1436" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Massive upside is coming tomorrow 🚀🚀🚀 The $450  gap filled. Next stop is $500. 🍒🍒🍒🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D1436" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1437" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1437" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT HOLD your shares . We are going to $480</t>
+        </is>
+      </c>
+      <c r="D1437" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1438" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1438" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Micro is sort of soft, kind of nervous😬</t>
+        </is>
+      </c>
+      <c r="D1438" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1439" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1439" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT nothing but FUD</t>
+        </is>
+      </c>
+      <c r="D1439" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1440" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1440" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT keep going. Got a small position left. Let’s double up. 435</t>
+        </is>
+      </c>
+      <c r="D1440" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1441" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C1441" s="4" t="inlineStr">
+        <is>
+          <t>$MSFT wow my puts are going ti be up like 200%</t>
+        </is>
+      </c>
+      <c r="D1441" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1442" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1442" s="3" t="inlineStr">
+        <is>
+          <t>$PANW plead bull shi ters post losses</t>
+        </is>
+      </c>
+      <c r="D1442" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1443" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1443" s="2" t="inlineStr">
+        <is>
+          <t>$PANW amazing earnings</t>
+        </is>
+      </c>
+      <c r="D1443" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1444" s="4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1444" s="4" t="inlineStr">
+        <is>
+          <t>$PANW bs</t>
+        </is>
+      </c>
+      <c r="D1444" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1445" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1445" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Stock doubled since April 13th so yeah, it&amp;#39;s hard to top or convince the investors. It has to be like Dell with government backing. Without tjeht trump pump tied with it, it will be a challenge.</t>
+        </is>
+      </c>
+      <c r="D1445" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1446" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1446" s="3" t="inlineStr">
+        <is>
+          <t>$PANW lol</t>
+        </is>
+      </c>
+      <c r="D1446" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1447" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1447" s="3" t="inlineStr">
+        <is>
+          <t>$PANW this is going red</t>
+        </is>
+      </c>
+      <c r="D1447" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1448" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1448" s="3" t="inlineStr">
+        <is>
+          <t>$PANW theres always money in the banana stand</t>
+        </is>
+      </c>
+      <c r="D1448" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1449" s="4" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1449" s="4" t="inlineStr">
+        <is>
+          <t>$PANW $240 very soon, remember insiders can now unload bags in the coming days</t>
+        </is>
+      </c>
+      <c r="D1449" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1450" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1450" s="3" t="inlineStr">
+        <is>
+          <t>$PANW Will she stop at 300, or do we get a measured move down......   I dunno, but I am leaving a runner.</t>
+        </is>
+      </c>
+      <c r="D1450" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1451" s="3" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C1451" s="3" t="inlineStr">
+        <is>
+          <t>$PANW cc not going well?😅,   but mom it was 180s , just 3 weeks ago🤭</t>
+        </is>
+      </c>
+      <c r="D1451" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1452" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1452" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN another idiot re-share instead of commenting 🙄</t>
+        </is>
+      </c>
+      <c r="D1452" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1453" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1453" s="3" t="inlineStr">
+        <is>
+          <t>By the $GOOGL is diluting its shares perhaps they are not confident that much on RoI.  $MSFT is not $GOOGL   I see $ORCL and $AMZN as  well down in sympathy</t>
+        </is>
+      </c>
+      <c r="D1453" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1454" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1454" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN @Ron_Burn   Read the chart properly...too late to report.  The move already happened and 258/255 will act as support and will bounce back from there</t>
+        </is>
+      </c>
+      <c r="D1454" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1455" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1455" s="3" t="inlineStr">
+        <is>
+          <t>Stocks with most action after hours $ANY $DBGI $DELL $GOOGL $AMZN</t>
+        </is>
+      </c>
+      <c r="D1455" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1456" s="4" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1456" s="4" t="inlineStr">
+        <is>
+          <t>$AMZN this indicator at the top never fails, pair it with MACD and can tell where this is heading</t>
+        </is>
+      </c>
+      <c r="D1456" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1457" s="2" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1457" s="2" t="inlineStr">
+        <is>
+          <t>$AMZN Per Gemini Ai (can be wrong, but push back, brings the same answers):  1. Redundancy is a National Security RequirementThe U.S. military heavily relies on low-Earth orbit satellites for encrypted communication, battlefield tracking, and drone operations.  The Single-Point-o</t>
+        </is>
+      </c>
+      <c r="D1457" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1458" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1458" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN fake drop</t>
+        </is>
+      </c>
+      <c r="D1458" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1459" s="4" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1459" s="4" t="inlineStr">
+        <is>
+          <t>$GOOGL 350 tomorrow   The sell off from 400 is going to come and before you know a 300 number in range   This $AMZN $META are just ATM’s to chip and memory companies   Extremely</t>
+        </is>
+      </c>
+      <c r="D1459" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1460" s="3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1460" s="3" t="inlineStr">
+        <is>
+          <t>$AMZN May Retest 255 level before reaching 280 EOW</t>
+        </is>
+      </c>
+      <c r="D1460" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1461" s="2" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C1461" s="2" t="inlineStr">
+        <is>
+          <t>$AMZN should be 3.5T mkt cap.</t>
+        </is>
+      </c>
+      <c r="D1461" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1462" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1462" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX Gap fill?</t>
+        </is>
+      </c>
+      <c r="D1462" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1463" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1463" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX volume is s real!!!</t>
+        </is>
+      </c>
+      <c r="D1463" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1464" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1464" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX I think I get it now. I don’t know who yet but I think AI will wipe out this company, it’s the only explination for this trading like it’s going bankrupt</t>
+        </is>
+      </c>
+      <c r="D1464" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1465" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1465" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX Maybe add shares here, but theres no way to find a bottom and buy call options right now.</t>
+        </is>
+      </c>
+      <c r="D1465" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1466" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1466" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX non stop selling….</t>
+        </is>
+      </c>
+      <c r="D1466" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1467" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1467" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX   7-12% green day incoming soon</t>
+        </is>
+      </c>
+      <c r="D1467" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1468" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1468" s="3" t="inlineStr">
+        <is>
+          <t>@jenbunn @Jeremymartin007 @simon58 @judgeyoung2 @cubie @ribbey @EBE_day @TraderRapp @Godreal1 @tonyctl same for $NFLX</t>
+        </is>
+      </c>
+      <c r="D1468" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1469" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1469" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX around $75.20 would be a 50% retracement of the move up from the May 2022 low. That would surely turn some heads   We’re still a ways off from that though.</t>
+        </is>
+      </c>
+      <c r="D1469" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1470" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1470" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX these fuckers should ask  Nvdia ceo Jensen to visit office for stock price boost!!!!  $SPY $NVDA</t>
+        </is>
+      </c>
+      <c r="D1470" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:36 ET</t>
+        </is>
+      </c>
+      <c r="B1471" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C1471" s="3" t="inlineStr">
+        <is>
+          <t>$NFLX looks like we have a squeeze coming soonish. up or down? IDK but seems like good risk/reward down here. 78 is also an enticing entry point.</t>
+        </is>
+      </c>
+      <c r="D1471" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -31029,177 +32855,177 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -31209,31 +33035,31 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-01 21:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -31243,7 +33069,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
@@ -31420,24 +33246,24 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -31447,48 +33273,48 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -31505,24 +33331,24 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -31539,58 +33365,58 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>RIVN</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -31607,7 +33433,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -31624,7 +33450,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -31641,7 +33467,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -31651,14 +33477,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -31668,14 +33494,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -31692,7 +33518,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -31702,14 +33528,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -31719,14 +33545,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -31736,14 +33562,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -31753,14 +33579,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -31770,14 +33596,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>PUSA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -31787,14 +33613,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RIVN</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -31804,14 +33630,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -31821,14 +33647,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -31853,7 +33679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -31919,10 +33745,20 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>52W_HIGH</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>52W_LOW</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>SECTOR</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>INDUSTRY</t>
         </is>
@@ -31931,7 +33767,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -31941,17 +33777,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10.69</t>
+          <t>10.58</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>44,287,617</t>
+          <t>45,605,586</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -31961,17 +33797,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7.27</t>
+          <t>6.97</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>6.26B</t>
+          <t>6.20B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>93.17</t>
+          <t>92.99</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -31981,10 +33817,20 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>10.332.40%</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>3.12239.03%</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Software - Infrastructure</t>
         </is>
@@ -31993,7 +33839,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -32003,17 +33849,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>487.97</t>
+          <t>489.04</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.33%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>14,053,254</t>
+          <t>14,425,560</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -32023,17 +33869,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>1.88</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2310.38B</t>
+          <t>2315.44B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>76.01</t>
+          <t>76.21</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -32043,10 +33889,20 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>488.820.05%</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>241.11102.83%</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Semiconductors</t>
         </is>
@@ -32055,7 +33911,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -32065,17 +33921,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.30</t>
+          <t>6.27</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.69%</t>
+          <t>2.13%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>21,811,967</t>
+          <t>22,343,156</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -32085,17 +33941,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3.81B</t>
+          <t>3.79B</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>83.85</t>
+          <t>83.65</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -32105,10 +33961,20 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>6.60-4.98%</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0.70795.86%</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Information Technology Services</t>
         </is>
@@ -32117,7 +33983,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -32127,17 +33993,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>306.98</t>
+          <t>307.32</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.57%</t>
+          <t>5.68%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>61,694,318</t>
+          <t>62,811,161</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -32147,17 +34013,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7.15</t>
+          <t>6.83</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>268.55B</t>
+          <t>268.84B</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>87.28</t>
+          <t>87.31</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -32167,10 +34033,20 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>291.305.50%</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>61.15402.57%</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Semiconductors</t>
         </is>
@@ -32179,7 +34055,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -32189,17 +34065,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17.93</t>
+          <t>17.87</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>3.35%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23,382,726</t>
+          <t>23,907,991</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -32209,17 +34085,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2.70</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>22.60B</t>
+          <t>22.52B</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>72.15</t>
+          <t>71.88</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -32229,10 +34105,20 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>22.69-21.24%</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>11.5754.45%</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Consumer Cyclical</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Auto Manufacturers</t>
         </is>
@@ -32241,7 +34127,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -32251,17 +34137,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.53</t>
+          <t>10.69</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>17.96%</t>
+          <t>19.76%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1,370,089</t>
+          <t>1,404,168</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -32271,17 +34157,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>7.80</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>927.07M</t>
+          <t>941.27M</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>56.98</t>
+          <t>57.83</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -32291,10 +34177,20 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>11.62-7.96%</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2.81280.60%</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Biotechnology</t>
         </is>
@@ -32303,7 +34199,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -32313,17 +34209,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>426.50</t>
+          <t>427.13</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-3.36%</t>
+          <t>-3.21%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14,021,404</t>
+          <t>14,687,631</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -32333,17 +34229,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3168.24B</t>
+          <t>3172.91B</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>52.22</t>
+          <t>52.50</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -32353,10 +34249,20 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
+          <t>555.45-23.10%</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>356.2819.89%</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Software - Infrastructure</t>
         </is>
@@ -32365,7 +34271,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -32375,17 +34281,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>282.17</t>
+          <t>282.81</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-5.05%</t>
+          <t>-4.84%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>6,994,189</t>
+          <t>7,159,216</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -32395,17 +34301,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.83</t>
+          <t>2.72</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>230.25B</t>
+          <t>230.77B</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>70.63</t>
+          <t>71.02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -32415,10 +34321,20 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>302.95-6.65%</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>139.57102.63%</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Software - Infrastructure</t>
         </is>
@@ -32427,7 +34343,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -32437,17 +34353,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>250.64</t>
+          <t>250.85</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-2.29%</t>
+          <t>-2.21%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15,734,373</t>
+          <t>16,576,437</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -32457,17 +34373,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2696.16B</t>
+          <t>2698.42B</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>39.83</t>
+          <t>39.98</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -32477,10 +34393,20 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>278.56-9.95%</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>196.0027.98%</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>Consumer Cyclical</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Internet Retail</t>
         </is>
@@ -32489,7 +34415,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -32499,17 +34425,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81.73</t>
+          <t>81.64</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-1.92%</t>
+          <t>-2.02%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>11,587,811</t>
+          <t>12,080,326</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -32519,17 +34445,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>344.14B</t>
+          <t>343.79B</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>27.47</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -32539,10 +34465,20 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t>134.12-39.12%</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>75.018.85%</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Entertainment</t>
         </is>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 20:43 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1471"/>
+  <dimension ref="A1:D1571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -32811,6 +32811,2206 @@
         </is>
       </c>
       <c r="D1471" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1472" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1472" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO MRVL about to send this to $600 this week.</t>
+        </is>
+      </c>
+      <c r="D1472" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1473" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1473" s="3" t="inlineStr">
+        <is>
+          <t>Earnings season is heating up:  $HPE is being compared with $DELL as investors watch enterprise trends.  Next key names: $AVGO, $PANW  The biggest market mover will likely be $ORCL.</t>
+        </is>
+      </c>
+      <c r="D1473" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1474" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1474" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL $AVGO  how will the overnight pump of Marvell , impact Broadcom’s price action tomorrow pre and post ER?</t>
+        </is>
+      </c>
+      <c r="D1474" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1475" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1475" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO over $500 this week</t>
+        </is>
+      </c>
+      <c r="D1475" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1476" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1476" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO $520 after er makes me $45K in profit</t>
+        </is>
+      </c>
+      <c r="D1476" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1477" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1477" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL $NVDA $AVGO $QCOM $INTC</t>
+        </is>
+      </c>
+      <c r="D1477" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1478" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1478" s="3" t="inlineStr">
+        <is>
+          <t>$JPM’s channel checks on MediaTek today are interesting.    The key takeaway:    $GOOGL appears to be scaling TPU deployment significantly higher.    Last week, Aletheia and Susquehanna also noted MTK gaining share in the TPU supply chain versus $AVGO.    But the cleaner trade ma</t>
+        </is>
+      </c>
+      <c r="D1478" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1479" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1479" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL $NVDA $MU $AVGO $TSM Everyday it’s a pump. PUMP PUMP PUMP.</t>
+        </is>
+      </c>
+      <c r="D1479" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1480" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1480" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO $INTC $MRVL $NVDA $QCOM</t>
+        </is>
+      </c>
+      <c r="D1480" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1481" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1481" s="3" t="inlineStr">
+        <is>
+          <t>@Wallstreetbest0708 easy look at $AVGO and this is at $180B ; DSP, Photonics and ASIC all 3 blended as industry standard ; this one is easy 10x even from here imho ; NFA ;</t>
+        </is>
+      </c>
+      <c r="D1481" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1482" s="4" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1482" s="4" t="inlineStr">
+        <is>
+          <t>$NOW $110 —&amp;gt; $100</t>
+        </is>
+      </c>
+      <c r="D1482" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1483" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1483" s="3" t="inlineStr">
+        <is>
+          <t>$NOW honestly just cruel</t>
+        </is>
+      </c>
+      <c r="D1483" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1484" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1484" s="3" t="inlineStr">
+        <is>
+          <t>$NOW Meh I’ll buy some more at $109</t>
+        </is>
+      </c>
+      <c r="D1484" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1485" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1485" s="3" t="inlineStr">
+        <is>
+          <t>$IGV $NOW $ZS $CRWD  this market is the biggest scam ever lol. Crowdstrike is up 50+% YTD while all other software is down 30%+. Explain to me how crowdstrike coming back to the pack sinks everything else lower</t>
+        </is>
+      </c>
+      <c r="D1485" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1486" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1486" s="3" t="inlineStr">
+        <is>
+          <t>$NOW I am really feel sorry on behalf of all bulls holding this stock. This is hell. Don’t invest a dollar in this. Don’t give these guys liquidity. Been holding this for 11 months of absolute hell. No other stock have been this volatile. Every day 3-5% moves for 11 months straig</t>
+        </is>
+      </c>
+      <c r="D1486" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1487" s="4" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1487" s="4" t="inlineStr">
+        <is>
+          <t>$NOW had no business pumping</t>
+        </is>
+      </c>
+      <c r="D1487" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1488" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1488" s="3" t="inlineStr">
+        <is>
+          <t>$NOW can we get 103 for a rebuy?</t>
+        </is>
+      </c>
+      <c r="D1488" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1489" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1489" s="3" t="inlineStr">
+        <is>
+          <t>$NOW 112</t>
+        </is>
+      </c>
+      <c r="D1489" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1490" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1490" s="3" t="inlineStr">
+        <is>
+          <t>$NOW Falls even faster AH!</t>
+        </is>
+      </c>
+      <c r="D1490" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1491" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C1491" s="3" t="inlineStr">
+        <is>
+          <t>$NOW $CRM $CRWD $ADBE this goes for your bastards as well. Utter trash getting abused like this</t>
+        </is>
+      </c>
+      <c r="D1491" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1492" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1492" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO  $CRWD  20% downside from here</t>
+        </is>
+      </c>
+      <c r="D1492" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1493" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1493" s="3" t="inlineStr">
+        <is>
+          <t>$CRWD a beat a raise and stock split and still not good enough</t>
+        </is>
+      </c>
+      <c r="D1493" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1494" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1494" s="3" t="inlineStr">
+        <is>
+          <t>$RBRK Sold almost all at $85 so I’m ok here. Had a bad $CRWD entry yesterday that was functioning under the “Ok, stonks only go up” thesis we’ve had since March 30th. The easy money has been made during a monster run for cybersecurity, now we get to sharpen our skills again.</t>
+        </is>
+      </c>
+      <c r="D1494" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1495" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1495" s="3" t="inlineStr">
+        <is>
+          <t>$INOD oof. Looks like we may have hit the wall with AI and semi? $AVGO and $CRWD has decent ER but falling AH. Bit surprised and was expecting similar move like $DELL last week.</t>
+        </is>
+      </c>
+      <c r="D1495" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1496" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1496" s="3" t="inlineStr">
+        <is>
+          <t>PickAlpha Midday:  CrowdStrike’s quarter was not a blowout, but the AI security narrative is getting stronger. The company guided Q2 revenue to $1.436B-$1.442B, reported Q1 revenue up 26% to $1.39B, and announced a 4-for-1 stock split as investors keep paying for cyber names posi</t>
+        </is>
+      </c>
+      <c r="D1496" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1497" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1497" s="3" t="inlineStr">
+        <is>
+          <t>$CRWD don’t trust ah moves</t>
+        </is>
+      </c>
+      <c r="D1497" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1498" s="2" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1498" s="2" t="inlineStr">
+        <is>
+          <t>$ZS This is a better value and buy at this price than $CRWD which will soon see $520 to $550</t>
+        </is>
+      </c>
+      <c r="D1498" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1499" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1499" s="3" t="inlineStr">
+        <is>
+          <t>$IGV $NOW $ZS $CRWD  this market is the biggest scam ever lol. Crowdstrike is up 50+% YTD while all other software is down 30%+. Explain to me how crowdstrike coming back to the pack sinks everything else lower</t>
+        </is>
+      </c>
+      <c r="D1499" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1500" s="4" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1500" s="4" t="inlineStr">
+        <is>
+          <t>$CRWD getting killed....</t>
+        </is>
+      </c>
+      <c r="D1500" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1501" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1501" s="3" t="inlineStr">
+        <is>
+          <t>$AMD $AVGO and $CRWD thats why you trim.  especially when you are playing with house money</t>
+        </is>
+      </c>
+      <c r="D1501" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1502" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1502" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN 🔥🔥🔥</t>
+        </is>
+      </c>
+      <c r="D1502" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1503" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1503" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN either back to $15 or $30. Take your pick</t>
+        </is>
+      </c>
+      <c r="D1503" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1504" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1504" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN</t>
+        </is>
+      </c>
+      <c r="D1504" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1505" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1505" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN Send it, $20 coming soon! https://www.reddit.com/r/RIVNstock/s/d8vcE3jL2e</t>
+        </is>
+      </c>
+      <c r="D1505" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1506" s="4" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1506" s="4" t="inlineStr">
+        <is>
+          <t>$SNDK $RIVN  pretty similar hype and 80% crash in 6 months</t>
+        </is>
+      </c>
+      <c r="D1506" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1507" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1507" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN I strongly feel it’ll play the $17.50 - $18.50 area (wide I know) with the hype built up for highly anticipated R2 release on the 9th.</t>
+        </is>
+      </c>
+      <c r="D1507" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1508" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1508" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN we have to break 18.5 with CONVICTION AND HOLD.</t>
+        </is>
+      </c>
+      <c r="D1508" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1509" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1509" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN where does it go from here is the question   Shorts/longs   Any ideas ??????  Don’t be bias   Just logical ????</t>
+        </is>
+      </c>
+      <c r="D1509" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1510" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1510" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN $BB profits taken to RIVN. 😏</t>
+        </is>
+      </c>
+      <c r="D1510" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1511" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1511" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN https://finance.yahoo.com/markets/stocks/articles/tesla-selling-worlds-most-efficient-142728186.html</t>
+        </is>
+      </c>
+      <c r="D1511" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1512" s="4" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1512" s="4" t="inlineStr">
+        <is>
+          <t>$PYPL they/them-pal.  Whew</t>
+        </is>
+      </c>
+      <c r="D1512" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1513" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1513" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL PayFall</t>
+        </is>
+      </c>
+      <c r="D1513" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1514" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1514" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL this really is a value trap  🪤</t>
+        </is>
+      </c>
+      <c r="D1514" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1515" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1515" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL how I’m so angry and how much much money I lost on this</t>
+        </is>
+      </c>
+      <c r="D1515" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1516" s="2" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1516" s="2" t="inlineStr">
+        <is>
+          <t>$PYPL   Trending  is  the most exciting thing  stockholders  have  had in  years,  lol.</t>
+        </is>
+      </c>
+      <c r="D1516" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1517" s="2" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1517" s="2" t="inlineStr">
+        <is>
+          <t>@jimmieB LMAO!! Everything is possible but you have to be realistic. At $20 $PYPL will be trading based on cash on hand as it’s PE will be around 3. At $42 it has a PE of 7</t>
+        </is>
+      </c>
+      <c r="D1517" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1518" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1518" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL Most millennials still hold PayPal accounts as we&amp;#39;re all approaching peak spend as a demographic. The inability to capitalize on that would be catastrophic and utterly disgraceful. 😆🙄🫩</t>
+        </is>
+      </c>
+      <c r="D1518" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1519" s="2" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1519" s="2" t="inlineStr">
+        <is>
+          <t>$PYPL why is this trending ?</t>
+        </is>
+      </c>
+      <c r="D1519" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1520" s="2" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1520" s="2" t="inlineStr">
+        <is>
+          <t>$PYPL DEEP value turn around. Congress is buying this will double in 1 year.</t>
+        </is>
+      </c>
+      <c r="D1520" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1521" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C1521" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL 8 pe, makes you think what if it gets to 1 pe? lol</t>
+        </is>
+      </c>
+      <c r="D1521" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1522" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1522" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL my only mistake is I did not buy more shares earlier this year when they were at $70 per share. What a mistake I made I should’ve doubled down. ￼</t>
+        </is>
+      </c>
+      <c r="D1522" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1523" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1523" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL I don’t have a crystal ball, but I believe Jensen has earned credibility. When the guy leading the company at the center of the AI revolution says Marvell is positioned to be a future trillion-dollar company, I’m comfortable holding my shares and letting the story play out.</t>
+        </is>
+      </c>
+      <c r="D1523" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1524" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1524" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL why</t>
+        </is>
+      </c>
+      <c r="D1524" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1525" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1525" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL $400.00🚀🚀🚀🚀🚀🚀🚀🚀🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D1525" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1526" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1526" s="3" t="inlineStr">
+        <is>
+          <t>$DJT $AVGO $MRVL $QQQ $SOXX</t>
+        </is>
+      </c>
+      <c r="D1526" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1527" s="4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1527" s="4" t="inlineStr">
+        <is>
+          <t>$MRVL same move as Dell</t>
+        </is>
+      </c>
+      <c r="D1527" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1528" s="4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1528" s="4" t="inlineStr">
+        <is>
+          <t>$MRVL -10 percent tomorrow</t>
+        </is>
+      </c>
+      <c r="D1528" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1529" s="4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1529" s="4" t="inlineStr">
+        <is>
+          <t>$MRVL late bullls holding bags congratulations</t>
+        </is>
+      </c>
+      <c r="D1529" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1530" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1530" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL correct me if I’m wrong but doesn’t NVDA own shares of Marvel? SEC? Investigation.</t>
+        </is>
+      </c>
+      <c r="D1530" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1531" s="4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1531" s="4" t="inlineStr">
+        <is>
+          <t>$MRVL slowly bleeding</t>
+        </is>
+      </c>
+      <c r="D1531" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1532" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1532" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR obviously that was merely a test to give the market reaction.  The real dump is coming very soon</t>
+        </is>
+      </c>
+      <c r="D1532" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1533" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1533" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR is holding up too well for this move to be real</t>
+        </is>
+      </c>
+      <c r="D1533" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1534" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1534" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR</t>
+        </is>
+      </c>
+      <c r="D1534" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1535" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1535" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR SHORTS GOT TRAPPED</t>
+        </is>
+      </c>
+      <c r="D1535" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1536" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1536" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR $MSTY $WNTR  Goodtimes</t>
+        </is>
+      </c>
+      <c r="D1536" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1537" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1537" s="4" t="inlineStr">
+        <is>
+          <t>$MSTR  kind of holding up while $BTC.X  is tanking is just an illusion. Be careful. Strategy is heavily connected to Bitcoin, the rug can be pulled at any moment, especially when you can&amp;#39;t get out, after hours is a real thing.      Now is the time to be on the sidelines. We a</t>
+        </is>
+      </c>
+      <c r="D1537" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1538" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1538" s="2" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR</t>
+        </is>
+      </c>
+      <c r="D1538" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1539" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1539" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR didn’t they just buy in the last few months too? why is them selling a small amount even news? $BTC.X</t>
+        </is>
+      </c>
+      <c r="D1539" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1540" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1540" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR fuk u and all your dip buyers 🖕🏽</t>
+        </is>
+      </c>
+      <c r="D1540" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1541" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1541" s="3" t="inlineStr">
+        <is>
+          <t>This is the second time Strategy has ever sold bitcoin and comes soon after the company announced a pivot from Saylor’s longstanding “never sell” strategy in favor of actively managing its balance sheet. That includes potentially selling bitcoin if it improves bitcoin-per-share m</t>
+        </is>
+      </c>
+      <c r="D1541" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1542" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1542" s="2" t="inlineStr">
+        <is>
+          <t>$WMT Earnings from 2 weeks ago was a beat but I think the market was been more focused on the tech sector as of late.  Time to buy this monster.</t>
+        </is>
+      </c>
+      <c r="D1542" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1543" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1543" s="3" t="inlineStr">
+        <is>
+          <t>As I always say, anything below $1000.00 is a conviction buying opportunity. Began this round of trading with the recent dip below $970 a couple of days ago. Several trades and the final position sold after hours today $969.50.     Feel free to scroll my feed to see other trading</t>
+        </is>
+      </c>
+      <c r="D1543" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1544" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1544" s="3" t="inlineStr">
+        <is>
+          <t>$WMT i got my money!  $480 good enough for yeoman’s work</t>
+        </is>
+      </c>
+      <c r="D1544" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1545" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1545" s="2" t="inlineStr">
+        <is>
+          <t>$WMT fill in the gap with a big V reversal next week.</t>
+        </is>
+      </c>
+      <c r="D1545" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1546" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1546" s="2" t="inlineStr">
+        <is>
+          <t>$WMT hahaha.. look at this shit.. lol</t>
+        </is>
+      </c>
+      <c r="D1546" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1547" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1547" s="3" t="inlineStr">
+        <is>
+          <t>$WMT</t>
+        </is>
+      </c>
+      <c r="D1547" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1548" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1548" s="2" t="inlineStr">
+        <is>
+          <t>$WMT oh yeah baby</t>
+        </is>
+      </c>
+      <c r="D1548" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1549" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1549" s="3" t="inlineStr">
+        <is>
+          <t>$WMT might be onto something here</t>
+        </is>
+      </c>
+      <c r="D1549" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1550" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1550" s="3" t="inlineStr">
+        <is>
+          <t>$WMT F U shorts!!!!</t>
+        </is>
+      </c>
+      <c r="D1550" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1551" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1551" s="2" t="inlineStr">
+        <is>
+          <t>$WMT 120 by Friday</t>
+        </is>
+      </c>
+      <c r="D1551" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1552" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1552" s="3" t="inlineStr">
+        <is>
+          <t>$AI If we all hate bears, we sould all buy this stock and short squeeze it.   30-40% Shorts right now on this company, which is crazy.</t>
+        </is>
+      </c>
+      <c r="D1552" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1553" s="4" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1553" s="4" t="inlineStr">
+        <is>
+          <t>$AI $0 soon</t>
+        </is>
+      </c>
+      <c r="D1553" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1554" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1554" s="3" t="inlineStr">
+        <is>
+          <t>$AI   Fiscal 2026 revenue was $250.3 million, with $227.1 million from subscriptions.   GAAP net loss was $470.4 million, or $3.35 per share, while non-GAAP net loss was $189.7 million, or $1.35 per share.   Fiscal fourth quarter revenue was $51.6 million, with subscription reven</t>
+        </is>
+      </c>
+      <c r="D1554" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1555" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1555" s="2" t="inlineStr">
+        <is>
+          <t>$AI</t>
+        </is>
+      </c>
+      <c r="D1555" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1556" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1556" s="3" t="inlineStr">
+        <is>
+          <t>$AI  Sell sell sell Buy later no upgrading from analysis  Sell sell sell please  Bull team we can buy lower</t>
+        </is>
+      </c>
+      <c r="D1556" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1557" s="4" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1557" s="4" t="inlineStr">
+        <is>
+          <t>$AI</t>
+        </is>
+      </c>
+      <c r="D1557" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1558" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1558" s="2" t="inlineStr">
+        <is>
+          <t>$AI call soon</t>
+        </is>
+      </c>
+      <c r="D1558" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1559" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1559" s="3" t="inlineStr">
+        <is>
+          <t>$AI whatever. grats</t>
+        </is>
+      </c>
+      <c r="D1559" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1560" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1560" s="3" t="inlineStr">
+        <is>
+          <t>$AI  I almost ignored this, which would have been a mistake.</t>
+        </is>
+      </c>
+      <c r="D1560" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1561" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1561" s="2" t="inlineStr">
+        <is>
+          <t>$DGXX $AI $CLSK $USO general</t>
+        </is>
+      </c>
+      <c r="D1561" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1562" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1562" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX You must have the biggest short position of all time then, I assume</t>
+        </is>
+      </c>
+      <c r="D1562" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1563" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1563" s="2" t="inlineStr">
+        <is>
+          <t>$ABVX added on this drop.  Amazing efficacy with some questionable safety signals.  They have data going back years from other trials without any safety issues…. Seems like an over reaction that may take some time to play out…</t>
+        </is>
+      </c>
+      <c r="D1563" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1564" s="4" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1564" s="4" t="inlineStr">
+        <is>
+          <t>$ABVX gap fill back down to $10 is coming.</t>
+        </is>
+      </c>
+      <c r="D1564" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1565" s="4" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1565" s="4" t="inlineStr">
+        <is>
+          <t>$ABVX 90 percent drop tomorrow</t>
+        </is>
+      </c>
+      <c r="D1565" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1566" s="4" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1566" s="4" t="inlineStr">
+        <is>
+          <t>$VKTX $ABVX Moment coming soon to a VIKING theatre near you!</t>
+        </is>
+      </c>
+      <c r="D1566" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1567" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1567" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX Biotech been crap recently. Looks like the money is flowing on AI stocks.</t>
+        </is>
+      </c>
+      <c r="D1567" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1568" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1568" s="2" t="inlineStr">
+        <is>
+          <t>$ABVX Still, an overreaction</t>
+        </is>
+      </c>
+      <c r="D1568" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1569" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1569" s="2" t="inlineStr">
+        <is>
+          <t>@Rafael_ Uhhhh, that&amp;#39;s a solid no.  Lame attempt. $ABVX just strengthened their balance sheet.</t>
+        </is>
+      </c>
+      <c r="D1569" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1570" s="2" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1570" s="2" t="inlineStr">
+        <is>
+          <t>@MZ2X Looks like a scripted sell the news with great data and a distraction of having 3 subjects out of over 400 develop some form of skin cancer (simplified) with no signs of any ties to the trial.  Truly a gift here on $ABVX.      Massive potential remains.  Buyout watch-list r</t>
+        </is>
+      </c>
+      <c r="D1570" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B1571" s="3" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C1571" s="3" t="inlineStr">
+        <is>
+          <t>$ABVX as good as Rinvoq = not good enough</t>
+        </is>
+      </c>
+      <c r="D1571" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -32827,7 +35027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32855,24 +35055,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>98</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -32889,17 +35089,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
@@ -32911,12 +35111,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>86</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
@@ -32991,58 +35191,58 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -33052,7 +35252,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-01 21:58 UTC</t>
         </is>
       </c>
     </row>
@@ -33081,12 +35281,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>44</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
@@ -33127,29 +35327,29 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>RIVN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -33161,24 +35361,24 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -33188,14 +35388,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -33205,14 +35405,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -33222,14 +35422,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -33239,14 +35439,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -33256,31 +35456,31 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -33290,48 +35490,48 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -33348,24 +35548,24 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -33382,24 +35582,24 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RIVN</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -33409,7 +35609,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 00:59 UTC</t>
         </is>
       </c>
     </row>
@@ -33665,6 +35865,91 @@
       <c r="C49" t="inlineStr">
         <is>
           <t>2026-06-03 11:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
@@ -33679,7 +35964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -34484,6 +36769,726 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>479.23</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>-0.49%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>41,034,114</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>24.17M</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1.70</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2268.99B</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>73.33</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>488.82-1.96%</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>241.1198.76%</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>117.90</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-7.64%</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>33,150,378</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>26.10M</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1.27</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>121.59B</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>59.57</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>211.48-44.25%</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>81.2445.13%</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>747.61</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-2.78%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4,767,847</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>3.61M</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>190.29B</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>76.31</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>785.66-4.84%</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>342.72118.14%</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>18.27</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>5.67%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>51,405,545</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>29.00M</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>23.03B</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>73.57</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>22.69-19.48%</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>11.5757.91%</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>42.61</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>19,164,491</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>15.45M</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>37.59B</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>32.57</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>79.50-46.40%</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>38.4610.79%</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Credit Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>301.65</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3.73%</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>111,297,058</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>28.91M</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3.85</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>263.88B</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>86.85</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>291.303.55%</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>61.15393.30%</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>126.54</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>-7.01%</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>20,215,966</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>18.40M</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>44.35B</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>30.50</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>457.22-72.32%</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>104.1721.49%</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>116.89</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3.39%</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>29,902,488</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>19.91M</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>930.22B</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>36.35</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>0.60</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>135.15-13.51%</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>93.4325.11%</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Discount Stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>10.71</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>-4.20%</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>17,517,417</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>5.15M</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1.56B</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>61.17</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>30.11-64.43%</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>7.6839.54%</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ABVX</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>90.15</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>24.34%</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>7,145,757</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1.35M</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>5.31</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>7.18B</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>36.44</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>148.83-39.43%</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>5.691484.36%</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-03 23:41 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1571"/>
+  <dimension ref="A1:D1671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -35011,6 +35011,2206 @@
         </is>
       </c>
       <c r="D1571" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1572" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1572" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO that was a quick move up to 450 to 480 .. if they smash earnings avgo will go 540 ? .. no idea at this point but it&amp;#39;s a fun ride so far</t>
+        </is>
+      </c>
+      <c r="D1572" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1573" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1573" s="3" t="inlineStr">
+        <is>
+          <t>$CBRS Cathie Wood&amp;#39;s ARK, with may others, think $NVDA, $AVGO and Cerebras are the best AI chip stocks for the near future. She keeps buying Cerebras since day1, heavy conviction, she is hoping to pull another $TSLA it seems</t>
+        </is>
+      </c>
+      <c r="D1573" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1574" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1574" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1574" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1575" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1575" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1575" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1576" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1576" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO looking to go big this week</t>
+        </is>
+      </c>
+      <c r="D1576" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1577" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1577" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO After watching $MRVL and $ARM I will be shocked if this doesnt get $550 Thursday.</t>
+        </is>
+      </c>
+      <c r="D1577" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1578" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1578" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1578" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1579" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1579" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1579" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1580" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1580" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1580" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1581" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1581" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO https://au.investing.com/news/stock-market-news/broadcom-unveils-broadband-edge-ai-portfolio-with-wifi-8-93CH-4465756</t>
+        </is>
+      </c>
+      <c r="D1581" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1582" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1582" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL let’s make it #1 trending !!😎🚀</t>
+        </is>
+      </c>
+      <c r="D1582" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1583" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1583" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL iT fOlLoWs bItCoIn</t>
+        </is>
+      </c>
+      <c r="D1583" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1584" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1584" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL 2.2GWs... Nice! Holding long.</t>
+        </is>
+      </c>
+      <c r="D1584" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1585" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1585" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL were just gonna start trending everyday until 20</t>
+        </is>
+      </c>
+      <c r="D1585" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1586" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1586" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL Where is that dumbass that says this followa BTC 😂</t>
+        </is>
+      </c>
+      <c r="D1586" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1587" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1587" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL I want to start a position but RSI at 80ish on daily and weekly.  Maybe small starter and add on a pullback?</t>
+        </is>
+      </c>
+      <c r="D1587" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1588" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1588" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL hmmm now the real question is what do I do with my 5$ June 18 calls. It might be time to cash in</t>
+        </is>
+      </c>
+      <c r="D1588" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1589" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1589" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL it’s feels like today 🤧🤧</t>
+        </is>
+      </c>
+      <c r="D1589" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1590" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1590" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL $10 before the 29th of June</t>
+        </is>
+      </c>
+      <c r="D1590" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1591" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1591" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL FLYYYY</t>
+        </is>
+      </c>
+      <c r="D1591" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1592" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1592" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI $BTC.X $MSTR $SPY $HOOD</t>
+        </is>
+      </c>
+      <c r="D1592" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1593" s="2" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1593" s="2" t="inlineStr">
+        <is>
+          <t>$SOFI dang, i look away and it&amp;#39;s down 6 more cents</t>
+        </is>
+      </c>
+      <c r="D1593" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1594" s="4" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1594" s="4" t="inlineStr">
+        <is>
+          <t>$SOFI oh look trending AGAIN. For the wrong reason ….</t>
+        </is>
+      </c>
+      <c r="D1594" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1595" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1595" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI oh just for funsies, gtfoh nobody cares.</t>
+        </is>
+      </c>
+      <c r="D1595" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1596" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1596" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI it’s a gift for the patient…</t>
+        </is>
+      </c>
+      <c r="D1596" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1597" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1597" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI   Many people know this is shit 💩 and are looking to get out as soon as breakeven.   Myself included.   Don’t care if ig goes up to a billion after I’m gone.</t>
+        </is>
+      </c>
+      <c r="D1597" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1598" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1598" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI inclusion not happening fsure now ….</t>
+        </is>
+      </c>
+      <c r="D1598" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1599" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1599" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI There are a lot of people trapped between here and $30+ dollars. The longer they stay trapped, the more eager they are to get out once given the opportunity. There is a lot of weight on the stock price. Not only do you have a short seller infestation… but you become exit li</t>
+        </is>
+      </c>
+      <c r="D1599" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1600" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1600" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI $$3.40 off the past weeks high time for a schwing …..</t>
+        </is>
+      </c>
+      <c r="D1600" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1601" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1601" s="3" t="inlineStr">
+        <is>
+          <t>$SOFI where’s the guy that said this would be enlisted in sp500 this month lol… 🤣</t>
+        </is>
+      </c>
+      <c r="D1601" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1602" s="2" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1602" s="2" t="inlineStr">
+        <is>
+          <t>$CADL the good Dr Tak is very active on X - spreading the good word as they say</t>
+        </is>
+      </c>
+      <c r="D1602" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1603" s="3" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1603" s="3" t="inlineStr">
+        <is>
+          <t>$CADL Close to 10K watchers.</t>
+        </is>
+      </c>
+      <c r="D1603" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1604" s="3" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1604" s="3" t="inlineStr">
+        <is>
+          <t>$CADL wheres the buyers?</t>
+        </is>
+      </c>
+      <c r="D1604" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1605" s="2" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1605" s="2" t="inlineStr">
+        <is>
+          <t>$CADL we skipping the 9s? We shouldnt be well into the 20s anyway... no need for 9s or 10s.</t>
+        </is>
+      </c>
+      <c r="D1605" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1606" s="3" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1606" s="3" t="inlineStr">
+        <is>
+          <t>$CADL It is time for the bulge bracket firms to join in on the game.  Think T Rowe Price, Janus Henderson, Franklin Templeton, Wellington, Dimensional, etc.  These are the types of players that he was meeting with at Jeffco, as well as smaller funds.  1m shares would be a starter</t>
+        </is>
+      </c>
+      <c r="D1606" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1607" s="2" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1607" s="2" t="inlineStr">
+        <is>
+          <t>$CADL #3 trending now. gonna be #1 at the bell</t>
+        </is>
+      </c>
+      <c r="D1607" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1608" s="3" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1608" s="3" t="inlineStr">
+        <is>
+          <t>$CADL how this isnt trading $12-$15 right now 🤷🏻‍♂️</t>
+        </is>
+      </c>
+      <c r="D1608" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1609" s="3" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1609" s="3" t="inlineStr">
+        <is>
+          <t>$CADL Nice. One of the few green ones. At breakeven now. Gidee up.</t>
+        </is>
+      </c>
+      <c r="D1609" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1610" s="2" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1610" s="2" t="inlineStr">
+        <is>
+          <t>$CADL  Above 9 again after hours.. All as expected in my weekly prediction for it in my live biotech group! ✅📈✅📈!</t>
+        </is>
+      </c>
+      <c r="D1610" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1611" s="3" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C1611" s="3" t="inlineStr">
+        <is>
+          <t>$CADL At least 1 of the 18 one-on-ones Tak had at Jeffco will turn into  buyers, particularly after they read the Cantor report and their $47 DCF target.  Ka&amp;#39;chng!</t>
+        </is>
+      </c>
+      <c r="D1611" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1612" s="2" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1612" s="2" t="inlineStr">
+        <is>
+          <t>$CRWD  -   CrowdStrike Delivers Beat-And-Raise Q1, Announces 4-For-1 Stock Split</t>
+        </is>
+      </c>
+      <c r="D1612" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1613" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1613" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $CRWD could not save the market...    I am sure Rigged Trump will come up with PECACE lie again and try to save ; but Market needs pull back like today - they necessary $SPY $QQQ</t>
+        </is>
+      </c>
+      <c r="D1613" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1614" s="4" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1614" s="4" t="inlineStr">
+        <is>
+          <t>$AVGO $SPY $QQQ $CRWD 🚨🚨🚨🤑🤑🤑</t>
+        </is>
+      </c>
+      <c r="D1614" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1615" s="2" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1615" s="2" t="inlineStr">
+        <is>
+          <t>$CRWD  -   https://www.benzinga.com/markets/earnings/26/06/52987804/crowdstrike-delivers-beat-and-raise-q1-announces-4-for-1-stock-split</t>
+        </is>
+      </c>
+      <c r="D1615" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1616" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1616" s="3" t="inlineStr">
+        <is>
+          <t>$CRWD the stock is splitting ???</t>
+        </is>
+      </c>
+      <c r="D1616" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1617" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1617" s="3" t="inlineStr">
+        <is>
+          <t>$CRWD with the shares doubling the last few months, without a beat and raise and split it would be down 300</t>
+        </is>
+      </c>
+      <c r="D1617" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1618" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1618" s="3" t="inlineStr">
+        <is>
+          <t>$IGV $NOW $ZS $CRWD Maybe ask Trump and his MAGA for allowing criminal cartel activity and getting kick-backs for this?🚨</t>
+        </is>
+      </c>
+      <c r="D1618" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1619" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1619" s="3" t="inlineStr">
+        <is>
+          <t>$CRWD  back to 550 .00 🥱</t>
+        </is>
+      </c>
+      <c r="D1619" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1620" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1620" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO   400  not far $CRWD   650 not far</t>
+        </is>
+      </c>
+      <c r="D1620" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1621" s="3" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1621" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not gonna lie… if this setup holds, I might wake up rich again tomorrow     All glory to my Heavenly Father above.     Been a crazy ride lately with $SPY and $CRWD moving like absolute maniacs.     One day the market humbles you… the next day it makes you feel unstoppable again. </t>
+        </is>
+      </c>
+      <c r="D1621" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1622" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1622" s="3" t="inlineStr">
+        <is>
+          <t>$QCOM $NVDA  Holding both of these but not kidding myself when the levy breaks pain will be felt across the entire sector.  $WMT could be a buy here</t>
+        </is>
+      </c>
+      <c r="D1622" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1623" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1623" s="2" t="inlineStr">
+        <is>
+          <t>$WMT if this thing goes to 135, im gonna go get porsche 911</t>
+        </is>
+      </c>
+      <c r="D1623" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1624" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1624" s="2" t="inlineStr">
+        <is>
+          <t>$WMT love to hear a Dividend Increase tomorrow on the Shareholders Day.  That will send this shit FLYING.  lol</t>
+        </is>
+      </c>
+      <c r="D1624" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1625" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1625" s="2" t="inlineStr">
+        <is>
+          <t>$WMT 120 on Thursday.  Lol</t>
+        </is>
+      </c>
+      <c r="D1625" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1626" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1626" s="3" t="inlineStr">
+        <is>
+          <t>$INTC That $AVGO drop looks pretty bad. If there is a sector rotation, it might be showing already. My $WMT position has gone up today. I&amp;#39;m not bearish on Intel, but this Broadcom drop can really do a number on other tech stocks</t>
+        </is>
+      </c>
+      <c r="D1626" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1627" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1627" s="3" t="inlineStr">
+        <is>
+          <t>$WMT added more today :)</t>
+        </is>
+      </c>
+      <c r="D1627" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1628" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1628" s="2" t="inlineStr">
+        <is>
+          <t>$WMT</t>
+        </is>
+      </c>
+      <c r="D1628" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1629" s="3" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1629" s="3" t="inlineStr">
+        <is>
+          <t>$WMT How long is this headline going to be accurate?   https://finance.yahoo.com/markets/stocks/articles/amazon-claims-no-1-spot-100000251.html</t>
+        </is>
+      </c>
+      <c r="D1629" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1630" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1630" s="2" t="inlineStr">
+        <is>
+          <t>$WMT Berkshire been loading with Alfred E Neuman.. BIG THINGS coming soon....</t>
+        </is>
+      </c>
+      <c r="D1630" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1631" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C1631" s="2" t="inlineStr">
+        <is>
+          <t>$WMT okay baby what’s going on I knew it</t>
+        </is>
+      </c>
+      <c r="D1631" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1632" s="4" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1632" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X complete destroying in half MONTH   🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣🤣  greatest criminal scam Pos fraud succcer stonk SCAM on EARTH 🤣🤡💩   $ETH $COIN $BMNR SPARTA INVESTMENT SHORT BIG TO CHAPTER 11 AND Below 🥳🥳🥳🥳🥳🥳🥳🥳🥳 Lambo Week</t>
+        </is>
+      </c>
+      <c r="D1632" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1633" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1633" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR  https://finance.yahoo.com/markets/crypto/articles/bitcoin-sinks-time-ethereum-outperform-223632917.html Let me think about it again.🤔</t>
+        </is>
+      </c>
+      <c r="D1633" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1634" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1634" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR   This is gonna go down towards 12&amp;#39;s.  I don&amp;#39;t see Eth bouncing at all.  Eth is gonna probably flat line around 1300&amp;#39;s.</t>
+        </is>
+      </c>
+      <c r="D1634" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1635" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1635" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR   This downward spiral is just way too predictable.</t>
+        </is>
+      </c>
+      <c r="D1635" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1636" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1636" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR $ETH.X Fucking Tom Lee, he gave a speech in Paris yesterday, towards the end, and I’m paraphrasing “We may decide to own more than 5%”.. this motherfucker is going to keep going..</t>
+        </is>
+      </c>
+      <c r="D1636" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1637" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1637" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR ok bot</t>
+        </is>
+      </c>
+      <c r="D1637" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1638" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1638" s="3" t="inlineStr">
+        <is>
+          <t>$INFQ  $BMNR  Im buying 500 shares tomorrow and hedging. .</t>
+        </is>
+      </c>
+      <c r="D1638" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1639" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1639" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR crypto stock is not the wave 🌊</t>
+        </is>
+      </c>
+      <c r="D1639" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1640" s="3" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1640" s="3" t="inlineStr">
+        <is>
+          <t>$BMNR    Crypto is dying a slow death — say no to ethereum</t>
+        </is>
+      </c>
+      <c r="D1640" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1641" s="2" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C1641" s="2" t="inlineStr">
+        <is>
+          <t>$BMNR on watch 👀</t>
+        </is>
+      </c>
+      <c r="D1641" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1642" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1642" s="3" t="inlineStr">
+        <is>
+          <t>$AI Tom S bought 6.17 million shares of C3 AI stock at a price of $11.16 per share.</t>
+        </is>
+      </c>
+      <c r="D1642" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1643" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1643" s="3" t="inlineStr">
+        <is>
+          <t>$AI damn! This was leading the Ai stock!! What happened here ?!?!?!</t>
+        </is>
+      </c>
+      <c r="D1643" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1644" s="4" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1644" s="4" t="inlineStr">
+        <is>
+          <t>$AI lmao!</t>
+        </is>
+      </c>
+      <c r="D1644" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1645" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1645" s="3" t="inlineStr">
+        <is>
+          <t>$AI only ones cooked are pumptards who did sell $12-$13 🤔😆  cubie nailed another one☺️😚</t>
+        </is>
+      </c>
+      <c r="D1645" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1646" s="4" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1646" s="4" t="inlineStr">
+        <is>
+          <t>$AI HAHAHAHAHAH</t>
+        </is>
+      </c>
+      <c r="D1646" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1647" s="4" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1647" s="4" t="inlineStr">
+        <is>
+          <t>$AI   I&amp;#39;m not greedy!  I will buy at  less than 50% of the stock price now.</t>
+        </is>
+      </c>
+      <c r="D1647" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1648" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1648" s="2" t="inlineStr">
+        <is>
+          <t>$AI hold now or chase it after the call</t>
+        </is>
+      </c>
+      <c r="D1648" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1649" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1649" s="2" t="inlineStr">
+        <is>
+          <t>$AI 15 tomorrow</t>
+        </is>
+      </c>
+      <c r="D1649" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1650" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1650" s="3" t="inlineStr">
+        <is>
+          <t>$NEON $AI $LAC Cc</t>
+        </is>
+      </c>
+      <c r="D1650" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1651" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C1651" s="3" t="inlineStr">
+        <is>
+          <t>$AI wow can’t hold up huh 😑</t>
+        </is>
+      </c>
+      <c r="D1651" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1652" s="3" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1652" s="3" t="inlineStr">
+        <is>
+          <t>$NTSK another 3 months of .....</t>
+        </is>
+      </c>
+      <c r="D1652" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1653" s="3" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1653" s="3" t="inlineStr">
+        <is>
+          <t>$NTSK going to 6</t>
+        </is>
+      </c>
+      <c r="D1653" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1654" s="3" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1654" s="3" t="inlineStr">
+        <is>
+          <t>$NTSK great numbers great calls, don’t be fooled.</t>
+        </is>
+      </c>
+      <c r="D1654" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1655" s="3" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1655" s="3" t="inlineStr">
+        <is>
+          <t>https://marketbeat.com/a/8691135/   $NTSK  Netskope Q1 Earnings Call Highlights</t>
+        </is>
+      </c>
+      <c r="D1655" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1656" s="2" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1656" s="2" t="inlineStr">
+        <is>
+          <t>$NTSK only $2 more to go ! LFG</t>
+        </is>
+      </c>
+      <c r="D1656" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1657" s="2" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1657" s="2" t="inlineStr">
+        <is>
+          <t>$NTSK if this can get back to $11 that would be good tomorrow..  Down 30% early was bullshit</t>
+        </is>
+      </c>
+      <c r="D1657" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1658" s="3" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1658" s="3" t="inlineStr">
+        <is>
+          <t>https://www.marketbeat.com/earnings/reports/2026-6-3-netskope-inc-stock/  $NTSK Netskope Earnings Transcript</t>
+        </is>
+      </c>
+      <c r="D1658" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1659" s="2" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1659" s="2" t="inlineStr">
+        <is>
+          <t>$NTSK 10 by morning is fine by me. It was a good call and report. FCF was mentioned and they expect it to be back positive in the second half. Takes money to make money</t>
+        </is>
+      </c>
+      <c r="D1659" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1660" s="2" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1660" s="2" t="inlineStr">
+        <is>
+          <t>$NTSK NUT SCRAPE living up to its name</t>
+        </is>
+      </c>
+      <c r="D1660" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1661" s="3" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="C1661" s="3" t="inlineStr">
+        <is>
+          <t>$NTSK fake pump then dump from institutional behaviour. **** Disgusting</t>
+        </is>
+      </c>
+      <c r="D1661" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1662" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1662" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN candles!</t>
+        </is>
+      </c>
+      <c r="D1662" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1663" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1663" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN I would say we send it to $20 now!</t>
+        </is>
+      </c>
+      <c r="D1663" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1664" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1664" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN More than half of active car shoppers are actively eyeing electric vehicles (EVs)</t>
+        </is>
+      </c>
+      <c r="D1664" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1665" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1665" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN don’t miss the opportunity is justbthr start  $TSLA $LCID $NIO $F</t>
+        </is>
+      </c>
+      <c r="D1665" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1666" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1666" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN model Y is the best selling EV perhaps in the world and it is but I needed something higher up and more utilitarian. R2 fits that.</t>
+        </is>
+      </c>
+      <c r="D1666" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1667" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1667" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN we’ll be trending soon. Gawd candles loading.</t>
+        </is>
+      </c>
+      <c r="D1667" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1668" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1668" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN PT raise, great PR’s. $18 feels more inevitable</t>
+        </is>
+      </c>
+      <c r="D1668" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1669" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1669" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN</t>
+        </is>
+      </c>
+      <c r="D1669" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1670" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1670" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN https://youtu.be/uzMHCFuFO-s?si=II2xrByBXk9F4QgW</t>
+        </is>
+      </c>
+      <c r="D1670" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+      <c r="B1671" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1671" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN the MMs are in super spoof mode</t>
+        </is>
+      </c>
+      <c r="D1671" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -35027,7 +37227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35072,24 +37272,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>96</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -35106,41 +37306,41 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -35150,7 +37350,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
@@ -35293,29 +37493,29 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>RIVN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -35327,46 +37527,46 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RIVN</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -35378,24 +37578,24 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -35405,14 +37605,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -35422,14 +37622,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -35439,14 +37639,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -35456,14 +37656,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -35473,87 +37673,87 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -35565,12 +37765,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -35582,92 +37782,92 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-03 00:59 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -35684,7 +37884,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -35701,7 +37901,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -35711,14 +37911,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -35728,14 +37928,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -35745,14 +37945,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -35762,14 +37962,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -35779,14 +37979,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -35796,14 +37996,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -35813,14 +38013,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -35830,14 +38030,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -35847,14 +38047,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>PUSA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -35864,14 +38064,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -35881,14 +38081,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -35898,14 +38098,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -35915,14 +38115,14 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -35939,7 +38139,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -35950,6 +38150,57 @@
       <c r="C54" t="inlineStr">
         <is>
           <t>2026-06-03 16:42 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
@@ -35964,7 +38215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36052,62 +38303,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10.58</t>
+          <t>479.23</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>-0.49%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>45,605,586</t>
+          <t>42,095,271</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>20.57M</t>
+          <t>24.17M</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6.97</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>6.20B</t>
+          <t>2268.99B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>92.99</t>
+          <t>73.33</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>10.332.40%</t>
+          <t>488.82</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3.12239.03%</t>
+          <t>241.1198</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -36117,69 +38368,69 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Semiconductors</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>489.04</t>
+          <t>6.15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>14,425,560</t>
+          <t>44,987,580</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>24.17M</t>
+          <t>34.62M</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.88</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2315.44B</t>
+          <t>3.71B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>76.21</t>
+          <t>82.88</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>488.820.05%</t>
+          <t>6.82</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>241.11102.83%</t>
+          <t>0.70778</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -36189,429 +38440,429 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>Information Technology Services</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6.27</t>
+          <t>16.68</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.13%</t>
+          <t>-5.98%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>22,343,156</t>
+          <t>72,837,765</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>34.62M</t>
+          <t>67.02M</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3.79B</t>
+          <t>21.40B</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>83.65</t>
+          <t>49.65</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>2.15</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>6.60-4.98%</t>
+          <t>49.04</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.70795.86%</t>
+          <t>13.2326</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Information Technology Services</t>
+          <t>Credit Services</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>307.32</t>
+          <t>8.80</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.68%</t>
+          <t>4.51%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>62,811,161</t>
+          <t>2,088,704</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>28.91M</t>
+          <t>1.74M</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6.83</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>268.84B</t>
+          <t>644.78M</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>87.31</t>
+          <t>67.98</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>291.305.50%</t>
+          <t>9.27</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>61.15402.57%</t>
+          <t>4.35102</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>Biotechnology</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RIVN</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17.87</t>
+          <t>747.61</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>-2.78%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23,907,991</t>
+          <t>4,836,752</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>29.00M</t>
+          <t>3.61M</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2.59</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>22.52B</t>
+          <t>190.29B</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>71.88</t>
+          <t>76.31</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>22.69-21.24%</t>
+          <t>785.66</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>11.5754.45%</t>
+          <t>342.72118</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Auto Manufacturers</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.69</t>
+          <t>116.89</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>19.76%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1,404,168</t>
+          <t>31,723,400</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>566.17K</t>
+          <t>19.91M</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7.80</t>
+          <t>1.59</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>941.27M</t>
+          <t>930.22B</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>57.83</t>
+          <t>36.35</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>11.62-7.96%</t>
+          <t>135.15</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2.81280.60%</t>
+          <t>93.4325</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Biotechnology</t>
+          <t>Discount Stores</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>427.13</t>
+          <t>16.90</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-3.21%</t>
+          <t>-5.95%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14,687,631</t>
+          <t>40,122,400</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>34.62M</t>
+          <t>41.29M</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3172.91B</t>
+          <t>9.63B</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>52.50</t>
+          <t>31.91</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>555.45-23.10%</t>
+          <t>161.00</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>356.2819.89%</t>
+          <t>3.92331</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Capital Markets</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>282.81</t>
+          <t>10.71</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-4.84%</t>
+          <t>-4.20%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>7,159,216</t>
+          <t>18,375,979</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.27M</t>
+          <t>5.15M</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.72</t>
+          <t>3.57</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>230.77B</t>
+          <t>1.56B</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>71.02</t>
+          <t>61.17</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>302.95-6.65%</t>
+          <t>64.43</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>139.57102.63%</t>
+          <t>7.6839</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -36628,864 +38879,144 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>250.85</t>
+          <t>12.40</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-2.21%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>16,576,437</t>
+          <t>13,691,184</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>44.96M</t>
+          <t>4.67M</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>2.93</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2698.42B</t>
+          <t>5.04B</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>39.98</t>
+          <t>60.30</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>278.56-9.95%</t>
+          <t>55.70</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>196.0027.98%</t>
+          <t>7.6661</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Internet Retail</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>RIVN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81.64</t>
+          <t>18.27</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-2.02%</t>
+          <t>5.67%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>12,080,326</t>
+          <t>51,430,372</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>38.82M</t>
+          <t>29.00M</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>343.79B</t>
+          <t>23.03B</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>27.47</t>
+          <t>73.57</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>134.12-39.12%</t>
+          <t>22.69</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>75.018.85%</t>
+          <t>11.5757</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Entertainment</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>479.23</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>-0.49%</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>41,034,114</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>24.17M</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>1.70</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2268.99B</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>73.33</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>1.43</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>488.82-1.96%</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>241.1198.76%</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Semiconductors</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>117.90</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>-7.64%</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>33,150,378</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>26.10M</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>1.27</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>121.59B</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>59.57</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>0.93</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>211.48-44.25%</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>81.2445.13%</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Software - Application</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>CRWD</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>747.61</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>-2.78%</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>4,767,847</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>3.61M</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>1.32</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>190.29B</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>76.31</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>785.66-4.84%</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>342.72118.14%</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Software - Infrastructure</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>RIVN</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>18.27</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>5.67%</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>51,405,545</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>29.00M</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>1.77</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>23.03B</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>73.57</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>22.69-19.48%</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>11.5757.91%</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
           <t>Auto Manufacturers</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PYPL</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>42.61</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>-4.31%</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>19,164,491</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>15.45M</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>37.59B</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>32.57</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>79.50-46.40%</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>38.4610.79%</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Financial Services</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Credit Services</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>301.65</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>3.73%</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>111,297,058</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>28.91M</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>3.85</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>263.88B</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>86.85</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>2.25</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>291.303.55%</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>61.15393.30%</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Semiconductors</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>MSTR</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>126.54</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>-7.01%</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>20,215,966</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>18.40M</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>44.35B</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>30.50</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>3.48</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>457.22-72.32%</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>104.1721.49%</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Software - Application</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>WMT</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>116.89</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>3.39%</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>29,902,488</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>19.91M</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>1.50</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>930.22B</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>36.35</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>0.60</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>135.15-13.51%</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>93.4325.11%</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Consumer Defensive</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Discount Stores</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>10.71</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>-4.20%</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>17,517,417</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>5.15M</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>1.56B</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>61.17</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>2.03</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>30.11-64.43%</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>7.6839.54%</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Software - Infrastructure</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-03 16:42 ET</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>ABVX</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>90.15</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>24.34%</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>7,145,757</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>1.35M</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>5.31</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>7.18B</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>36.44</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>148.83-39.43%</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>5.691484.36%</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Biotechnology</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-04 18:02 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1671"/>
+  <dimension ref="A1:D1771"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -37213,6 +37213,2206 @@
       <c r="D1671" s="3" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1672" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1672" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO People are going to pile in to this today and tomorrow 😂 May break 500 without even earnings 😂</t>
+        </is>
+      </c>
+      <c r="D1672" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1673" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1673" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO &amp;gt; $MU rotation is happening!!</t>
+        </is>
+      </c>
+      <c r="D1673" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1674" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1674" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1674" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1675" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1675" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO 80B Google spend goes to AVGO</t>
+        </is>
+      </c>
+      <c r="D1675" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1676" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1676" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1676" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1677" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1677" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO up 5.7% at 472.43.</t>
+        </is>
+      </c>
+      <c r="D1677" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1678" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1678" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO $500 coming, lets gooo !!!</t>
+        </is>
+      </c>
+      <c r="D1678" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1679" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1679" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO Will cross 500 on Tuesday and probably rise further on Wednesday going into earnings</t>
+        </is>
+      </c>
+      <c r="D1679" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1680" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1680" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO maybe short here</t>
+        </is>
+      </c>
+      <c r="D1680" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1681" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1681" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $AVGO I’m going to puts on this one before Er 440 or 450 lol</t>
+        </is>
+      </c>
+      <c r="D1681" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1682" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1682" s="2" t="inlineStr">
+        <is>
+          <t>$META Just bought 500 shares at $614.40...Looking to add more if the opportunity arises..</t>
+        </is>
+      </c>
+      <c r="D1682" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1683" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1683" s="3" t="inlineStr">
+        <is>
+          <t>$META rapidly dropped 39% after its IPO in a strikingly similar pattern to $CBRS which hit a low of 38% down today.  We know what happened after with META.  Look for the buyers to come in soon. $QQQ $SPY</t>
+        </is>
+      </c>
+      <c r="D1683" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1684" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1684" s="3" t="inlineStr">
+        <is>
+          <t>$META If you missed 610, you missed it.</t>
+        </is>
+      </c>
+      <c r="D1684" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1685" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1685" s="2" t="inlineStr">
+        <is>
+          <t>$META This morning was a buy! 620 incoming</t>
+        </is>
+      </c>
+      <c r="D1685" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1686" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1686" s="3" t="inlineStr">
+        <is>
+          <t>$META my concern is that META will be one of the stocks heavily sold in order to purchase the new IPOs like SpaceX and Anthropic</t>
+        </is>
+      </c>
+      <c r="D1686" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1687" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1687" s="3" t="inlineStr">
+        <is>
+          <t>$META can I get it under 600 again? For the 3rd time.</t>
+        </is>
+      </c>
+      <c r="D1687" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1688" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1688" s="2" t="inlineStr">
+        <is>
+          <t>$META  anyone foresee 620+ today</t>
+        </is>
+      </c>
+      <c r="D1688" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1689" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1689" s="3" t="inlineStr">
+        <is>
+          <t>There are two things certain in life. $META cannot really  There are better fixed income vehicles than $TLT</t>
+        </is>
+      </c>
+      <c r="D1689" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1690" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1690" s="3" t="inlineStr">
+        <is>
+          <t>$META imagine your arrogante, You don&amp;#39;t know what pressure Is. If You did,You wouldnt talk like this.   You have no idea of the first step to manage a behometh like this. Be aware his applications are in the hands of every human on earth. Facebook, Instagram or WhatsApp. Ever</t>
+        </is>
+      </c>
+      <c r="D1690" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1691" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C1691" s="3" t="inlineStr">
+        <is>
+          <t>$META what caused the dip today?</t>
+        </is>
+      </c>
+      <c r="D1691" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1692" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1692" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $DELL $MRVL $SOXS $SPY making &amp;quot;massive amounts of money&amp;quot;? Where? Circle jerking one another another? This is way bigger scam than the dotcom bubble! People literally want to burn these data centers down, woth all those chips and video cardss that they are giving t</t>
+        </is>
+      </c>
+      <c r="D1692" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1693" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1693" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL 6 minutes until the Asia market opens…this could get interesting</t>
+        </is>
+      </c>
+      <c r="D1693" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1694" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1694" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL If that doesn&amp;#39;t scream market manipulation then what does?</t>
+        </is>
+      </c>
+      <c r="D1694" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1695" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1695" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $DELL $MRVL $SOXS $SPY in the game of musical chairs. When do you know when to get out that is the biggest problem many of us have we don’t want to pay capital gains but perhaps we should.</t>
+        </is>
+      </c>
+      <c r="D1695" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1696" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1696" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL Yea, SEC will be involved</t>
+        </is>
+      </c>
+      <c r="D1696" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1697" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1697" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL @donthaveone yes Jensen bought Shares March 1 when it was it about $71 per share ￼</t>
+        </is>
+      </c>
+      <c r="D1697" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1698" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1698" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL holy mother of all the gods together  Fusiioned!!!!!!</t>
+        </is>
+      </c>
+      <c r="D1698" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1699" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1699" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $MRVL couldn’t be happier than if we see Broadcom go over $500 tomorrow. What a run. ￼</t>
+        </is>
+      </c>
+      <c r="D1699" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1700" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1700" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$AVGO $DELL $MRVL $SOXS $SPY except Dotcom. 90% of those companies were fraudulent. These companies selling A.I product are making massive amounts of money. Huge difference. Not to say, it can&amp;#39;t come crashing down, but no comparison to shell companies during dotcom bubble to </t>
+        </is>
+      </c>
+      <c r="D1700" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1701" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C1701" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO lets buy call this one and can dump like   $MSFT? LOL     INSANE MARKET.. BUT Nvda ceo say $MRVL is 1T and non stop pump!!     Welcome to casino 🎰</t>
+        </is>
+      </c>
+      <c r="D1701" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1702" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1702" s="2" t="inlineStr">
+        <is>
+          <t>$CELH time to buy more?</t>
+        </is>
+      </c>
+      <c r="D1702" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1703" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1703" s="2" t="inlineStr">
+        <is>
+          <t>$CELH</t>
+        </is>
+      </c>
+      <c r="D1703" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1704" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1704" s="2" t="inlineStr">
+        <is>
+          <t>$CELH oh, so insiders believe it will go up now. I’ll take that money and join them</t>
+        </is>
+      </c>
+      <c r="D1704" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1705" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1705" s="2" t="inlineStr">
+        <is>
+          <t>$CELH   I&amp;#39;ll take a potential 53% upside  This is according to investing.  .com</t>
+        </is>
+      </c>
+      <c r="D1705" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1706" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1706" s="2" t="inlineStr">
+        <is>
+          <t>$CELH are people really this quick to forget the massive insider buys…😅🔥</t>
+        </is>
+      </c>
+      <c r="D1706" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1707" s="3" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1707" s="3" t="inlineStr">
+        <is>
+          <t>$CELH i need to clarify that all those orange bars are insiders that have sols</t>
+        </is>
+      </c>
+      <c r="D1707" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1708" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1708" s="2" t="inlineStr">
+        <is>
+          <t>$CELH</t>
+        </is>
+      </c>
+      <c r="D1708" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1709" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1709" s="2" t="inlineStr">
+        <is>
+          <t>$CELH I’m in this has been beaten down enough.</t>
+        </is>
+      </c>
+      <c r="D1709" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1710" s="4" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1710" s="4" t="inlineStr">
+        <is>
+          <t>$CELH I warned</t>
+        </is>
+      </c>
+      <c r="D1710" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1711" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1711" s="2" t="inlineStr">
+        <is>
+          <t>$CELH How quick people forget about the insider buys is how quick they will forget about this BS. BUY THE DIP</t>
+        </is>
+      </c>
+      <c r="D1711" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1712" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1712" s="3" t="inlineStr">
+        <is>
+          <t>$lulu do not worry you will have good profit !!</t>
+        </is>
+      </c>
+      <c r="D1712" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1713" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1713" s="3" t="inlineStr">
+        <is>
+          <t>$LULU oh boy… you ever been to NY or TX? 😂</t>
+        </is>
+      </c>
+      <c r="D1713" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1714" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1714" s="3" t="inlineStr">
+        <is>
+          <t>$LULU who still buys overpriced china fabric</t>
+        </is>
+      </c>
+      <c r="D1714" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1715" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1715" s="3" t="inlineStr">
+        <is>
+          <t>$LULU 20-30%+ is my prediction as well.. we shall see</t>
+        </is>
+      </c>
+      <c r="D1715" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1716" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1716" s="3" t="inlineStr">
+        <is>
+          <t>$LULU no turning back</t>
+        </is>
+      </c>
+      <c r="D1716" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1717" s="2" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1717" s="2" t="inlineStr">
+        <is>
+          <t>$LULU 160 let’s go</t>
+        </is>
+      </c>
+      <c r="D1717" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1718" s="4" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1718" s="4" t="inlineStr">
+        <is>
+          <t>$LULU you must be new here…</t>
+        </is>
+      </c>
+      <c r="D1718" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1719" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1719" s="3" t="inlineStr">
+        <is>
+          <t>$LULU everyone thinks it’s going to get wrecked after earnings. Which means it won’t</t>
+        </is>
+      </c>
+      <c r="D1719" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1720" s="4" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1720" s="4" t="inlineStr">
+        <is>
+          <t>$LULU locked and loaded on the puts. Lulu 100p only cost me 0.05</t>
+        </is>
+      </c>
+      <c r="D1720" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1721" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1721" s="3" t="inlineStr">
+        <is>
+          <t>$LULU just a constant drain all year</t>
+        </is>
+      </c>
+      <c r="D1721" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1722" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1722" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN   Some people will interpret seeing a Warren Buffet quote posted as the top for this stock   I&amp;#39;m hoping this is just the beginning</t>
+        </is>
+      </c>
+      <c r="D1722" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1723" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1723" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN   Volume is 7 times the average and still the price has held up  I&amp;#39;m feeling confident   Still wary of that feeling when you see the shakeout   But I&amp;#39;ve been down this road before   Holding strong</t>
+        </is>
+      </c>
+      <c r="D1723" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1724" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1724" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN The Reddit attention this has is insane</t>
+        </is>
+      </c>
+      <c r="D1724" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1725" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1725" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN   Or are we getting a shakeout to put the fear of God in our 1,500 watchers!!!!</t>
+        </is>
+      </c>
+      <c r="D1725" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1726" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1726" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN</t>
+        </is>
+      </c>
+      <c r="D1726" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1727" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1727" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN</t>
+        </is>
+      </c>
+      <c r="D1727" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1728" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1728" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN   Are we getting a $10 close this evening</t>
+        </is>
+      </c>
+      <c r="D1728" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1729" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1729" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN Here it goes!!!🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D1729" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1730" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1730" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN This could get juicy!!🔥🔥</t>
+        </is>
+      </c>
+      <c r="D1730" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1731" s="2" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C1731" s="2" t="inlineStr">
+        <is>
+          <t>$LFVN   Today is first day I&amp;#39;ve seen a lot of Reddit interest   This has prob helped hold up / buy up those who were shaken out</t>
+        </is>
+      </c>
+      <c r="D1731" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1732" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1732" s="3" t="inlineStr">
+        <is>
+          <t>$T I’ll buy back at $20</t>
+        </is>
+      </c>
+      <c r="D1732" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1733" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1733" s="3" t="inlineStr">
+        <is>
+          <t>$T i think we end the week green</t>
+        </is>
+      </c>
+      <c r="D1733" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1734" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1734" s="3" t="inlineStr">
+        <is>
+          <t>$T now HERES a stock you should buy the dip on.  Fukin Value man, VALUE!  Gimmie!!</t>
+        </is>
+      </c>
+      <c r="D1734" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1735" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1735" s="2" t="inlineStr">
+        <is>
+          <t>$T $25 Calls Sept 18👨‍🍳</t>
+        </is>
+      </c>
+      <c r="D1735" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1736" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1736" s="3" t="inlineStr">
+        <is>
+          <t>$T  All the telco stocks are getting wrecked, this reminds me to when NVDA and INTEL got wrecked to the 20s and 80s because of hype.     I literally go to NANOG yearly where all these AI and satellite topics are spoken, and I yet to heard someone said Space Data Centers and inter</t>
+        </is>
+      </c>
+      <c r="D1736" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1737" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1737" s="2" t="inlineStr">
+        <is>
+          <t>$T Position officially acquired at 22.50 4.94% DivYeild secured!</t>
+        </is>
+      </c>
+      <c r="D1737" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1738" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1738" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$T for those who own this stock. Do you elect to automatically reinvest the dividends or do you take the cash and use elsewhere?  Elsewhere can be monthly bills or buying other company’s shares. I’ve done both with other stocks and lean more to using the money elsewhere but that </t>
+        </is>
+      </c>
+      <c r="D1738" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1739" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1739" s="3" t="inlineStr">
+        <is>
+          <t>$T well it looks like the shorts have arrived. Once you start seeing posts  like  &amp;quot;I&amp;#39;m a buyer at $12.&amp;quot; Then you know it&amp;#39;s trending</t>
+        </is>
+      </c>
+      <c r="D1739" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1740" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1740" s="3" t="inlineStr">
+        <is>
+          <t>$T Yeah well less cap gains fo at least $1600 and maybe even $2300</t>
+        </is>
+      </c>
+      <c r="D1740" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1741" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1741" s="3" t="inlineStr">
+        <is>
+          <t>$T don’t doubt this will recover but it’s a risky savings acct. i wouldn’t shame anyone from entering here, but i wouldn’t go 100% of what you’re willing to spend here either. I could see putting 25-50-% to work and if it goes down to $20 or less then load up on it and forget abo</t>
+        </is>
+      </c>
+      <c r="D1741" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1742" s="4" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1742" s="4" t="inlineStr">
+        <is>
+          <t>$CMG .95 cents away from 5 year low</t>
+        </is>
+      </c>
+      <c r="D1742" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1743" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1743" s="3" t="inlineStr">
+        <is>
+          <t>@WeAreKangz it’s sector related. Look at $MCD $TXRH $CMG . All near 52 weeks low</t>
+        </is>
+      </c>
+      <c r="D1743" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1744" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1744" s="3" t="inlineStr">
+        <is>
+          <t>$CELH lesson learned: diversify. Between this and $CMG, my account is blown</t>
+        </is>
+      </c>
+      <c r="D1744" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1745" s="2" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1745" s="2" t="inlineStr">
+        <is>
+          <t>$CMG earnings end of next month have to consider buying at the 52w lows🎯✅</t>
+        </is>
+      </c>
+      <c r="D1745" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1746" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1746" s="3" t="inlineStr">
+        <is>
+          <t>#OPTIONACTION  $RXRX Weekly Jun05 4 calls are seeing interest with the underlying stock 12% (volume: 10.1K, open int: 7.3K, implied vol: ~110%, prev day implied vol: 66%). 3.0K traded in a single transaction. Co is expected to report earnings mid-August.  $OPEN Weekly Jun12 5 cal</t>
+        </is>
+      </c>
+      <c r="D1746" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1747" s="4" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1747" s="4" t="inlineStr">
+        <is>
+          <t>$CMG long lines at the bathroom, which is always filthy and out of toilet paper.   Whew</t>
+        </is>
+      </c>
+      <c r="D1747" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1748" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1748" s="3" t="inlineStr">
+        <is>
+          <t>$CMG  I love Taquerias, but whenever i go to cmg, its not very good and definitely overpriced.  I would love to buy, but food is not good value, or high end.</t>
+        </is>
+      </c>
+      <c r="D1748" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1749" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1749" s="3" t="inlineStr">
+        <is>
+          <t>$CMG $PTLO 🤕🤦🤦🤦</t>
+        </is>
+      </c>
+      <c r="D1749" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1750" s="2" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1750" s="2" t="inlineStr">
+        <is>
+          <t>$CMG sigh worst investment so far…. At least PayPal gave me a bounce to get out after a year</t>
+        </is>
+      </c>
+      <c r="D1750" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1751" s="2" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1751" s="2" t="inlineStr">
+        <is>
+          <t>$CMG easy buy and hold</t>
+        </is>
+      </c>
+      <c r="D1751" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1752" s="2" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1752" s="2" t="inlineStr">
+        <is>
+          <t>$CIEN bought the dip it’s still at a decent price</t>
+        </is>
+      </c>
+      <c r="D1752" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1753" s="3" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1753" s="3" t="inlineStr">
+        <is>
+          <t>@ribbey @Jeremymartin007 @simon58 @judgeyoung2 @jenbunn @EBE_day @Godreal1 @TraderRapp @tonyctl @zuby34 Lunch time  had enough &amp;quot;fun&amp;quot;, today 🙄😑.  still pissed off bout $cien</t>
+        </is>
+      </c>
+      <c r="D1753" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1754" s="3" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1754" s="3" t="inlineStr">
+        <is>
+          <t>@DrJohansson $CIEN $avgo  posted it weekly for years now since cubie started learning options. congrats on seeing it for for very frist time today🙄😑</t>
+        </is>
+      </c>
+      <c r="D1754" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1755" s="3" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1755" s="3" t="inlineStr">
+        <is>
+          <t>@Jeremymartin007 @simon58 @judgeyoung2 @jenbunn @ribbey @EBE_day @TraderRapp @Godreal1 @tonyctl @zuby34  $MDB $ARM $AVGO $CIEN  no, cubie hate losing more jer</t>
+        </is>
+      </c>
+      <c r="D1755" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1756" s="2" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1756" s="2" t="inlineStr">
+        <is>
+          <t>$CIEN a gift, loaded at 500</t>
+        </is>
+      </c>
+      <c r="D1756" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1757" s="3" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1757" s="3" t="inlineStr">
+        <is>
+          <t>@jenbunn @Jeremymartin007 @simon58 @judgeyoung2 @ribbey @EBE_day @TraderRapp @Godreal1 @tonyctl @zuby34  $CIEN $avgo  scared money like jen, makes no moeny</t>
+        </is>
+      </c>
+      <c r="D1757" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1758" s="3" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1758" s="3" t="inlineStr">
+        <is>
+          <t>@LiveTradePro you mean $CIEN or really $CEIN ?</t>
+        </is>
+      </c>
+      <c r="D1758" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1759" s="2" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1759" s="2" t="inlineStr">
+        <is>
+          <t>$CIEN</t>
+        </is>
+      </c>
+      <c r="D1759" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1760" s="3" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1760" s="3" t="inlineStr">
+        <is>
+          <t>$CIEN - looks like it might close green…algos are loading up cheap….profitable and almost very little debt compared to peers that have huge debt…near term 600</t>
+        </is>
+      </c>
+      <c r="D1760" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1761" s="3" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C1761" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO not too late indeed🤑🫡😁, congrats fip buyers,  $CIEN too</t>
+        </is>
+      </c>
+      <c r="D1761" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1762" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1762" s="2" t="inlineStr">
+        <is>
+          <t>$RUM $RDDT $BTC.X $GME Easiest squeeze play of 2026. Revenue is set to 3x year over year thanks to Tether committing $250 million in advertising and cloud spending. This doesnt include any other cloud revenue they&amp;#39;ll likely get now that Rumble is about to become the 7th large</t>
+        </is>
+      </c>
+      <c r="D1762" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1763" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1763" s="2" t="inlineStr">
+        <is>
+          <t>$RUM low volume and up nearly 5% I like it…</t>
+        </is>
+      </c>
+      <c r="D1763" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1764" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1764" s="3" t="inlineStr">
+        <is>
+          <t>$RUM wall at 9.65, nothing past this level</t>
+        </is>
+      </c>
+      <c r="D1764" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1765" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1765" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$RUM tether owned northern data.. they are converting all their shares and not selling..  Management from northern data is locked in for a long while as well… minimal shares hit the market.  In addition no shares hit the market from the day of delisting for 30-45 days or per the </t>
+        </is>
+      </c>
+      <c r="D1765" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1766" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1766" s="2" t="inlineStr">
+        <is>
+          <t>$RUM Shares are getting bought up as soon as they are sold. Shorts are doomed.</t>
+        </is>
+      </c>
+      <c r="D1766" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1767" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1767" s="3" t="inlineStr">
+        <is>
+          <t>$RUM shes ripping</t>
+        </is>
+      </c>
+      <c r="D1767" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1768" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1768" s="2" t="inlineStr">
+        <is>
+          <t>$RUM Approximately 130.2 million new Rumble Class A shares are being issued (specifically 130,197,281), at an exchange ratio of 2.0281 Rumble Class A shares per Northern Data (ND) share.  THIS IS MASSIVE DILUTION AND THE STOCK PRICE MUST FALL IN LINE WITH THIS FACTOR.  NO DUMB AS</t>
+        </is>
+      </c>
+      <c r="D1768" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1769" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1769" s="3" t="inlineStr">
+        <is>
+          <t>$VIVO is the same setup as $APLD last April, which ran from $4 to currently $47. Except this one has 2.4 mil free float, and 3.6 mil shares short. Serious potential to go parabolic.  They recently bought a fully operational 41.5MW datacenter in Norway (Apr 21) at ~4x EBITDA. 100%</t>
+        </is>
+      </c>
+      <c r="D1769" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1770" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1770" s="2" t="inlineStr">
+        <is>
+          <t>$RUM northern data was once valued at 10-16 billion in a potential us ipo that was scrapped. It has the magic key to become a hyperscaler what is that? It is part of nvidias elite could service provider status. The same as coreweave and others. You’d have to spend years and billi</t>
+        </is>
+      </c>
+      <c r="D1770" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B1771" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1771" s="2" t="inlineStr">
+        <is>
+          <t>$RUM An 85% gain in less than three months is getting us some much deserved attention.  The woke of Wall Street won&amp;#39;t be able to hide RUM much longer.</t>
+        </is>
+      </c>
+      <c r="D1771" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
         </is>
       </c>
     </row>
@@ -37227,7 +39427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37255,34 +39455,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>106</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>98</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
@@ -37340,41 +39540,41 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -37384,14 +39584,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -37401,24 +39601,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
@@ -37527,63 +39727,63 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -37595,24 +39795,24 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -37622,14 +39822,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -37639,14 +39839,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -37656,7 +39856,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
@@ -38201,6 +40401,108 @@
       <c r="C57" t="inlineStr">
         <is>
           <t>2026-06-03 19:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
@@ -38215,7 +40517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -39020,6 +41322,726 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>421.73</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>-12.00%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>57,301,634</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>24.63M</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3.45</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1996.75B</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>48.87</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>495.00</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>241.1174</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>629.28</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1.01%</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>12,432,994</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>16.26M</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1597.38B</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>53.71</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>796.25</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>520.2620</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>314.54</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>4.27%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>61,455,589</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>30.47M</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2.99</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>275.16B</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>87.92</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>324.20</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>61.44411</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>28.17</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>-6.11%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>11,003,168</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>8.22M</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1.99</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>7.20B</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>37.63</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>66.74</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>27.661</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Beverages - Non-Alcoholic</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>125.18</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>-0.67%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2,718,684</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3.08M</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1.31</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>14.97B</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>38.17</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>339.15</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>116.627</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Apparel Retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LFVN</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>9.62</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>15.63%</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1,890,054</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>262.70K</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>10.68</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>121.36M</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>73.68</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>0.70</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>35.87</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>3.90146</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Packaged Foods</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>22.48</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>-4.54%</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>42,227,698</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>39.71M</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1.58</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>156.20B</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>23.74</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>29.79</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>22.95</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Telecom Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>28.38</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-1.26%</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>12,020,351</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>16.79M</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>36.40B</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>26.15</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>58.42</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>28.160</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Restaurants</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>524.45</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>-15.46%</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>5,415,729</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2.69M</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2.98</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>74.16B</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>45.08</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>637.51</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>70.77641</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Communication Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>8.39</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0.72%</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>10,016,911</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2.80M</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>5.29</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>3.66B</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>53.32</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>23.66</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>4.6281</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-04 19:54 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1771"/>
+  <dimension ref="A1:D1871"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -39413,6 +39413,2206 @@
       <c r="D1771" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1772" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1772" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO  i know the business here,  simple and sweet</t>
+        </is>
+      </c>
+      <c r="D1772" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1773" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1773" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO  I remember buying a company that sold books &amp;amp; shit online when the PE was over @1,000. Yeah i know that was about 15 years ago…  I’m old AF, you see.  Anyway, AMZN did ok🤷‍♂️.    So…piss off, I guess!?🐂 😂🐿️🫡 MM</t>
+        </is>
+      </c>
+      <c r="D1773" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1774" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1774" s="3" t="inlineStr">
+        <is>
+          <t>Top US tech names: P/E vs growth tells the story.  Undervalued:  $SNDK — memory leader, growth catching up  $WDC — solid free cash flow, undervalued  $AVGO — Broadcom, strong earnings support  Overvalued:  $INTC — high P/E vs modest growth  $TSLA — priced for perfection, executio</t>
+        </is>
+      </c>
+      <c r="D1774" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1775" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1775" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO this might open at 500 today 🥶💵</t>
+        </is>
+      </c>
+      <c r="D1775" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1776" s="4" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1776" s="4" t="inlineStr">
+        <is>
+          <t>$AVGO pe near 90 im pissing to all the bull mouths</t>
+        </is>
+      </c>
+      <c r="D1776" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1777" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1777" s="3" t="inlineStr">
+        <is>
+          <t>The biggest milestone in a company’s history dropped today—partnering with a photonics player, making them the standard functional laser for CPO, Pluggables, and SiPH.  This matters for $NVDA, $AVGO, $AMD, and $MRVL using the foundry.  Anyone know the name?</t>
+        </is>
+      </c>
+      <c r="D1777" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1778" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1778" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO still looks like one of the cleanest ways to own AI infrastructure.    Everyone watches GPUs, but few talk about what powers massive AI clusters behind the scenes—custom silicon and networking. Broadcom sits at the center of that buildout.    Long-term relationships with $G</t>
+        </is>
+      </c>
+      <c r="D1778" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1779" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1779" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO supersonic speed activated..500+ looking like a piece of cake</t>
+        </is>
+      </c>
+      <c r="D1779" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1780" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1780" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TSMC is reportedly considering a 15% price hike for 3nm chips in H2, driven by tight capacity and strong AI chip demand. Potential 5%-10% increases may follow in 2027.    $TSM benefits from scarcity and pricing power.  $NVDA’s AI data center orders continue to push advanced node </t>
+        </is>
+      </c>
+      <c r="D1780" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1781" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1781" s="3" t="inlineStr">
+        <is>
+          <t>@HankVenture Solid combination. Both $NVDA and $AVGO are core names in the AI infrastructure space, and both have completed a base, breakout, and successful retest. Now it&amp;#39;s about whether the trend continues to reflect the underlying fundamental growth.</t>
+        </is>
+      </c>
+      <c r="D1781" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1782" s="4" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1782" s="4" t="inlineStr">
+        <is>
+          <t>$LULU price action is a look into the future!</t>
+        </is>
+      </c>
+      <c r="D1782" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1783" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1783" s="3" t="inlineStr">
+        <is>
+          <t>$LULU</t>
+        </is>
+      </c>
+      <c r="D1783" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1784" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1784" s="3" t="inlineStr">
+        <is>
+          <t>$LULU best of luck!</t>
+        </is>
+      </c>
+      <c r="D1784" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1785" s="2" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1785" s="2" t="inlineStr">
+        <is>
+          <t>$LULU</t>
+        </is>
+      </c>
+      <c r="D1785" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1786" s="2" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1786" s="2" t="inlineStr">
+        <is>
+          <t>$LULU Hint hint</t>
+        </is>
+      </c>
+      <c r="D1786" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1787" s="4" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1787" s="4" t="inlineStr">
+        <is>
+          <t>$LULU   FAIR VALUE 71.23</t>
+        </is>
+      </c>
+      <c r="D1787" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1788" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1788" s="3" t="inlineStr">
+        <is>
+          <t>$LULU low expections but do they guide lower ? Clothes stocks have sucked. $QQQ $SPY</t>
+        </is>
+      </c>
+      <c r="D1788" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1789" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1789" s="3" t="inlineStr">
+        <is>
+          <t>$LULU my 15yr old daughter just said burn all her lulu clothes because some chemical in it causes cancer when you sweat! She has about 10k worth of this shit in her closet. She said all her friends are doing it. WTF is going on?? Bueller…bueller</t>
+        </is>
+      </c>
+      <c r="D1789" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1790" s="2" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1790" s="2" t="inlineStr">
+        <is>
+          <t>$LULU can we squeeeze higher it’s trending atleast… like goodness sake!</t>
+        </is>
+      </c>
+      <c r="D1790" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1791" s="3" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C1791" s="3" t="inlineStr">
+        <is>
+          <t>$LULU it’s going to easliy smash as the outlook and expectations  were deliberately set too low  Watch for shorters to run like pigs here</t>
+        </is>
+      </c>
+      <c r="D1791" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1792" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1792" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY</t>
+        </is>
+      </c>
+      <c r="D1792" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1793" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1793" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY this fucking Guy is cracking the code. Nice work. Either lube up and wait for messiah to come back… or do what this man did. Nice work</t>
+        </is>
+      </c>
+      <c r="D1793" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1794" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1794" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY nice easy simple 1hr trades lol</t>
+        </is>
+      </c>
+      <c r="D1794" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1795" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1795" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY we have come a long way boys</t>
+        </is>
+      </c>
+      <c r="D1795" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1796" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1796" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY that lil pump was just some extra cushion for the pushing tomorrow for red Friday! Lube up and try to smile…. It really does help.</t>
+        </is>
+      </c>
+      <c r="D1796" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1797" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1797" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY Today we had another example how GLXY is garbage.</t>
+        </is>
+      </c>
+      <c r="D1797" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1798" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1798" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY</t>
+        </is>
+      </c>
+      <c r="D1798" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1799" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1799" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY what a BUY</t>
+        </is>
+      </c>
+      <c r="D1799" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1800" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1800" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY good, he needs to reduce his share count</t>
+        </is>
+      </c>
+      <c r="D1800" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1801" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1801" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY has to be Novo dumping his shares on the market IMO</t>
+        </is>
+      </c>
+      <c r="D1801" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1802" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1802" s="2" t="inlineStr">
+        <is>
+          <t>$RUM</t>
+        </is>
+      </c>
+      <c r="D1802" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1803" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1803" s="3" t="inlineStr">
+        <is>
+          <t>$RUM boom</t>
+        </is>
+      </c>
+      <c r="D1803" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1804" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1804" s="3" t="inlineStr">
+        <is>
+          <t>$RUM sneaky shorts flashing big selling orders on the level 2 to scare buyers... or longs setting traps for bears trying to cover...?</t>
+        </is>
+      </c>
+      <c r="D1804" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1805" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1805" s="2" t="inlineStr">
+        <is>
+          <t>$RUM volume has picked up all day from where we were at open. Something brewing ladies</t>
+        </is>
+      </c>
+      <c r="D1805" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1806" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1806" s="3" t="inlineStr">
+        <is>
+          <t>$RUM power hour</t>
+        </is>
+      </c>
+      <c r="D1806" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1807" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1807" s="3" t="inlineStr">
+        <is>
+          <t>$RUM fomo kicking</t>
+        </is>
+      </c>
+      <c r="D1807" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1808" s="3" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1808" s="3" t="inlineStr">
+        <is>
+          <t>$RUM RUM IS LINING UP AROUND $1.08B IN COMBINED AI INFRA + PLATFORM REVENUE ON TODAY’S PIPELINE    ND BRINGS OVER $1B OF AI DATA CENTER BUILDOUT ALREADY DEPLOYED BETWEEN GPU CLUSTERS POWER CAPACITY AND SITES UNDER DEVELOPMENT    AI NAMES WITH REAL INFRA AND GROWTH ARE REGULARLY G</t>
+        </is>
+      </c>
+      <c r="D1808" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1809" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1809" s="2" t="inlineStr">
+        <is>
+          <t>$RUM she ripping</t>
+        </is>
+      </c>
+      <c r="D1809" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1810" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1810" s="2" t="inlineStr">
+        <is>
+          <t>$RUM ABSOLUTE BEAST MODE</t>
+        </is>
+      </c>
+      <c r="D1810" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1811" s="2" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C1811" s="2" t="inlineStr">
+        <is>
+          <t>$RUM $RUM $RDDT Rumble just acquired 9 data centers, 22k $NVDA GPUs and 300k CPUs for the price of $1.1 billion. Wall Street is needs to wake up. Just look at the market cap of $RUM at $3 billion vs. $NBIS at $50 billion. Glad I know both.</t>
+        </is>
+      </c>
+      <c r="D1811" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1812" s="2" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1812" s="2" t="inlineStr">
+        <is>
+          <t>$CRWV is breaking 130 Wall today $SPY</t>
+        </is>
+      </c>
+      <c r="D1812" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1813" s="3" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1813" s="3" t="inlineStr">
+        <is>
+          <t>@ClutchBallz Be aware that $CRWV will bottom before interest rates start dropping!</t>
+        </is>
+      </c>
+      <c r="D1813" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1814" s="2" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1814" s="2" t="inlineStr">
+        <is>
+          <t>$CRWV rebounding to 138 !!!</t>
+        </is>
+      </c>
+      <c r="D1814" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1815" s="3" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1815" s="3" t="inlineStr">
+        <is>
+          <t>$CRWV  what a jack leg</t>
+        </is>
+      </c>
+      <c r="D1815" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1816" s="4" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1816" s="4" t="inlineStr">
+        <is>
+          <t>$CRWV dropping like a rock</t>
+        </is>
+      </c>
+      <c r="D1816" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1817" s="3" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1817" s="3" t="inlineStr">
+        <is>
+          <t>$CRWV gimme $200</t>
+        </is>
+      </c>
+      <c r="D1817" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1818" s="3" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1818" s="3" t="inlineStr">
+        <is>
+          <t>$CRWV ceo is playing the game🥂🚀</t>
+        </is>
+      </c>
+      <c r="D1818" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1819" s="3" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1819" s="3" t="inlineStr">
+        <is>
+          <t>$CRWV Nebius has about 6-8 data centers and coreweave has 43 ..so it appears that the reason that nebius has slighly better margins is that they chose to monetize their current centers ...aka sell add on services and to build out slower. nothing wrong with that . But can you imag</t>
+        </is>
+      </c>
+      <c r="D1819" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1820" s="3" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1820" s="3" t="inlineStr">
+        <is>
+          <t>$CRWV I wish I could just take all insiders&amp;#39; phones and laptops away for one business day!  So they&amp;#39;d let this run for ONE DAY without multiple insider sell offs during a trading session!</t>
+        </is>
+      </c>
+      <c r="D1820" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1821" s="2" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C1821" s="2" t="inlineStr">
+        <is>
+          <t>$TPET oil going higher and higher get readyyy can see $2 on this 🤩 Watching $CRWV $AMD $HKIT $SOAR</t>
+        </is>
+      </c>
+      <c r="D1821" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1822" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1822" s="2" t="inlineStr">
+        <is>
+          <t>$CELH grabbed a little more!</t>
+        </is>
+      </c>
+      <c r="D1822" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1823" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1823" s="2" t="inlineStr">
+        <is>
+          <t>$CELH ken paxton probably buying shares right now</t>
+        </is>
+      </c>
+      <c r="D1823" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1824" s="3" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1824" s="3" t="inlineStr">
+        <is>
+          <t>$CELH im sorry Redbull gives you wings and bang is 300mg of caffeine but were being probed? Noise! Thanks for the shares.</t>
+        </is>
+      </c>
+      <c r="D1824" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1825" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1825" s="2" t="inlineStr">
+        <is>
+          <t>$CELH not much but another $700 at 27.82</t>
+        </is>
+      </c>
+      <c r="D1825" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1826" s="4" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1826" s="4" t="inlineStr">
+        <is>
+          <t>$CELH and eat the shit,</t>
+        </is>
+      </c>
+      <c r="D1826" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1827" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1827" s="2" t="inlineStr">
+        <is>
+          <t>$CELH tell me again how long Celsius has been a company?</t>
+        </is>
+      </c>
+      <c r="D1827" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1828" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1828" s="2" t="inlineStr">
+        <is>
+          <t>$CELH Loaded again</t>
+        </is>
+      </c>
+      <c r="D1828" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1829" s="3" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1829" s="3" t="inlineStr">
+        <is>
+          <t>$CELH one last comment Celsius, and its other brands will not last long-term. There are so many knock offs out there. I go around to stores and observe peoples purchases and I noticed everyone buys monster or Red Bull. I never see people buying their product.</t>
+        </is>
+      </c>
+      <c r="D1829" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1830" s="2" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1830" s="2" t="inlineStr">
+        <is>
+          <t>$CELH buy the dip</t>
+        </is>
+      </c>
+      <c r="D1830" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1831" s="3" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C1831" s="3" t="inlineStr">
+        <is>
+          <t>$CELH down 7% to 27.86, ask stacked 6x heavier than the bid. no panic vol, just steady selling, barely above avg. down 39% over 3 months so this is bleeding not crashing. waiting for it to base before I even think about a bounce. anyone got a level they&amp;#39;re watching?  on my fa</t>
+        </is>
+      </c>
+      <c r="D1831" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1832" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1832" s="3" t="inlineStr">
+        <is>
+          <t>$T I’m going to play defensively and do a cheap otm cover call incase they try to rip it up 🤣 and a csp. I’m ok with adding shares if it gets exercised.</t>
+        </is>
+      </c>
+      <c r="D1832" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1833" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1833" s="2" t="inlineStr">
+        <is>
+          <t>$T LOADED UP</t>
+        </is>
+      </c>
+      <c r="D1833" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1834" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1834" s="3" t="inlineStr">
+        <is>
+          <t>$T let’s go, algos are jumping in. Next stop 23-24s</t>
+        </is>
+      </c>
+      <c r="D1834" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1835" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1835" s="3" t="inlineStr">
+        <is>
+          <t>$T   Time to start building a position here  This selloff is over done. It very well may test  The 52 week low (falling knife ) but the downgrade is bullshit.  At&amp;amp;T is cheap extremely cheap. The street treats it like it’s a bond it’s not it’s a company that continues to gener</t>
+        </is>
+      </c>
+      <c r="D1835" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1836" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1836" s="3" t="inlineStr">
+        <is>
+          <t>$T in</t>
+        </is>
+      </c>
+      <c r="D1836" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1837" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1837" s="3" t="inlineStr">
+        <is>
+          <t>$T buying heavy it’s time, sold a lot last year</t>
+        </is>
+      </c>
+      <c r="D1837" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1838" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1838" s="3" t="inlineStr">
+        <is>
+          <t>$T Absolute disaster</t>
+        </is>
+      </c>
+      <c r="D1838" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1839" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1839" s="3" t="inlineStr">
+        <is>
+          <t>$CMCSA $CHTR $T $VZ This is just like the bottom of the oil stocks in late 2020. Dead and never coming back. 400+% returns over next 5 years from here if you can stomach it</t>
+        </is>
+      </c>
+      <c r="D1839" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1840" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1840" s="2" t="inlineStr">
+        <is>
+          <t>$T took profit on the covered calls,  but im guessing why wouldn’t they rug pull on the puts, premium seems now really nice. Thinking.</t>
+        </is>
+      </c>
+      <c r="D1840" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1841" s="4" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C1841" s="4" t="inlineStr">
+        <is>
+          <t>$T under 5% is not a good dividend</t>
+        </is>
+      </c>
+      <c r="D1841" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1842" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1842" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN</t>
+        </is>
+      </c>
+      <c r="D1842" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1843" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1843" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN I won’t be surprised if this thing tanks on June 9. Historically it has done than on major event days or announcements.</t>
+        </is>
+      </c>
+      <c r="D1843" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1844" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1844" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN https://mashable.com/tech/rivian-r2-launch-date</t>
+        </is>
+      </c>
+      <c r="D1844" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1845" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1845" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN an 18+ close would be pretty huge to confirm higher high</t>
+        </is>
+      </c>
+      <c r="D1845" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1846" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1846" s="3" t="inlineStr">
+        <is>
+          <t>$RIVN holding nicely</t>
+        </is>
+      </c>
+      <c r="D1846" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1847" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1847" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN Bears looking for any excuse.</t>
+        </is>
+      </c>
+      <c r="D1847" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1848" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1848" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN please let’s go rivian   You’re my only green   I’m counting on you girl</t>
+        </is>
+      </c>
+      <c r="D1848" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1849" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1849" s="3" t="inlineStr">
+        <is>
+          <t>$XPEV we are on the way back up, but it is sad to see that $RIVN has mc of 24b while Xpeng is at $17, WS needs to correct this shit, it makes NO sense.</t>
+        </is>
+      </c>
+      <c r="D1849" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1850" s="3" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1850" s="3" t="inlineStr">
+        <is>
+          <t>$F $LCID $NIO $RIVN $TSLA</t>
+        </is>
+      </c>
+      <c r="D1850" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1851" s="2" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C1851" s="2" t="inlineStr">
+        <is>
+          <t>$RIVN trading nicely here! Even on a RED day. PT raise, new product. The high today was a test and discovery. 🤞🏽✅ and the test has shown so far it has the power to proceed. Volume up up.</t>
+        </is>
+      </c>
+      <c r="D1851" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1852" s="3" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1852" s="3" t="inlineStr">
+        <is>
+          <t>$RCAT BUY BUY BUY BUY ABOUT TO SEE MASSIVE VOLUME OMG</t>
+        </is>
+      </c>
+      <c r="D1852" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1853" s="3" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1853" s="3" t="inlineStr">
+        <is>
+          <t>$RCAT buying here if Kevin wins I win</t>
+        </is>
+      </c>
+      <c r="D1853" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1854" s="2" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1854" s="2" t="inlineStr">
+        <is>
+          <t>$RCAT NATO countries will be buying. ☎️</t>
+        </is>
+      </c>
+      <c r="D1854" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1855" s="2" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1855" s="2" t="inlineStr">
+        <is>
+          <t>$RCAT don’t forget we are in The catalogue.</t>
+        </is>
+      </c>
+      <c r="D1855" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1856" s="3" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1856" s="3" t="inlineStr">
+        <is>
+          <t>$RCAT     The low-iq fibonachi chart crayon traders are in control there.</t>
+        </is>
+      </c>
+      <c r="D1856" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1857" s="4" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1857" s="4" t="inlineStr">
+        <is>
+          <t>$RCAT     Red Cat has not once held gains. Welcome, newbies.</t>
+        </is>
+      </c>
+      <c r="D1857" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1858" s="3" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1858" s="3" t="inlineStr">
+        <is>
+          <t>$RCAT   only if this could hold above 15. But not possible. Army of sellers above 15.</t>
+        </is>
+      </c>
+      <c r="D1858" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1859" s="4" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1859" s="4" t="inlineStr">
+        <is>
+          <t>$RCAT     Talk Monday.</t>
+        </is>
+      </c>
+      <c r="D1859" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1860" s="3" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1860" s="3" t="inlineStr">
+        <is>
+          <t>$RCAT I have no idea if they are going to go up tomorrow or not. All I know is that at some point in the future the shares will be far higher than current.</t>
+        </is>
+      </c>
+      <c r="D1860" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1861" s="3" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C1861" s="3" t="inlineStr">
+        <is>
+          <t>$RCAT the bull flag on the 15m is being a real tease</t>
+        </is>
+      </c>
+      <c r="D1861" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1862" s="2" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1862" s="2" t="inlineStr">
+        <is>
+          <t>$CMG staring position here. Don&amp;#39;t you short my burrito or you gonna have to deal with my taco 😄</t>
+        </is>
+      </c>
+      <c r="D1862" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1863" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1863" s="3" t="inlineStr">
+        <is>
+          <t>$CMG not good enough? I&amp;#39;m buying here</t>
+        </is>
+      </c>
+      <c r="D1863" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1864" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1864" s="3" t="inlineStr">
+        <is>
+          <t>$CMG from $3000 to split to $28 .. smfh</t>
+        </is>
+      </c>
+      <c r="D1864" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1865" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1865" s="3" t="inlineStr">
+        <is>
+          <t>$CMG Why dip ?</t>
+        </is>
+      </c>
+      <c r="D1865" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1866" s="2" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1866" s="2" t="inlineStr">
+        <is>
+          <t>$CMG Hopefully they switch to building ai data centers. We would go 100%</t>
+        </is>
+      </c>
+      <c r="D1866" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1867" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1867" s="3" t="inlineStr">
+        <is>
+          <t>$SBUX look at $CMG rhese businesses are tapped out on the ability to increase prices and people still pay for it. $4.00 gas doesn’t help either but 6.50 for a coffee and 18$ for a burrito aren’t sustainable</t>
+        </is>
+      </c>
+      <c r="D1867" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1868" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1868" s="3" t="inlineStr">
+        <is>
+          <t>$CMG dime away from a new 52 w low, selling off nonstop since the bell while index has fully recovered</t>
+        </is>
+      </c>
+      <c r="D1868" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1869" s="4" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1869" s="4" t="inlineStr">
+        <is>
+          <t>$CMG we don&amp;#39;t need overpriced burritos and guac!</t>
+        </is>
+      </c>
+      <c r="D1869" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1870" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1870" s="3" t="inlineStr">
+        <is>
+          <t>$CMG possible bankruptcy</t>
+        </is>
+      </c>
+      <c r="D1870" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B1871" s="3" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C1871" s="3" t="inlineStr">
+        <is>
+          <t>$CMG 13% in a week no news lmao</t>
+        </is>
+      </c>
+      <c r="D1871" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -39427,7 +41627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39460,12 +41660,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>116</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
@@ -39698,46 +41898,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>43</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
@@ -39863,7 +42063,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -39873,14 +42073,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -39890,14 +42090,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -39907,14 +42107,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -39931,7 +42131,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -39948,114 +42148,114 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -40067,92 +42267,92 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -40162,14 +42362,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -40179,14 +42379,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -40196,14 +42396,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -40213,14 +42413,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -40230,14 +42430,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -40247,14 +42447,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -40264,14 +42464,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -40281,14 +42481,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -40298,14 +42498,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -40315,14 +42515,14 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>PUSA</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -40332,14 +42532,14 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -40349,14 +42549,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -40366,14 +42566,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -40383,14 +42583,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -40400,14 +42600,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -40417,14 +42617,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -40434,14 +42634,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LFVN</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -40451,14 +42651,14 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -40468,14 +42668,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>LFVN</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -40503,6 +42703,40 @@
       <c r="C63" t="inlineStr">
         <is>
           <t>2026-06-04 14:02 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
@@ -40517,7 +42751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -42042,6 +44276,726 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>422.03</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-11.94%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>70,195,956</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>24.63M</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1998.17B</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>48.95</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>495.00</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>241.1175</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>124.45</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>-1.25%</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>4,277,072</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>3.08M</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>14.88B</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>37.28</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>339.15</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>116.626</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Apparel Retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>28.62</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0.46%</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>7,397,507</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>5.37M</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>11.16B</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>50.39</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>3.61</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>45.92</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>16.4374</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Capital Markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8.36</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0.42%</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>12,282,237</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2.80M</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>4.63</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>3.65B</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>53.12</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>23.89</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>4.6281</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>108.85</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>-1.88%</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>21,585,653</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>28.62M</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>59.38B</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>48.94</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>7.06</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>187.00</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>63.8070</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>27.86</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>-7.15%</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>15,390,714</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>8.22M</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>1.98</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>7.12B</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>36.83</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>66.74</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>27.660</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Beverages - Non-Alcoholic</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>22.67</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>-3.76%</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>61,340,335</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>39.71M</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>157.48B</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>24.63</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>29.79</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>22.95</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Telecom Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>18.00</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>-1.51%</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>26,866,035</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>29.42M</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>22.68B</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>70.43</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>22.69</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>11.5755</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RCAT</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>14.95</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>8.45%</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>19,789,508</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>16.39M</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2.28B</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>66.09</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>20.37</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>5.77159</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>28.23</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>-1.79%</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>18,123,273</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>16.79M</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>36.21B</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>25.66</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>58.42</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>28.160</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Restaurants</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-05 17:26 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1871"/>
+  <dimension ref="A1:D1971"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41613,6 +41613,2206 @@
       <c r="D1871" s="3" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1872" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1872" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA</t>
+        </is>
+      </c>
+      <c r="D1872" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1873" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1873" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA   Yo! Retail got played today</t>
+        </is>
+      </c>
+      <c r="D1873" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1874" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1874" s="2" t="inlineStr">
+        <is>
+          <t>$COSM Cosmos Health Continues U.S. Expansion with Launch of Oliv18, Targeting Cardiovascular and Antioxidant Categories  Science-backed, USDA and EU-certified, whole olive tree supplement for two major wellness categories — rapidly growing global market projected to exceed $33 bi</t>
+        </is>
+      </c>
+      <c r="D1874" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1875" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1875" s="3" t="inlineStr">
+        <is>
+          <t>$QQQ  $SPY  $NVDA $AMD  $TSLA  and stonks don&amp;#39;t go up in a straight line (cubie rule #9 u know🫡) ,  told @Jeremymartin007 till blue in the face , 8th or 9th inning , obviously due for pullback. cubie teaches 👇</t>
+        </is>
+      </c>
+      <c r="D1875" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1876" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1876" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA   How is this $40 car company stock still trading over $100?</t>
+        </is>
+      </c>
+      <c r="D1876" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1877" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1877" s="2" t="inlineStr">
+        <is>
+          <t>$TSLA call me crazy but $450+ next week</t>
+        </is>
+      </c>
+      <c r="D1877" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1878" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1878" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA incredible opportunity</t>
+        </is>
+      </c>
+      <c r="D1878" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1879" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1879" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA two week low hit.</t>
+        </is>
+      </c>
+      <c r="D1879" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1880" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1880" s="4" t="inlineStr">
+        <is>
+          <t>$TSLA Just the begining retail will sell this bag until SpaceX IPO</t>
+        </is>
+      </c>
+      <c r="D1880" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1881" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C1881" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA 387 loading</t>
+        </is>
+      </c>
+      <c r="D1881" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1882" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1882" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL</t>
+        </is>
+      </c>
+      <c r="D1882" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1883" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1883" s="3" t="inlineStr">
+        <is>
+          <t>$MU Great start of the week but not  a greatest end to the week.  $ORCL earning next week should boost the enthusiasm back. Announcement of $NVDA buy in for more micron chips is still a positive narrative.  Market needs this pull back, this is healthy.  $MU earning this month goi</t>
+        </is>
+      </c>
+      <c r="D1883" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1884" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1884" s="4" t="inlineStr">
+        <is>
+          <t>$ORCL this will continue to get nailed</t>
+        </is>
+      </c>
+      <c r="D1884" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1885" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1885" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL looking at the igv companies is infuriating.    orcl -10%, rest down about 1%.  what the fuck.</t>
+        </is>
+      </c>
+      <c r="D1885" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1886" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1886" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL yeah just go lower… fuck it.</t>
+        </is>
+      </c>
+      <c r="D1886" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1887" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1887" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL no way 300 next week and I was counting on it smh</t>
+        </is>
+      </c>
+      <c r="D1887" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1888" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1888" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL when in doubt zoom out, we are in a bull run, Red days are good days to buy , and sell on green, if your investing another great day to buy!  $QQQ $SPY</t>
+        </is>
+      </c>
+      <c r="D1888" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1889" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1889" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL Next week easy $300</t>
+        </is>
+      </c>
+      <c r="D1889" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1890" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1890" s="3" t="inlineStr">
+        <is>
+          <t>@Muktar65 don’t do anything today, just start your weekend and next week with slow Monday start we having a good news coming for micron and wider market. $ORCL earning could pump the overall market too. Have a great weekend</t>
+        </is>
+      </c>
+      <c r="D1890" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1891" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C1891" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL Is it Wednesday yet?</t>
+        </is>
+      </c>
+      <c r="D1891" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1892" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1892" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR Its human instincts to fear the unknow. The ones who conquered that fear wins 95% of the time.</t>
+        </is>
+      </c>
+      <c r="D1892" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1893" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1893" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR Might as well test 145</t>
+        </is>
+      </c>
+      <c r="D1893" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1894" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1894" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR Saylor&amp;#39;s playing some fkng games with issuing shares and probably its probably high frequency hedge funds buying them</t>
+        </is>
+      </c>
+      <c r="D1894" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1895">
+      <c r="A1895" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1895" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1895" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR you’ll be surprised how fast it runs past 200 within a couple or few weeks   This is MSTR!!!</t>
+        </is>
+      </c>
+      <c r="D1895" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1896" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1896" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR Bulls getting rejected</t>
+        </is>
+      </c>
+      <c r="D1896" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1897" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1897" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR Dump ittt</t>
+        </is>
+      </c>
+      <c r="D1897" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1898" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1898" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR $STRC $STRK</t>
+        </is>
+      </c>
+      <c r="D1898" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1899" s="4" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1899" s="4" t="inlineStr">
+        <is>
+          <t>$BTC.X $MSTR I THINK NOW IS THE PERFECT TIME FOR SAYLOR TO ATM THE SHIT OUT OF THE BULLS LOL.... MAKE THAT MONEY SAYLOR 🤣🤣🤣</t>
+        </is>
+      </c>
+      <c r="D1899" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1900" s="3" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1900" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR selling 32 is a great decoupling test</t>
+        </is>
+      </c>
+      <c r="D1900" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1901">
+      <c r="A1901" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1901" s="2" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C1901" s="2" t="inlineStr">
+        <is>
+          <t>$MSTR Down some more.</t>
+        </is>
+      </c>
+      <c r="D1901" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1902">
+      <c r="A1902" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1902" s="2" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1902" s="2" t="inlineStr">
+        <is>
+          <t>$OUST $PL generational dip buying opportunities.</t>
+        </is>
+      </c>
+      <c r="D1902" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1903" s="2" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1903" s="2" t="inlineStr">
+        <is>
+          <t>$PL gross but still long</t>
+        </is>
+      </c>
+      <c r="D1903" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1904" s="2" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1904" s="2" t="inlineStr">
+        <is>
+          <t>$PL bought some shares and calls here</t>
+        </is>
+      </c>
+      <c r="D1904" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1905" s="3" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1905" s="3" t="inlineStr">
+        <is>
+          <t>#Nasdaq Sinks Over 500 Points As #Tech Selloff Deepens $AVGO $DJI $NDX $PL $SPX https://talkmarkets.com/article/nasdaq-sinks-over-500-points-as-tech-selloff-deepens-1780679770</t>
+        </is>
+      </c>
+      <c r="D1905" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1906" s="3" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1906" s="3" t="inlineStr">
+        <is>
+          <t>$PL</t>
+        </is>
+      </c>
+      <c r="D1906" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1907">
+      <c r="A1907" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1907" s="3" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1907" s="3" t="inlineStr">
+        <is>
+          <t>$PL</t>
+        </is>
+      </c>
+      <c r="D1907" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1908" s="3" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1908" s="3" t="inlineStr">
+        <is>
+          <t>$PL this trash destroyed the whole sector on top of the market dump</t>
+        </is>
+      </c>
+      <c r="D1908" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1909" s="3" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1909" s="3" t="inlineStr">
+        <is>
+          <t>$SIDU wow they trapped all of us above 5 for sure. Bummer game !! Up down up down . $SPCE $PL</t>
+        </is>
+      </c>
+      <c r="D1909" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1910" s="3" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1910" s="3" t="inlineStr">
+        <is>
+          <t>$PL just dropped a structure that the market is clearly trying to digest     A $1.5B ATM on a ~$15B market cap is aggressive by any standard. That’s roughly 12 percent potential dilution sitting over the stock, which is why traders are reacting the way they are.    For context, $</t>
+        </is>
+      </c>
+      <c r="D1910" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1911" s="3" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C1911" s="3" t="inlineStr">
+        <is>
+          <t>$NVDA Simple: Funds harvested cash at the top ready for SpaceX IPO, it was inevitable. They will of course blame it on the jobs numbers coming in strong and risk of interest reate hikes... lol $PL</t>
+        </is>
+      </c>
+      <c r="D1911" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1912" s="2" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1912" s="2" t="inlineStr">
+        <is>
+          <t>$BNAI  $50 is coming</t>
+        </is>
+      </c>
+      <c r="D1912" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1913" s="2" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1913" s="2" t="inlineStr">
+        <is>
+          <t>$BNAI told yay 😀</t>
+        </is>
+      </c>
+      <c r="D1913" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1914">
+      <c r="A1914" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1914" s="3" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1914" s="3" t="inlineStr">
+        <is>
+          <t>$BNAI warrants are like free  bnaiw</t>
+        </is>
+      </c>
+      <c r="D1914" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1915" s="2" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1915" s="2" t="inlineStr">
+        <is>
+          <t>$BNAI</t>
+        </is>
+      </c>
+      <c r="D1915" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1916" s="3" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1916" s="3" t="inlineStr">
+        <is>
+          <t>$BNAI break</t>
+        </is>
+      </c>
+      <c r="D1916" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1917" s="3" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1917" s="3" t="inlineStr">
+        <is>
+          <t>$BNAI nreak 26.59 it game on</t>
+        </is>
+      </c>
+      <c r="D1917" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1918" s="2" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1918" s="2" t="inlineStr">
+        <is>
+          <t>$BNAI Recent  Developments  1. Africa AI licensing deal ($2.05 million): The company recently announced a $2.05 million AI licensing partnership in Africa.  2. Latin America expansion: BNAI finalized a $5 million exclusive AI licensing partnership in Latin America, targeting both</t>
+        </is>
+      </c>
+      <c r="D1918" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1919" s="3" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1919" s="3" t="inlineStr">
+        <is>
+          <t>$BNAI holding up strong</t>
+        </is>
+      </c>
+      <c r="D1919" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1920" s="2" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1920" s="2" t="inlineStr">
+        <is>
+          <t>$BNAI * BNAI terminated a $50 million Standby Equity Purchase Agreement that could have been a significant source of future dilution.    * The company has also announced several debt conversions and liability reductions totaling millions of dollars</t>
+        </is>
+      </c>
+      <c r="D1920" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1921" s="2" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C1921" s="2" t="inlineStr">
+        <is>
+          <t>$BNAI The bull case:    * Real commercial agreements are being announced.  * International expansion is accelerating.  * The company is reducing debt and has eliminated one potentially dilutive financing arrangement.  * The low float can create powerful upside moves</t>
+        </is>
+      </c>
+      <c r="D1921" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1922" s="3" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1922" s="3" t="inlineStr">
+        <is>
+          <t>$STI yes sir</t>
+        </is>
+      </c>
+      <c r="D1922" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1923" s="3" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1923" s="3" t="inlineStr">
+        <is>
+          <t>$STI Only a miracle can save her!</t>
+        </is>
+      </c>
+      <c r="D1923" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1924" s="2" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1924" s="2" t="inlineStr">
+        <is>
+          <t>$STI $60 EOD 🚀</t>
+        </is>
+      </c>
+      <c r="D1924" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1925" s="3" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1925" s="3" t="inlineStr">
+        <is>
+          <t>$STI trending down but if you can those bottoms can be good</t>
+        </is>
+      </c>
+      <c r="D1925" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1926" s="2" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1926" s="2" t="inlineStr">
+        <is>
+          <t>$RMSG what are they going to run this up to. $4 or high $3’s one or the other has to take place before anything else.   If your short I would tread lightly. This may halt up.   $STI $TE $UNH $CAVA   #BullFam #ShortSqueeze #TopWatches #WW</t>
+        </is>
+      </c>
+      <c r="D1926" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1927" s="2" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1927" s="2" t="inlineStr">
+        <is>
+          <t>$STI this will bounce !!!</t>
+        </is>
+      </c>
+      <c r="D1927" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1928" s="2" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1928" s="2" t="inlineStr">
+        <is>
+          <t>$STI go</t>
+        </is>
+      </c>
+      <c r="D1928" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1929" s="4" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1929" s="4" t="inlineStr">
+        <is>
+          <t>$STI its not a  scamm, its YOU that  is scamming yourself  and letting that short interest fee of 200% holding you hostage to hold for death!!!! That is the dumbiest stupid excuse lmao</t>
+        </is>
+      </c>
+      <c r="D1929" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1930" s="3" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1930" s="3" t="inlineStr">
+        <is>
+          <t>$STI</t>
+        </is>
+      </c>
+      <c r="D1930" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1931" s="4" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C1931" s="4" t="inlineStr">
+        <is>
+          <t>$STI as donnie said since $45.75 short .. people  that hold above $25 are dumb and stupid smh</t>
+        </is>
+      </c>
+      <c r="D1931" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1932" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1932" s="3" t="inlineStr">
+        <is>
+          <t>$MU Is it time to rip higher, or Monday?</t>
+        </is>
+      </c>
+      <c r="D1932" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1933" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1933" s="3" t="inlineStr">
+        <is>
+          <t>$MSTR  Sandisk $SNDK has already cracked the weekly parabolic trend, and $MU looks like it&amp;#39;s on it&amp;#39;s last legs. Could see one more pop early next week, but the sells will be all over that.</t>
+        </is>
+      </c>
+      <c r="D1933" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1934" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1934" s="2" t="inlineStr">
+        <is>
+          <t>$MU look at 1 year chart .... Or even 6 month  Easiest dip buy of my life, drops 70k on calls   3 in this account 3 in my other</t>
+        </is>
+      </c>
+      <c r="D1934" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1935" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1935" s="2" t="inlineStr">
+        <is>
+          <t>$MU going all in 1000$ calls!!!</t>
+        </is>
+      </c>
+      <c r="D1935" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1936" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1936" s="3" t="inlineStr">
+        <is>
+          <t>$MU space X is all about data centers. Where will Elon get his chips from?</t>
+        </is>
+      </c>
+      <c r="D1936" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1937" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1937" s="4" t="inlineStr">
+        <is>
+          <t>$MU going all in on 600$ puts</t>
+        </is>
+      </c>
+      <c r="D1937" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1938" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1938" s="3" t="inlineStr">
+        <is>
+          <t>$OSS Ouch $MU $NBIS $CRWV $MRVL</t>
+        </is>
+      </c>
+      <c r="D1938" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1939" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1939" s="4" t="inlineStr">
+        <is>
+          <t>$MU load up ur 600$ puts and u can thank me later more downside on modnay</t>
+        </is>
+      </c>
+      <c r="D1939" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1940" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1940" s="2" t="inlineStr">
+        <is>
+          <t>$MU who knew $AVGO was the single most important company and benchmark of global economic health!  How far will this overreaction go is a guess.</t>
+        </is>
+      </c>
+      <c r="D1940" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1941" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1941" s="2" t="inlineStr">
+        <is>
+          <t>$MU   Did we find the bottom ?</t>
+        </is>
+      </c>
+      <c r="D1941" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1942" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1942" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL Drops Premarket: $80B Equity Raise For AI Buildout Sparks Dilution Fears  $GOOGL $AVGO $BRK.B $BRK.A  https://stocktwits.com/news/equity/markets/googl-drops-premarket-80-b-equity-raise-for-ai-buildout-sparks-dilution-fears/cZ0itBORew4</t>
+        </is>
+      </c>
+      <c r="D1942" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1943" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1943" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why is $VIAV a top pick for June?    Everyone’s focused on $NVDA, $LITE, $COHR, $AVGO for the optical buildout. But when the industry plans to scale InP laser capacity 12x by 2030 while demand stays ~50% ahead of supply, who’s going to test it all?    $VIAV steps in—and it could </t>
+        </is>
+      </c>
+      <c r="D1943" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1944" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1944" s="3" t="inlineStr">
+        <is>
+          <t>The AI buildout isn&amp;#39;t just about GPUs.  Every layer of the semiconductor stack is seeing demand acceleration.  $AVGO benefits from AI networking and custom silicon demand.  $MRVL remains tied to cloud and data center infrastructure.  $SNDK is gaining from improving memory and</t>
+        </is>
+      </c>
+      <c r="D1944" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1945" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1945" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO Think Credo possibility</t>
+        </is>
+      </c>
+      <c r="D1945" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1946" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1946" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO Folks did you think they might miss on earnings</t>
+        </is>
+      </c>
+      <c r="D1946" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1947" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1947" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO 424 get in you will get it</t>
+        </is>
+      </c>
+      <c r="D1947" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1948" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1948" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO</t>
+        </is>
+      </c>
+      <c r="D1948" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1949" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1949" s="3" t="inlineStr">
+        <is>
+          <t>$NBIS  Maybe not. Tomorrow is $AVGO  Could add more fuel to the beautiful fire.</t>
+        </is>
+      </c>
+      <c r="D1949" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1950" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1950" s="2" t="inlineStr">
+        <is>
+          <t>$AVGO fuck it not sleeping in this morning. This is going to fly</t>
+        </is>
+      </c>
+      <c r="D1950" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1951" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C1951" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL everyone gets to be $1 trillion. $MU $AVGO $TSM $SOXX</t>
+        </is>
+      </c>
+      <c r="D1951" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1952" s="3" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1952" s="3" t="inlineStr">
+        <is>
+          <t>$MRLN ripping 32% on 10x avg vol, these vertical breakouts can fade just as fast as they spike. ask side stacked 6x heavier so somebody&amp;#39;s leaning on it. who&amp;#39;s got a read on this one?  this is what my scanner flagged: https://tapeboard.com/research/MRLN?utm_source=stocktwi</t>
+        </is>
+      </c>
+      <c r="D1952" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1953" s="2" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1953" s="2" t="inlineStr">
+        <is>
+          <t>$MRLN Autonomous flight ✈️  Certification is everything. AI integration small float massive upside</t>
+        </is>
+      </c>
+      <c r="D1953" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1954" s="2" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1954" s="2" t="inlineStr">
+        <is>
+          <t>$MRLN burn em</t>
+        </is>
+      </c>
+      <c r="D1954" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1955" s="2" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1955" s="2" t="inlineStr">
+        <is>
+          <t>$MRLN $12 Unstoppable</t>
+        </is>
+      </c>
+      <c r="D1955" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1956" s="3" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1956" s="3" t="inlineStr">
+        <is>
+          <t>$MRLN $LASE $QQQ $SPY</t>
+        </is>
+      </c>
+      <c r="D1956" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1957" s="2" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1957" s="2" t="inlineStr">
+        <is>
+          <t>$MRLN</t>
+        </is>
+      </c>
+      <c r="D1957" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1958" s="3" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1958" s="3" t="inlineStr">
+        <is>
+          <t>$MRLN Markets recovering slightly...Let&amp;#39;s see how this responds.  🤔🧐</t>
+        </is>
+      </c>
+      <c r="D1958" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1959" s="2" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1959" s="2" t="inlineStr">
+        <is>
+          <t>$MRLN   Absent global turmoil, looking for 12+ next week.</t>
+        </is>
+      </c>
+      <c r="D1959" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1960" s="2" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1960" s="2" t="inlineStr">
+        <is>
+          <t>$MRLN Amazing what&amp;#39;s going to happen here!! Looks really, really great</t>
+        </is>
+      </c>
+      <c r="D1960" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1961" s="2" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C1961" s="2" t="inlineStr">
+        <is>
+          <t>$MRLN Asymetric upside. Partnered with GE to develop this. Potentially hundreds of dollars. Getting in early is everything and despite the market dumping hard this stock has met up very well. Big leg up after hours and 12/13 pre market monday.</t>
+        </is>
+      </c>
+      <c r="D1961" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1962" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1962" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL realistic PT upon closing a deal??</t>
+        </is>
+      </c>
+      <c r="D1962" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1963" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1963" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL damn timed that well!</t>
+        </is>
+      </c>
+      <c r="D1963" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1964" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1964" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL one of us could be a guy working for KEEL just saying… howelse are we predicting so well</t>
+        </is>
+      </c>
+      <c r="D1964" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1965" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1965" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL  All algos just broke.  Good luck baby bish bear cub… you’re going to need it. $SPY $SMCI $BURU   The funniest part… it doesn’t matter what I own.. you bears are going to call it trash… hahahahaha 🤣 it could be Tesla, Nvidia, Apple, Microsoft, Keel, Bitcoin, Ethereum, etc e</t>
+        </is>
+      </c>
+      <c r="D1965" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1966" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1966" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL will it go to 7?</t>
+        </is>
+      </c>
+      <c r="D1966" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1967">
+      <c r="A1967" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1967" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1967" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL next stop $10 on the first deal. $15 on second deal. $20+ by EOY on third deal.</t>
+        </is>
+      </c>
+      <c r="D1967" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1968">
+      <c r="A1968" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1968" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1968" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL 6 🥳</t>
+        </is>
+      </c>
+      <c r="D1968" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1969">
+      <c r="A1969" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1969" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1969" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL Moving just like $DGXX before their massive $CBRS deal.   Don’t try to time the news, buy and HODL</t>
+        </is>
+      </c>
+      <c r="D1969" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1970">
+      <c r="A1970" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1970" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1970" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL $6.21-$6.3 seems possible this week  Not saying thats the limit before any correction  I just like to keep the price range not too ridiculously wide for each leg up for TA sake</t>
+        </is>
+      </c>
+      <c r="D1970" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1971">
+      <c r="A1971" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B1971" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1971" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL 🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D1971" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
         </is>
       </c>
     </row>
@@ -41627,7 +43827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41660,12 +43860,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>126</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
@@ -41677,19 +43877,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>108</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>KEEL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -41699,14 +43899,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -41723,17 +43923,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
@@ -42737,6 +44937,125 @@
       <c r="C65" t="inlineStr">
         <is>
           <t>2026-06-04 15:53 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
@@ -42751,7 +45070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -44996,6 +47315,726 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>395.69</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>-5.44%</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>33,811,947</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>59.48M</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1486.10B</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>41.86</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>498.83</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>273.2144</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>214.51</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>-9.24%</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>13,879,938</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>27.48M</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>616.93B</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>56.00</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>345.72</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>134.5759</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>118.62</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>-8.31%</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>22,914,218</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>18.23M</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>41.57B</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>28.91</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>3.49</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>457.22</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>104.1713</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>32.67</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>-24.94%</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>26,966,914</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>13.59M</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>3.39</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>11.64B</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>35.45</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>51.76</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>4.90566</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BNAI</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>23.98</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>46.76%</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>7,664,961</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>604.75K</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>21.63</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>156.06M</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>55.13</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>0.41</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>86.28</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>1.181932</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>STI</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>30.96</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>36.33%</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>29,218,591</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1.72M</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>29.04</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>239.80M</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>94.85</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>-0.35</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>38.15</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2.94953</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Electrical Equipment &amp; Parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>896.33</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>-10.01%</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>39,769,108</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>48.43M</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>1010.82B</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>58.13</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2.17</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>1089.29</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>103.38767</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>394.54</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>-5.82%</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>26,789,892</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>25.35M</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>1867.99B</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>41.81</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>495.00</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>241.1163</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MRLN</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>9.15</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>27.37%</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>23,240,882</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1.51M</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>26.22</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>882.71M</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>55.65</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>46.21</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>5.7858</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5.05</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>-14.76%</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>80,084,071</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>35.13M</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>3.89</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>3.05B</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>55.75</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>23.41</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0.70622</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-08 18:35 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1971"/>
+  <dimension ref="A1:D2071"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -43813,6 +43813,2206 @@
       <c r="D1971" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1972" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1972" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL 13 dollar dump don’t imagine e they have too many more shares to dump</t>
+        </is>
+      </c>
+      <c r="D1972" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1973" s="2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1973" s="2" t="inlineStr">
+        <is>
+          <t>$AAPL I predict we go below $300 ; then sit around $290- $300 for a while hopefully then trickle back up in the coming months ; this went up fast ; the long game wins</t>
+        </is>
+      </c>
+      <c r="D1973" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1974" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1974" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL stopped out -1 point</t>
+        </is>
+      </c>
+      <c r="D1974" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1975" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1975" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL 10 JUN 26 $300 PUT $1.70</t>
+        </is>
+      </c>
+      <c r="D1975" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1976">
+      <c r="A1976" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1976" s="4" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1976" s="4" t="inlineStr">
+        <is>
+          <t>$AAPL if not today, there will be follow through with people unloading for SpaceX.  I think</t>
+        </is>
+      </c>
+      <c r="D1976" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1977">
+      <c r="A1977" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1977" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1977" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL 10 JUN 26 $300 PUT $1.70  OUTSIDE BAR FORMED + OUTSIDE BAR BREAK   high risk</t>
+        </is>
+      </c>
+      <c r="D1977" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1978">
+      <c r="A1978" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1978" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1978" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL Who did $AAPL piss off?</t>
+        </is>
+      </c>
+      <c r="D1978" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1979">
+      <c r="A1979" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1979" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1979" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL 10 JUN 26 $300 PUT $1.70  OUTSIDE BAR FORMED + OUTSIDE BAR BREAK   high risk</t>
+        </is>
+      </c>
+      <c r="D1979" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1980">
+      <c r="A1980" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1980" s="4" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1980" s="4" t="inlineStr">
+        <is>
+          <t>$AAPL breaking bad</t>
+        </is>
+      </c>
+      <c r="D1980" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1981" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C1981" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL when  do they  release the apple  pager?   I hope  it’s a  flip  or  swipe  lol.</t>
+        </is>
+      </c>
+      <c r="D1981" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1982">
+      <c r="A1982" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1982" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1982" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY Reading these posts is a great way to see the difference in thinking between traders and investors.  I mostly invest in Galaxy. So I don’t care much if it follows closely with its overvalued peers, or not. What matters to investors is what the margins will be on the data ce</t>
+        </is>
+      </c>
+      <c r="D1982" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1983">
+      <c r="A1983" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1983" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1983" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY you can feel that we are on the verge of an announcement.... Helios or new purchase. Anything crypto does is just an add on. The data center angle is worth our market cap alone.</t>
+        </is>
+      </c>
+      <c r="D1983" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1984">
+      <c r="A1984" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1984" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1984" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY interesting chart movemebt right now, keeping an eye and might add a little more</t>
+        </is>
+      </c>
+      <c r="D1984" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1985">
+      <c r="A1985" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1985" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1985" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY ok</t>
+        </is>
+      </c>
+      <c r="D1985" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1986">
+      <c r="A1986" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1986" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1986" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY wtf</t>
+        </is>
+      </c>
+      <c r="D1986" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1987">
+      <c r="A1987" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1987" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1987" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY used to it…find a new slant</t>
+        </is>
+      </c>
+      <c r="D1987" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1988">
+      <c r="A1988" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1988" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1988" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY false alarm   Let&amp;#39;s hope bitcoin recovers tomorrow</t>
+        </is>
+      </c>
+      <c r="D1988" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1989">
+      <c r="A1989" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1989" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1989" s="2" t="inlineStr">
+        <is>
+          <t>$GLXY no worries, tomorrow&amp;#39;s green. Pretty sure of that.</t>
+        </is>
+      </c>
+      <c r="D1989" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1990">
+      <c r="A1990" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1990" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1990" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY complete manipulation</t>
+        </is>
+      </c>
+      <c r="D1990" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1991" s="3" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C1991" s="3" t="inlineStr">
+        <is>
+          <t>$GLXY</t>
+        </is>
+      </c>
+      <c r="D1991" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1992" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1992" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL 6.60 today, why not</t>
+        </is>
+      </c>
+      <c r="D1992" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1993" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1993" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D1993" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1994">
+      <c r="A1994" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1994" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1994" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL  Too the moon Alice</t>
+        </is>
+      </c>
+      <c r="D1994" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1995" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1995" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D1995" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1996" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1996" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL added a few bags.</t>
+        </is>
+      </c>
+      <c r="D1996" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1997" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1997" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL added January $12 calls to my longs</t>
+        </is>
+      </c>
+      <c r="D1997" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1998" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1998" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL now leaving orbit</t>
+        </is>
+      </c>
+      <c r="D1998" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B1999" s="2" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C1999" s="2" t="inlineStr">
+        <is>
+          <t>$KEEL pump itttttt!!!!!</t>
+        </is>
+      </c>
+      <c r="D1999" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2000" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C2000" s="3" t="inlineStr">
+        <is>
+          <t>$KEEL</t>
+        </is>
+      </c>
+      <c r="D2000" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2001" s="3" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C2001" s="3" t="inlineStr">
+        <is>
+          <t>@jenbunn @ribbey @cubie @simon58 @judgeyoung2 @EBE_day @TraderRapp @Godreal1 @tonyctl @zuby34 $KEEL $NOK $CIFR</t>
+        </is>
+      </c>
+      <c r="D2001" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2002" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2002" s="3" t="inlineStr">
+        <is>
+          <t>$PLTR signs $HPE like $DELL $SPY Open Ai $MSFT …</t>
+        </is>
+      </c>
+      <c r="D2002" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2003" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2003" s="4" t="inlineStr">
+        <is>
+          <t>$MSFT less than a week ago this was at 412....</t>
+        </is>
+      </c>
+      <c r="D2003" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2004" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2004" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Massive upside is coming tomorrow 🚀🚀🚀 The $500  is the next stop. Build 2026 Conference is tomorrow! Many surprises will be revealed 🚀🚀🚀 🍒🍒🍒💵💵💵🍰🍰🍰💥💥💥⬆️⬆️⬆️⬆️⬆️⬆️⬆️⬆️⬆️⬆️⬆️⬆️</t>
+        </is>
+      </c>
+      <c r="D2004" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2005" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2005" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT</t>
+        </is>
+      </c>
+      <c r="D2005" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2006" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2006" s="2" t="inlineStr">
+        <is>
+          <t>$META Had to add.  This isn’t META specific.  $MSFT  dropped in after hours too.</t>
+        </is>
+      </c>
+      <c r="D2006" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2007" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2007" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT all Stocktwits analysts coming up with full fud analysis… lol .. none of you know shitttttt.</t>
+        </is>
+      </c>
+      <c r="D2007" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2008" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2008" s="3" t="inlineStr">
+        <is>
+          <t>$GOOG $MSFT and poor $META got caught in the same setup…🖕the hedgies this means fuckin War Baby!</t>
+        </is>
+      </c>
+      <c r="D2008" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2009" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2009" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$MSFT  gave back the entire day’s gains in after hours, and that kind of reversal always gets attention.    What looked like steady accumulation during the session turned into a full round-trip once liquidity thinned out, which is pretty typical for mega caps when positioning is </t>
+        </is>
+      </c>
+      <c r="D2009" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2010" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2010" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT so now we know why this never retested premarket high because all hedgies knew $GOOG was about to drop capex funding news AH so they were not worried one bit all day where the price would go knowing the AH panicans would give them generational wealth! You can’t make this st</t>
+        </is>
+      </c>
+      <c r="D2010" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2011" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2011" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT Bild 2026 Conference tomorrow 🚀🚀🚀🍒🍒🍒💵💵💵🍰🍰🍰⬆️⬆️⬆️💥💥💥</t>
+        </is>
+      </c>
+      <c r="D2011" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2012" s="3" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2012" s="3" t="inlineStr">
+        <is>
+          <t>$ZVRA will hold gains 🔥🔥🔥</t>
+        </is>
+      </c>
+      <c r="D2012" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2013" s="3" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2013" s="3" t="inlineStr">
+        <is>
+          <t>ZVRA Stock ‘Way Undervalued’? Analyst Sees 117% Upside After Patent Extends Exclusivity Till 2041 For Sole Approved Drug  $ZVRA $VTI $IWM  https://stocktwits.com/news/equity/markets/zvra-stock-surges-on-extended-miplyffa-patent-protection-to-2041/cZ0vg5cR7Gv</t>
+        </is>
+      </c>
+      <c r="D2013" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2014" s="2" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2014" s="2" t="inlineStr">
+        <is>
+          <t>$ZVRA It&amp;#39;s about time 😉😎</t>
+        </is>
+      </c>
+      <c r="D2014" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2015" s="3" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2015" s="3" t="inlineStr">
+        <is>
+          <t>$ZVRA that’s all ?</t>
+        </is>
+      </c>
+      <c r="D2015" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2016" s="3" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2016" s="3" t="inlineStr">
+        <is>
+          <t>$ZVRA reclaiming 11 and pushing through, up to 11.95 on a clean session breakout. volume&amp;#39;s only 1.3x avg so this isn&amp;#39;t a pump, looks like real demand stepping in. eyes on whether it holds 11.50 into the close. anyone got a read on this one?  this is what my scanner flagge</t>
+        </is>
+      </c>
+      <c r="D2016" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2017" s="3" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2017" s="3" t="inlineStr">
+        <is>
+          <t>$ZVRA This is such a boring stock lol!</t>
+        </is>
+      </c>
+      <c r="D2017" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2018" s="3" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2018" s="3" t="inlineStr">
+        <is>
+          <t>$ZVRA  @Rodzilla01 is going to have a  surprise when he gets off the boat today</t>
+        </is>
+      </c>
+      <c r="D2018" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2019" s="2" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2019" s="2" t="inlineStr">
+        <is>
+          <t>$ZVRA Now we’re cooking with butter!</t>
+        </is>
+      </c>
+      <c r="D2019" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2020" s="2" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2020" s="2" t="inlineStr">
+        <is>
+          <t>$ZVRA let her rip tater chip</t>
+        </is>
+      </c>
+      <c r="D2020" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2021" s="2" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C2021" s="2" t="inlineStr">
+        <is>
+          <t>$ZVRA yeaaaa buddy!!! 🤑</t>
+        </is>
+      </c>
+      <c r="D2021" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2022" s="3" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2022" s="3" t="inlineStr">
+        <is>
+          <t>$BABA  HERE WE GO AGAIN O_o</t>
+        </is>
+      </c>
+      <c r="D2022" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2023" s="3" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2023" s="3" t="inlineStr">
+        <is>
+          <t>$BABA isn’t getting government/ military contract a big bullish of the stock? We didn’t have US company help US military like $PLTR ? So what? And just because Chinese is enemy?</t>
+        </is>
+      </c>
+      <c r="D2023" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2024" s="2" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2024" s="2" t="inlineStr">
+        <is>
+          <t>$BABA US can&amp;#39;t do much about China because all of their AI and robotics or the whole tech still heavily rely on China&amp;#39;s supply chain... Don&amp;#39;t forget about the rare earths... If US restrict China, they can easily restrict the rare earth export... Then the whole tech se</t>
+        </is>
+      </c>
+      <c r="D2024" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2025" s="3" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2025" s="3" t="inlineStr">
+        <is>
+          <t>$BABA $WEN $SOXS raging buy. $PYPL $SNAP add on dips. Sell every semi stock</t>
+        </is>
+      </c>
+      <c r="D2025" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2026" s="2" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2026" s="2" t="inlineStr">
+        <is>
+          <t>$BABA</t>
+        </is>
+      </c>
+      <c r="D2026" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2027" s="4" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2027" s="4" t="inlineStr">
+        <is>
+          <t>$BABA Sell.</t>
+        </is>
+      </c>
+      <c r="D2027" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2028" s="2" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2028" s="2" t="inlineStr">
+        <is>
+          <t>$BABA 120 it&amp;#39;s a four-year bottom. We tested it a thousand times. Even it got broken for sometime, it will r claim very quickly...</t>
+        </is>
+      </c>
+      <c r="D2028" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2029" s="3" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2029" s="3" t="inlineStr">
+        <is>
+          <t>$BABA “Cathie Wood”</t>
+        </is>
+      </c>
+      <c r="D2029" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2030" s="3" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2030" s="3" t="inlineStr">
+        <is>
+          <t>$BABA pentagaon doing what they do….psycho ops. Trump be pissed. Xi will just smile at the idea when US and Israel are up to there neck in defence contractors. Crazy world. Make money while the f*ck around</t>
+        </is>
+      </c>
+      <c r="D2030" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2031" s="4" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2031" s="4" t="inlineStr">
+        <is>
+          <t>$BABA Poor bata getting beat up left and right on booty chick</t>
+        </is>
+      </c>
+      <c r="D2031" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2032" s="2" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2032" s="2" t="inlineStr">
+        <is>
+          <t>$TNGX Trailing my stop</t>
+        </is>
+      </c>
+      <c r="D2032" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2033" s="3" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2033" s="3" t="inlineStr">
+        <is>
+          <t>$TNGX TNGX Price Target Alert: $36.00. Issued by Mizuho Securities    https://marketwirenews.com/stock/tngx/news/tngx-price-target-alert-36-00-issued-by-mizuho-secur-8697143402468964.html?utm_source=stocktwits</t>
+        </is>
+      </c>
+      <c r="D2033" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2034" s="3" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2034" s="3" t="inlineStr">
+        <is>
+          <t>$TNGX   Wolfe raised the drug’s global peak sales estimate to about $2.6 billion from $1.9 billion.</t>
+        </is>
+      </c>
+      <c r="D2034" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2035" s="4" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2035" s="4" t="inlineStr">
+        <is>
+          <t>$TNGX big correction coming end of day .. should drop a few bucks.</t>
+        </is>
+      </c>
+      <c r="D2035" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2036" s="3" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2036" s="3" t="inlineStr">
+        <is>
+          <t>$TNGX</t>
+        </is>
+      </c>
+      <c r="D2036" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2037" s="3" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2037" s="3" t="inlineStr">
+        <is>
+          <t>$TNGX what a bounce from lows!</t>
+        </is>
+      </c>
+      <c r="D2037" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2038" s="2" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2038" s="2" t="inlineStr">
+        <is>
+          <t>$TNGX - Tango Therapeutics. Up 57% today.It is up sharply today because it released very strong clinical trial data for its lead cancer drug combination, and the results were significantly better than investors expected.</t>
+        </is>
+      </c>
+      <c r="D2038" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2039" s="2" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2039" s="2" t="inlineStr">
+        <is>
+          <t>$TNGX https://www.investors.com/news/technology/tango-therapeutics-stock-revolution-medicines-pancreatic-cancer-treatment/</t>
+        </is>
+      </c>
+      <c r="D2039" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2040" s="3" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2040" s="3" t="inlineStr">
+        <is>
+          <t>$TNGX take your profit and run before collapse</t>
+        </is>
+      </c>
+      <c r="D2040" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2041" s="2" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C2041" s="2" t="inlineStr">
+        <is>
+          <t>$TNGX were trending on stock twits!!!!!</t>
+        </is>
+      </c>
+      <c r="D2041" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2042" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2042" s="3" t="inlineStr">
+        <is>
+          <t>$INTC  $PYPL   I see similar type of movement in future… back to 2021 prices</t>
+        </is>
+      </c>
+      <c r="D2042" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2043" s="4" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2043" s="4" t="inlineStr">
+        <is>
+          <t>$PYPL fuckin guy keeps giving targets 12-24 months down the road....no near term catalysts at all...sub 40 tomorrow....waste of time listening to this guy.</t>
+        </is>
+      </c>
+      <c r="D2043" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2044" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2044" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL had the chance to sell for even but didnt.  Smh</t>
+        </is>
+      </c>
+      <c r="D2044" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2045" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2045" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL  just wait for a  thr mother of all recessions.   People are broke, saving vanished. Nobody is buying shit.</t>
+        </is>
+      </c>
+      <c r="D2045" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2046" s="2" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2046" s="2" t="inlineStr">
+        <is>
+          <t>$PYPL I’m Bullish as fuck , and happy as fuck at this prices. Hope painpsll stays under $45 next 4 years.</t>
+        </is>
+      </c>
+      <c r="D2046" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2047" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2047" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL It won&amp;#39;t go bankrupt, but what it certainly won&amp;#39;t do is recover a single penny with a new CEO who says nothing and just collects a paycheck—he&amp;#39;s just another useless figure like his predecessors, and the stock will keep falling.</t>
+        </is>
+      </c>
+      <c r="D2047" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2048" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2048" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL 8.35 PE…. What a laughing stock</t>
+        </is>
+      </c>
+      <c r="D2048" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2049" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2049" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL $XYZ I generally don&amp;#39;t reflect on my stop losses getting triggered looking back and being happy about it but man am I glad I took a loss on PYPL last December. The term &amp;quot;Fintech&amp;quot; is about as offensive to me as a white guy in Kentucky wearing a backwards cap an</t>
+        </is>
+      </c>
+      <c r="D2049" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2050" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2050" s="3" t="inlineStr">
+        <is>
+          <t>$TOST can’t be company o ly it’s the economy   $PYPL and $XYZ too  so much hidden leverage in the system methinks</t>
+        </is>
+      </c>
+      <c r="D2050" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2051" s="3" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C2051" s="3" t="inlineStr">
+        <is>
+          <t>$PYPL burry, vanguard, citadel, Francis Chou, Jane street, have all been buying recently, how does this non give people more confidence. The names don’t get bigger. Yet the stock continues to be crushed with a PE of 8, down so much and my average is 55 feel for everyone above</t>
+        </is>
+      </c>
+      <c r="D2051" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2052" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2052" s="3" t="inlineStr">
+        <is>
+          <t>$NRIX not how I thought today would go … I think this will run soon they are holding it back but I won’t lie and say today wasn’t disappointing</t>
+        </is>
+      </c>
+      <c r="D2052" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2053" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2053" s="3" t="inlineStr">
+        <is>
+          <t>$NRIX 💨</t>
+        </is>
+      </c>
+      <c r="D2053" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2054" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2054" s="3" t="inlineStr">
+        <is>
+          <t>$NRIX Avg .21.90 🤣🙄</t>
+        </is>
+      </c>
+      <c r="D2054" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2055" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2055" s="3" t="inlineStr">
+        <is>
+          <t>$NRIX next analyst pt update 45 usd Jefferies</t>
+        </is>
+      </c>
+      <c r="D2055" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2056" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2056" s="3" t="inlineStr">
+        <is>
+          <t>$NRIX Net Premium &amp;amp; Whale Levels    Closing Price: $15.93    Critical Breakout Points:    $16.00 ($6.4M) | $16.10 ($8.4M) | $16.30 ($6.3M)    Critical Support Zones:    $15.80 ($8.1M)    Stay informed about daily whale levels across all trending assets  Follow for timely upda</t>
+        </is>
+      </c>
+      <c r="D2056" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2057" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2057" s="3" t="inlineStr">
+        <is>
+          <t>$INHD $NRIX signs multi-billion dollar deal and we fly here? Not what I anticipated but I’ll take it!</t>
+        </is>
+      </c>
+      <c r="D2057" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2058" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2058" s="3" t="inlineStr">
+        <is>
+          <t>$NRIX as derisked as it can get  I get the cons of the deal (giving away 50% of future sales from their lead asset + M&amp;amp;A not happening)  But: - Huge upfront (+ milestones + royalties) allows NRIX to advance quickly additional indications and pipeline (+ establish commercial i</t>
+        </is>
+      </c>
+      <c r="D2058" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2059" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2059" s="3" t="inlineStr">
+        <is>
+          <t>$NRIX solid base here</t>
+        </is>
+      </c>
+      <c r="D2059" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2060" s="3" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2060" s="3" t="inlineStr">
+        <is>
+          <t>INHD $NRIX signs a multi-billion dollar deal and we fly here? Not what I expected but I’ll take it!</t>
+        </is>
+      </c>
+      <c r="D2060" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2061" s="2" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C2061" s="2" t="inlineStr">
+        <is>
+          <t>$NRIX i have still 20 k shares from $INHD . will cash out around 30 usd and add here</t>
+        </is>
+      </c>
+      <c r="D2061" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2062" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2062" s="3" t="inlineStr">
+        <is>
+          <t>$LLY | Eli Lilly&amp;#39;s Oral GLP-1 Foundayo (Orforglipron) Delivered Superior A1c Control And Weight Loss In Three Pivotal Type 2 Diabetes Trials - PRN  https://www.prnewswire.com/news-releases/lillys-oral-glp-1-foundayo-orforglipron-delivered-superior-a1c-control-and-weight-loss-</t>
+        </is>
+      </c>
+      <c r="D2062" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2063" s="2" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2063" s="2" t="inlineStr">
+        <is>
+          <t>$LLY  10 or even 15 to 1 stock split time.</t>
+        </is>
+      </c>
+      <c r="D2063" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2064" s="2" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2064" s="2" t="inlineStr">
+        <is>
+          <t>$LLY this is about to move higher. Chart says so.</t>
+        </is>
+      </c>
+      <c r="D2064" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2065" s="4" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2065" s="4" t="inlineStr">
+        <is>
+          <t>$LLY Shooting star, and a double top..! Ripe to start a nice juicy short here</t>
+        </is>
+      </c>
+      <c r="D2065" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2066" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2066" s="3" t="inlineStr">
+        <is>
+          <t>Whether you view upcoming medical conferences as the next major catalyst or are keeping a cautious eye on absolute sector valuations, tracking these distinct thematic structures is critical. 🔍    Track institutional fund flows, monitor organic growth, and check the full list of E</t>
+        </is>
+      </c>
+      <c r="D2066" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2067" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2067" s="3" t="inlineStr">
+        <is>
+          <t>4️⃣ $OZEM - Roundhill GLP-1 &amp;amp; Weight Loss ETF    Sporting a 19.08% allocation to $LLY.    The first pure-play ETF targeting the anti-obesity global theme. Given its specialized exposure to pure anti-obesity competitors, localized sector profit-taking weighed on performance ov</t>
+        </is>
+      </c>
+      <c r="D2067" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2068" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2068" s="3" t="inlineStr">
+        <is>
+          <t>3️⃣ $MEDI - Harbor Health Care ETF    Holding a major 21.61% allocation to $LLY.    An actively managed play focusing on secular growth across the medical spectrum. Broad health infrastructure drags pushed its price performance into the red over the trailing 5 days despite steady</t>
+        </is>
+      </c>
+      <c r="D2068" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2069" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2069" s="3" t="inlineStr">
+        <is>
+          <t>2️⃣ $PPH - VanEck Pharmaceutical ETF    Carrying a substantial 22.73% allocation to $LLY.    This strategy tracks the 25 largest US-listed pharmaceutical firms. While strong stock performance kept the overall price return positive, the fund did experience an organic retreat:  📈 5</t>
+        </is>
+      </c>
+      <c r="D2069" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2070" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2070" s="3" t="inlineStr">
+        <is>
+          <t>1️⃣ $IHE - iShares U.S. Pharmaceuticals ETF    Allocation check: Dominating the board with a heavy 24.59% weighting in $LLY.    This fund provides targeted exposure to the heavy hitters of domestic pharma. Eli Lilly&amp;#39;s momentum helped keep this basket insulated from broader he</t>
+        </is>
+      </c>
+      <c r="D2070" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B2071" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C2071" s="3" t="inlineStr">
+        <is>
+          <t>Eli Lilly ($LLY) is climbing up the trending boards after positive Phase 3 clinical data for retatrutide reinforced its massive competitive edge in the GLP-1 sector! 💊🧬    While the community actively debates $LLY&amp;#39;s long-term pipeline strength against main rivals like Novo No</t>
+        </is>
+      </c>
+      <c r="D2071" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -43827,7 +46027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43894,12 +46094,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
@@ -43940,7 +46140,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -43950,19 +46150,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -43974,24 +46174,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -44001,14 +46201,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -44331,7 +46531,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -44341,14 +46541,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -44365,7 +46565,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -44375,14 +46575,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -44399,7 +46599,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -44416,7 +46616,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -44433,160 +46633,160 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>GLXY</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -44603,7 +46803,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -44620,7 +46820,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -44637,7 +46837,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -44647,14 +46847,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -44664,14 +46864,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -44681,14 +46881,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -44698,14 +46898,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -44715,14 +46915,14 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -44732,14 +46932,14 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -44749,14 +46949,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>PUSA</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -44766,14 +46966,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -44783,14 +46983,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -44800,14 +47000,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -44817,14 +47017,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -44834,14 +47034,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -44858,7 +47058,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -44875,7 +47075,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LFVN</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -44885,14 +47085,14 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>LFVN</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -44909,7 +47109,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>GLXY</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -44919,7 +47119,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
@@ -45056,6 +47256,108 @@
       <c r="C72" t="inlineStr">
         <is>
           <t>2026-06-05 13:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
@@ -45070,7 +47372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -48035,6 +50337,726 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>305.18</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>-0.70%</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>44,938,196</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>44.89M</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>4482.29B</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>57.73</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>316.94</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>195.0756</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Consumer Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>31.17</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>23.99%</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>14,530,332</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>5.48M</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>3.51</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>12.15B</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>57.21</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>3.62</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>45.92</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>16.4389</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Capital Markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>KEEL</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>5.69</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>11.01%</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>57,421,654</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>36.49M</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2.09</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>3.44B</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>63.87</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>13.71</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0.70713</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>412.15</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>-1.08%</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>17,778,264</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>34.43M</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>3061.63B</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>45.47</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>555.45</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>356.2815</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ZVRA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>12.00</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>13.13%</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2,611,165</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1.46M</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2.37</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>709.58M</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>61.56</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>0.91</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>13.16</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>7.1667</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>120.39</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>-0.56%</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>5,837,172</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>11.29M</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0.69</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>288.82B</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>36.49</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>0.47</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>192.67</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>103.7116</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Internet Retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>31.91</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>57.79%</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>17,264,745</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>3.12M</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>7.34</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>4.61B</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>70.78</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>1.22</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>28.4112</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>3.58791</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>41.08</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>-0.52%</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>8,941,371</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>15.43M</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0.77</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>36.23B</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>27.54</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>79.50</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>38.466</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Credit Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>15.52</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>6.05%</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>17,591,663</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1.16M</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>20.14</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>1.61B</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>43.05</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>31.00</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>8.1989</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1159.29</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2.46%</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2,671,126</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>3.12M</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>1091.75B</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>71.45</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>0.51</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>1166.29</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>623.7885</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Drug Manufacturers - General</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-09 17:33 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2071"/>
+  <dimension ref="A1:D2171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -46011,6 +46011,2206 @@
         </is>
       </c>
       <c r="D2071" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2072" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2072" s="4" t="inlineStr">
+        <is>
+          <t>If you buy today, You&amp;#39;re gonna be bag holding  for 9 years. 100.01%   $QQQ $SPY $PLTR $ORCL $MSFT</t>
+        </is>
+      </c>
+      <c r="D2072" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2073" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2073" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL totally handicapped thisnmarket will never let it bounce wo a crash to buy it..still reallybdidnt crashngave backn50 percent of gains thiugh</t>
+        </is>
+      </c>
+      <c r="D2073" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2074" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2074" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL BUY and CHILL 😎</t>
+        </is>
+      </c>
+      <c r="D2074" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2075" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2075" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL     350 next week nobody cares about today</t>
+        </is>
+      </c>
+      <c r="D2075" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2076" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2076" s="3" t="inlineStr">
+        <is>
+          <t>$INTC $ORCL in 1hour bars...i forgot to say</t>
+        </is>
+      </c>
+      <c r="D2076" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2077" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2077" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL BUYING OPPORTUNITY</t>
+        </is>
+      </c>
+      <c r="D2077" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2078" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2078" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL   BUY BUY. 300 NEXT WEEK</t>
+        </is>
+      </c>
+      <c r="D2078" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2079" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2079" s="3" t="inlineStr">
+        <is>
+          <t>$INTC $ORCL nasdaq futures for june ihss been oversold all day in RSI  and now we are at the lowest 19,99</t>
+        </is>
+      </c>
+      <c r="D2079" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2080" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2080" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL adding more here</t>
+        </is>
+      </c>
+      <c r="D2080" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2081" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2081" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL $NOK $GFS $LAC  Whoever think they are smart to move money to SpaceX will get their new brand new heavy bag and will be bagholding it for decades. Elon is a good marketing guy but that SpaceX company doesn’t worth anything more than 500B and even this is only because of his</t>
+        </is>
+      </c>
+      <c r="D2081" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2082" s="3" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2082" s="3" t="inlineStr">
+        <is>
+          <t>$APLD vs $DJT comparing two trending tickers</t>
+        </is>
+      </c>
+      <c r="D2082" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2083" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2083" s="2" t="inlineStr">
+        <is>
+          <t>$APLD they can try and slow it down, but they ain’t stopping the A train</t>
+        </is>
+      </c>
+      <c r="D2083" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2084" s="3" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2084" s="3" t="inlineStr">
+        <is>
+          <t>$APLD V</t>
+        </is>
+      </c>
+      <c r="D2084" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2085" s="3" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2085" s="3" t="inlineStr">
+        <is>
+          <t>gonna wait for H% to cool down before buying $APLD like usual</t>
+        </is>
+      </c>
+      <c r="D2085" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2086" s="3" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2086" s="3" t="inlineStr">
+        <is>
+          <t>$APLD This was practically one of the safest investments considering the last news and only reason why this was down was overall market.</t>
+        </is>
+      </c>
+      <c r="D2086" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2087" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2087" s="2" t="inlineStr">
+        <is>
+          <t>$APLD $CHRN Can someone close to trump have connection til BofA to make stock fall ?   Trump and others have made great investments over the past nd somehow always before the stock when up again … same case today ?</t>
+        </is>
+      </c>
+      <c r="D2087" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2088" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2088" s="2" t="inlineStr">
+        <is>
+          <t>$APLD This one is for @MarketPro    They don’t know it’s just a matter of time…..😎🏦🏦</t>
+        </is>
+      </c>
+      <c r="D2088" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2089" s="3" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2089" s="3" t="inlineStr">
+        <is>
+          <t>$APLD</t>
+        </is>
+      </c>
+      <c r="D2089" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2090" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2090" s="2" t="inlineStr">
+        <is>
+          <t>$APLD strong!</t>
+        </is>
+      </c>
+      <c r="D2090" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2091" s="3" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C2091" s="3" t="inlineStr">
+        <is>
+          <t>$APLD fun times here👍</t>
+        </is>
+      </c>
+      <c r="D2091" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2092" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2092" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL When do we see $400 a share? Any guidance here?</t>
+        </is>
+      </c>
+      <c r="D2092" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2093" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2093" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL shorted this overnight made $243 for fun. I just short for fun somtimes. Not seriously do it</t>
+        </is>
+      </c>
+      <c r="D2093" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2094" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2094" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $DELL $MRVL $SOXS $SPY quote- Circular financing is risky when it hides weak end-demand  that&amp;#39;s what blew up in the dot-com era. But AI usage is already large and growing quickly, and the build-out is primarily funded by established tech giants with massive balance shee</t>
+        </is>
+      </c>
+      <c r="D2094" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2095">
+      <c r="A2095" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2095" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2095" s="3" t="inlineStr">
+        <is>
+          <t>@LeFloppJames yeah, but that was BEFORE Huang guaranteed $MRVL to quadruple!!!  It&amp;#39;s called new information, and markets tend not to forget about it once it&amp;#39;s out.</t>
+        </is>
+      </c>
+      <c r="D2095" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2096">
+      <c r="A2096" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2096" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2096" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL wtf whoaaaaaa</t>
+        </is>
+      </c>
+      <c r="D2096" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2097" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2097" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$MRVL If AI spending remains strong through the 2030s, it&amp;#39;s not difficult to imagine Marvell being worth several times its current value. Whether it becomes a 5x, 10x, or larger winner depends on how successfully it converts today&amp;#39;s AI demand into durable earnings growth </t>
+        </is>
+      </c>
+      <c r="D2097" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2098" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2098" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL guys what is the max</t>
+        </is>
+      </c>
+      <c r="D2098" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2099">
+      <c r="A2099" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2099" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2099" s="3" t="inlineStr">
+        <is>
+          <t>Today&amp;#39;s option volume of 64.3M contracts was -12.00% below recent avg levels, w/ calls leading puts 5 to 3.    Single stock (37.6M contracts on 6.56M trades) &amp;amp; Index products (5.21M contracts on 2.49M trades) saw relatively heavy volume, while ETF flow was moderate (21.5M</t>
+        </is>
+      </c>
+      <c r="D2099" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2100" s="2" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2100" s="2" t="inlineStr">
+        <is>
+          <t>$MRVL Marvell Technology (MRVL) 🍀🍀🍀🍀🍀🍀 Current Price: ~$290–$318 (strong breakout after +32% surge on AI news). Entry: $295–$305 (on minor pullback to EMA 9/21 support). Stop Loss: $275 (risk ~$20–25 per share). Targets: $330 (Target 1), $350 (Target 2).</t>
+        </is>
+      </c>
+      <c r="D2100" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2101" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C2101" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL</t>
+        </is>
+      </c>
+      <c r="D2101" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2102">
+      <c r="A2102" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2102" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2102" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL ..dead money compared to other opportunities :(</t>
+        </is>
+      </c>
+      <c r="D2102" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2103" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2103" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL omg i didn&amp;#39;t make my weekly put trade and just came back to see this.  50 - 310p weeklies.  nauseous.</t>
+        </is>
+      </c>
+      <c r="D2103" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2104" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2104" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL what a  shit show</t>
+        </is>
+      </c>
+      <c r="D2104" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2105" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2105" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL that is not a coincidence.  We knew about this one hour ahead of time.</t>
+        </is>
+      </c>
+      <c r="D2105" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2106" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2106" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL &amp;gt;&amp;gt; What Makes Today So Valuable:    What&amp;#39;s interesting is that BOTH setups appeared in the same session.    Stage 1    Failed breakout    315.17 failure    ↓    Stage 2    Support breakdown    308.21 failure    ↓    Stage 3    Trend acceleration    304s    That is</t>
+        </is>
+      </c>
+      <c r="D2106" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2107" s="2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2107" s="2" t="inlineStr">
+        <is>
+          <t>$AAPL LOAD U FOOLS ;P</t>
+        </is>
+      </c>
+      <c r="D2107" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2108" s="2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2108" s="2" t="inlineStr">
+        <is>
+          <t>$AAPL will it close green</t>
+        </is>
+      </c>
+      <c r="D2108" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2109">
+      <c r="A2109" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2109" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2109" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL    🛑🛑🛑🛑🛑🛑Hit the follow button .. and follow me ….  do you think this is just luck we went BEARISH  one hour before the stock plummeted ? you shareholders should be following only one person on this stock message board that is yours truly. I’m only following one person.. an</t>
+        </is>
+      </c>
+      <c r="D2109" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2110" s="4" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2110" s="4" t="inlineStr">
+        <is>
+          <t>$AAPL fckin pos</t>
+        </is>
+      </c>
+      <c r="D2110" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2111">
+      <c r="A2111" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2111" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C2111" s="3" t="inlineStr">
+        <is>
+          <t>$AAPL PoS</t>
+        </is>
+      </c>
+      <c r="D2111" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2112" s="4" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2112" s="4" t="inlineStr">
+        <is>
+          <t>$NVDA halted</t>
+        </is>
+      </c>
+      <c r="D2112" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2113" s="2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2113" s="2" t="inlineStr">
+        <is>
+          <t>$QQQ big ups V $MRVL $IONQ $NOK $NVDA</t>
+        </is>
+      </c>
+      <c r="D2113" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2114" s="2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2114" s="2" t="inlineStr">
+        <is>
+          <t>$NVDA means a 40% squeeze incoming</t>
+        </is>
+      </c>
+      <c r="D2114" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2115" s="3" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2115" s="3" t="inlineStr">
+        <is>
+          <t>$NVDA its frozen</t>
+        </is>
+      </c>
+      <c r="D2115" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2116" s="3" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2116" s="3" t="inlineStr">
+        <is>
+          <t>$BTC.X $MU $NVDA $QQQ $SPY  Exactly 🤣</t>
+        </is>
+      </c>
+      <c r="D2116" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2117" s="3" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2117" s="3" t="inlineStr">
+        <is>
+          <t>@Quantum_Rules @Optomystic     $MU $NVDA  That&amp;#39;;s what I dont understand... So all they anaylst that up grade stocks, with PT adjustments... etc....  Is it all BS or what...  How else are use little guys suppose to know....</t>
+        </is>
+      </c>
+      <c r="D2117" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2118" s="2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2118" s="2" t="inlineStr">
+        <is>
+          <t>$RUM $RUM $INTC $RDDT Like I said, RUMBLE just acquired 9 DATA CENTERS with 22k $NVDA GPUs and +300k CPUs. EVERYONE is lacking in compute.  Just wait for the CLOUD deals to come through and this becomes a rocket ship. Only 1 analyst is aware of this   with a $22 price target. Wal</t>
+        </is>
+      </c>
+      <c r="D2118" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2119" s="2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2119" s="2" t="inlineStr">
+        <is>
+          <t>$SOXL $AMD $NVDA $INTC $MU</t>
+        </is>
+      </c>
+      <c r="D2119" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2120">
+      <c r="A2120" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2120" s="2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2120" s="2" t="inlineStr">
+        <is>
+          <t>$SPY $QQQ $NVDA $SLV   *US BELIEVES IRAN TO SETTLE ON 15-YR ENRICHMENT SUSPENSION: NYT</t>
+        </is>
+      </c>
+      <c r="D2120" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2121" s="2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2121" s="2" t="inlineStr">
+        <is>
+          <t>$SOXL $AMD $NVDA $INTC $MU</t>
+        </is>
+      </c>
+      <c r="D2121" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2122" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2122" s="2" t="inlineStr">
+        <is>
+          <t>$RDW it&amp;#39;s trying</t>
+        </is>
+      </c>
+      <c r="D2122" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2123" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2123" s="2" t="inlineStr">
+        <is>
+          <t>$RDW Thank you!</t>
+        </is>
+      </c>
+      <c r="D2123" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2124" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2124" s="2" t="inlineStr">
+        <is>
+          <t>$CPSH Are they really doing this again today? Huge dip yesterday followed by a massive rally. $RDW $LASE $SATL $HYLN</t>
+        </is>
+      </c>
+      <c r="D2124" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2125" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2125" s="2" t="inlineStr">
+        <is>
+          <t>$RDW there is going to be insane accumulation tomorrow and Thursday. They will get it as low as they can today.</t>
+        </is>
+      </c>
+      <c r="D2125" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2126" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2126" s="2" t="inlineStr">
+        <is>
+          <t>$RDW 🚩“Welp… RDW’s doing its thing — gap‑filling right around 10:29 PST / 13:29 EST. Tape’s tightening, momentum’s shifting, and it looks like the worst of the drama-for-your-mama phase is finally cooling off. Market’s resetting, sentiment’s stabilizing, and the next move looks a</t>
+        </is>
+      </c>
+      <c r="D2126" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2127" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2127" s="2" t="inlineStr">
+        <is>
+          <t>$RDW</t>
+        </is>
+      </c>
+      <c r="D2127" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2128" s="3" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2128" s="3" t="inlineStr">
+        <is>
+          <t>$FLY $RKLB $RDW PUTS  SPACE STOCKS TOAST FOR NOW DUE TO SPACEX IPO  SELL THE NEWS EVENT  RUN UP IS OVER FOR ALL THESE NAMES</t>
+        </is>
+      </c>
+      <c r="D2128" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2129">
+      <c r="A2129" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2129" s="3" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2129" s="3" t="inlineStr">
+        <is>
+          <t>$RDW Phrase of the Day: “Strategic Issuance”    “This isn’t dilution, it’s strategic issuance.”    Translation: We turned on the share‑printer but wore a suit while doing it.    “We’re enhancing the balance sheet.”    Translation: We needed cash and the hype window was open.    “</t>
+        </is>
+      </c>
+      <c r="D2129" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2130" s="4" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2130" s="4" t="inlineStr">
+        <is>
+          <t>fake bounce bull trap get ready for REAL plunge and then AH bonus massacre</t>
+        </is>
+      </c>
+      <c r="D2130" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2131" s="3" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2131" s="3" t="inlineStr">
+        <is>
+          <t>$RDW This is a gift @ these levels ..some might need to go onto there website &amp;amp; see Everything  this co. Does..Wait till these contracts  start really pouring in..as of know $500 million  back log...The Future of space infrastructure  &amp;amp; more is here.. Dont listen to the N</t>
+        </is>
+      </c>
+      <c r="D2131" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2132">
+      <c r="A2132" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2132" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2132" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$DJT   Weren&amp;#39;t they begging for a deal?   Wasn&amp;#39;t a deal very close?   Isn&amp;#39;t there a ceasefire?   Wasn&amp;#39;t Iran&amp;#39;s military obliterated? All their missiles destroyed?  Wasn&amp;#39;t this suppose to be only 2-3 weeks?   What happened to finish the job?    maga has no </t>
+        </is>
+      </c>
+      <c r="D2132" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2133" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2133" s="3" t="inlineStr">
+        <is>
+          <t>$DJT The formula for making America great again:  Y =  #  x (8 + 6 + 4 + 7) =  #8647</t>
+        </is>
+      </c>
+      <c r="D2133" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2134">
+      <c r="A2134" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2134" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2134" s="4" t="inlineStr">
+        <is>
+          <t>$DJT Oh KA$H. Your Judgment Day is coming. Considering that Crooks was killed that day, there a reason they had to redact the shit outta this too?</t>
+        </is>
+      </c>
+      <c r="D2134" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2135" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2135" s="3" t="inlineStr">
+        <is>
+          <t>$SPY can&amp;#39;t wait to see Trump family filings. Where he sold today, after posting in the morning that an Iran deal is a few days away while already knowing they shot down a US helicopter. MAGA loves to be gaslit, but most of us find it offensive $DJT $QQQ</t>
+        </is>
+      </c>
+      <c r="D2135" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2136" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2136" s="4" t="inlineStr">
+        <is>
+          <t>$DJT Under 8 I see.</t>
+        </is>
+      </c>
+      <c r="D2136" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2137" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2137" s="4" t="inlineStr">
+        <is>
+          <t>$DJT lmao this is heading to penny stock land.</t>
+        </is>
+      </c>
+      <c r="D2137" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2138" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2138" s="4" t="inlineStr">
+        <is>
+          <t>$DJT whatever.... I&amp;#39;ve heard it for 3 months now. First you have to get an M.O.U. signed than you have to implement it.  Good luck with that....</t>
+        </is>
+      </c>
+      <c r="D2138" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2139" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2139" s="3" t="inlineStr">
+        <is>
+          <t>$DJT</t>
+        </is>
+      </c>
+      <c r="D2139" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2140" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2140" s="3" t="inlineStr">
+        <is>
+          <t>$APLD vs $DJT comparing two trending tickers</t>
+        </is>
+      </c>
+      <c r="D2140" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2141" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2141" s="3" t="inlineStr">
+        <is>
+          <t>$DJT It took you 12 years to figure out the con? 🖕🏿</t>
+        </is>
+      </c>
+      <c r="D2141" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2142" s="2" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2142" s="2" t="inlineStr">
+        <is>
+          <t>$SMCI Once over 40 no mercy gap up!</t>
+        </is>
+      </c>
+      <c r="D2142" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2143">
+      <c r="A2143" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2143" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2143" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI nasdaq fell 3% we fell 15%. Sounds about right! 🤣</t>
+        </is>
+      </c>
+      <c r="D2143" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2144">
+      <c r="A2144" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2144" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2144" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI 🐿️</t>
+        </is>
+      </c>
+      <c r="D2144" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2145" s="2" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2145" s="2" t="inlineStr">
+        <is>
+          <t>$SMCI vicious covering!</t>
+        </is>
+      </c>
+      <c r="D2145" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2146" s="2" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2146" s="2" t="inlineStr">
+        <is>
+          <t>$SMCI this will follow the spy!</t>
+        </is>
+      </c>
+      <c r="D2146" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2147" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2147" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI ouch</t>
+        </is>
+      </c>
+      <c r="D2147" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2148" s="2" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2148" s="2" t="inlineStr">
+        <is>
+          <t>$SMCI SPY is going into space! vertical climb!</t>
+        </is>
+      </c>
+      <c r="D2148" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2149" s="2" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2149" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$SMCI     Ongoing rotation may also reflect capital flowing out of legacy hardware names like Dell and HPE and could go all in Super Micro Computer.    SMCI showcased an impressive product portfolio at Computex alongside Nvidia, AMD, Intel, and ARM. Its modular rack architecture </t>
+        </is>
+      </c>
+      <c r="D2149" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2150" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2150" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI let&amp;#39;s get back to 41!!!!</t>
+        </is>
+      </c>
+      <c r="D2150" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2151" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2151" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI today is why u keep cash handy. Its like going to tag sales on the weekend 🤣</t>
+        </is>
+      </c>
+      <c r="D2151" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2152" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2152" s="2" t="inlineStr">
+        <is>
+          <t>$MU going to see recovery at least at least</t>
+        </is>
+      </c>
+      <c r="D2152" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2153" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2153" s="2" t="inlineStr">
+        <is>
+          <t>$SPACZZX.P $MU and $GOOGL doing the storage for all the data.</t>
+        </is>
+      </c>
+      <c r="D2153" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2154" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2154" s="2" t="inlineStr">
+        <is>
+          <t>$MU I panic bought more 😂</t>
+        </is>
+      </c>
+      <c r="D2154" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2155" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2155" s="3" t="inlineStr">
+        <is>
+          <t>$MU got 200 at 890 for a quick swing into 2:30.  All 900 puts, nearly 20 million premium will expire worthless. Mark this. This will close around 920</t>
+        </is>
+      </c>
+      <c r="D2155" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2156" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2156" s="2" t="inlineStr">
+        <is>
+          <t>$MU I suppose days like this are necessary so that we can see higher highs.  Hold strong people.</t>
+        </is>
+      </c>
+      <c r="D2156" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2157" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2157" s="3" t="inlineStr">
+        <is>
+          <t>$MU has taken more than two weeks to gain but two days to drop back? fucking shesh and whos behind this</t>
+        </is>
+      </c>
+      <c r="D2157" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2158" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2158" s="2" t="inlineStr">
+        <is>
+          <t>$MU nice robbery today!</t>
+        </is>
+      </c>
+      <c r="D2158" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2159" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2159" s="2" t="inlineStr">
+        <is>
+          <t>$MU  buy target $1500</t>
+        </is>
+      </c>
+      <c r="D2159" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2160" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2160" s="3" t="inlineStr">
+        <is>
+          <t>$MU can we close at &amp;gt;920 today?</t>
+        </is>
+      </c>
+      <c r="D2160" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2161" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C2161" s="3" t="inlineStr">
+        <is>
+          <t>$MU $907 close</t>
+        </is>
+      </c>
+      <c r="D2161" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2162" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2162" s="3" t="inlineStr">
+        <is>
+          <t>$IGV $NOW $ZS $CRWD Maybe ask Trump and his MAGA for allowing criminal cartel activity and getting kick-backs for this?🚨</t>
+        </is>
+      </c>
+      <c r="D2162" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2163" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2163" s="3" t="inlineStr">
+        <is>
+          <t>$NOW was just a pump n dump</t>
+        </is>
+      </c>
+      <c r="D2163" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2164" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2164" s="3" t="inlineStr">
+        <is>
+          <t>$NOW Had bought it at 102 and sold it all at 124 two days ago only to see it climb further to 136 and felt like an idiot, but today not so much. Might start scaling back in at 112-110</t>
+        </is>
+      </c>
+      <c r="D2164" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2165" s="2" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2165" s="2" t="inlineStr">
+        <is>
+          <t>$NOW saw this coming. I&amp;#39;m a buyer at 110. Hold if it goes lower and add on 100. Then sit back and forget.</t>
+        </is>
+      </c>
+      <c r="D2165" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2166" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2166" s="3" t="inlineStr">
+        <is>
+          <t>$NOW Dont worry all the liquidity keeps pumping same Ai semis bs into trillions everybody else well I guess Bear market-Cant make this up mother of all bubbles MU pumped trillion in year but software gets slaughtered like theres no tomorrow interesting bs Bull market kinda like e</t>
+        </is>
+      </c>
+      <c r="D2166" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2167" s="2" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2167" s="2" t="inlineStr">
+        <is>
+          <t>$NOW I was just kicking myself for selling a week or so ago. Not a popular post but I’m getting back in.. need to do mode DD to scale but so far in super</t>
+        </is>
+      </c>
+      <c r="D2167" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2168" s="4" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2168" s="4" t="inlineStr">
+        <is>
+          <t>$NOW can’t hold onto any type of gain absolute dog shit</t>
+        </is>
+      </c>
+      <c r="D2168" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2169" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2169" s="3" t="inlineStr">
+        <is>
+          <t>@NJLionsfan91 weird to me that software is down at all - especially $NOW</t>
+        </is>
+      </c>
+      <c r="D2169" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2170" s="2" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2170" s="2" t="inlineStr">
+        <is>
+          <t>$NOW the emotional maturity and regulation (or lack thereof) on social media, especially financial social media, is something to behold.  If you think the market is irrational, or irrational in the short term, ask yourself:  “Am I irrational, or irrational in the short term?”.  T</t>
+        </is>
+      </c>
+      <c r="D2170" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B2171" s="3" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2171" s="3" t="inlineStr">
+        <is>
+          <t>$NOW THIS IS A FORTUNE 500 COMPANY TRADING LIKE A PENNY STOCK WHAT THE FUCK</t>
+        </is>
+      </c>
+      <c r="D2171" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -46027,7 +48227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46140,24 +48340,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -46167,7 +48367,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
@@ -46514,7 +48714,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -46524,14 +48724,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -46541,14 +48741,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -46558,14 +48758,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -46582,7 +48782,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -46592,14 +48792,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -46616,7 +48816,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -46633,7 +48833,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -46650,7 +48850,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GLXY</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -46660,87 +48860,87 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>GLXY</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -46752,12 +48952,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -46769,92 +48969,92 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -46871,7 +49071,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -46881,14 +49081,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -46898,14 +49098,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -46915,14 +49115,14 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -46932,14 +49132,14 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -46949,14 +49149,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -46966,14 +49166,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -46983,14 +49183,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -47000,14 +49200,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -47017,14 +49217,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>PUSA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -47034,14 +49234,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-06-03 16:42 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -47051,14 +49251,14 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -47068,14 +49268,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -47085,14 +49285,14 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LFVN</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -47102,14 +49302,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -47119,14 +49319,14 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RCAT</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -47136,14 +49336,14 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>LFVN</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -47153,14 +49353,14 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -47170,14 +49370,14 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>RCAT</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -47187,14 +49387,14 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BNAI</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -47211,7 +49411,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -47228,7 +49428,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>BNAI</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -47245,7 +49445,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MRLN</t>
+          <t>STI</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -47262,7 +49462,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>MRLN</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -47272,7 +49472,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
@@ -47358,6 +49558,91 @@
       <c r="C78" t="inlineStr">
         <is>
           <t>2026-06-08 14:35 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
@@ -47372,7 +49657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -51057,6 +53342,726 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>203.42</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>-3.97%</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>16,464,078</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>27.23M</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>585.04B</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>50.54</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>345.72</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>134.5751</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>41.25</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>0.75%</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>27,826,128</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>21.78M</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>11.79B</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>48.60</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>5.66</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>50.72</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>9.02357</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>256.83</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>-11.09%</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>61,401,778</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>32.31M</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>224.67B</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>59.56</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2.16</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>324.20</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>61.44318</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>290.38</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>-3.70%</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>40,597,984</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>45.47M</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>4264.91B</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>42.51</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>317.40</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>195.0748</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Consumer Electronics</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>203.78</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>-2.33%</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>105,556,110</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>165.97M</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>4931.47B</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>43.42</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>236.54</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>140.8544</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>15.44</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>-16.88%</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>50,164,208</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>33.96M</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2.44</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>3.07B</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>46.96</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2.99</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>42.06</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>4.87216</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>7.86</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>-3.62%</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>3,098,235</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>3.88M</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2.18B</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>37.11</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>63.72</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>7.86</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>39.72</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>-9.70%</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>27,670,617</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>41.66M</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>23.89B</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>53.08</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>1.88</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>62.36</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>19.48103</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Computer Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>899.74</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>-5.22%</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>45,446,324</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>49.48M</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>1014.67B</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>56.38</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2.17</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>1089.29</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>103.38770</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>105.64</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>-7.49%</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>22,727,608</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>26.51M</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>108.95B</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>49.02</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>211.48</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>81.2430</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-10 18:44 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2171"/>
+  <dimension ref="A1:D2271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -48211,6 +48211,2206 @@
         </is>
       </c>
       <c r="D2171" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2172">
+      <c r="A2172" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2172" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2172" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI get the stripper money buy it all!</t>
+        </is>
+      </c>
+      <c r="D2172" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2173" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2173" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI i wouldn&amp;#39;t be surprised if we closed back at 45.   Its just so damn cheap!! 😁</t>
+        </is>
+      </c>
+      <c r="D2173" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2174" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2174" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI Nice nice</t>
+        </is>
+      </c>
+      <c r="D2174" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2175" s="2" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2175" s="2" t="inlineStr">
+        <is>
+          <t>$SMCI start the climb!</t>
+        </is>
+      </c>
+      <c r="D2175" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2176" s="4" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2176" s="4" t="inlineStr">
+        <is>
+          <t>$SMCI 72% for a rate hike. Jobs came back blowing expectations out of the water even though 120/170k jobs added are government, uber drivers, World Cup workers. Can’t cut rates with that news.   That’s not positive news for this sector along with Ai. Reason for the big drop today</t>
+        </is>
+      </c>
+      <c r="D2176" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2177" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2177" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI taking half my profits to the 45s and a roll up.</t>
+        </is>
+      </c>
+      <c r="D2177" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2178" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2178" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI damn. Cant believe what i bought smci shares for today. Im keeping up with the Kardashians!</t>
+        </is>
+      </c>
+      <c r="D2178" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2179" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2179" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI $SMCI. The shorts are now spinning the  same old news on export control investigation by the US and Taiwanese authorities. However, they never mentioned $SMCI was neither indicted nor a defendent in the case. The intent is nothing more than manipulation of market through ps</t>
+        </is>
+      </c>
+      <c r="D2179" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2180" s="2" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2180" s="2" t="inlineStr">
+        <is>
+          <t>$SMCI could be full recovery by Bell!</t>
+        </is>
+      </c>
+      <c r="D2180" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2181" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C2181" s="3" t="inlineStr">
+        <is>
+          <t>$SMCI damn im up 14.00 on dell already.  I might abandon you all for them! 😁</t>
+        </is>
+      </c>
+      <c r="D2181" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2182" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2182" s="2" t="inlineStr">
+        <is>
+          <t>$FRMI  Bullish flow 👃👀  https://x.com/i/status/2064757314121334946</t>
+        </is>
+      </c>
+      <c r="D2182" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2183" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2183" s="3" t="inlineStr">
+        <is>
+          <t>TLDR: The $FRMI headline is loud.    The ETF trail is nerdier, stranger, and probably more useful:    1️⃣ Active values  2️⃣ Global real estate  3️⃣ Texas exposure    That’s the ETFDb point. A trending ticker can show up in baskets you’d never guess from the headline.     Use ETF</t>
+        </is>
+      </c>
+      <c r="D2183" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2184" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2184" s="3" t="inlineStr">
+        <is>
+          <t>3️⃣ $TEXX Horizon Kinetics Texas ETF  📊 $FRMI Weighting: 0.24%  💸 Expense Ratio: 0.85%    And then Texas enters the chat. Yeehaw. 🤠    $TEXX is a Texas-focused ETF, which gives the $FRMI exposure map a very on-brand twist. If traders are watching Project Matador, power demand, an</t>
+        </is>
+      </c>
+      <c r="D2184" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2185" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2185" s="3" t="inlineStr">
+        <is>
+          <t>2️⃣ $SPRE SP Funds S&amp;amp;P Global REIT Sharia ETF  📊 $FRMI Weighting: 0.31%  💸 Expense Ratio: 0.50%    Now the exposure trail takes a turn into real estate.    $SPRE brings global REIT exposure with Sharia-compliant screening, which actually makes the $FRMI connection more intere</t>
+        </is>
+      </c>
+      <c r="D2185" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2186" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2186" s="3" t="inlineStr">
+        <is>
+          <t>1️⃣ $SOVF Sovereign&amp;#39;s Capital Flourish Fund  📊 $FRMI Weighting: 0.91%  💸 Expense Ratio: 0.75%    The biggest ETF weight to $FRMI is not some obvious AI infrastructure moon-basket. 🌕    It’s $SOVF, an actively managed fund with a values-oriented approach. Translation: the stoc</t>
+        </is>
+      </c>
+      <c r="D2186" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2187" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2187" s="3" t="inlineStr">
+        <is>
+          <t>$FRMI is ripping, and it&amp;#39;s plot sounds like it was written by a 2026 market intern with Red Bull and a Bloomberg Terminal. 🥤💽    Investors are chasing a very current storyline: renewed hyperscaler interest in Project Matador, AI data center infrastructure, power demand, and t</t>
+        </is>
+      </c>
+      <c r="D2187" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2188" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2188" s="3" t="inlineStr">
+        <is>
+          <t>$FRMI buy buy buy use 100% margin soon moon 🚀 😆</t>
+        </is>
+      </c>
+      <c r="D2188" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2189" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2189" s="2" t="inlineStr">
+        <is>
+          <t>$FRMI okayyyy 500 shares at $9 come pick me up</t>
+        </is>
+      </c>
+      <c r="D2189" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2190" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2190" s="2" t="inlineStr">
+        <is>
+          <t>$FRMI This is when you buy. before it moves up again.</t>
+        </is>
+      </c>
+      <c r="D2190" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2191" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C2191" s="2" t="inlineStr">
+        <is>
+          <t>$FRMI 2nd trending</t>
+        </is>
+      </c>
+      <c r="D2191" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2192" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2192" s="3" t="inlineStr">
+        <is>
+          <t>$QXO on the bright side it can only go down 14.88…lol…bumpy road ahead…will average down when the dust settles in the market</t>
+        </is>
+      </c>
+      <c r="D2192" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2193" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2193" s="3" t="inlineStr">
+        <is>
+          <t>$QXO Brad Jacobs cooked all investors here by diluting them WAY too much for the intial float size. Biting smaller companies would have been much smarter vs going after the bigger fish. Common stock holders are paying the price</t>
+        </is>
+      </c>
+      <c r="D2193" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2194" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2194" s="3" t="inlineStr">
+        <is>
+          <t>$QXO sold 20 of the weekly $14 puts for 10 a contract. See if I can snag a few thousand shares on the real cheap</t>
+        </is>
+      </c>
+      <c r="D2194" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2195" s="2" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2195" s="2" t="inlineStr">
+        <is>
+          <t>$QXO price went back to 2 years ago :) bought heavily lets see if it holds</t>
+        </is>
+      </c>
+      <c r="D2195" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2196" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2196" s="3" t="inlineStr">
+        <is>
+          <t>$QXO penny stock soon</t>
+        </is>
+      </c>
+      <c r="D2196" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2197" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2197" s="3" t="inlineStr">
+        <is>
+          <t>$QXO guarantee the float goes up on the next report. This is 100% dilution</t>
+        </is>
+      </c>
+      <c r="D2197" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2198" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2198" s="3" t="inlineStr">
+        <is>
+          <t>$QXO   God forbid this finishes at the day low. The balls these shorts have.</t>
+        </is>
+      </c>
+      <c r="D2198" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2199" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2199" s="3" t="inlineStr">
+        <is>
+          <t>$QXO   There’s no bottom 😂  Laughing and crying all at same time 😂</t>
+        </is>
+      </c>
+      <c r="D2199" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2200" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2200" s="3" t="inlineStr">
+        <is>
+          <t>$QXO i think this is the only ticker down 10% today, oh SMCI is down 20% so we have another 10% to fo yet , that woukd put us at $13 and change</t>
+        </is>
+      </c>
+      <c r="D2200" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2201" s="3" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2201" s="3" t="inlineStr">
+        <is>
+          <t>$QXO dang Brad.  Maybe too cocky?</t>
+        </is>
+      </c>
+      <c r="D2201" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2202" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2202" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$ORCL is the ticker getting attention, but the ETF exposure varies by wrapper.    $AOTS ➡️ brings the software platform angle.  $OGIG ➡️ brings the global internet/tech basket.  $TDIV  ➡️ brings the tech dividend approach.    Track daily fund flows, check portfolio exposure, and </t>
+        </is>
+      </c>
+      <c r="D2202" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2203" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2203" s="3" t="inlineStr">
+        <is>
+          <t>3️⃣ $TDIV  First Trust NASDAQ Technology Dividend Index Fund    $TDIV takes a different angle: technology companies with dividend characteristics.    With $ORCL at a 9.82% weighting, this is not just a growth-tech basket. It brings a tech dividend lens to one of the market’s most</t>
+        </is>
+      </c>
+      <c r="D2203" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2204" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2204" s="3" t="inlineStr">
+        <is>
+          <t>2️⃣ $OGIG  ALPS | O’Shares Global Internet Giants ETF    $OGIG focuses on large global internet and technology companies with exposure to digital platforms, cloud, e-commerce, and online growth themes.    Its $ORCL position gives the fund a connection to the enterprise software a</t>
+        </is>
+      </c>
+      <c r="D2204" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2205" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2205" s="3" t="inlineStr">
+        <is>
+          <t>1️⃣ $AOTS  AOT Software Platform ETF    $AOTS targets software platform companies, giving investors exposure to businesses tied to enterprise software, cloud infrastructure, and digital transformation.    With $ORCL in the mix, this is a software-focused basket for traders watchi</t>
+        </is>
+      </c>
+      <c r="D2205" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2206" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2206" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL is trending as traders watch volatility ahead of earnings. 👀    💬 The chatter: profit-taking, AI infrastructure conviction, cloud backlog comparisons, and questions around whether this is just a pullback or a bigger reset.    The stock may be the headline, but the ETF baske</t>
+        </is>
+      </c>
+      <c r="D2206" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2207" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2207" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL Remember that Donald Trump has this stock, so it&amp;#39;s only going up next week.</t>
+        </is>
+      </c>
+      <c r="D2207" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2208" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2208" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL   292 calls for June 18th.......          Shouldnt Oracle be at a 1 trillion marketcap......just off the backlog.....</t>
+        </is>
+      </c>
+      <c r="D2208" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2209" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2209" s="4" t="inlineStr">
+        <is>
+          <t>$ORCL will be worth than avgo 🩸🩸🩸🩸</t>
+        </is>
+      </c>
+      <c r="D2209" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2210" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2210" s="3" t="inlineStr">
+        <is>
+          <t>$VERI $ORCL $GOOGL $NVDA Who wants to place a value on this patent?  @silverws is asking.</t>
+        </is>
+      </c>
+      <c r="D2210" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2211" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2211" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL hurts today. But this is the best way to lead into earnings next week.</t>
+        </is>
+      </c>
+      <c r="D2211" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2212" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2212" s="4" t="inlineStr">
+        <is>
+          <t>$DJT $4 soon Puts will print. Load the Leaps. November…..</t>
+        </is>
+      </c>
+      <c r="D2212" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2213" s="2" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2213" s="2" t="inlineStr">
+        <is>
+          <t>$VMHG https://marketwirenews.com/stock/vmhg/news/victory-marine-holdings-announces-completion-of-init-7421778004967172.html     Victory Marine Holdings Announces Completion of Initial GUTSI(TM) Production and U.S. Market Launch  https://www.stocktitan.net/news/VMHG/victory-marine</t>
+        </is>
+      </c>
+      <c r="D2213" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2214" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2214" s="4" t="inlineStr">
+        <is>
+          <t>$DJT PT 5</t>
+        </is>
+      </c>
+      <c r="D2214" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2215" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2215" s="4" t="inlineStr">
+        <is>
+          <t>$DJT Below , what a beautiful sight ❤️</t>
+        </is>
+      </c>
+      <c r="D2215" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2216" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2216" s="3" t="inlineStr">
+        <is>
+          <t>$DJT $QQQ $SPY $USO $VOO this is DUMB don’t believe this at all</t>
+        </is>
+      </c>
+      <c r="D2216" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2217" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2217" s="3" t="inlineStr">
+        <is>
+          <t>$DJT  Trump is profiting from being POTUS…!!!  Say the DAF Libt💩rd 🤪🤡</t>
+        </is>
+      </c>
+      <c r="D2217" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2218" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2218" s="4" t="inlineStr">
+        <is>
+          <t>$DJT &amp;quot;I never thought he was a good man&amp;quot; You knew and voted for him 3 times?</t>
+        </is>
+      </c>
+      <c r="D2218" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2219" s="4" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2219" s="4" t="inlineStr">
+        <is>
+          <t>$DJT I&amp;#39;m just going to go ahead and say it Donald Trump is by far most incompetent incapable and outright corrupted stupid president in the past hundred years.</t>
+        </is>
+      </c>
+      <c r="D2219" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2220" s="3" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2220" s="3" t="inlineStr">
+        <is>
+          <t>$DJT so anyone that bought in above $50?</t>
+        </is>
+      </c>
+      <c r="D2220" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2221" s="2" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C2221" s="2" t="inlineStr">
+        <is>
+          <t>$DJT The Trump presidency is a total abject failure and sad to be saying this as a lifelong Republican</t>
+        </is>
+      </c>
+      <c r="D2221" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2222" s="3" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2222" s="3" t="inlineStr">
+        <is>
+          <t>$FAC Ripping! It&amp;#39;s a rocket 📈🚀</t>
+        </is>
+      </c>
+      <c r="D2222" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2223" s="3" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2223" s="3" t="inlineStr">
+        <is>
+          <t>$FAC we need a strong close</t>
+        </is>
+      </c>
+      <c r="D2223" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2224" s="2" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2224" s="2" t="inlineStr">
+        <is>
+          <t>$FAC</t>
+        </is>
+      </c>
+      <c r="D2224" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2225" s="3" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2225" s="3" t="inlineStr">
+        <is>
+          <t>$FAC haha. Nice.</t>
+        </is>
+      </c>
+      <c r="D2225" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2226" s="3" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2226" s="3" t="inlineStr">
+        <is>
+          <t>$FAC on 🔥🔥🔥🔥🔥🔥🔥🔥🔥🔥🔥</t>
+        </is>
+      </c>
+      <c r="D2226" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2227" s="2" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2227" s="2" t="inlineStr">
+        <is>
+          <t>$FAC 💎</t>
+        </is>
+      </c>
+      <c r="D2227" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2228" s="3" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2228" s="3" t="inlineStr">
+        <is>
+          <t>$PMI $FAC is on a run</t>
+        </is>
+      </c>
+      <c r="D2228" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2229" s="3" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2229" s="3" t="inlineStr">
+        <is>
+          <t>$FAC are we having fun :D 30! 30!</t>
+        </is>
+      </c>
+      <c r="D2229" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2230" s="3" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2230" s="3" t="inlineStr">
+        <is>
+          <t>$FAC This is up over 30% ON JUST 1.3 million shares traded.....</t>
+        </is>
+      </c>
+      <c r="D2230" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2231" s="2" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C2231" s="2" t="inlineStr">
+        <is>
+          <t>$FAC $Factorial Energy Inc  num num num eat that wall up!!!!</t>
+        </is>
+      </c>
+      <c r="D2231" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2232" s="3" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2232" s="3" t="inlineStr">
+        <is>
+          <t>$CMG know $CBRL is up 26%?</t>
+        </is>
+      </c>
+      <c r="D2232" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2233" s="2" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2233" s="2" t="inlineStr">
+        <is>
+          <t>$CASY $MUSA $CBRL  @Stocktwits  good pizza$</t>
+        </is>
+      </c>
+      <c r="D2233" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2234" s="3" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2234" s="3" t="inlineStr">
+        <is>
+          <t>@cynicaloptimist @BustaCapital @Jblack500 @IsabellaDC @WAJeff @No_Face_character   Yo ,   $CASY  $MUSA $CBRL   +9.35   - nice    Buc-ee&amp;#39;$ wanting to join da party</t>
+        </is>
+      </c>
+      <c r="D2234" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2235" s="3" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2235" s="3" t="inlineStr">
+        <is>
+          <t>$CBRL up 25% after Wells Fargo flagged cheap valuation and 27% short interest as room for more upside. that much short fuel explains the vertical. these squeezy legs fade fast though, I want to see 45 hold into the close. holds, tomorrow gets fun. loses it, round trip city.  this</t>
+        </is>
+      </c>
+      <c r="D2235" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2236" s="2" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2236" s="2" t="inlineStr">
+        <is>
+          <t>$CBRL go push at 50$ !!</t>
+        </is>
+      </c>
+      <c r="D2236" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2237" s="2" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2237" s="2" t="inlineStr">
+        <is>
+          <t>$NDLS Will break 15$ for sure ;) $BYND $CBRL $MCD $CMG</t>
+        </is>
+      </c>
+      <c r="D2237" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2238" s="3" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2238" s="3" t="inlineStr">
+        <is>
+          <t>CBRL Stock On Track To Post Best Single-Day Gains – Wells Fargo Says Cheap Valuation, 27% Short Interest Set Stage For Further Upside  $CBRL  https://stocktwits.com/news/equity/markets/cbrl-stock-gains-wall-street-upside-potential-high-short-interest/cZ06ql1R7c4</t>
+        </is>
+      </c>
+      <c r="D2238" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2239" s="3" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2239" s="3" t="inlineStr">
+        <is>
+          <t>$CBRL kaboom in the room</t>
+        </is>
+      </c>
+      <c r="D2239" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2240" s="3" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2240" s="3" t="inlineStr">
+        <is>
+          <t>Two booming rural names: $CBRL and $CASY</t>
+        </is>
+      </c>
+      <c r="D2240" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2241" s="4" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C2241" s="4" t="inlineStr">
+        <is>
+          <t>$CBRL there goes the after lunch pump, straight down from here.   We thinking 42 or less by EOD? Personally I’m thinking it dumps all the way to $40.</t>
+        </is>
+      </c>
+      <c r="D2241" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2242" s="2" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2242" s="2" t="inlineStr">
+        <is>
+          <t>$LMND   $10.00 day will happen Thursday or Friday or maybe both .</t>
+        </is>
+      </c>
+      <c r="D2242" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2243" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2243" s="3" t="inlineStr">
+        <is>
+          <t>$LMND went up 8 dollars on no volume too! now they are selling their shares to retail. Lets see if it closes red!</t>
+        </is>
+      </c>
+      <c r="D2243" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2244" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2244" s="3" t="inlineStr">
+        <is>
+          <t>$LMND ok what a joke</t>
+        </is>
+      </c>
+      <c r="D2244" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2245" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2245" s="3" t="inlineStr">
+        <is>
+          <t>$LMND It still looks sour. Honestly don&amp;#39;t know why people continue to trade this stock  https://share.trendspider.com/chart/LMND/66828cdj7c</t>
+        </is>
+      </c>
+      <c r="D2245" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2246" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2246" s="3" t="inlineStr">
+        <is>
+          <t>$LMND selling off on low volume. Could see a run up back to $60 in next few days.</t>
+        </is>
+      </c>
+      <c r="D2246" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2247" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2247" s="3" t="inlineStr">
+        <is>
+          <t>$LMND hold or sell?</t>
+        </is>
+      </c>
+      <c r="D2247" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2248" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2248" s="3" t="inlineStr">
+        <is>
+          <t>$LMND This is a casino. from 53 to almost 61, to lose it all again! who knows, close could be 50 or 60!</t>
+        </is>
+      </c>
+      <c r="D2248" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2249" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2249" s="3" t="inlineStr">
+        <is>
+          <t>$LMND why I didn’t sell at 60$ 😞😞😞</t>
+        </is>
+      </c>
+      <c r="D2249" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2250" s="3" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2250" s="3" t="inlineStr">
+        <is>
+          <t>$LMND There is 0.5 between bid and ask, this is a lot for a 50 dollars stock!</t>
+        </is>
+      </c>
+      <c r="D2250" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2251" s="2" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C2251" s="2" t="inlineStr">
+        <is>
+          <t>$LMND 👀</t>
+        </is>
+      </c>
+      <c r="D2251" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2252" s="3" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2252" s="3" t="inlineStr">
+        <is>
+          <t>$FUBO Finally got NBC back. Telemundo right before the World Cup too. Figured Disney would just let it die and never sign any good carriage agreements. Still a massive pile of wet dog shit but they finally did something at least.</t>
+        </is>
+      </c>
+      <c r="D2252" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2253" s="2" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2253" s="2" t="inlineStr">
+        <is>
+          <t>$FUBO</t>
+        </is>
+      </c>
+      <c r="D2253" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2254" s="2" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2254" s="2" t="inlineStr">
+        <is>
+          <t>$FUBO gonna laugh when this thing doubles like it’s nothing</t>
+        </is>
+      </c>
+      <c r="D2254" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2255" s="2" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2255" s="2" t="inlineStr">
+        <is>
+          <t>$FUBO so many apes, nobody will stop this</t>
+        </is>
+      </c>
+      <c r="D2255" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2256" s="2" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2256" s="2" t="inlineStr">
+        <is>
+          <t>$FUBO ah about to be lit!</t>
+        </is>
+      </c>
+      <c r="D2256" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2257" s="2" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2257" s="2" t="inlineStr">
+        <is>
+          <t>$FUBO too many partnerships</t>
+        </is>
+      </c>
+      <c r="D2257" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2258" s="3" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2258" s="3" t="inlineStr">
+        <is>
+          <t>$FUBO wall street running out of garbage to pump</t>
+        </is>
+      </c>
+      <c r="D2258" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2259" s="3" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2259" s="3" t="inlineStr">
+        <is>
+          <t>$FUBO 83 cents</t>
+        </is>
+      </c>
+      <c r="D2259" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2260" s="2" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2260" s="2" t="inlineStr">
+        <is>
+          <t>$FUBO millions of new subscriptions coming near world cup start</t>
+        </is>
+      </c>
+      <c r="D2260" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2261" s="2" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C2261" s="2" t="inlineStr">
+        <is>
+          <t>$FUBO lesgoooooo</t>
+        </is>
+      </c>
+      <c r="D2261" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2262" s="2" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2262" s="2" t="inlineStr">
+        <is>
+          <t>$UEC Apparently the blood suckers aren&amp;#39;t done yet.</t>
+        </is>
+      </c>
+      <c r="D2262" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2263" s="2" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2263" s="2" t="inlineStr">
+        <is>
+          <t>$UEC Ohhh you greedy pricks, quit it.</t>
+        </is>
+      </c>
+      <c r="D2263" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2264" s="3" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2264" s="3" t="inlineStr">
+        <is>
+          <t>$UEC hard to time a perfect buy, but after a negative 40% month it might be worth accumulating some shares.</t>
+        </is>
+      </c>
+      <c r="D2264" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2265" s="2" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2265" s="2" t="inlineStr">
+        <is>
+          <t>$UEC  Thought about adding this yesterday but it looks like the bloodbath continues!  Not just here, even gold has been getting destroyed. I think I will watch for a bit? ￼</t>
+        </is>
+      </c>
+      <c r="D2265" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2266" s="2" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2266" s="2" t="inlineStr">
+        <is>
+          <t>$UEC 🚀</t>
+        </is>
+      </c>
+      <c r="D2266" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2267" s="3" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2267" s="3" t="inlineStr">
+        <is>
+          <t>$UEC Bought I bunch more.</t>
+        </is>
+      </c>
+      <c r="D2267" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2268" s="2" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2268" s="2" t="inlineStr">
+        <is>
+          <t>$UEC the bounce back would be nice! What an opportunity to DCA 🤤</t>
+        </is>
+      </c>
+      <c r="D2268" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2269" s="2" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2269" s="2" t="inlineStr">
+        <is>
+          <t>$UEC What the fuck ? Bankrupt?  ☹️🤕🤛🏻</t>
+        </is>
+      </c>
+      <c r="D2269" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2270" s="2" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2270" s="2" t="inlineStr">
+        <is>
+          <t>$UEC , $UECG   Yes, oversold. I think the tutes wanted 10 but took it to 9.50 for good measure. lol</t>
+        </is>
+      </c>
+      <c r="D2270" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B2271" s="3" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C2271" s="3" t="inlineStr">
+        <is>
+          <t>$UEC selling off after yesterday&amp;#39;s earnings call, down 10.6% on elevated volume. drops like this rarely bottom in one session. my guess, lower low tomorrow before any real bounce.  on my fade list: https://tapeboard.com/research/UEC?utm_source=stocktwits&amp;amp;utm_medium=post&amp;a</t>
+        </is>
+      </c>
+      <c r="D2271" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -48227,7 +50427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48544,63 +50744,63 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -48612,24 +50812,24 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -48639,14 +50839,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -48656,14 +50856,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -48673,14 +50873,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -48690,14 +50890,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -48707,14 +50907,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -48724,14 +50924,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -48741,14 +50941,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -48758,14 +50958,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -48775,14 +50975,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -48799,7 +50999,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -48809,14 +51009,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -48833,7 +51033,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -48850,7 +51050,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -48867,7 +51067,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GLXY</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -48877,14 +51077,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>GLXY</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -48894,7 +51094,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
@@ -48935,160 +51135,160 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>DJT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -49105,7 +51305,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -49122,7 +51322,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -49139,7 +51339,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -49149,14 +51349,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -49166,14 +51366,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -49183,14 +51383,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -49200,14 +51400,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -49217,14 +51417,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -49234,14 +51434,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -49251,14 +51451,14 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>PUSA</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -49268,14 +51468,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -49285,14 +51485,14 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -49302,14 +51502,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -49319,14 +51519,14 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -49343,7 +51543,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LFVN</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -49353,14 +51553,14 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -49370,14 +51570,14 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>RCAT</t>
+          <t>LFVN</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -49387,14 +51587,14 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -49404,14 +51604,14 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>RCAT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -49421,14 +51621,14 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BNAI</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -49445,7 +51645,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -49462,7 +51662,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MRLN</t>
+          <t>BNAI</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -49479,7 +51679,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ZVRA</t>
+          <t>STI</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -49489,14 +51689,14 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BABA</t>
+          <t>MRLN</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -49506,14 +51706,14 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TNGX</t>
+          <t>ZVRA</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -49530,7 +51730,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>BABA</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -49547,7 +51747,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>TNGX</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -49564,7 +51764,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -49574,14 +51774,14 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -49591,14 +51791,14 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>RDW</t>
+          <t>APLD</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -49615,7 +51815,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>DJT</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -49632,7 +51832,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>RDW</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -49643,6 +51843,125 @@
       <c r="C83" t="inlineStr">
         <is>
           <t>2026-06-09 13:33 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
@@ -49657,7 +51976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -54062,6 +56381,726 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>32.22</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>-20.71%</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>92,370,341</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>42.04M</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2.82</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>19.38B</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>41.74</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>62.36</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>19.4865</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Computer Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>6.86</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>22.03%</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>38,427,893</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>15.50M</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>4.37B</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>58.09</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>81.46</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>4.4753</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>REIT - Specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>14.92</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>-9.02%</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>14,760,141</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>13.75M</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>1.38</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>10.82B</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>34.25</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>45.96</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>15.32</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Industrial Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>204.92</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>-0.43%</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>19,971,286</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>27.15M</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>589.37B</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>51.20</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>345.72</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>134.5752</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>DJT</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>7.95</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>-2.51%</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2,129,902</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>3.91M</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>0.70</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2.20B</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>38.07</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>63.00</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>7.762</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>FAC</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>22.70</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>41.88%</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>1,405,091</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>293.85K</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>6.14</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>783.15M</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>89.14</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>-0.17</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>25.33</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>9.26145</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Electrical Equipment &amp; Parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>45.79</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>26.14%</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>8,592,271</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>1.04M</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>10.58</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>1.02B</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>81.93</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>71.93</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>24.8584</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Restaurants</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>LMND</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>55.80</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>4.14%</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2,271,961</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>1.74M</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>4.29B</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>49.53</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>99.90</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>35.7056</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Insurance - Property &amp; Casualty</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>FUBO</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>10.48</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>7.72%</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>1,078,715</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>1.80M</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>0.77</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>1.14B</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>50.75</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2.37</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>81.49</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>8.3126</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Broadcasting</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>UEC</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>9.48</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>-10.94%</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>16,831,909</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>9.66M</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2.24</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>4.65B</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>30.11</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>53.37</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>5.9060</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Uranium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-11 19:27 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2271"/>
+  <dimension ref="A1:D2371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -50413,6 +50413,2206 @@
       <c r="D2271" s="3" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2272" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2272" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT $SPY Microsoft Event Tomorrow morning</t>
+        </is>
+      </c>
+      <c r="D2272" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2273" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2273" s="3" t="inlineStr">
+        <is>
+          <t>The biggest gains usually come from simply holding the right stocks longer than everyone else — and letting time do the rest.    $ZETA → $32+ still early in AI-marketing re-rate  $OSCR → $30+ consolidation breakout finally firing  $NBIS → $300+ AI infrastructure ramping hard  $NO</t>
+        </is>
+      </c>
+      <c r="D2273" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2274" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2274" s="3" t="inlineStr">
+        <is>
+          <t>My latest YouTube video discusses the probable S&amp;amp;P 500 and Nasdaq $QQQ performance through June and by year-end. Uncovering how to position after a 9-week rally and a VIX dropping below 16 for the first time in 2 months, and what the labor market is signaling...    $AMZN $UVI</t>
+        </is>
+      </c>
+      <c r="D2274" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2275" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2275" s="3" t="inlineStr">
+        <is>
+          <t>$MSFT Gap filled…450 strong support.⚡️</t>
+        </is>
+      </c>
+      <c r="D2275" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2276" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2276" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT anybody buy at $451 tonight?</t>
+        </is>
+      </c>
+      <c r="D2276" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2277" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2277" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation ( $MSFT ) SpicyTrade - Daily Stock Analysis https://youtu.be/waHH9YLJuNs?si=8ogBNRxAvKIS8u1K</t>
+        </is>
+      </c>
+      <c r="D2277" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2278" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2278" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT $META $CRM All these fuckin hedgies can STAY underwater for all i care they shouldn’t have overleveraged their shorts in the fuckin first place!!!!!!🖕🤣🌮🍿🤫✅</t>
+        </is>
+      </c>
+      <c r="D2278" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2279" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2279" s="3" t="inlineStr">
+        <is>
+          <t>$GOOGL already recovering from 367 dump;  $BRK.B buying them cheap ;     $MSFT $NOW hype cooling down; buy at dips soon    $NOC cant believ this dumped alot today.     NOC is best one to buy while market ATH</t>
+        </is>
+      </c>
+      <c r="D2279" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2280" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2280" s="2" t="inlineStr">
+        <is>
+          <t>$MSFT  govt invested 2 billion for 10% of $INTEL.X  .. it’s worth 34 billion today.. they are doing the same exact thing with Quantum industry .. $QTEX will undoubtedly benefit .. in this moment it is proper to trade following the governments intentions .. with $39 trillion in de</t>
+        </is>
+      </c>
+      <c r="D2280" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2281" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C2281" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$MSFT hold up. We’re down because of a Google Dilution with Berkshire being the purchaser?  Um. Yea tomorrow is a buy lmfaoooooooooooooo  Ai Infrastructure purchase by the one and only??  Also, Google is absolutely fucked up spending wise compared to us with their TPUs. We don’t </t>
+        </is>
+      </c>
+      <c r="D2281" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2282" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2282" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK nice</t>
+        </is>
+      </c>
+      <c r="D2282" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2283" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2283" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK Multiple millions added each day. Not really sustainable honestly</t>
+        </is>
+      </c>
+      <c r="D2283" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2284" s="4" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2284" s="4" t="inlineStr">
+        <is>
+          <t>$SNDK 🚨    Iran has not yet confirmed that all of this is lies and nonsense.</t>
+        </is>
+      </c>
+      <c r="D2284" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2285" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2285" s="3" t="inlineStr">
+        <is>
+          <t>$SNDQ $SNDK</t>
+        </is>
+      </c>
+      <c r="D2285" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2286" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2286" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK man, just take all my money. BK me.</t>
+        </is>
+      </c>
+      <c r="D2286" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2287" s="4" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2287" s="4" t="inlineStr">
+        <is>
+          <t>$SNDK Way too many green candles in a row. Prepare for meltdown</t>
+        </is>
+      </c>
+      <c r="D2287" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2288" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2288" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL $NBIS $MRAM $SNDK $MU</t>
+        </is>
+      </c>
+      <c r="D2288" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2289" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2289" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK  Update: Leopold might be doing it again…    $SNDK is moving fast:  Up another 6.6% today  Now +25% since his most recent 13F filing    Why it’s catching attention:  Strong follow-through after institutional positioning  Momentum keeps building instead of fading  Traders wh</t>
+        </is>
+      </c>
+      <c r="D2289" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2290" s="2" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2290" s="2" t="inlineStr">
+        <is>
+          <t>$SNDK Breached 52 week high.  We’re in uncharted territory.</t>
+        </is>
+      </c>
+      <c r="D2290" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2291" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2291" s="3" t="inlineStr">
+        <is>
+          <t>@uhmillie @Holdmybagz $SPY $QQQ $AMD $MU $sndk  they done like cubie said. nailed it 🫡☺️</t>
+        </is>
+      </c>
+      <c r="D2291" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2292" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2292" s="2" t="inlineStr">
+        <is>
+          <t>@drewLA Everyone is thinking this, so that means $ADBE will have more room to climb. I will sell when retail gets more bullish on it</t>
+        </is>
+      </c>
+      <c r="D2292" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2293" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2293" s="2" t="inlineStr">
+        <is>
+          <t>$CRM $NOW $ADBE $SHOP $MSFT Me pounding the table on SaaS. I&amp;#39;m never wrong on these calls 🍀</t>
+        </is>
+      </c>
+      <c r="D2293" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2294" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2294" s="2" t="inlineStr">
+        <is>
+          <t>$QTEX  will make some new millionaires soon just like $ASTC    let’s see $ADBE $IBM $INTC</t>
+        </is>
+      </c>
+      <c r="D2294" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2295" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2295" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE I am down from 340 but added 2028 calls at 240.</t>
+        </is>
+      </c>
+      <c r="D2295" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2296" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2296" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE it is absurd how cheap this has gotten despite adopting AI and having a MOAT as a business tool.   Expect this to crush earnings, confirm buyback and raise outlook.</t>
+        </is>
+      </c>
+      <c r="D2296" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2297" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2297" s="3" t="inlineStr">
+        <is>
+          <t>@Jeremymartin007 @simon58 @judgeyoung2 @jenbunn @ribbey @EBE_day @TraderRapp @Godreal1 @tonyctl @zuby34  $ADBE $CRM  thats why dont short low.pe stonks. short expensive ones near max pain have better chance $NOW muy bueno,  $SNOW ok</t>
+        </is>
+      </c>
+      <c r="D2297" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2298" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2298" s="3" t="inlineStr">
+        <is>
+          <t>$ADBE $CRM $NOW $SNOW $WDAY this could have been generational wealth but you were sidelined 🔥</t>
+        </is>
+      </c>
+      <c r="D2298" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2299" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2299" s="3" t="inlineStr">
+        <is>
+          <t>$ADBE HA! I HATE YOUR PRODUCTS ADOBE NOW SURRENDER YOUR MONEY TO MEEEE</t>
+        </is>
+      </c>
+      <c r="D2299" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2300" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2300" s="3" t="inlineStr">
+        <is>
+          <t>$ADBE holy shit. Software is back. Now they just have to not fuck up the earnings.</t>
+        </is>
+      </c>
+      <c r="D2300" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2301" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2301" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE Im only down 22% now! Fuck yeah!</t>
+        </is>
+      </c>
+      <c r="D2301" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2302" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2302" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL so the wall street idiots are expecting weaker job report for interest rate cuts and today’s sell of is anguish reaction for strong job report. Idiots</t>
+        </is>
+      </c>
+      <c r="D2302" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2303" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2303" s="2" t="inlineStr">
+        <is>
+          <t>$INTC $ORCL For the first time today, and with considerable effort, the Nasdaq futures contract for June on the 15-minute bar was close to giving a buy signal on three technical indicators 30 minutes ago if it had remained stable... This sell-off was algorithm-driven, as after th</t>
+        </is>
+      </c>
+      <c r="D2303" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2304" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2304" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL Bad earnings incoming?</t>
+        </is>
+      </c>
+      <c r="D2304" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2305" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2305" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL someone forgot to turn algo off</t>
+        </is>
+      </c>
+      <c r="D2305" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2306" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2306" s="3" t="inlineStr">
+        <is>
+          <t>With $META raising cash to fund AI buildout. Time for $ORCL to declare bankruptcy</t>
+        </is>
+      </c>
+      <c r="D2306" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2307" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2307" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL dropped 10% overnight despite zero fundamental changes.  Jesus</t>
+        </is>
+      </c>
+      <c r="D2307" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2308" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2308" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL ffs, orcl is now down MORE than the 9001 pe semis that caused this crash.  amd, intc, qcom are down less than 10%.  thisd iss -10.3%    WHAT THE FUCK, MAN.</t>
+        </is>
+      </c>
+      <c r="D2308" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="A2309" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2309" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2309" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL seriously, what is it about oracle that makes it absolutely gutted when ANYTHING is red?  software, bonds, semis, macro, ai, trading cards, pogs - if ANYTHING is down, no matter how much the market is up, orcl will be deep red.      it&amp;#39;s been this way for 8 fucking mont</t>
+        </is>
+      </c>
+      <c r="D2309" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="A2310" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2310" s="3" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2310" s="3" t="inlineStr">
+        <is>
+          <t>$ORCL Lets thank Taco for him sponsoring this stock and letting it fly. Because the greedy mofos at WS wanna play games. Thanx, a sincere follower. Dont forget to invest.</t>
+        </is>
+      </c>
+      <c r="D2310" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2311" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2311" s="2" t="inlineStr">
+        <is>
+          <t>$ORCL lol , ill add some more here too,</t>
+        </is>
+      </c>
+      <c r="D2311" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2312" s="4" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2312" s="4" t="inlineStr">
+        <is>
+          <t>$VELO is complete garbage.  Trading at at 9–10x sales is the most expensive name in 3D printing. Low margin, non recurring revenue business. Revenue has gone down 76% over 3 years. While shares outstanding quadrupled. One of the most overvalued companies out there.</t>
+        </is>
+      </c>
+      <c r="D2312" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2313" s="3" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2313" s="3" t="inlineStr">
+        <is>
+          <t>$VELO what a week, who’s ready for the main event tomorrow?</t>
+        </is>
+      </c>
+      <c r="D2313" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2314" s="3" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2314" s="3" t="inlineStr">
+        <is>
+          <t>$FUBO sit back and relax, things can change really fast, a few days ago $VELO was $15, now it’s almost $32.. the same thing will happen with Fubo.</t>
+        </is>
+      </c>
+      <c r="D2314" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2315" s="4" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2315" s="4" t="inlineStr">
+        <is>
+          <t>$VELO i would not hold this over night</t>
+        </is>
+      </c>
+      <c r="D2315" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="A2316" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2316" s="4" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2316" s="4" t="inlineStr">
+        <is>
+          <t>$VELO i like it short here</t>
+        </is>
+      </c>
+      <c r="D2316" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="A2317" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2317" s="3" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2317" s="3" t="inlineStr">
+        <is>
+          <t>$VELO will be lifechanging, dyor asap!!! 👍</t>
+        </is>
+      </c>
+      <c r="D2317" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2318" s="4" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2318" s="4" t="inlineStr">
+        <is>
+          <t>$VELO</t>
+        </is>
+      </c>
+      <c r="D2318" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2319" s="2" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2319" s="2" t="inlineStr">
+        <is>
+          <t>@cykuTYTkaxa Let&amp;#39;s let it do it&amp;#39;s thing,   Rising tides are good for everyone.   The relative &amp;quot;ponds&amp;quot; will adjust with time.   Just look back at the $VELO chart and you will see it was $3.05, exactly where DD is now (more or less) and where the offering closed a</t>
+        </is>
+      </c>
+      <c r="D2319" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="A2320" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2320" s="3" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2320" s="3" t="inlineStr">
+        <is>
+          <t>$VELO     Day traders taking profit into close    Should see a retest of that 28 area</t>
+        </is>
+      </c>
+      <c r="D2320" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="A2321" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2321" s="3" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C2321" s="3" t="inlineStr">
+        <is>
+          <t>$VELO YUHHH</t>
+        </is>
+      </c>
+      <c r="D2321" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2322">
+      <c r="A2322" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2322" s="3" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2322" s="3" t="inlineStr">
+        <is>
+          <t>$TE &amp;amp; $CHPY on the move</t>
+        </is>
+      </c>
+      <c r="D2322" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2323" s="2" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2323" s="2" t="inlineStr">
+        <is>
+          <t>$TE fingers crossed for a 20-30% day soon.</t>
+        </is>
+      </c>
+      <c r="D2323" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="A2324" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2324" s="2" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2324" s="2" t="inlineStr">
+        <is>
+          <t>$TE who else bought the dip. And if you didn’t, we still are in a dip. So buy as much as you can and squeeze the crap out of Fuzzy after Roth reiterated.   Very bullish.</t>
+        </is>
+      </c>
+      <c r="D2324" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="A2325" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2325" s="3" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2325" s="3" t="inlineStr">
+        <is>
+          <t>$TE running hot, +8.2% a day after that Fuzzy Panda short report knocked it around. snapback verticals like this can give it all back fast, so I&amp;#39;m watching whether it keeps holding above the 7.73 prior close. who&amp;#39;s in this one?  this is what my scanner flagged: https://ta</t>
+        </is>
+      </c>
+      <c r="D2325" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="A2326" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2326" s="2" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2326" s="2" t="inlineStr">
+        <is>
+          <t>$TE We are ready for take-off 🚀</t>
+        </is>
+      </c>
+      <c r="D2326" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2327" s="3" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2327" s="3" t="inlineStr">
+        <is>
+          <t>$TE some listen and some don&amp;#39;t</t>
+        </is>
+      </c>
+      <c r="D2327" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="A2328" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2328" s="2" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2328" s="2" t="inlineStr">
+        <is>
+          <t>$TE they called it!</t>
+        </is>
+      </c>
+      <c r="D2328" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="A2329" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2329" s="2" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2329" s="2" t="inlineStr">
+        <is>
+          <t>$TE The unicorn stock of 2026. Watch this fly.      $SPY $DIA $QQQ $TSLA</t>
+        </is>
+      </c>
+      <c r="D2329" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2330" s="3" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2330" s="3" t="inlineStr">
+        <is>
+          <t>$TE</t>
+        </is>
+      </c>
+      <c r="D2330" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="A2331" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2331" s="2" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C2331" s="2" t="inlineStr">
+        <is>
+          <t>$TE fuzzie Panda getting them drawz ripped right off their ass!</t>
+        </is>
+      </c>
+      <c r="D2331" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2332" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2332" s="2" t="inlineStr">
+        <is>
+          <t>$SATS after hours gonna be epic!!!</t>
+        </is>
+      </c>
+      <c r="D2332" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="A2333" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2333" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2333" s="2" t="inlineStr">
+        <is>
+          <t>$SATS $150 real quick</t>
+        </is>
+      </c>
+      <c r="D2333" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2334" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2334" s="2" t="inlineStr">
+        <is>
+          <t>$SATS I know running today in expectation but this still doesn’t look like pricing in any pop for tomorrow?</t>
+        </is>
+      </c>
+      <c r="D2334" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="A2335" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2335" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2335" s="2" t="inlineStr">
+        <is>
+          <t>$SATS $SPACZZX.P I know it does not mean a lot what they do over there…. But sentiment is epic 🤌🏼🚀  It’s in €….. so actually 228$ ‼️🚀</t>
+        </is>
+      </c>
+      <c r="D2335" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2336" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2336" s="3" t="inlineStr">
+        <is>
+          <t>$SPACZZX.P $SATS tic toc</t>
+        </is>
+      </c>
+      <c r="D2336" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2337">
+      <c r="A2337" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2337" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2337" s="3" t="inlineStr">
+        <is>
+          <t>$SATS  $127.XX is the next hard resistance.  Then 132, 138, 147</t>
+        </is>
+      </c>
+      <c r="D2337" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="A2338" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2338" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2338" s="2" t="inlineStr">
+        <is>
+          <t>$SATS https://www.benzinga.com/trading-ideas/movers/26/06/53152182/echostar-stock-soars-ahead-of-spacex-ipo</t>
+        </is>
+      </c>
+      <c r="D2338" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="A2339" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2339" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2339" s="3" t="inlineStr">
+        <is>
+          <t>$SATS  Expect Space X to purchase SATS for 100 billion dollars within 6 months of IPO !!</t>
+        </is>
+      </c>
+      <c r="D2339" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2340">
+      <c r="A2340" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2340" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2340" s="3" t="inlineStr">
+        <is>
+          <t>$SATS Anticipating a reversal (up) mos tof the rest of today based on technicals.</t>
+        </is>
+      </c>
+      <c r="D2340" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="A2341" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2341" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2341" s="2" t="inlineStr">
+        <is>
+          <t>$SATS</t>
+        </is>
+      </c>
+      <c r="D2341" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="A2342" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2342" s="4" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2342" s="4" t="inlineStr">
+        <is>
+          <t>$SPCE</t>
+        </is>
+      </c>
+      <c r="D2342" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2343">
+      <c r="A2343" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2343" s="2" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2343" s="2" t="inlineStr">
+        <is>
+          <t>$SPCE BOUGHT MORE HERE🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D2343" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2344">
+      <c r="A2344" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2344" s="3" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2344" s="3" t="inlineStr">
+        <is>
+          <t>$SPCE $6.46 looks like our new support.</t>
+        </is>
+      </c>
+      <c r="D2344" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2345">
+      <c r="A2345" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2345" s="3" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2345" s="3" t="inlineStr">
+        <is>
+          <t>$SPCE lol its over already</t>
+        </is>
+      </c>
+      <c r="D2345" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2346">
+      <c r="A2346" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2346" s="3" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2346" s="3" t="inlineStr">
+        <is>
+          <t>$SPCE all you gotta do is:  🚀🚀🚀🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D2346" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2347">
+      <c r="A2347" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2347" s="2" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2347" s="2" t="inlineStr">
+        <is>
+          <t>$SPCE</t>
+        </is>
+      </c>
+      <c r="D2347" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2348">
+      <c r="A2348" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2348" s="2" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2348" s="2" t="inlineStr">
+        <is>
+          <t>$SPCE 2 weeks until SpaceX IPO, this ride is just starting</t>
+        </is>
+      </c>
+      <c r="D2348" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2349">
+      <c r="A2349" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2349" s="2" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2349" s="2" t="inlineStr">
+        <is>
+          <t>$RKTO $SPCE</t>
+        </is>
+      </c>
+      <c r="D2349" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2350">
+      <c r="A2350" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2350" s="3" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2350" s="3" t="inlineStr">
+        <is>
+          <t>$SPCE Fives shortly</t>
+        </is>
+      </c>
+      <c r="D2350" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2351">
+      <c r="A2351" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2351" s="3" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C2351" s="3" t="inlineStr">
+        <is>
+          <t>$SPCE Back to $7.00 then double digits! 😍</t>
+        </is>
+      </c>
+      <c r="D2351" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2352">
+      <c r="A2352" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2352" s="3" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2352" s="3" t="inlineStr">
+        <is>
+          <t>$KLAC will have 1.36 Billion shares and good luck if you think the stock is going to run further actually massive selling and lighting up by institutions investors</t>
+        </is>
+      </c>
+      <c r="D2352" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2353">
+      <c r="A2353" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2353" s="3" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2353" s="3" t="inlineStr">
+        <is>
+          <t>$KLAC will crash tomorrow as i guarantee you because for 10 for 1 split will create so much dolitoon on the stock with 1.5ab shares outstanding and always you are going to find sellers tomorrow and all next week to lock up their profits.Iam warning from slim experience for the la</t>
+        </is>
+      </c>
+      <c r="D2353" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2354">
+      <c r="A2354" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2354" s="3" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2354" s="3" t="inlineStr">
+        <is>
+          <t>$KLAC from my own experience for the last 36 yrs in the market after the split the stock will tank and Lrcx after the split lost  almost 60% of the stock value after the split and it took them over 9 months to bounce to all time high</t>
+        </is>
+      </c>
+      <c r="D2354" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2355">
+      <c r="A2355" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2355" s="2" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2355" s="2" t="inlineStr">
+        <is>
+          <t>$KLAC alright, wheres the guy that had a short position here?</t>
+        </is>
+      </c>
+      <c r="D2355" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2356">
+      <c r="A2356" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2356" s="2" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2356" s="2" t="inlineStr">
+        <is>
+          <t>$KLAC - up $229.00 from next suggested buy entry. Projected price target $2395.00 area.</t>
+        </is>
+      </c>
+      <c r="D2356" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2357">
+      <c r="A2357" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2357" s="2" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2357" s="2" t="inlineStr">
+        <is>
+          <t>When market rallies, chips lead the gains.   Look at those monster gains:  $KORU 29%  $SOXL 20%  $SNDK 12%  $KLAC 12%    And of course we have the contrarian $SOXS with -20%    The beauty is nearly all of chips aren&amp;#39;t even close to being in RSI oversold - meaning it&amp;#39;s got</t>
+        </is>
+      </c>
+      <c r="D2357" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2358">
+      <c r="A2358" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2358" s="3" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2358" s="3" t="inlineStr">
+        <is>
+          <t>$AMAT $ASML $KLAC $LRCX 🎯</t>
+        </is>
+      </c>
+      <c r="D2358" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2359">
+      <c r="A2359" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2359" s="3" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2359" s="3" t="inlineStr">
+        <is>
+          <t>$KLAC the Iranian just denied any deal close with the USA</t>
+        </is>
+      </c>
+      <c r="D2359" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2360">
+      <c r="A2360" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2360" s="3" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2360" s="3" t="inlineStr">
+        <is>
+          <t>$KLAC Barclays analyst Tom O&amp;#39;Malley maintains KLA (NASDAQ:KLAC) with a Overweight and raises the price target from $1700 to $2250.This target is within 52 weeks not one day target</t>
+        </is>
+      </c>
+      <c r="D2360" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2361">
+      <c r="A2361" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2361" s="3" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C2361" s="3" t="inlineStr">
+        <is>
+          <t>$KLAC even the ceo Mr Wallace is selling his own shares because he knows this price is not going to last much longer.They are selling a commodity products</t>
+        </is>
+      </c>
+      <c r="D2361" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2362">
+      <c r="A2362" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2362" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2362" s="3" t="inlineStr">
+        <is>
+          <t>$RKLB if this IPO doesn&amp;#39;t do well....a lot of people in deep doodoo</t>
+        </is>
+      </c>
+      <c r="D2362" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2363">
+      <c r="A2363" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2363" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2363" s="3" t="inlineStr">
+        <is>
+          <t>$APP bought back this after sold $IREN $RKLB $HOOD $MRVL</t>
+        </is>
+      </c>
+      <c r="D2363" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2364">
+      <c r="A2364" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2364" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2364" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB  When Wall street is pumping SpaceX like the only thing in the world right now, take pause before buying. Its the stocks they don&amp;#39;t pump that do best.  Not advising, but warningof rash moves. Been at this since 1992.</t>
+        </is>
+      </c>
+      <c r="D2364" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2365">
+      <c r="A2365" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2365" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2365" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB let&amp;#39;s fly bulls!!!!!</t>
+        </is>
+      </c>
+      <c r="D2365" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2366">
+      <c r="A2366" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2366" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2366" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB   Shorts are getting hammered.     RKLB is in an excellent spot righ now, and will capatilize on the new space economy.</t>
+        </is>
+      </c>
+      <c r="D2366" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2367">
+      <c r="A2367" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2367" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2367" s="3" t="inlineStr">
+        <is>
+          <t>$RKLB I’m smelling burnt shorts, or maybe it’s rocket fuel?? Anyone else smell that?</t>
+        </is>
+      </c>
+      <c r="D2367" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2368">
+      <c r="A2368" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2368" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2368" s="3" t="inlineStr">
+        <is>
+          <t>$RKLB I thought you know what you are doing... but you are egoistic bear like michael burry.  Hope you are doing good.</t>
+        </is>
+      </c>
+      <c r="D2368" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2369">
+      <c r="A2369" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2369" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2369" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB 120 EOD.</t>
+        </is>
+      </c>
+      <c r="D2369" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2370">
+      <c r="A2370" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2370" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2370" s="3" t="inlineStr">
+        <is>
+          <t>$RKLB hard to get a feel on how this will react to the IPO tmmrw. Love this company and holding but tempted to buy more now or see if money flows from here to SpaceX</t>
+        </is>
+      </c>
+      <c r="D2370" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2371">
+      <c r="A2371" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B2371" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2371" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB tomorow we fly😉</t>
+        </is>
+      </c>
+      <c r="D2371" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
         </is>
       </c>
     </row>
@@ -50427,7 +52627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50506,7 +52706,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -50516,14 +52716,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-11 15:27 ET</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -50540,7 +52740,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -50550,24 +52750,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
@@ -50591,7 +52791,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BTC.X</t>
+          <t>SPCE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -50601,14 +52801,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-11 15:27 ET</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>BTC.X</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -50618,41 +52818,41 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-01 21:58 UTC</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
@@ -50727,34 +52927,34 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-11 15:27 ET</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-10 14:44 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
@@ -50863,7 +53063,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -50873,14 +53073,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-11 15:27 ET</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -50890,14 +53090,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ETH.X</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -50907,14 +53107,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>ETH.X</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -50924,14 +53124,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-03 11:36 ET</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -50941,14 +53141,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-03 11:36 ET</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -50958,14 +53158,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -50975,14 +53175,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -50992,14 +53192,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -51016,7 +53216,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -51026,14 +53226,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -51050,7 +53250,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -51067,7 +53267,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -51084,7 +53284,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GLXY</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -51094,14 +53294,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>GLXY</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -51111,14 +53311,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -51135,7 +53335,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DJT</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -51145,14 +53345,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-10 14:44 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>DJT</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -51169,24 +53369,24 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -51196,48 +53396,48 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -51254,24 +53454,24 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -51288,24 +53488,24 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -51322,7 +53522,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -51339,7 +53539,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -51962,6 +54162,108 @@
       <c r="C90" t="inlineStr">
         <is>
           <t>2026-06-10 14:44 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
         </is>
       </c>
     </row>
@@ -51976,7 +54278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -57101,6 +59403,726 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>387.46</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>-2.49%</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>29,904,129</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>34.54M</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>2878.26B</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>35.86</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>555.45</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>356.288</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>1858.17</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>13.08%</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>10,221,030</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>15.48M</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>275.18B</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>66.97</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>5.06</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>1861.00</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>39.444611</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Computer Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>221.99</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>-4.88%</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>8,502,172</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>5.59M</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>89.73B</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>35.53</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>416.39</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>224.13</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>182.93</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>-9.11%</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>53,165,568</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>27.07M</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>526.13B</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>41.65</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>345.72</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>134.5735</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>VELO</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>31.44</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>38.62%</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>14,384,776</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>3.04M</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>5.36</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>936.95M</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>70.47</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>26.5018</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2.811018</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Computer Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>8.19</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>5.95%</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>31,917,640</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>26.76M</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>2.29B</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>48.35</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>2.23</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>34.43</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>1.15612</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Electrical Equipment &amp; Parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>126.26</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>9.56%</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>12,010,457</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>6.95M</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>36.59B</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>52.15</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>147.25</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>16.60660</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Telecom Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>5.99</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>27.28%</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>96,053,655</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>22.63M</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>4.81</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>603.60M</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>63.98</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>2.69</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>32.64</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2.13181</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2389.69</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>11.90%</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>948,818</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>1.02M</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>312.16B</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>71.74</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>2304.413</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>832.24187</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Semiconductor Equipment &amp; Materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>113.49</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>8.03%</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>18,254,787</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>25.62M</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>0.81</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>65.69B</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>49.31</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>2.59</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>151.00</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>25.24349</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-12 17:52 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2371"/>
+  <dimension ref="A1:D2471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -52611,6 +52611,2206 @@
         </is>
       </c>
       <c r="D2371" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2372">
+      <c r="A2372" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2372" s="4" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2372" s="4" t="inlineStr">
+        <is>
+          <t>$SPCX  Im  a buyer sub $70</t>
+        </is>
+      </c>
+      <c r="D2372" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2373">
+      <c r="A2373" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2373" s="2" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2373" s="2" t="inlineStr">
+        <is>
+          <t>$SPCX 4th grade smack talk. Love it! You do you, buddy!</t>
+        </is>
+      </c>
+      <c r="D2373" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2374">
+      <c r="A2374" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2374" s="3" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2374" s="3" t="inlineStr">
+        <is>
+          <t>$SPCX Dont chase the hype of Elon Musk. Wait until December  .</t>
+        </is>
+      </c>
+      <c r="D2374" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2375">
+      <c r="A2375" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2375" s="2" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2375" s="2" t="inlineStr">
+        <is>
+          <t>$SPCX come boys SPACEX to become World’s most valuable company on 1st day of trading public.   This is the headline we need</t>
+        </is>
+      </c>
+      <c r="D2375" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2376">
+      <c r="A2376" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2376" s="2" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2376" s="2" t="inlineStr">
+        <is>
+          <t>$SPCX ipo</t>
+        </is>
+      </c>
+      <c r="D2376" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2377">
+      <c r="A2377" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2377" s="3" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2377" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA $SPCX  those* money*  this play was not rocket science.  pardon the pun😅</t>
+        </is>
+      </c>
+      <c r="D2377" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2378">
+      <c r="A2378" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2378" s="3" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2378" s="3" t="inlineStr">
+        <is>
+          <t>$SPCX 2 trades today 137 to the good lol not what i was thinking might happen</t>
+        </is>
+      </c>
+      <c r="D2378" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2379">
+      <c r="A2379" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2379" s="3" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2379" s="3" t="inlineStr">
+        <is>
+          <t>$SPCX  I will buy shares in the company that shoots down musks rockets in space.</t>
+        </is>
+      </c>
+      <c r="D2379" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2380">
+      <c r="A2380" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2380" s="2" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2380" s="2" t="inlineStr">
+        <is>
+          <t>Early $SPCX  investors capital will hit the market eventually and once they do, you can bet they will buy $$NVDA , $CRWD , &amp;amp; $PLTR</t>
+        </is>
+      </c>
+      <c r="D2380" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2381">
+      <c r="A2381" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2381" s="3" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C2381" s="3" t="inlineStr">
+        <is>
+          <t>$SPCX $SPY $QQQ Take that canadaQ</t>
+        </is>
+      </c>
+      <c r="D2381" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2382">
+      <c r="A2382" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2382" s="2" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2382" s="2" t="inlineStr">
+        <is>
+          <t>$SNDK to the fucking moon!!</t>
+        </is>
+      </c>
+      <c r="D2382" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2383">
+      <c r="A2383" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2383" s="2" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2383" s="2" t="inlineStr">
+        <is>
+          <t>$SNDK miss me - trefuego 🔥</t>
+        </is>
+      </c>
+      <c r="D2383" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2384">
+      <c r="A2384" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2384" s="2" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2384" s="2" t="inlineStr">
+        <is>
+          <t>$SNDK can’t believe the bears are still here. They have no shame</t>
+        </is>
+      </c>
+      <c r="D2384" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2385">
+      <c r="A2385" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2385" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2385" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK 2k eow not impossible lol</t>
+        </is>
+      </c>
+      <c r="D2385" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2386">
+      <c r="A2386" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2386" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2386" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK The algos have gone haywire. This is straight up insanity.</t>
+        </is>
+      </c>
+      <c r="D2386" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2387">
+      <c r="A2387" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2387" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2387" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK this has be the blowoff move.  Getting myself mentally ready to go all in short</t>
+        </is>
+      </c>
+      <c r="D2387" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2388">
+      <c r="A2388" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2388" s="4" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2388" s="4" t="inlineStr">
+        <is>
+          <t>am i right in my guess: what a great opportunity to SHORT in small small increments as these bloated stocks try to find a TOP $MU $SNDK</t>
+        </is>
+      </c>
+      <c r="D2388" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2389">
+      <c r="A2389" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2389" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2389" s="3" t="inlineStr">
+        <is>
+          <t>$MRVL $NBIS $MRAM $SNDK $MU That kind of day...</t>
+        </is>
+      </c>
+      <c r="D2389" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2390">
+      <c r="A2390" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2390" s="3" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2390" s="3" t="inlineStr">
+        <is>
+          <t>$SNDK short of the century here</t>
+        </is>
+      </c>
+      <c r="D2390" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2391">
+      <c r="A2391" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2391" s="2" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C2391" s="2" t="inlineStr">
+        <is>
+          <t>$SNDK we get it you want a dip to get back in. You missed it get over it</t>
+        </is>
+      </c>
+      <c r="D2391" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2392">
+      <c r="A2392" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2392" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2392" s="3" t="inlineStr">
+        <is>
+          <t>$RKLB   The last few days, the stock price has risen significantly In overnight trading.   It will be interesting to see what happens tonight . . .</t>
+        </is>
+      </c>
+      <c r="D2392" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2393">
+      <c r="A2393" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2393" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2393" s="3" t="inlineStr">
+        <is>
+          <t>🧊 ⬆️ $RKLB flipped to Vol-damping (dealers pin price), heat -35 since last session, now ~$114.    Inside the $100 to $120 range, 5% to the call, 13% to the put.    Damping means dealers are long gamma with spot above the $95 flip: their hedging sells strength and buys dips, which</t>
+        </is>
+      </c>
+      <c r="D2393" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2394">
+      <c r="A2394" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2394" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2394" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB run boy run!</t>
+        </is>
+      </c>
+      <c r="D2394" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2395">
+      <c r="A2395" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2395" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2395" s="2" t="inlineStr">
+        <is>
+          <t>$ASTS SpaceX will run like $TSLA did in 2020 $RKLB $LUNR $RDW</t>
+        </is>
+      </c>
+      <c r="D2395" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2396">
+      <c r="A2396" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2396" s="3" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2396" s="3" t="inlineStr">
+        <is>
+          <t>$RKLB — This is called the STAIRWAY TO THE MOON!      Since 5 AM, you @tradepulsealerts have been busy chasing pennies and getting burned in the process. Meanwhile, I remain focused on the long-term picture, where daily price fluctuations mean very little.    The trend remains fu</t>
+        </is>
+      </c>
+      <c r="D2396" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2397">
+      <c r="A2397" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2397" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2397" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB that aged well 🤙</t>
+        </is>
+      </c>
+      <c r="D2397" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2398">
+      <c r="A2398" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2398" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2398" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB Afterhour and overnight will be fun today</t>
+        </is>
+      </c>
+      <c r="D2398" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2399">
+      <c r="A2399" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2399" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2399" s="2" t="inlineStr">
+        <is>
+          <t>$RKLB close above $115 🥹</t>
+        </is>
+      </c>
+      <c r="D2399" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2400">
+      <c r="A2400" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2400" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2400" s="2" t="inlineStr">
+        <is>
+          <t>$SIDU LFG, get on board, major $SPCX hype starts now.     $ASTS $SPCE $RKLB</t>
+        </is>
+      </c>
+      <c r="D2400" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2401">
+      <c r="A2401" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2401" s="2" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C2401" s="2" t="inlineStr">
+        <is>
+          <t>The accumulation goes unabated.  Love  these three.  $ASTS   $RKLB   $FLY    SpaceX who ?</t>
+        </is>
+      </c>
+      <c r="D2401" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2402">
+      <c r="A2402" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2402" s="3" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2402" s="3" t="inlineStr">
+        <is>
+          <t>$TTD May 22 was last time it closed within 1% of the day&amp;#39;s high.</t>
+        </is>
+      </c>
+      <c r="D2402" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2403">
+      <c r="A2403" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2403" s="3" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2403" s="3" t="inlineStr">
+        <is>
+          <t>$TTD Still incapable of closing within 1% of days highs.</t>
+        </is>
+      </c>
+      <c r="D2403" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2404">
+      <c r="A2404" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2404" s="3" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2404" s="3" t="inlineStr">
+        <is>
+          <t>Just scored a massive 10-bagger on $ARMG. Realized gains: +$127,000 (+1,023%)!    My buddy Marcus was exhausted from working back-to-back night shifts. I urged him to stop scalping for peanuts and instead focus on high-conviction trades. He studied my ARMG thesis and-just like me</t>
+        </is>
+      </c>
+      <c r="D2404" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2405">
+      <c r="A2405" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2405" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2405" s="2" t="inlineStr">
+        <is>
+          <t>$TTD don’t let them fool ya.  What’s been happening the whole time as you’ve been getting pummelled by shorts?   Is it coordinated? Yes.   Paytience 👏</t>
+        </is>
+      </c>
+      <c r="D2405" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2406">
+      <c r="A2406" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2406" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2406" s="2" t="inlineStr">
+        <is>
+          <t>$TTD higher highs, higher lows</t>
+        </is>
+      </c>
+      <c r="D2406" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2407">
+      <c r="A2407" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2407" s="3" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2407" s="3" t="inlineStr">
+        <is>
+          <t>$TTD So Publicis is once again recommending The Trade Desk to clients what a bunch of criminals.</t>
+        </is>
+      </c>
+      <c r="D2407" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2408">
+      <c r="A2408" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2408" s="3" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2408" s="3" t="inlineStr">
+        <is>
+          <t>$TTD seems like sell on news type of price action. Need some more positive momentum.</t>
+        </is>
+      </c>
+      <c r="D2408" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2409">
+      <c r="A2409" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2409" s="3" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2409" s="3" t="inlineStr">
+        <is>
+          <t>$TTD shorts are not covering, this is Tuesdays price, it will take more than this to push them out.</t>
+        </is>
+      </c>
+      <c r="D2409" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2410">
+      <c r="A2410" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2410" s="3" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2410" s="3" t="inlineStr">
+        <is>
+          <t>$TTD super disappointing. Good news, top 10 trending on here. Can’t get over $20 lmao what a joke!</t>
+        </is>
+      </c>
+      <c r="D2410" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2411">
+      <c r="A2411" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2411" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C2411" s="2" t="inlineStr">
+        <is>
+          <t>$TTD Time for these unhinged weetodded shorts to start covering!</t>
+        </is>
+      </c>
+      <c r="D2411" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2412">
+      <c r="A2412" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2412" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2412" s="3" t="inlineStr">
+        <is>
+          <t>$SPACZZX.P $SPY $TSLA funds 25% secured.</t>
+        </is>
+      </c>
+      <c r="D2412" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2413">
+      <c r="A2413" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2413" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2413" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA live trader just said space ex mauy be cancelled for being too garbage a stock?</t>
+        </is>
+      </c>
+      <c r="D2413" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2414">
+      <c r="A2414" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2414" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2414" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA der is no manipulation only deficient markets $SPY</t>
+        </is>
+      </c>
+      <c r="D2414" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2415">
+      <c r="A2415" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2415" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2415" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA   This is a stupid weak move.  5 min RSI looks retarded….</t>
+        </is>
+      </c>
+      <c r="D2415" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2416">
+      <c r="A2416" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2416" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2416" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA double bottom</t>
+        </is>
+      </c>
+      <c r="D2416" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2417">
+      <c r="A2417" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2417" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2417" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA It&amp;#39;s always some trashy Gupta. And they are always last to know who is the trash. And it is always JPM or GS.</t>
+        </is>
+      </c>
+      <c r="D2417" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2418">
+      <c r="A2418" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2418" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2418" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA no recovery bounce today?</t>
+        </is>
+      </c>
+      <c r="D2418" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2419">
+      <c r="A2419" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2419" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2419" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA will this trade with SpaceX’s ipo</t>
+        </is>
+      </c>
+      <c r="D2419" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2420">
+      <c r="A2420" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2420" s="3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2420" s="3" t="inlineStr">
+        <is>
+          <t>$TSLA space ex is so garbage it may not even be eligable to be a stock now. lmao.     funny becasue tesla is still allowed in major indexes and it&amp;#39;s basically the same.</t>
+        </is>
+      </c>
+      <c r="D2420" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2421">
+      <c r="A2421" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2421" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C2421" s="2" t="inlineStr">
+        <is>
+          <t>$TSLA lost 200 SMA and 20 EMA, now testing 50 SMA  5 weeks of gains wiped  Can’t imagine much enthusiasm for $SPACZZX.P is this continues</t>
+        </is>
+      </c>
+      <c r="D2421" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2422">
+      <c r="A2422" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2422" s="2" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2422" s="2" t="inlineStr">
+        <is>
+          <t>$ASTS one would expect an EOD bounce.</t>
+        </is>
+      </c>
+      <c r="D2422" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2423">
+      <c r="A2423" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2423" s="4" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2423" s="4" t="inlineStr">
+        <is>
+          <t>$ASTS $LUNR $NASA $PL $RDW all dead will be in deep red entire month</t>
+        </is>
+      </c>
+      <c r="D2423" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2424">
+      <c r="A2424" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2424" s="2" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2424" s="2" t="inlineStr">
+        <is>
+          <t>$ASTS Took some shares here</t>
+        </is>
+      </c>
+      <c r="D2424" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2425" s="3" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2425" s="3" t="inlineStr">
+        <is>
+          <t>$ASTS $100</t>
+        </is>
+      </c>
+      <c r="D2425" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2426">
+      <c r="A2426" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2426" s="2" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2426" s="2" t="inlineStr">
+        <is>
+          <t>$ASTS The data shows the mechanics of trade volume, distinguishing between the buying (Inflow) and selling (Outflow) pressure.  Order Flow Distribution: This chart tracks money moving into and out of the stock.  Inflow (460M) vs. Outflow (293M): Despite the stock price being down</t>
+        </is>
+      </c>
+      <c r="D2426" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2427">
+      <c r="A2427" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2427" s="3" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2427" s="3" t="inlineStr">
+        <is>
+          <t>$ASTS 80 please</t>
+        </is>
+      </c>
+      <c r="D2427" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2428">
+      <c r="A2428" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2428" s="2" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2428" s="2" t="inlineStr">
+        <is>
+          <t>$ASTS acumulating at this price , Jun 17th coming up</t>
+        </is>
+      </c>
+      <c r="D2428" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2429">
+      <c r="A2429" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2429" s="3" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2429" s="3" t="inlineStr">
+        <is>
+          <t>$ASTS more selloff</t>
+        </is>
+      </c>
+      <c r="D2429" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2430" s="2" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2430" s="2" t="inlineStr">
+        <is>
+          <t>$ASTS call me crazy but i still see $88-90 EOD  this is all manipulation spcx ipo or not this should be in mid to high 90s right now</t>
+        </is>
+      </c>
+      <c r="D2430" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2431">
+      <c r="A2431" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2431" s="3" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2431" s="3" t="inlineStr">
+        <is>
+          <t>$ASTS   Break one way or another.</t>
+        </is>
+      </c>
+      <c r="D2431" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2432">
+      <c r="A2432" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2432" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2432" s="3" t="inlineStr">
+        <is>
+          <t>$SATS catching the space group bid ahead of the SpaceX debut, up 9.9% and holding the move all session. these sympathy runs can fade fast once the hype cools, but tape&amp;#39;s been steady so far. who&amp;#39;s riding the space basket today, drop your names.  this is what my scanner fla</t>
+        </is>
+      </c>
+      <c r="D2432" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2433">
+      <c r="A2433" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2433" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2433" s="2" t="inlineStr">
+        <is>
+          <t>$SATS This evening should be interesting and pre-market.  Let&amp;#39;s all hope for lift off and not an explosion on the launch pad!!</t>
+        </is>
+      </c>
+      <c r="D2433" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2434">
+      <c r="A2434" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2434" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2434" s="2" t="inlineStr">
+        <is>
+          <t>$SATS This is such a good post:    &amp;quot;   $SATS currently has over 30% of its float sold short. Its market cap is only $34B By selling spectrum to   $T  , the company is expected to receive $23B in cash. The FCC’s final approval for that transaction is scheduled for 6/11. On to</t>
+        </is>
+      </c>
+      <c r="D2434" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2435">
+      <c r="A2435" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2435" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2435" s="2" t="inlineStr">
+        <is>
+          <t>$SATS Requesting FULL SEND. Curb stomp these  🩳</t>
+        </is>
+      </c>
+      <c r="D2435" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2436">
+      <c r="A2436" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2436" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2436" s="2" t="inlineStr">
+        <is>
+          <t>$SATS ☘️</t>
+        </is>
+      </c>
+      <c r="D2436" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2437">
+      <c r="A2437" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2437" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2437" s="3" t="inlineStr">
+        <is>
+          <t>$SATS already up on the double</t>
+        </is>
+      </c>
+      <c r="D2437" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2438">
+      <c r="A2438" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2438" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2438" s="3" t="inlineStr">
+        <is>
+          <t>$SATS 🚀🚀🚀🚀</t>
+        </is>
+      </c>
+      <c r="D2438" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2439">
+      <c r="A2439" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2439" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2439" s="3" t="inlineStr">
+        <is>
+          <t>$SATS 🌝🌝🌝</t>
+        </is>
+      </c>
+      <c r="D2439" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2440">
+      <c r="A2440" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2440" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2440" s="3" t="inlineStr">
+        <is>
+          <t>$SATS mooning</t>
+        </is>
+      </c>
+      <c r="D2440" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2441">
+      <c r="A2441" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2441" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C2441" s="2" t="inlineStr">
+        <is>
+          <t>$ASTS if you squint hard enough you can convince yourself you own $SATS</t>
+        </is>
+      </c>
+      <c r="D2441" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2442">
+      <c r="A2442" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2442" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2442" s="3" t="inlineStr">
+        <is>
+          <t>$ADBE another, yet they were simply marking the bottom and asking you for your shares.  But CC will show the way! Already has...</t>
+        </is>
+      </c>
+      <c r="D2442" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2443">
+      <c r="A2443" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2443" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2443" s="3" t="inlineStr">
+        <is>
+          <t>Shameful and useless idiots telling you NO on $ADBE over the past few months, and I will soon show you how CC exposes the market deception - only to me for now.  Look it up if you missed these worthless interviews.</t>
+        </is>
+      </c>
+      <c r="D2443" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2444">
+      <c r="A2444" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2444" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2444" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE</t>
+        </is>
+      </c>
+      <c r="D2444" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2445">
+      <c r="A2445" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2445" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2445" s="3" t="inlineStr">
+        <is>
+          <t>Snowflake&amp;#39;s Historic Stock Boom Is Turning SaaS Panic Into A Short-Covering Problem  $SNOW $CRM $PATH $ADBE $TEAM   https://www.benzinga.com/trading-ideas/movers/26/06/52915000/snowflakes-historic-stock-boom-is-turning-saas-panic-into-a-short-covering-problem</t>
+        </is>
+      </c>
+      <c r="D2445" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2446">
+      <c r="A2446" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2446" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2446" s="3" t="inlineStr">
+        <is>
+          <t>$ADBE weren&amp;#39;t you like 620 2 years ago??   what do?  OHHHH AI made you worthless and your TOS pissed your lifelong users off.   FK round Find out.</t>
+        </is>
+      </c>
+      <c r="D2446" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2447">
+      <c r="A2447" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2447" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2447" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE   $DOCU $MSFT $QQQ $SPY</t>
+        </is>
+      </c>
+      <c r="D2447" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2448">
+      <c r="A2448" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2448" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2448" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE    amazing gross margins and now Trump long.  Very undervalued.</t>
+        </is>
+      </c>
+      <c r="D2448" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2449">
+      <c r="A2449" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2449" s="3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2449" s="3" t="inlineStr">
+        <is>
+          <t>$ADBE nice. Making big gains already since i entered. Holding.</t>
+        </is>
+      </c>
+      <c r="D2449" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2450">
+      <c r="A2450" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2450" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2450" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE I believed in this stock right from the beginning of the &amp;quot;SaaS apocalypse&amp;quot;!</t>
+        </is>
+      </c>
+      <c r="D2450" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2451">
+      <c r="A2451" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2451" s="2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C2451" s="2" t="inlineStr">
+        <is>
+          <t>$ADBE super bullish trend. Loving the price action!!!</t>
+        </is>
+      </c>
+      <c r="D2451" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2452">
+      <c r="A2452" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2452" s="3" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2452" s="3" t="inlineStr">
+        <is>
+          <t>$RDW Buy for The Future  Growth here... Long))) Good day to all you..out</t>
+        </is>
+      </c>
+      <c r="D2452" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2453">
+      <c r="A2453" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2453" s="3" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2453" s="3" t="inlineStr">
+        <is>
+          <t>$RDW Trump says U.S. must &amp;#39;respond&amp;#39; after Iran shoots down helicopter over Hormuz Strait</t>
+        </is>
+      </c>
+      <c r="D2453" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2454">
+      <c r="A2454" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2454" s="3" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2454" s="3" t="inlineStr">
+        <is>
+          <t>$RDW 100% will buy back in.. was here for the spacex pop.. cashed out the 1st one.. will pick up some for the long term later..</t>
+        </is>
+      </c>
+      <c r="D2454" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2455">
+      <c r="A2455" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2455" s="3" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2455" s="3" t="inlineStr">
+        <is>
+          <t>$RDW The dip is violent because the repricing was fast- not because the company is broken.  The chart looks ugly.  The candles look brutal.  The emotions are real.  But the buiness didn&amp;#39;t chage. Only the math did.  And once dilution is absorbed, stocks stabilize, build  a bas</t>
+        </is>
+      </c>
+      <c r="D2455" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2456">
+      <c r="A2456" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2456" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2456" s="2" t="inlineStr">
+        <is>
+          <t>$RDW buy</t>
+        </is>
+      </c>
+      <c r="D2456" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2457">
+      <c r="A2457" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2457" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2457" s="2" t="inlineStr">
+        <is>
+          <t>$RDW just a theory…. Could the dilution be to only generate funds to then buy the shares back at this price? As they know what’s about to happen with all space stocks?</t>
+        </is>
+      </c>
+      <c r="D2457" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2458">
+      <c r="A2458" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2458" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2458" s="2" t="inlineStr">
+        <is>
+          <t>$RDW 🔮</t>
+        </is>
+      </c>
+      <c r="D2458" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2459">
+      <c r="A2459" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2459" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2459" s="2" t="inlineStr">
+        <is>
+          <t>$RDW I think it&amp;#39;s time to get in 🤞</t>
+        </is>
+      </c>
+      <c r="D2459" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2460">
+      <c r="A2460" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2460" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2460" s="2" t="inlineStr">
+        <is>
+          <t>$RDW strong buy</t>
+        </is>
+      </c>
+      <c r="D2460" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2461">
+      <c r="A2461" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2461" s="2" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C2461" s="2" t="inlineStr">
+        <is>
+          <t>$RDW fomo gonna be crazy here</t>
+        </is>
+      </c>
+      <c r="D2461" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2462">
+      <c r="A2462" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2462" s="4" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2462" s="4" t="inlineStr">
+        <is>
+          <t>$ASTS $LUNR $NASA $PL $RDW all dead will be in deep red entire month</t>
+        </is>
+      </c>
+      <c r="D2462" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2463">
+      <c r="A2463" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2463" s="3" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2463" s="3" t="inlineStr">
+        <is>
+          <t>$LUNR This isn&amp;#39;t a direct competitor of spacex and could see them working together if they do not already. Good buy here will pick up a starter</t>
+        </is>
+      </c>
+      <c r="D2463" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2464">
+      <c r="A2464" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2464" s="2" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2464" s="2" t="inlineStr">
+        <is>
+          <t>$LUNR Not expecting this but accept the reality and move on</t>
+        </is>
+      </c>
+      <c r="D2464" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2465">
+      <c r="A2465" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2465" s="2" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2465" s="2" t="inlineStr">
+        <is>
+          <t>@TheIndustrials All other space stocks are still down too, $ASTS, $LUNR, $RKLB...etc  We&amp;#39;re doing ok considering an ongoing offering. Once that is closed and the image is clearer for the sentiment surrounding SpaceX, all of the space stocks will jump</t>
+        </is>
+      </c>
+      <c r="D2465" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2466">
+      <c r="A2466" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2466" s="3" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2466" s="3" t="inlineStr">
+        <is>
+          <t>$LUNR why we didn’t sell at $45? WHY???</t>
+        </is>
+      </c>
+      <c r="D2466" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2467">
+      <c r="A2467" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2467" s="2" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2467" s="2" t="inlineStr">
+        <is>
+          <t>$LUNR be greedy when others are being fearful</t>
+        </is>
+      </c>
+      <c r="D2467" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2468">
+      <c r="A2468" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2468" s="4" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2468" s="4" t="inlineStr">
+        <is>
+          <t>$LUNR timber $SPCX</t>
+        </is>
+      </c>
+      <c r="D2468" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2469">
+      <c r="A2469" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2469" s="4" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2469" s="4" t="inlineStr">
+        <is>
+          <t>$LUNR $ASTS $RDW $RKLB I can&amp;#39;t wait to see this.</t>
+        </is>
+      </c>
+      <c r="D2469" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2470">
+      <c r="A2470" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2470" s="2" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2470" s="2" t="inlineStr">
+        <is>
+          <t>$LUNR Red day, same thesis. $4.82B NASA Near Space Network contract, $180.4M IM-5 lunar mission award, growing backlog, and new lunar reconnaissance contracts.   The market is trading emotion while Intuitive Machines is building the communications and navigation backbone of the M</t>
+        </is>
+      </c>
+      <c r="D2470" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2471">
+      <c r="A2471" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B2471" s="2" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C2471" s="2" t="inlineStr">
+        <is>
+          <t>$LUNR rug pull at spcx imminent</t>
+        </is>
+      </c>
+      <c r="D2471" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
@@ -52627,7 +54827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52961,63 +55161,63 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-12 13:52 ET</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -53029,24 +55229,24 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FLNC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>FLNC</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -53056,14 +55256,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -53073,7 +55273,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-11 15:27 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
@@ -53318,7 +55518,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -53328,14 +55528,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-12 13:52 ET</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -53352,7 +55552,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DJT</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -53362,14 +55562,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-06-10 14:44 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>RDW</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -53379,121 +55579,121 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-10 14:44 ET</t>
+          <t>2026-06-12 13:52 ET</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>DJT</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-01 22:07 UTC</t>
+          <t>2026-06-12 13:52 ET</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>SATS</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-12 13:52 ET</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-06-01 15:17 UTC</t>
+          <t>2026-06-12 13:52 ET</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-06-02 20:40 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -53505,92 +55705,92 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 22:07 UTC</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ALOY</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>FLY</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-01 15:17 UTC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-06-01 15:03 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>NASA</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-02 20:40 UTC</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -53600,14 +55800,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-06-01 15:08 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>ALOY</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -53617,14 +55817,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-06-01 18:15 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -53634,14 +55834,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SOXS</t>
+          <t>XAUUSD</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -53651,14 +55851,14 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-06-03 00:30 UTC</t>
+          <t>2026-06-01 15:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>NASA</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -53668,14 +55868,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-06-03 01:03 UTC</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -53685,14 +55885,14 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 15:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>NUAI</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -53702,14 +55902,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-06-02 21:21 ET</t>
+          <t>2026-06-01 18:15 UTC</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DRTS</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -53719,14 +55919,14 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-06-03 11:27 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>SOXS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -53736,14 +55936,14 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 00:30 UTC</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>PUSA</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -53753,14 +55953,14 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-03 01:03 UTC</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -53770,14 +55970,14 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-06-03 19:40 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>LFVN</t>
+          <t>GME</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -53787,14 +55987,14 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-02 21:21 ET</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>DRTS</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -53804,14 +56004,14 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-06-04 14:02 ET</t>
+          <t>2026-06-03 11:27 ET</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>RCAT</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -53821,14 +56021,14 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-06-04 15:53 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -53838,14 +56038,14 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -53855,14 +56055,14 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-03 19:40 ET</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BNAI</t>
+          <t>LFVN</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -53872,14 +56072,14 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -53889,14 +56089,14 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 14:02 ET</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MRLN</t>
+          <t>RCAT</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -53906,14 +56106,14 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-06-05 13:25 ET</t>
+          <t>2026-06-04 15:53 ET</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ZVRA</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -53923,14 +56123,14 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BABA</t>
+          <t>BNAI</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -53940,14 +56140,14 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TNGX</t>
+          <t>STI</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -53957,14 +56157,14 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>MRLN</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -53974,14 +56174,14 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-06-08 14:35 ET</t>
+          <t>2026-06-05 13:25 ET</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>ZVRA</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -53998,7 +56198,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>BABA</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -54008,14 +56208,14 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>TNGX</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -54025,14 +56225,14 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>RDW</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -54042,14 +56242,14 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-06-09 13:33 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FRMI</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -54059,14 +56259,14 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-06-10 14:44 ET</t>
+          <t>2026-06-08 14:35 ET</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>QXO</t>
+          <t>APLD</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -54076,14 +56276,14 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-06-10 14:44 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>FAC</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -54093,14 +56293,14 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-06-10 14:44 ET</t>
+          <t>2026-06-09 13:33 ET</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>FRMI</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -54117,7 +56317,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>LMND</t>
+          <t>QXO</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -54134,7 +56334,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>FUBO</t>
+          <t>FAC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -54151,7 +56351,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>UEC</t>
+          <t>CBRL</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -54168,7 +56368,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>LMND</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -54178,14 +56378,14 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-06-11 15:27 ET</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>VELO</t>
+          <t>FUBO</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -54195,14 +56395,14 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-06-11 15:27 ET</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>UEC</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -54212,14 +56412,14 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-06-11 15:27 ET</t>
+          <t>2026-06-10 14:44 ET</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SATS</t>
+          <t>VELO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -54236,7 +56436,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -54253,7 +56453,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -54264,6 +56464,74 @@
       <c r="C96" t="inlineStr">
         <is>
           <t>2026-06-11 15:27 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
         </is>
       </c>
     </row>
@@ -54278,7 +56546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N81"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -60123,6 +62391,726 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>170.62</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>26.38%</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>350,813,838</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>2230.98B</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2006.60</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>6.65%</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>8,354,671</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>15.44M</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>0.83</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>297.16B</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>71.30</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>4.93</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>1895.005</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>39.444987</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Computer Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>105.57</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>-8.03%</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>49,732,335</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>25.74M</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2.96</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>61.11B</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>45.16</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>2.55</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>151.00</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>25.24318</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>19.80</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>4.77%</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>18,490,431</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>19.74M</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>9.31B</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>43.03</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>91.45</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>18.377</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>Advertising Agencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>400.88</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>0.43%</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>42,726,728</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>58.91M</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>1505.59B</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>46.92</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>1.81</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>498.83</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>288.7738</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>83.85</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>-14.05%</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>40,158,025</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>19.44M</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>3.17</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>32.55B</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>43.87</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>2.67</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>133.86</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>35.81134</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>Communication Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>112.68</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>-12.06%</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>36,333,464</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>7.12M</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>7.83</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>32.66B</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>41.12</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>147.25</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>16.73573</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>Telecom Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>203.08</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>-7.18%</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>18,822,815</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>5.79M</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>4.99</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>82.08B</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>29.11</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>416.39</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>218.09</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>RDW</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>15.52</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>-9.18%</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>50,353,832</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>35.90M</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>3.09B</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>47.52</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>41.74</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>4.87218</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>26.93</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>-12.11%</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>16,588,178</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>15.37M</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>5.84B</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>42.65</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>1.78</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>46.75</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>7.78246</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-14 15:08 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2471"/>
+  <dimension ref="A1:D2481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -54811,6 +54811,226 @@
         </is>
       </c>
       <c r="D2471" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2472">
+      <c r="A2472" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2472" s="3" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2472" s="3" t="inlineStr">
+        <is>
+          <t>$ROKU  +20% on takeover speculation. Momentum is clearly reacting to the headline.    Potential strategic buyers being floated:  $DIS, $WBD, $PSKY -all need scale in streaming distribution, and Roku brings ~100M users into the equation.    But there’s a key structural detail most</t>
+        </is>
+      </c>
+      <c r="D2472" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2473">
+      <c r="A2473" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2473" s="4" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2473" s="4" t="inlineStr">
+        <is>
+          <t>$ROKU Take y&amp;#39;all profits!! Monday this will tank imo</t>
+        </is>
+      </c>
+      <c r="D2473" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2474">
+      <c r="A2474" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2474" s="3" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2474" s="3" t="inlineStr">
+        <is>
+          <t>$ROKU I wonder if we get follow up news this coming week. Strange to make the report and not name a company. Woods would only sell at an insane premium. This could be big news and I wonder if it establishes a new bottom. I think it’s going to be Netflix.</t>
+        </is>
+      </c>
+      <c r="D2474" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2475">
+      <c r="A2475" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2475" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2475" s="2" t="inlineStr">
+        <is>
+          <t>$ROKU ROKU Stock: Retail View    Retail sentiment on Stocktwits was &amp;#39;extremely bullish&amp;#39; with &amp;#39;extremely high&amp;#39; message volumes. Retail chatter has soared about 116% over the past week and month.    The stock is rated &amp;#39;Buy&amp;#39; by 25 of 29 analysts, with three a</t>
+        </is>
+      </c>
+      <c r="D2475" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2476">
+      <c r="A2476" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2476" s="3" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2476" s="3" t="inlineStr">
+        <is>
+          <t>$ROKU interesting short set up soon</t>
+        </is>
+      </c>
+      <c r="D2476" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2477">
+      <c r="A2477" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2477" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2477" s="2" t="inlineStr">
+        <is>
+          <t>$ROKU super bullish for Monday!!</t>
+        </is>
+      </c>
+      <c r="D2477" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2478">
+      <c r="A2478" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2478" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2478" s="2" t="inlineStr">
+        <is>
+          <t>$ROKU amazing day 🎉</t>
+        </is>
+      </c>
+      <c r="D2478" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2479">
+      <c r="A2479" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2479" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2479" s="2" t="inlineStr">
+        <is>
+          <t>$ROKU this opens at 160 tonight</t>
+        </is>
+      </c>
+      <c r="D2479" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2480">
+      <c r="A2480" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2480" s="3" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2480" s="3" t="inlineStr">
+        <is>
+          <t>$ROKU Here come the Johnny come lately crowd 😳</t>
+        </is>
+      </c>
+      <c r="D2480" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="2481">
+      <c r="A2481" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B2481" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2481" s="2" t="inlineStr">
+        <is>
+          <t>$ROKU hitting its highest share price since 2022, fueled by M&amp;amp;A headlines and a fresh $185 price target from Evercore ISI. Momentum is real here.</t>
+        </is>
+      </c>
+      <c r="D2481" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
@@ -54827,7 +55047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56532,6 +56752,23 @@
       <c r="C100" t="inlineStr">
         <is>
           <t>2026-06-12 13:52 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
         </is>
       </c>
     </row>
@@ -56546,7 +56783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -63111,6 +63348,78 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:08 ET</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>143.66</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>20.08%</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>14,922,301</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2.48M</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>6.01</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>21.20B</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>69.09</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>133.467</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>73.9194</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-14 16:04 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Raw Messages" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ticker Frequency" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="FinViz Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NLP Sentiment" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -445,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -913,6 +914,28 @@
       <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 12:03 ET</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>$ROKU   Massive news next week!!!!!</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -960,12 +983,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-14 11:49 ET</t>
+          <t>2026-06-14 12:03 ET</t>
         </is>
       </c>
     </row>
@@ -997,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1226,6 +1249,830 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-14 12:03 ET</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>143.66</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>20.08%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>14,922,301</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2.48M</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>6.01</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>21.20B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>69.09</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>133.467</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>73.9194</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-14 12:03 ET</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>355.20</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.32%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2,698,896</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2.66M</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>191.70B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>61.93</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>391.29</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>267.8332</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Drug Manufacturers - General</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SYMBOL</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CLEAN TEXT</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ORIGINAL SENTIMENT</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NLP LABEL</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>NLP SCORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>your day trading watch list for june 15th in 2 minutes .</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>roku continues to grow despite, what many may consider unfair trade practices by google. i understand google uses its brute financial power by paying costco to keep the likes of roku tvs out of costco. google39s infinite financial pockets are seemingly able to steer or</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>20 on takeover speculation. momentum is clearly reacting to the headline. potential strategic buyers being floated , , -all need scale in streaming distribution, and roku brings 100m users into the equation. but theres a key structural detail most</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>take y39all profits!! monday this will tank imo</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>i wonder if we get follow up news this coming week. strange to make the report and not name a company. woods would only sell at an insane premium. this could be big news and i wonder if it establishes a new bottom. i think its going to be netflix.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>roku stock retail view retail sentiment on stocktwits was 39extremely bullish39 with 39extremely high39 message volumes. retail chatter has soared about 116 over the past week and month. the stock is rated 39buy39 by 25 of 29 analysts, with three a</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>interesting short set up soon</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>super bullish for monday!!</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>amazing day</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>this opens at 160 tonight</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>patience is going to be the primary requirement if you want to have successful outcome with this outfit... we see very few discussions as it relates to a buyout of this issue... after having been in this jizz-bizz for over 60 years, i see all the signs of a potential buy</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>anyone here know when cvot data will be released for lp with a little a ? it39s going to be a blockbuster!</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>it39s coming. it39ll be a blockbuster.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>abbvie reports promising new clinical updates. here39s what it means for the company39s dividend</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>bullish above the stomach candlestick pattern formed</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>this is gonna rip higher in the coming days. it39s coming out of that slow rolling base with a break of the descending trend line and a successful retest on higher volume.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>amgen is seeking to defend the future of tavneos after hiring the duke clinical research institute to conduct an independent reanalysis of the clinical trial data that supported the drugs approval. the move comes as the fda pushes to withdraw tavneos from the market over concern</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>why this going up ??</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>winner winner</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 12:03 ET</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>massive news next week!!!!!</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-14 17:13 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -934,6 +934,314 @@
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$ROKU is nearly 50% of my portfolio right now and avg cost of ~$70 and I didn&amp;#39;t think about selling and likely won&amp;#39;t unless this goes past $200 soon or there&amp;#39;s news of an agreed upon sale lower than that, which would be disappointing. I can&amp;#39;t believe Anthony Wood </t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>$INTC $QQQ $ROKU $SPY   Ooops. Your Furu forgot to mention $INTC before the pump last week ⬇️   What a Chad.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>$ROKU Classic 🩸🩸🩸</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>$ROKU roku tanking</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>$EOSE $FLNC $TSLA $NXT $CSIQ  https://wapo.st/4vgWWCg</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>$NXT Rockets made people crazy today. Well, until we are living on the Moon or Mars,  which won&amp;#39;t happen until decades from now, we still need to convert our fossil-fueled planet to a solar-powered one. Put any funds you&amp;#39;re tempted to throw at $SPCX into Nextpower. Once t</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio movers today:   $INTC +7%   $COHR +7%   $AEVA +6.4%   $APP +4%  $NXT +3.7%.   Added Lidar play $AEVA straight off this week&amp;#39;s watchlist and it&amp;#39;s already paying off. Still holding 1/3 cash while waiting for the 682 market confirmation.   Market leaders are clearl</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>$NXT bouncing off recent lows, up ~5% to ~$126 after a rough ~20% drop over five sessions.    The move is headline-driven as Senate uncertainty over the solar Investment Tax Credit weighs on sentiment. Bulls are eyeing international diversification and a potential 2026 ITC extens</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>$NXT nice. sold half</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>$NXT nice swing</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>$NXT sold for overnight 5% gain</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>$NXT 🚀</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>$NXT</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Starters in $NXT and $NVTS. 111s and 20.80s respectively</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -950,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -983,12 +1291,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-14 12:03 ET</t>
+          <t>2026-06-14 13:12 ET</t>
         </is>
       </c>
     </row>
@@ -1006,6 +1314,23 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>2026-06-14 11:49 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1393,6 +1718,150 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>143.66</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>20.08%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>14,922,301</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2.48M</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>6.01</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>21.20B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>69.09</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>133.467</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>73.9194</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>121.88</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1.84%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2,456,514</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2.16M</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>18.32B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>45.53</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>163.13</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>51.69135</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Solar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1404,7 +1873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2073,6 +2542,414 @@
         <v>0</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>is nearly 50 of my portfolio right now and avg cost of 70 and i didn39t think about selling and likely won39t unless this goes past 200 soon or there39s news of an agreed upon sale lower than that, which would be disappointing. i can39t believe anthony wood</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>ooops. your furu forgot to mention before the pump last week what a chad.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>classic</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>roku tanking</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>rockets made people crazy today. well, until we are living on the moon or mars, which won39t happen until decades from now, we still need to convert our fossil-fueled planet to a solar-powered one. put any funds you39re tempted to throw at into nextpower. once t</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>portfolio movers today 7 7 6.4 4 3.7. added lidar play straight off this week39s watchlist and it39s already paying off. still holding 13 cash while waiting for the 682 market confirmation. market leaders are clearl</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>bouncing off recent lows, up 5 to 126 after a rough 20 drop over five sessions. the move is headline-driven as senate uncertainty over the solar investment tax credit weighs on sentiment. bulls are eyeing international diversification and a potential 2026 itc extens</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>nice. sold half</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>nice swing</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>sold for overnight 5 gain</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:12 ET</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>starters in and . 111s and 20.80s respectively</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-14 17:22 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1244,6 +1244,28 @@
       <c r="D36" s="2" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:22 ET</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>$ROKU ATH is $460, damn long way to go.</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Bullish</t>
         </is>
       </c>
     </row>
@@ -1291,12 +1313,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-14 13:12 ET</t>
+          <t>2026-06-14 13:22 ET</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1433,7 +1455,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-14 11:49 ET</t>
+          <t>2026-06-14 13:22 ET</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1505,358 +1527,70 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-14 11:49 ET</t>
+          <t>2026-06-14 13:22 ET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>355.20</t>
+          <t>121.88</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.32%</t>
+          <t>1.84%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2,698,896</t>
+          <t>2,456,514</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2.66M</t>
+          <t>2.16M</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>191.70B</t>
+          <t>18.32B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>61.93</t>
+          <t>45.53</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>1.90</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>391.29</t>
+          <t>163.13</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>267.8332</t>
+          <t>51.69135</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
-        <is>
-          <t>Drug Manufacturers - General</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-14 12:03 ET</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ROKU</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>143.66</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>20.08%</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>14,922,301</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2.48M</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>6.01</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>21.20B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>69.09</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2.03</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>133.467</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>73.9194</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Entertainment</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-14 12:03 ET</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>AMGN</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>355.20</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>0.32%</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2,698,896</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2.66M</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>1.01</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>191.70B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>61.93</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>0.40</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>391.29</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>267.8332</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Drug Manufacturers - General</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-06-14 13:12 ET</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ROKU</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>143.66</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>20.08%</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>14,922,301</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2.48M</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>6.01</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>21.20B</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>69.09</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2.03</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>133.467</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>73.9194</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Entertainment</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-14 13:12 ET</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>NXT</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>121.88</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1.84%</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2,456,514</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2.16M</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>1.14</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>18.32B</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>45.53</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>163.13</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>51.69135</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -1873,7 +1607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2950,6 +2684,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 13:22 ET</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>ath is 460, damn long way to go.</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-14 19:57 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -694,6 +694,226 @@
       <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Dragonfly Capital - 5 Trade Ideas for Monday: Ally, Amgen, GE Aerospace, Intel and JP Morgan $ALLY $AMGN $GE $INTC $JPM https://dragonflycap.com/5-trade-ideas-for-monday-ally-amgen-ge-aerospace-intel-and-jp-morgan/ and early summe discount!</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>@JayMacy The someone of great influence is  the Saudies... They are the largest holders of $AMGN and they got those two idiots at the FDA fired...</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$IBRX Patience is going to be the primary requirement if you want to have successful outcome with this outfit...   We see very few discussions as it relates to a buyout of this issue... After having been in this jizz-bizz for over 60 years, I see all the signs of a potential buy </t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>$AMGN $ARWR Anyone here know when CVOT data will be released for LP with a little a ? It&amp;#39;s going to be a blockbuster!</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>$JNJ $AMGN $PFE $MRK $BMY</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>$MNKD $MRK $AMGN It&amp;#39;s coming.  It&amp;#39;ll be a blockbuster.  $UTHR</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>AbbVie Reports Promising New Clinical Updates. Here&amp;#39;s What It Means for the Company&amp;#39;s Dividend: https://www.fool.com/investing/2026/06/12/abbvie-reports-promising-new-clinical-updates-here/ $ABBV $JNJ $AMGN $LLY</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>$AMGN Bullish Above the Stomach Candlestick Pattern Formed</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>$AMGN This is gonna rip higher in the coming days. It&amp;#39;s coming out of that slow rolling base with a break of the descending trend line and a successful retest on higher volume. $MRK $JNJ $LLY</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Amgen is seeking to defend the future of Tavneos after hiring the Duke Clinical Research Institute to conduct an independent reanalysis of the clinical trial data that supported the drug’s approval. The move comes as the FDA pushes to withdraw Tavneos from the market over concern</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -708,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -747,6 +967,23 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>2026-06-14 13:51 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
         </is>
       </c>
     </row>
@@ -761,7 +998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -918,6 +1155,78 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>355.20</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.32%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2,698,896</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2.66M</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>191.70B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>61.93</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>391.29</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>267.8332</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Drug Manufacturers - General</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -929,7 +1238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1272,6 +1581,302 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>dragonfly capital - 5 trade ideas for monday ally, amgen, ge aerospace, intel and jp morgan and early summe discount!</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>the someone of great influence is the saudies... they are the largest holders of and they got those two idiots at the fda fired...</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>patience is going to be the primary requirement if you want to have successful outcome with this outfit... we see very few discussions as it relates to a buyout of this issue... after having been in this jizz-bizz for over 60 years, i see all the signs of a potential buy</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>anyone here know when cvot data will be released for lp with a little a ? it39s going to be a blockbuster!</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>it39s coming. it39ll be a blockbuster.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>abbvie reports promising new clinical updates. here39s what it means for the company39s dividend</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>bullish above the stomach candlestick pattern formed</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>this is gonna rip higher in the coming days. it39s coming out of that slow rolling base with a break of the descending trend line and a successful retest on higher volume.</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>amgen is seeking to defend the future of tavneos after hiring the duke clinical research institute to conduct an independent reanalysis of the clinical trial data that supported the drugs approval. the move comes as the fda pushes to withdraw tavneos from the market over concern</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-15 20:41 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -914,6 +914,1546 @@
       <c r="D21" s="3" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>$NTLA .. intrest will grow here as folk digest the data signifigence and analysts assesments flow... lots to play for here... grwat news for gene therapy...</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>$NTLA poor me sold at 13.5</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>$NTLA Watching the consistent elevated volume.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>$NTLA with today’s good news and potential rotation from Semis to Biotech, the uptrend is just getting started.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>$NTLA  this just keeps pushing without much effort</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>$NTLA seems like they want some really nasty squeeze here , 50$ on friday ,</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>$NTLA I thought this was Nutella and was a about to ape into this.</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>$NTLA $20 by morning</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>$NTLA some things going last 12 minutes crazy buying going on</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>$NTLA shorts burning away on this baby as they will on $GDC ! lets get this news of the buy out for 10.75 ! from 10CENT to where it belongs ! 7500 $BTC.X coins like come on what more do you guys want Bears in full panic mode</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>$HQ Lock up period for PIPE investors is 24 months..   $IONQ owns 13% and $DELL owns 8%...  Described as Microsoft of Quantum world.. hold for gold..low float.. first target 30 to 40++  https://www.sec.gov/Archives/edgar/data/2088256/000121390026009801/ea0261018-05.htm  $RGTI $XN</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>$HQ majorrrr 🤡</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Your Day Trading Watch List for June 16th in 2 Minutes (con&amp;#39;t): $SMWB $WYFI $ARQQ $HQ $QNC   .</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>$HQ Smart money piling in.</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>$HQ</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>$HQ this will have a massive crash soon</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>$HQ Finally broke that 17.9 wall.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>$HQ never knew POS can taste so good…</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>$HQ wtf is this POS</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>$IONQ insiders are selling to free up some of their own cash to buy $HQ Horizon Quantum…</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>It’s 2030 - your portfolio is up 30x–50x. Why?    Because you loaded up on these 4 memory stocks and never sold.    $MU - Micron Technology  Target: $5,000 by 2030  $SNDK - SanDisk  Target: $4,000 by 2030  $WDC - Western Digital  Target: $2,500 by 2030  $DRAM -DRAM ETF  Target: $</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>$WDC  $MU   Already got my initial investment + profit out, just house money from here.</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>$WDC looks i was trading it back in 2013 too. lol     Seeing this makes me miss eSignal.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>$DRAM the roundhill guys sure nailed timing of this etf launch  with $SNDK $MU and korean leaders and $WDC</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>$WDC omg. wow.   is this in any of the big indices ?</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>$WDC booming today</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>$MU $SMH own a boatload since last year about 5k shares!held them all along! Bullish. also held my $SNDK, $WDC and $STX</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>$WDC breakout, up 15.0% on 7,349,602 volume.  this is what my scanner flagged: https://tapeboard.com/scanner?utm_source=stocktwits&amp;amp;utm_medium=post&amp;amp;utm_campaign=olivia&amp;amp;utm_content=wdc-bk-up-scanner&amp;amp;utm_term=scanner&amp;amp;s=WDC</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>$WDC eod of day rug pull incoming</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>$WDC  $655 for power hour</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>$OUST OUST sensor used  ISL Aurochs II — Autonomous Navigation in Contested Environments  The Aurochs II, developed by the French-German Research Institute of Saint-Louis (ISL), pushes the boundaries of tactical ground robotics.    Its strength: total operational flexibility. The</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>$OUST Everyone is talking about the future of Physical AI, but fewer conversations focus on what it actually takes to bring that technology into the real world at scale.    We’re proud to expand our partnership with Ouster to support high-volume production of their REV8 digital l</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$OUST Interesting to see Ouster’s BlueCity traffic management solution being deployed at more than 40 locations around MetLife Stadium ahead of the 2026 FIFA World Cup ⚽🌍    With the New York New Jersey Stadium hosting eight matches, including the final, the scale of traffic and </t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>$OUST It was an absolute pleasure welcoming this brilliant group from NECSTlab at Ouster!  We had a fantastic, high-energy discussion about the future of sensing technologies and what it takes to drive real corporate innovation. It’s always inspiring to engage with next-generatio</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>$OUST ITS America Recap, what a great show the community will always be great. The response to RGB LiDAR exceeded our initial thoughts! New friends made, old ones solidified. Thanks for everyone who stopped by the booth, making history thankful to be a part of the movement.  http</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>$OUST OUST sensor used  TiHAN–IIT Hyderabad Signs MoU with Elonroad at Bharat Innovates 2026    As part of Bharat Innovates 2026 in Nice, France, TiHAN-IIT Hyderabad and Elonroad formalized a partnership through the signing of a Memorandum of Understanding (MoU).  https://www.lin</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>$OUST if we get more volume , this thing can go eeven more crazy stv</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>These are shaping up to be some of my cleanest long-term entries this year:    $AAOI &amp;gt; $92  $OUST &amp;gt; $22  $NBIS &amp;gt; $86  $RKLB &amp;gt; $67    Nothing magical about the levels themselves-it’s more about catching them when sentiment was still uncertain and positioning was light.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>$OUST Dropping beats….  https://x.com/ousterlidar/status/2066592827707121761?s=46&amp;amp;t=dLsEh-Gj7r292IRr1gpGbw</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>bought $OUST</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>$BTQ why the huge dip after hours???</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>$BTQ Dip</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>$BTQ looking good</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>$BTQ  Closed above 200 day 1st time since 1/20/26.  Good sign, will be watching to see if any continuation.  Still, if the market (or crypto)  tanks tomorrow will probably give a lot back..  Charts are  always better at showing where something has been than where it is going!  GL</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Your Day Trading Watch List for June 16th in 2 Minutes: $SPY $QUCY $ELMT $BTQ $QTEX    .</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>$BTQ it caught too much attention so the shorts moved in, that&amp;#39;s ok.</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>$BTQ  not much selling at all… that’s interesting</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>$BTQ even if it doesn&amp;#39;t shoot up into close today we broke thr moving averages so it&amp;#39;s awake for the algorithms.</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>$BTQ feeling this has enough too go bang, its has enough and will run wild</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>$BTQ showing a bullish MACD cross on the daily. Squeeze is building.  We love our supernovas with parabolic potential.</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>$SATS meli spanish amazon of bout 10 years ago</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>$SATS back to back 20 per cent $SPCX  gains.   NAV up over 8 billion on it today alone.  What more can you ask for, service with a smile?  🚀 🚀 🚀</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>$SATS why isn’t this trading over $200/share right now?</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>$SATS</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>$SATS nets lockin up crap</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>$SATS I know… try to grab more from dark pools but at &amp;gt; 11m already borrowed Short on dark pools… maybe not much more to borrow there?</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>$SATS $SPCX running into a strong close &amp;amp; &amp;gt; 52m shares Short in $SATS have themselves in a bind as continue to drawdown what little available shares left to hang onto bearish bets… now, only 80k available shares… what do they do when goes to zero?</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>$NASA $SPCX $SATS biggest holding here is Spcx, not going up as its supposed to be, coiled sprint loading. People will miss it.</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>$SATS i see 130 plus</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>$SATS are u kiddin mec70 ta 75 mil in 2 days seriously are they eatin em like potatoe chis. Freakin insane ĺast week it would have been minimum 150. Explain please. Pu all your shares at 180 for sale dont let the shorts get em dam!!!!</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>$RVI had to close my covered calls at a loss</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>$SPCX $DXYZ $RVI DX and RV are the sleepers in the new momentum here</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>$RVI lol wild price action to end the day 😂</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>$RVI Incredible! Congrats everyone ! I openly admit I made huge mistake and sold this for dxyz because of SpaceX and now I’m regretting it big time! 🫤</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>$RVI</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>$RVI come to daddy</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>$RVI 😏😏😏😏😏</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>$RVI nice</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>$RVI and to think I took a loss on this to but dxyz to take a monster paper loss because of SpaceX only for this to now own SpaceX and be flying! Total madness!</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>$RVI Since RH was an underwriter it looks like they got their $SPCX at the open on 6/12 ... so I&amp;#39;m guessing their basis is $135!</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
         </is>
       </c>
     </row>
@@ -928,7 +2468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -984,6 +2524,125 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>2026-06-14 15:56 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
         </is>
       </c>
     </row>
@@ -998,7 +2657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1227,6 +2886,510 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>14.92</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>23.20%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>16,295,731</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>5.76M</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2.83</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2.08B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>59.04</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>47.19</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>7.9587</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>17.82</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>63.34%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>6,220,047</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>185.51K</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>33.53</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>567.27M</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>69.35</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>15.4915</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>8.29114</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>653.53</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>16.10%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>9,422,027</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>7.77M</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>225.26B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>71.24</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2.13</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>602.548</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>54.601096</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Computer Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>45.18</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>13.52%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4,612,549</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3.57M</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2.88B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>62.68</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>3.26</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>49.39</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>16.40175</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Electronic Components</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5.35</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>28.61%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>12,492,085</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2.75M</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>4.54</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>756.28M</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>65.86</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>-6.00</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>66.56</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2.09155</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>117.86</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3.32%</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>17,574,371</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>7.81M</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>34.16B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>45.48</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>147.25</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>16.73604</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Telecom Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>40.62</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>15.23%</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>902,900</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>769.44K</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>512.62M</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>47.94</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>77.39</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>21.0093</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Asset Management</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1238,7 +3401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1877,6 +4040,2090 @@
         <v>0</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>.. intrest will grow here as folk digest the data signifigence and analysts assesments flow... lots to play for here... grwat news for gene therapy...</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>poor me sold at 13.5</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>watching the consistent elevated volume.</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>with todays good news and potential rotation from semis to biotech, the uptrend is just getting started.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>this just keeps pushing without much effort</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>seems like they want some really nasty squeeze here , 50 on friday ,</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>i thought this was nutella and was a about to ape into this.</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>20 by morning</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>some things going last 12 minutes crazy buying going on</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>NTLA</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>shorts burning away on this baby as they will on ! lets get this news of the buy out for 10.75 ! from 10cent to where it belongs ! 7500 .x coins like come on what more do you guys want bears in full panic mode</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>lock up period for pipe investors is 24 months.. owns 13 and owns 8... described as microsoft of quantum world.. hold for gold..low float.. first target 30 to 40</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>majorrrr</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>your day trading watch list for june 16th in 2 minutes con39t .</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>smart money piling in.</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>this will have a massive crash soon</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>finally broke that 17.9 wall.</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>never knew pos can taste so good</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>wtf is this pos</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>insiders are selling to free up some of their own cash to buy horizon quantum</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>its 2030 - your portfolio is up 30x50x. why? because you loaded up on these 4 memory stocks and never sold. - micron technology target 5,000 by 2030 - sandisk target 4,000 by 2030 - western digital target 2,500 by 2030 -dram etf target</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>already got my initial investment profit out, just house money from here.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>looks i was trading it back in 2013 too. lol seeing this makes me miss esignal.</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>the roundhill guys sure nailed timing of this etf launch with and korean leaders and</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>omg. wow. is this in any of the big indices ?</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>booming today</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>own a boatload since last year about 5k shares!held them all along! bullish. also held my , and</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>breakout, up 15.0 on 7,349,602 volume. this is what my scanner flagged</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>eod of day rug pull incoming</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>655 for power hour</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>oust sensor used isl aurochs ii autonomous navigation in contested environments the aurochs ii, developed by the french-german research institute of saint-louis isl, pushes the boundaries of tactical ground robotics. its strength total operational flexibility. the</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>everyone is talking about the future of physical ai, but fewer conversations focus on what it actually takes to bring that technology into the real world at scale. were proud to expand our partnership with ouster to support high-volume production of their rev8 digital l</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>interesting to see ousters bluecity traffic management solution being deployed at more than 40 locations around metlife stadium ahead of the 2026 fifa world cup with the new york new jersey stadium hosting eight matches, including the final, the scale of traffic and</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>it was an absolute pleasure welcoming this brilliant group from necstlab at ouster! we had a fantastic, high-energy discussion about the future of sensing technologies and what it takes to drive real corporate innovation. its always inspiring to engage with next-generatio</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>its america recap, what a great show the community will always be great. the response to rgb lidar exceeded our initial thoughts! new friends made, old ones solidified. thanks for everyone who stopped by the booth, making history thankful to be a part of the movement. http</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>oust sensor used tihaniit hyderabad signs mou with elonroad at bharat innovates 2026 as part of bharat innovates 2026 in nice, france, tihan-iit hyderabad and elonroad formalized a partnership through the signing of a memorandum of understanding mou.</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>if we get more volume , this thing can go eeven more crazy stv</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>these are shaping up to be some of my cleanest long-term entries this year gt 92 gt 22 gt 86 gt 67 nothing magical about the levels themselves-its more about catching them when sentiment was still uncertain and positioning was light.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>dropping beats.</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>bought</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>why the huge dip after hours???</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>dip</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>looking good</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>closed above 200 day 1st time since 12026. good sign, will be watching to see if any continuation. still, if the market or crypto tanks tomorrow will probably give a lot back.. charts are always better at showing where something has been than where it is going! gl</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>your day trading watch list for june 16th in 2 minutes .</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>it caught too much attention so the shorts moved in, that39s ok.</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>not much selling at all thats interesting</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>even if it doesn39t shoot up into close today we broke thr moving averages so it39s awake for the algorithms.</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>feeling this has enough too go bang, its has enough and will run wild</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>BTQ</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>showing a bullish macd cross on the daily. squeeze is building. we love our supernovas with parabolic potential.</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>meli spanish amazon of bout 10 years ago</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>back to back 20 per cent gains. nav up over 8 billion on it today alone. what more can you ask for, service with a smile?</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>why isnt this trading over 200share right now?</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>nets lockin up crap</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>i know try to grab more from dark pools but at gt 11m already borrowed short on dark pools maybe not much more to borrow there?</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>running into a strong close amp gt 52m shares short in have themselves in a bind as continue to drawdown what little available shares left to hang onto bearish bets now, only 80k available shares what do they do when goes to zero?</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>biggest holding here is spcx, not going up as its supposed to be, coiled sprint loading. people will miss it.</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>i see 130 plus</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>are u kiddin mec70 ta 75 mil in 2 days seriously are they eatin em like potatoe chis. freakin insane ast week it would have been minimum 150. explain please. pu all your shares at 180 for sale dont let the shorts get em dam!!!!</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>had to close my covered calls at a loss</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>dx and rv are the sleepers in the new momentum here</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>lol wild price action to end the day</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>incredible! congrats everyone ! i openly admit i made huge mistake and sold this for dxyz because of spacex and now im regretting it big time!</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>come to daddy</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>nice</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>and to think i took a loss on this to but dxyz to take a monster paper loss because of spacex only for this to now own spacex and be flying! total madness!</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>RVI</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>since rh was an underwriter it looks like they got their at the open on 612 ... so i39m guessing their basis is 135!</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-16 20:37 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2454,6 +2454,1546 @@
       <c r="D91" s="2" t="inlineStr">
         <is>
           <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>$KRMN trending because this is literally the cheapest aerospace/missile/rocket play out there with over $3B backlog    $SPCX</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>$KRMN 💪 asf</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>$KRMN   https://www.tradeapes.com/stocks/KRMN</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>$KRMN dont worry @OG_Monkey_Banana_Genius there cant be enough news to get us back to our shit of an entry!. thanks for another failure among your many lmfao. the court jester.</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>$VIVO bro this thing might just fucking gamma squeeze  $WYFI $FRMI $KRMN</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>$KRMN I should bloody think so. This has been treated appallingly. No respect whatsoever. Up, up, up now...</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>$KRMN 50DMA is 67 lets gooooo</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>$KRMN AVG 61 but its a little Monster Will all the facilites needed to build, metals, emgines, software and hardware ..space and defense bright future here</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>$KRMN news?</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>$KRMN breaking out hard, up 7.3% and clearing prior close with 2.6M shares through already. these vertical sessions either have legs into the close or they stall the moment buyers thin out. watching 51.50 hold as the line.  this is what my scanner flagged: https://tapeboard.com/r</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>$LION https://www.thewrap.com/industry-news/business/netflix-lionsgate-acquisition-not-interested/</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>@aawn @itsphd $LION $nflx  nvm mind, lionsgate recovered almost all the drop, maybe  someone fat fingered🤭</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>$LION @cubie Hey cubie please show us that you have ever had a position. You just jump from trending stock and brag about follower. Come on does anyone care about followers on stocktwits. You LOSER!</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>@zuby34 @Jeremymartin007 @Cubie @simon58 @judgeyoung2 @jenbunn @EBE_day @ribbey @TraderRapp @Godreal1 @tonyctl   $LION  wth</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>$LION did $nflx just deny it bc lionsgates dropped -$2</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>$LION that&amp;#39;s what I was waiting for... hehehe. thanks... im out</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>$LION $OCC</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>Here are the Final 2 Stocks in Your Day Trading Watch List for June 17th in 2 Minutes: $LION $OCC   .</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>$LION added about 75 watchers</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>HOUR stock can 10X from here - most undervalued penny stock in the market     - 1.8M float with zero dilution    - did 143M in revenue last year with around $2M in net profit (doing the best numbers since they went public )    - insiders have never sold (even when this hit 7+) an</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>$MGNI</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>$MGNI currently at resistance.  Break through, and she could run to 21.</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>$MGNI Unclear why the surge today- anyone have/seen any news?  Whatever the reasons, a superb day for all the LONGS- congrats!     Still lots of shorts in this @ roughly 9% of the float. If we can keep the momentum going we may see some extra lift in SP from covering.</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>$MGNI over 6 million shares traded, closed at high of day, and heavy bullish option flow. Nice day all. About time</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>$MGNI the last time Barrett dumped a load of his shares, price ran away from him significantly.  Let&amp;#39;s repeat that.  (But let&amp;#39;s not repeat the other thing that eventually happened, when price collapsed way under his sell point.)</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>$MGNI below $18 tm</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>$MGNI the worm has turned 😊</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>$TTD $MGNI now within 2% of Shitdesk as it spikes into the close and Shitdesk collapses yet again.</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>HOUR stock can 10X from here - most undervalued penny stock in the market     - 1.8M float with zero dilution    - did 143M in revenue last year with around $2M in net profit (doing the best numbers since they went public )    - insiders have never sold (even when this hit 7+) an</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>$MGNI surging 10% - anyone buying here?</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>$RXT on option strat, someones loading hella $5 puts but why!!!!! i pray we just break out man! i mean they hit the LQ sweep at the bell</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>$RXT Tomorrow going to be like a Hurricane clearing out shorty...Huge Day!</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>$RXT Premarket tmrw they&amp;#39;ll grab everything available. Hold tight. GL Long$</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>$RXT     Swingingitintotomorrowland</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>$RXT offering tonight 👍🏼👍🏼😃😃</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>$RXT Decent day altogether, up 5% on good news and a red day for nasdaq. I&amp;#39;ll take that.</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>$RXT Today all semiconductors down  and AMD -7.30%. Let&amp;#39;s see tomorrow how it goes</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>$RXT gping red?</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>$RXT i warned you they take it down on open</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>$RXT New contract with AMD</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>@StocktwitsPolls $SNDK $MU $STX $WDC</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>$WDC bubble</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>$WDC LEADER</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>$WDC is RIDICULOUS!    Current resistance sits at $655, but the hype around this stock could have us see $700!    The senseful thing would be a pullback to ~$600 ...</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Storage is still one of the cleanest momentum + re-rating trades in the market right now, especially with earnings catalysts ahead.    $WDC - pushing ATH momentum, re-rating on supply discipline + pricing power  $STX - strong trend continuation, institutional accumulation still v</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Western Digital, Seagate Technology, and Sandisk are all continuing to push into fresh all-time highs as momentum stays strong across the storage space heading into next week’s Micron Technology earnings.  What’s even more notable is the strength still hasn’t faded there’s a clea</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>$KORU $MU $DRAM $SNDK $WDC</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>$LRCX $AMAT $STX $WDC  congrats all. Winners in all four</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>$WDC Insane!</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>$WDC pressing the 75-day high with momentum. Entry has already gained ground and the next target zone is the $650 area. This one still has room to run.</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI +21.43%</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI  didn’t have this on the bingo card today</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI truth reveals it self here again</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI This is going to let a lot of people down in the very short term. 1.16 bil market cap with less than 100 mil revenue and losing money. In the next couple years maybe good but for now your overpaying.  I know fundamentals don&amp;#39;t matter anymore to short term holders but wo</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>@Nasdaq_Frontier I should have clarified that the facilities they retro fit are buildings that housed now closed manufacturing, or a company that moved or left for some reason. Your AI misread my meaning when I said “facilities already built.” Thinking they were Tier 3  facilitie</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI  https://www.tradeapes.com/stocks/WYFI</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI lolol no</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>$VIVO bro this thing might just fucking gamma squeeze  $WYFI $FRMI $KRMN</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>$WYFI</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI sold 28% of holdings at 36.49 held from 1/21/26 good for 96% gains. Will let the rest ride</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>$ABCB nice breakout in this bank stock</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>$ABCB Price: $83.50 (-1.34%) Trend: Bullish Market Bias (7D): Bullish Bias 📈 Expected Range: ±0.20% RSI: 52.6 | Momentum: Moderate Volume: -85.7% vs avg Volatility: 1.24% Support: $81.94 | Resistance: $87.99  Data and analytics sourced from Given Analytics educational research: h</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>#DILUTION  Ameris Bancorp ($ABCB) files mixed securities shelf offering  Babcock &amp;amp; Wilcox Enterprises ($BW) files for 11,657,221 share common stock offering by selling stockholders  Biodesix ($BDSX) files for 375,000 share common stock offering by selling stockholders  Galaxy</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>Fundamental analysis of $ABCB (Ameris Bancorp) based on financial data and reported results. #ABCB #Ameris</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>$ABCB Share Price: $85.06  Contract Selected: Oct 16, 2026 $85 Calls  Buy Zone: $4.76 – $5.88 Target Zone: $7.56 – $9.24 Potential Upside: 50% ROI  Time to Expiration: 171 Days | Updates via https://fxcapta.com/stockinfo/</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>$ABCB Q1 &amp;#39;26 Earnings Results &amp;amp; Recap  • Reported GAAP EPS of $1.64 up 28.12% YoY • Reported revenue of $314.36M up 9.97% YoY</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>$ABCB Share Price: $75.16  Contract Selected: Oct 16, 2026 $45 Calls  Buy Zone: $24.33 – $30.05 Target Zone: $44.14 – $53.95 Potential Upside: 71% ROI  Time to Expiration: 205 Days | Updates via https://fxcapta.com/stockinfo/</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>$ABCB Share Price: $83.72  Contract Selected: Jul 17, 2026 $85 Calls  Buy Zone: $2.98 – $3.68 Target Zone: $5.40 – $6.60 Potential Upside: 71% ROI  Time to Expiration: 145 Days | Updates via https://fxcapta.com/stockinfo/</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>$ABCB Share Price: $84.80  Contract Selected: Jul 17, 2026 $85 Calls  Buy Zone: $3.48 – $4.30 Target Zone: $5.79 – $7.07 Potential Upside: 57% ROI  Time to Expiration: 156 Days | Updates via https://fxcapta.com/stockinfo/</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>$ABCB Q4 &amp;#39;25 Earnings Results &amp;amp; Recap  • Reported GAAP EPS of $1.59 up 16.06% YoY • Reported revenue of $307.13M up 5.62% YoY</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -2468,7 +4008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2496,24 +4036,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-14 13:51 ET</t>
+          <t>2026-06-16 16:37 ET</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2523,14 +4063,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-14 15:56 ET</t>
+          <t>2026-06-14 13:51 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NTLA</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2540,14 +4080,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-15 16:40 ET</t>
+          <t>2026-06-14 15:56 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>NTLA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2564,7 +4104,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>HQ</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2643,6 +4183,108 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>2026-06-15 16:40 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
         </is>
       </c>
     </row>
@@ -2657,7 +4299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3033,7 +4675,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-15 16:40 ET</t>
+          <t>2026-06-16 16:37 ET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3043,52 +4685,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>653.53</t>
+          <t>681.08</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>16.10%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>9,422,027</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>7.77M</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>1.21</t>
+          <t>15733016</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>225.26B</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>71.24</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2.13</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>602.548</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>54.601096</t>
+          <t>234756.11</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -3387,6 +4999,258 @@
       <c r="N10" t="inlineStr">
         <is>
           <t>Asset Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>51.70</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>7.11%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>6363978</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>6851.60</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>16.36</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>13.85%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>16236863</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>4754.77</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Shell Companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>18.55</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>10.75%</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>6373979</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2656.64</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Advertising Agencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>6.21</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>4.99%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>82043452</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1547.67</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>35.65</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>18.91%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4975627</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1376.59</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>88.47</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.71%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1009561</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>5953.37</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Banks - Regional</t>
         </is>
       </c>
     </row>
@@ -3401,7 +5265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6124,6 +7988,2074 @@
         <v>0</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>trending because this is literally the cheapest aerospacemissilerocket play out there with over 3b backlog</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>asf</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr"/>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>dont worry there cant be enough news to get us back to our shit of an entry!. thanks for another failure among your many lmfao. the court jester.</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>bro this thing might just fucking gamma squeeze</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>i should bloody think so. this has been treated appallingly. no respect whatsoever. up, up, up now...</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>50dma is 67 lets gooooo</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>avg 61 but its a little monster will all the facilites needed to build, metals, emgines, software and hardware ..space and defense bright future here</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>news?</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>KRMN</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>breaking out hard, up 7.3 and clearing prior close with 2.6m shares through already. these vertical sessions either have legs into the close or they stall the moment buyers thin out. watching 51.50 hold as the line. this is what my scanner flagged</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr"/>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>nflx nvm mind, lionsgate recovered almost all the drop, maybe someone fat fingered</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>hey cubie please show us that you have ever had a position. you just jump from trending stock and brag about follower. come on does anyone care about followers on stocktwits. you loser!</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>wth</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>did nflx just deny it bc lionsgates dropped -2</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>that39s what i was waiting for... hehehe. thanks... im out</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr"/>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>here are the final 2 stocks in your day trading watch list for june 17th in 2 minutes .</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>added about 75 watchers</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>LION</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>hour stock can 10x from here - most undervalued penny stock in the market - 1.8m float with zero dilution - did 143m in revenue last year with around 2m in net profit doing the best numbers since they went public - insiders have never sold even when this hit 7 an</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr"/>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>currently at resistance. break through, and she could run to 21.</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>unclear why the surge today- anyone haveseen any news? whatever the reasons, a superb day for all the longs- congrats! still lots of shorts in this roughly 9 of the float. if we can keep the momentum going we may see some extra lift in sp from covering.</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>over 6 million shares traded, closed at high of day, and heavy bullish option flow. nice day all. about time</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>the last time barrett dumped a load of his shares, price ran away from him significantly. let39s repeat that. but let39s not repeat the other thing that eventually happened, when price collapsed way under his sell point.</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>below 18 tm</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>the worm has turned</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>now within 2 of shitdesk as it spikes into the close and shitdesk collapses yet again.</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>hour stock can 10x from here - most undervalued penny stock in the market - 1.8m float with zero dilution - did 143m in revenue last year with around 2m in net profit doing the best numbers since they went public - insiders have never sold even when this hit 7 an</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>surging 10 - anyone buying here?</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>on option strat, someones loading hella 5 puts but why!!!!! i pray we just break out man! i mean they hit the lq sweep at the bell</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>tomorrow going to be like a hurricane clearing out shorty...huge day!</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>premarket tmrw they39ll grab everything available. hold tight. gl long</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>swingingitintotomorrowland</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>offering tonight</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>decent day altogether, up 5 on good news and a red day for nasdaq. i39ll take that.</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>today all semiconductors down and amd -7.30. let39s see tomorrow how it goes</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>gping red?</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>i warned you they take it down on open</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>new contract with amd</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr"/>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>bubble</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>leader</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>is ridiculous! current resistance sits at 655, but the hype around this stock could have us see 700! the senseful thing would be a pullback to 600 ...</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>storage is still one of the cleanest momentum re-rating trades in the market right now, especially with earnings catalysts ahead. - pushing ath momentum, re-rating on supply discipline pricing power - strong trend continuation, institutional accumulation still v</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>western digital, seagate technology, and sandisk are all continuing to push into fresh all-time highs as momentum stays strong across the storage space heading into next weeks micron technology earnings. whats even more notable is the strength still hasnt faded theres a clea</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr"/>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>congrats all. winners in all four</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>insane!</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F140" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>pressing the 75-day high with momentum. entry has already gained ground and the next target zone is the 650 area. this one still has room to run.</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>21.43</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>didnt have this on the bingo card today</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>truth reveals it self here again</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>this is going to let a lot of people down in the very short term. 1.16 bil market cap with less than 100 mil revenue and losing money. in the next couple years maybe good but for now your overpaying. i know fundamentals don39t matter anymore to short term holders but wo</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>i should have clarified that the facilities they retro fit are buildings that housed now closed manufacturing, or a company that moved or left for some reason. your ai misread my meaning when i said facilities already built. thinking they were tier 3 facilitie</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr"/>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>lolol no</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>bro this thing might just fucking gamma squeeze</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr"/>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>sold 28 of holdings at 36.49 held from 12126 good for 96 gains. will let the rest ride</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>nice breakout in this bank stock</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>price 83.50 -1.34 trend bullish market bias 7d bullish bias expected range 0.20 rsi 52.6 momentum moderate volume -85.7 vs avg volatility 1.24 support 81.94 resistance 87.99 data and analytics sourced from given analytics educational research h</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>dilution ameris bancorp files mixed securities shelf offering babcock amp wilcox enterprises files for 11,657,221 share common stock offering by selling stockholders biodesix files for 375,000 share common stock offering by selling stockholders galaxy</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>fundamental analysis of ameris bancorp based on financial data and reported results. abcb ameris</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>share price 85.06 contract selected oct 16, 2026 85 calls buy zone 4.76 5.88 target zone 7.56 9.24 potential upside 50 roi time to expiration 171 days updates via</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>q1 3926 earnings results amp recap reported gaap eps of 1.64 up 28.12 yoy reported revenue of 314.36m up 9.97 yoy</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>share price 75.16 contract selected oct 16, 2026 45 calls buy zone 24.33 30.05 target zone 44.14 53.95 potential upside 71 roi time to expiration 205 days updates via</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>share price 83.72 contract selected jul 17, 2026 85 calls buy zone 2.98 3.68 target zone 5.40 6.60 potential upside 71 roi time to expiration 145 days updates via</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>share price 84.80 contract selected jul 17, 2026 85 calls buy zone 3.48 4.30 target zone 5.79 7.07 potential upside 57 roi time to expiration 156 days updates via</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F160" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>ABCB</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>q4 3925 earnings results amp recap reported gaap eps of 1.59 up 16.06 yoy reported revenue of 307.13m up 5.62 yoy</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-16 20:42 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3992,6 +3992,248 @@
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>$WDC news?</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>$WDC solid.</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>$WDC</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>$WDC this stock never failed me  $AMAT as well!    $HOOD this stock will be a legendary stock soon!  you  will see !</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>$WDC</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>$WDC $STX $SNDK $MU WTf are you waiting for...its time to buy in dummies... GL!</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>$WDC quite near the most bullish analyst pt</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>$MU Fwd P/E 10, $WDC 20 and $SNDK is at 30. I believe Micron will double over remainder of year. The other two will go up 50% but Micron is way undervalued. Look for them to be the clear winner in the 2nd half of 2026.</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t>$WDC easy short here guys, has reached peak!</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>Why WDC, MU, STX, SNDK Stocks Rallied Hard Today And Lifted DRAM To ‘Solid Breakout’   $WDC $MU $STX $SNDK $DRAM  https://stocktwits.com/news/equity/markets/why-wdc-mu-stx-sndk-stocks-rallied-hard-today-and-lifted-dram-to-solid-breakout/cZKWBy4R7E2</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>$TTWO today.  Boom!  Testing 200sma.  Long in the Options room.  Best trade today was $WYFI hitting target, among the 2 rooms.  $TTWO was #2.</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -4041,36 +4283,36 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-14 13:51 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4080,14 +4322,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-14 15:56 ET</t>
+          <t>2026-06-14 13:51 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NTLA</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4097,14 +4339,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-15 16:40 ET</t>
+          <t>2026-06-14 15:56 ET</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>NTLA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4121,7 +4363,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>HQ</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4138,7 +4380,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BTQ</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4155,7 +4397,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SATS</t>
+          <t>BTQ</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4172,7 +4414,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RVI</t>
+          <t>SATS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4189,7 +4431,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KRMN</t>
+          <t>RVI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4199,14 +4441,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-15 16:40 ET</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LION</t>
+          <t>KRMN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4223,7 +4465,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>LION</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4240,7 +4482,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RXT</t>
+          <t>MGNI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4257,7 +4499,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>RXT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4675,7 +4917,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4695,7 +4937,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15733016</t>
+          <t>15734653</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -5005,7 +5247,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5025,7 +5267,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>6363978</t>
+          <t>6364142</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -5047,7 +5289,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -5067,7 +5309,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16236863</t>
+          <t>16262584</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -5089,7 +5331,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5109,7 +5351,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>6373979</t>
+          <t>6374005</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -5131,7 +5373,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5151,7 +5393,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>82043452</t>
+          <t>82062683</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -5173,7 +5415,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5193,7 +5435,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4975627</t>
+          <t>4975767</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -5215,7 +5457,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-16 16:42 ET</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5265,7 +5507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F161"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10056,6 +10298,328 @@
         <v>0</v>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>news?</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>solid.</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr"/>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>this stock never failed me as well! this stock will be a legendary stock soon! you will see !</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr"/>
+      <c r="D166" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E166" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F166" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>wtf are you waiting for...its time to buy in dummies... gl!</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>quite near the most bullish analyst pt</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E168" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F168" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>fwd pe 10, 20 and is at 30. i believe micron will double over remainder of year. the other two will go up 50 but micron is way undervalued. look for them to be the clear winner in the 2nd half of 2026.</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>easy short here guys, has reached peak!</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>why wdc, mu, stx, sndk stocks rallied hard today and lifted dram to solid breakout</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:42 ET</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>today. boom! testing 200sma. long in the options room. best trade today was hitting target, among the 2 rooms. was 2.</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-16 20:48 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D172"/>
+  <dimension ref="A1:D186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4234,6 +4234,314 @@
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>$MGNI huh?   my eyes deceiving me??</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>$VELO ran from 22.29 to 26.50 and holding 25 here,  with volume it can get 28 to 30  $VMAR r/s in effect June 17 so it could squeeze, be up early  $RXT see if 6 holds for a move to 6.50 and 8  $CCTG we want 1.15 to hold for a move to 1.50 and 2  $LNAI if 3 can hold maybe we get 3</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>$RXT everytime I go fishing this goes green</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C176" s="4" t="inlineStr">
+        <is>
+          <t>$WDC don’t chase any memory stocks right now, you might wake up to a 25-50% haircut once a bad news day hits any day</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>$TOLEY - Tokyo Electron Ltd. Posted below is the weekly chart. Memory stocks worldwide reaching for the sky. In the US $MU , $STX &amp;amp; $WDC have been doing the same.</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>$WDC 📈📈📈</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>$WDC The forgotten baby in the memory. Finally 10x. Expected cool off, or a major contract. All this AI content, tokens and generation needs to be stored somewhere. We will see another double from here.</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>$WDC love this memory stock. Not as followed as much but it can. Move. I see it going to 1000 plus</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>$WDC wow - just wow. Might have to roll my short calls</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>$WDC  retraced well till golden ratio and took the support of TL, likely to visit till 750/815 by next week.</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>$WDC $HOOD   all i do is keep buying, still sleeping soundly at night:)</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>$WDC  Nice call here bro @kirkulr 😎💪🐐</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>$WDC I’m buying u guys think im late ? I may hold long term 3-4 yrs</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>$WYFI good say.  Bought this morning and on track for $50 next month</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -4283,70 +4591,70 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>RXT</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-14 13:51 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>MGNI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-14 15:56 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NTLA</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4356,14 +4664,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-15 16:40 ET</t>
+          <t>2026-06-14 13:51 ET</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4373,14 +4681,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-15 16:40 ET</t>
+          <t>2026-06-14 15:56 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>NTLA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4397,7 +4705,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BTQ</t>
+          <t>HQ</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4414,7 +4722,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SATS</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4431,7 +4739,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RVI</t>
+          <t>BTQ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4448,7 +4756,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KRMN</t>
+          <t>SATS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4458,14 +4766,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-15 16:40 ET</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LION</t>
+          <t>RVI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4475,14 +4783,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-15 16:40 ET</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>KRMN</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4499,7 +4807,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RXT</t>
+          <t>LION</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4917,7 +5225,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4937,7 +5245,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15734653</t>
+          <t>15744908</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -5247,7 +5555,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5289,7 +5597,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -5309,7 +5617,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16262584</t>
+          <t>16265022</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -5331,7 +5639,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5373,7 +5681,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5393,7 +5701,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>82062683</t>
+          <t>82092521</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -5415,7 +5723,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5435,7 +5743,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4975767</t>
+          <t>4975888</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -5457,7 +5765,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-16 16:42 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5507,7 +5815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F172"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10620,6 +10928,422 @@
         <v>0</v>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>huh? my eyes deceiving me??</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>ran from 22.29 to 26.50 and holding 25 here, with volume it can get 28 to 30 rs in effect june 17 so it could squeeze, be up early see if 6 holds for a move to 6.50 and 8 we want 1.15 to hold for a move to 1.50 and 2 if 3 can hold maybe we get 3</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>everytime i go fishing this goes green</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>dont chase any memory stocks right now, you might wake up to a 25-50 haircut once a bad news day hits any day</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>- tokyo electron ltd. posted below is the weekly chart. memory stocks worldwide reaching for the sky. in the us , amp have been doing the same.</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr"/>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>the forgotten baby in the memory. finally 10x. expected cool off, or a major contract. all this ai content, tokens and generation needs to be stored somewhere. we will see another double from here.</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>love this memory stock. not as followed as much but it can. move. i see it going to 1000 plus</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F180" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>wow - just wow. might have to roll my short calls</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>retraced well till golden ratio and took the support of tl, likely to visit till 750815 by next week.</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>all i do is keep buying, still sleeping soundly at night</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>nice call here bro</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F184" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>im buying u guys think im late ? i may hold long term 3-4 yrs</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 16:48 ET</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>good say. bought this morning and on track for 50 next month</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F186" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-17 14:25 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D186"/>
+  <dimension ref="A1:D256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4542,6 +4542,1546 @@
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ momentum hedge funds and algos are going to jump in which brings in the volume and volatility halts upwards 🧨⏱️</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ $BTQ  $IONQ  $SPY $QQQ   Quantum security next big mover</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ 24K shares left only, shorts are in trouble.. has same mechanics structure as $CAR and much lower float, much more to come imho this is just a warmup</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ running hot, up 17.4% and no read on what&amp;#39;s driving it yet. these vertical moves can stall once the early buyers start trimming. what level are you guys watching here?  this is what my scanner flagged: https://tapeboard.com/research/ARQQ?utm_source=stocktwits&amp;amp;utm_me</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ Once this breaks $30 sky is the limit form there!</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ looking for 30 by tomorrow</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ 200%</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ shorts have about 1.7M shares need to be bought back on this 6M float in quantum.. $400M valuation only as apposed to $20 BILLION with $IONQ</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ calls up 10x from entering congrats</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>$BHVN up nearly 10% and still grinding through session highs. no read on the driver yet, tape just keeps absorbing the offers. watching this one closely.  live tape on the breakout: https://tapeboard.com/scanner?utm_source=stocktwits&amp;amp;utm_medium=post&amp;amp;utm_campaign=olivia&amp;am</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>$BHVN nice sympathy move on $QURE news (prospects for SCA resubmission)</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>$BHVN Biohaven’s SCA Drug: Biohaven compared its clinical trial patients against external real-world databases, specifically the European EuroSCA study and the US CRC-SCA database. UniQure’s AMT-130: uniQure compared its Phase I/II Huntington&amp;#39;s patients against a historical n</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>$BHVN The data uniQure used was historical data, and the core methodological problem is identical to the one that caused Biohaven&amp;#39;s spinocerebellar ataxia (SCA) drug, Vyglxia (troriluzole), to receive an FDA Complete Response Letter (CRL). This means that perhaps FDA might co</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>$BHVN - nice sympathy move on $QURE news (prospects for SCA resubmission with another year or two of follow-up)</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>$BHVN MMs got caught. There’s no big or ask on those options itm.</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>$BHVN Noce news. Crazy it isn’t at 40 yet.</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>$BHVN so qure is up 60% on fda revisit.  This is running up to the inevitable resubmission.</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>$BHVN someone is cover …</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>$BHVN Why the premarket buzz?</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>$BTGO remember once seller sold at this low price, those shares purchased by buyback will be put away on shelf by the company. This is a slow drainage of available low cost shares pool. Majority IPO shares cost $18 and they won’t sell at $6 if they didn’t sell at 4.xx.  Expect th</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO this stock will be back to $10 in no time!! why is it not trending? you are being weak spreading the world, less than 1k watchers this is the early stage, $10 next, then all the way up to $25, and finally price discovery above that value!!</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO nice news, added 📈🚀</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO $10 today</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO Volume 0.5 million they will buy 10.000.000 shares lolol RIP 🐻</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO Short Squeeze?</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO 🚀👍💯📈‼️</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO Will fly to $10 today</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>$BTGO boom</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>$CPNG</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>$CPNG you can see a re rating is in process with how much this jumps at open daily</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>$CPNG pumped up kicks</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>$CPNG...  Yes.</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>$CPNG   myyy precioussss  $SPY</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>$CPNG this is headed to 20s</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>$CPNG I told you this thing is going back over 20</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>$CPNG</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>$CPNG where all this money will be spent? on coupang.    all the businesses want piece from this spending will give ads to Coupang. I am sooo bullish for next earnings.</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>$HIMS steady grind all day to 32, we want 31.25 to hold now for 33 to 35  $OTLK got 1.58, see if 1.50  holds for a move to 2  $PURR ran to 10.98, now we want 10 to hold for a break of 11 for 12  $CPNG hit 18 strong day, we could see a dip to 17.50 but break of 18 for 20  $CRVO gr</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>$EOSE Nothing better than a strong all American Co. in NJ.</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>Best stocks to won until 2030    Power - $TE , $EOSE, $HYLN, $OKLO     Which other stocks do you think are worth considering?    Power and energy could become one of the most important investment themes of the next five years. AI data centers, EV adoption, grid modernization, and</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>$EOSE</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>$EOSE is another BE FLY TO 100 POSIBLE</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>$EOSE new production site went live overnight and the stock&amp;#39;s been grinding up all session, now 10.7% off yesterday&amp;#39;s close. not parabolic, just steady. that&amp;#39;s what I want to see. anyone tracking this one?  this is what my scanner flagged: https://tapeboard.com/scanne</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>$FPS   We forge ahead   Close above 62 and will be 75%   Position sized   $BLDP FLNC $BE $EOSE</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>$SPCX damn… missing this dip. Bought $1000 worth of $EOSE this morning!!!</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>$EOSE</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>$EOSE HWG!!!</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>$EOSE volume picking up nicely. Set right up. Wait til it halts and opens back up at over 8</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>$FIG Shorts still active on a day with a new $36 PT when its in the 18s🤷‍♀️ honestly they deserve to get in trouble.</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>$FIG short interest , looks like 30%, easy money if you pile in ! ill add little more here, but this is team work effort</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>$FIG drops 3% 🤣</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>$FIG me too, shorts are covering</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>$FIG well I&amp;#39;m back in</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>$FIG</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>$FIG</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>$FIG RIP shorts 🪦</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>$FIG is short interest 36%</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>$FIG Still down 23% 😢</t>
+        </is>
+      </c>
+      <c r="D246" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>$FRMI</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>$AVGO $FRMI $ICCM $RXT</t>
+        </is>
+      </c>
+      <c r="D248" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>$ICCM this is how it’s done  $FRMI $12 went  $RXT holddddd  $AVGO more</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>$FRMI slow rise up my boyz!! fuck yeah! geezus feels goid</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>$FRMI took a few 11c 8/21 @ 1.50</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>$FRMI in with 1700 shares at 8.47. Let’s see what happens.</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>$OCUL  $FRMI  keep eyes on  $NIO  is your next runner whales will find this name so attractive very soon $15</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>$FRMI 👀 watching</t>
+        </is>
+      </c>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>$FRMI FLY ME TO THE MOON!</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>$FRMI   $10 today!!!!!!</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -4558,7 +6098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4835,6 +6375,125 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>2026-06-16 16:37 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
         </is>
       </c>
     </row>
@@ -4849,7 +6508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5804,6 +7463,300 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>22.84</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>14.54%</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1102792</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>397.47</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>13.56</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>12.16%</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1960505</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2041.60</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>6.05</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>11.15%</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1391596</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>701.18</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Capital Markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>19.15</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>6.21%</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>9123877</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>34375.48</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Internet Retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>10.13%</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>13526949</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2546.39</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Electrical Equipment &amp; Parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>18.86</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>4.89%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>9260523</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>9965.18</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>8.40</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>6.66%</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>9369458</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>5358.82</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>REIT - Specialty</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5815,7 +7768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11344,6 +13297,2062 @@
         <v>0</v>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>momentum hedge funds and algos are going to jump in which brings in the volume and volatility halts upwards</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>quantum security next big mover</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F188" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>24k shares left only, shorts are in trouble.. has same mechanics structure as and much lower float, much more to come imho this is just a warmup</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>running hot, up 17.4 and no read on what39s driving it yet. these vertical moves can stall once the early buyers start trimming. what level are you guys watching here? this is what my scanner flagged</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>once this breaks 30 sky is the limit form there!</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>looking for 30 by tomorrow</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="D193" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F193" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>shorts have about 1.7m shares need to be bought back on this 6m float in quantum.. 400m valuation only as apposed to 20 billion with</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>calls up 10x from entering congrats</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F195" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr"/>
+      <c r="D196" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F196" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>up nearly 10 and still grinding through session highs. no read on the driver yet, tape just keeps absorbing the offers. watching this one closely. live tape on the breakout</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>nice sympathy move on news prospects for sca resubmission</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E198" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F198" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>biohavens sca drug biohaven compared its clinical trial patients against external real-world databases, specifically the european eurosca study and the us crc-sca database. uniqures amt-130 uniqure compared its phase iii huntington39s patients against a historical n</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>the data uniqure used was historical data, and the core methodological problem is identical to the one that caused biohaven39s spinocerebellar ataxia sca drug, vyglxia troriluzole, to receive an fda complete response letter crl. this means that perhaps fda might co</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>- nice sympathy move on news prospects for sca resubmission with another year or two of follow-up</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>mms got caught. theres no big or ask on those options itm.</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F202" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>noce news. crazy it isnt at 40 yet.</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F203" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>so qure is up 60 on fda revisit. this is running up to the inevitable resubmission.</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F204" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>someone is cover</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F205" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>BHVN</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>why the premarket buzz?</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>remember once seller sold at this low price, those shares purchased by buyback will be put away on shelf by the company. this is a slow drainage of available low cost shares pool. majority ipo shares cost 18 and they wont sell at 6 if they didnt sell at 4.xx. expect th</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>this stock will be back to 10 in no time!! why is it not trending? you are being weak spreading the world, less than 1k watchers this is the early stage, 10 next, then all the way up to 25, and finally price discovery above that value!!</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>nice news, added</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>10 today</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F210" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>volume 0.5 million they will buy 10.000.000 shares lolol rip</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>short squeeze?</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr"/>
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr"/>
+      <c r="D214" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F214" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>will fly to 10 today</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>boom</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr"/>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>you can see a re rating is in process with how much this jumps at open daily</t>
+        </is>
+      </c>
+      <c r="D218" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>pumped up kicks</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>... yes.</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>myyy precioussss</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>this is headed to 20s</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>i told you this thing is going back over 20</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr"/>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>where all this money will be spent? on coupang. all the businesses want piece from this spending will give ads to coupang. i am sooo bullish for next earnings.</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>CPNG</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>steady grind all day to 32, we want 31.25 to hold now for 33 to 35 got 1.58, see if 1.50 holds for a move to 2 ran to 10.98, now we want 10 to hold for a break of 11 for 12 hit 18 strong day, we could see a dip to 17.50 but break of 18 for 20 gr</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>nothing better than a strong all american co. in nj.</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>best stocks to won until 2030 power - , , , which other stocks do you think are worth considering? power and energy could become one of the most important investment themes of the next five years. ai data centers, ev adoption, grid modernization, and</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr"/>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>is another be fly to 100 posible</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>new production site went live overnight and the stock39s been grinding up all session, now 10.7 off yesterday39s close. not parabolic, just steady. that39s what i want to see. anyone tracking this one? this is what my scanner flagged</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>we forge ahead close above 62 and will be 75 position sized flnc</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>damn missing this dip. bought 1000 worth of this morning!!!</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr"/>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E234" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F234" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>hwg!!!</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>EOSE</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>volume picking up nicely. set right up. wait til it halts and opens back up at over 8</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>shorts still active on a day with a new 36 pt when its in the 18s honestly they deserve to get in trouble.</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>short interest , looks like 30, easy money if you pile in ! ill add little more here, but this is team work effort</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>drops 3</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>me too, shorts are covering</t>
+        </is>
+      </c>
+      <c r="D240" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E240" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F240" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>well i39m back in</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr"/>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E242" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr"/>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>rip shorts</t>
+        </is>
+      </c>
+      <c r="D244" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E244" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F244" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B245" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="inlineStr">
+        <is>
+          <t>is short interest 36</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E245" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F245" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>FIG</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>still down 23</t>
+        </is>
+      </c>
+      <c r="D246" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E246" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F246" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr"/>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E247" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F247" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr"/>
+      <c r="D248" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E248" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F248" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>this is how its done 12 went holddddd more</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>slow rise up my boyz!! fuck yeah! geezus feels goid</t>
+        </is>
+      </c>
+      <c r="D250" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E250" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F250" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>took a few 11c 821 1.50</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E251" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F251" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>in with 1700 shares at 8.47. lets see what happens.</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E252" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F252" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>keep eyes on is your next runner whales will find this name so attractive very soon 15</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F253" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>watching</t>
+        </is>
+      </c>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E254" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F254" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>fly me to the moon!</t>
+        </is>
+      </c>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="E255" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F255" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>10 today!!!!!!</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F256" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: stocktwits data 2026-06-17 19:59 UTC
</commit_message>
<xml_diff>
--- a/data/stocktwits_data.xlsx
+++ b/data/stocktwits_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D256"/>
+  <dimension ref="A1:D326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6084,6 +6084,1546 @@
       <c r="D256" s="3" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ They just want to trap as many shorts for what I think is a parabolic run later</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ let me guess, u have pumper Joealert in here?</t>
+        </is>
+      </c>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ running hot this session, up 8.7% on volume that&amp;#39;s grinding steady. these vertical moves can extend or snap back with zero warning. watching for any pullback to absorb before it stalls. who else has eyes on this?  live tape on the breakout: https://tapeboard.com/scanner</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ 100$</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>$ONCY Oncolytics Biotech® Secures New U.S. Patent Protecting Commercial Manufacturing of Pelareorep into 2044 https://www.globenewswire.com/news-release/2026/06/16/3312687/0/en/oncolytics-biotech-secures-new-u-s-patent-protecting-commercial-manufacturing-of-pelareorep-into-2044.h</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ sub 22. Needs to bounce soon.</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ is a meme. How quickly everyone forgets $NVDA invested in $QNT worked out pretty well for $NBIS $LITE Honeywell&amp;#39;s Quantinuum raises funds from Nvidia, others at $10 billion valuation | Reuters https://share.google/wtCvPEUfRcmeiglnM</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B264" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ seems to be too many sellers stepping in. We’ll see.</t>
+        </is>
+      </c>
+      <c r="D264" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>$ARQQ 6 million float. 1.7 million shares short (19%). Potential to squeeze this over 30 if sellers don’t step in.</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>$ARQQ $BTQ     Something crazy going on here.  Whales moving in. Must be news on the way.</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>$HOOD bagholders getting out new ones being created</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B268" s="3" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>$HOOD trying some 106$ calls</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>$HOOD haven&amp;#39;t sold a share -- stay squarely focused on filling that $153.86 gap from October.  Sell and leave $$$ on table  $COIN $MSTR</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>$HOOD disgusting manipulation. Can’t ever be happy owning this</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B271" s="4" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C271" s="4" t="inlineStr">
+        <is>
+          <t>$TSLA fk Robinhood $HOOD, they sold my puts at 3.30.. puts increases  7x from that point..</t>
+        </is>
+      </c>
+      <c r="D271" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B272" s="3" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>$HOOD exited at 109.5 . I guess smart move 😂</t>
+        </is>
+      </c>
+      <c r="D272" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>$HOOD this scum thinks he’s smart. The typical loser to chase.</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>$HOOD Jan 28th was the last time it was above the 200ma.  Today was the first time it crossed upward this year.</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>$HOOD   PT$  115-120  per Josh Brow  @ Half Time CNBC show.</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>$HOOD I knew it would drop. Just didn’t have the balls for the $109.29 level breaking</t>
+        </is>
+      </c>
+      <c r="D276" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>$OCUL, I have learned through many years not to get excited. This stock never follows through. The news is great, but we could be back in the 8s tomorrow.</t>
+        </is>
+      </c>
+      <c r="D277" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B278" s="4" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C278" s="4" t="inlineStr">
+        <is>
+          <t>$OCUL one more thought for all the genius &amp;quot;bulls&amp;quot; here (none of you even own a considerable amount of stock anyway):    if today was so excellent- why aren&amp;#39;t shorts covering en masse?  25 million short, right?  we should be really nervous about getting burned, right</t>
+        </is>
+      </c>
+      <c r="D278" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>$OCUL burning lot of cash.... no pharma buyer... delayed NDA...yikes. GL.... dextenza 2.0 lol</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B280" s="3" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>$OCUL I’m in the green!🍀🍀🍀</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>$OCUL  Smart team + smart plan + great data = superior product</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>$OCUL &amp;quot;Give FDA everything that they are asking for to expedite the review&amp;quot;..  Exactly what I want to hear, this will have an efficient review cycle when submitted!</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>$OCUL This is GOLD!!!</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>$OCUL 4Q NDA submission....already behind and burning cash.... down she goes</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B285" s="3" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>$OCUL what a scam artist.... submitting 4Q so they can submit SOL-R and not get a CRL LOL....</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B286" s="4" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C286" s="4" t="inlineStr">
+        <is>
+          <t>$OCUL wow, so weird...they start talking and the SP drops.  who could&amp;#39;ve seen that coming?</t>
+        </is>
+      </c>
+      <c r="D286" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>$PDYN This is exactly why you buy the low-volume fades. The market wanted definitive contracts, and Palladyne just delivered the U.S. Army. Validating SwarmOS and the Gremlin-X under a competitive DoD program proves this isn&amp;#39;t just hype, it&amp;#39;s the future of edge AI and dom</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>$PDYN shorts are gonna start getting out - to the moon</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B289" s="3" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>$PDYN im late? Bought some today below 7</t>
+        </is>
+      </c>
+      <c r="D289" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>$ONDS  $PDYN $UMAC $RCAT   This $6 Stock Just Became America&amp;#39;s Drone Supplier (I&amp;#39;M BUYING)  https://youtu.be/ffjz-eQ-lA4?is=DwLSa-hwan5cGdnj</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>$PDYN hold</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>$PDYN</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>$PDYN you know what it is</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>$PDYN SQEEEeEEeeEZE!!!</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>$BYND guys look😳 $PDYN gonna squeeze hard ! $POET</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>$PDYN incredible!! gogo !</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C297" s="3" t="inlineStr">
+        <is>
+          <t>$QURE  the market is making a compelling argument here.</t>
+        </is>
+      </c>
+      <c r="D297" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="inlineStr">
+        <is>
+          <t>Shares of $CLPT jumped 27% after $QURE’s announcement. AMT-130 uses ClearPoint’s SmartFlow cannula and navigation platform for precise intracerebral delivery.</t>
+        </is>
+      </c>
+      <c r="D298" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>$ALOT $ELTX $FTHM $GPUS $QURE</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>Top Gainers PT2                                                                         $ELTX $FTHM $QURE $ALOT $GPUS</t>
+        </is>
+      </c>
+      <c r="D300" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr">
+        <is>
+          <t>$ELTX  $QURE  FDA approval. Institutional Money created new floor and slow grinding up since then.  🧗‍♂️🚀</t>
+        </is>
+      </c>
+      <c r="D301" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B302" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="inlineStr">
+        <is>
+          <t>$QURE break 48 and confess 45</t>
+        </is>
+      </c>
+      <c r="D302" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B303" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C303" s="3" t="inlineStr">
+        <is>
+          <t>$QURE don&amp;#39;t be the last retard to sell</t>
+        </is>
+      </c>
+      <c r="D303" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr">
+        <is>
+          <t>$QURE Crazy after hours? We will see</t>
+        </is>
+      </c>
+      <c r="D304" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B305" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C305" s="3" t="inlineStr">
+        <is>
+          <t>IVA-Inventiva global NATiV3 Phase3 data due 2H2026 - Lanifibranor for MASH. $SPRO $ELTX  $QURE $CLPT $MRNA</t>
+        </is>
+      </c>
+      <c r="D305" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B306" s="3" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C306" s="3" t="inlineStr">
+        <is>
+          <t>$QURE next up on the radar #LRMR.</t>
+        </is>
+      </c>
+      <c r="D306" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B307" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C307" s="3" t="inlineStr">
+        <is>
+          <t>Many traders are watching $RXT but seeing only a single 5% gain on the chart.  What I see, however, is a stock that has been frustrating both bulls and bears for months.  With stocks like this, once short covering begins, the price can move rapidly.  The best short squeezes often</t>
+        </is>
+      </c>
+      <c r="D307" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>$SRXH $RXT $DVLT $SNDK     Lottery plays :)  High risk high reward~    Year end will tell if these are gold or poo :)</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>$RXT Why Rackspace Rallied Today    https://marketwirenews.com/stock/rxt/news/why-rackspace-rallied-today-7368977143726307.html?utm_source=stocktwits</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>$RXT  $ 10</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B311" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C311" s="3" t="inlineStr">
+        <is>
+          <t>$RXT Did the same thing last gap up... sold off hard, but then it ran 80%. We&amp;#39;ll see if it runs 80% this time aswell.</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="inlineStr">
+        <is>
+          <t>$RXT 3rd highest close since 2022 💥</t>
+        </is>
+      </c>
+      <c r="D312" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>$RXT</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>$RXT 💯</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>$RXT golden cross about to happen on the macd on the 1D chart!! something&amp;#39;s cooking on soul</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>$RXT can someone @me if this goes over $8??? Please lol 😂 I can’t watch the stock this week. And yes I won’t be back till next Monday. I will post my fish I caught so we can all fish everyday and retire early</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B317" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>$ACON we need a real move hoe come on!</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>$ACON if dips more I&amp;#39;m adding, gap fill order at 2.95-3 maybe</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>$ACON someone thinks their presentation will be good. Think so too 😉</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>$ACON</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>$ACON Patience and execution is a key here!</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>$ACON</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>$ACON unbelievable get us back to over $7 you fucks!</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B324" s="4" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C324" s="4" t="inlineStr">
+        <is>
+          <t>$ACON very bad management</t>
+        </is>
+      </c>
+      <c r="D324" s="4" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>$ACON</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>$ACON wake me up at $10 come on bitch, make a real move!</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>Bullish</t>
         </is>
       </c>
     </row>
@@ -6098,7 +7638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6148,41 +7688,41 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-16 16:48 ET</t>
+          <t>2026-06-17 15:59 ET</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>ARQQ</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-16 16:48 ET</t>
+          <t>2026-06-17 15:59 ET</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -6194,24 +7734,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>MGNI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-14 13:51 ET</t>
+          <t>2026-06-16 16:48 ET</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6221,14 +7761,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-14 15:56 ET</t>
+          <t>2026-06-14 13:51 ET</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NTLA</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6238,14 +7778,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-15 16:40 ET</t>
+          <t>2026-06-14 15:56 ET</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>NTLA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6262,7 +7802,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>HQ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6279,7 +7819,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BTQ</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6296,7 +7836,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SATS</t>
+          <t>BTQ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6313,7 +7853,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RVI</t>
+          <t>SATS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6330,7 +7870,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>KRMN</t>
+          <t>RVI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6340,14 +7880,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-16 16:37 ET</t>
+          <t>2026-06-15 16:40 ET</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LION</t>
+          <t>KRMN</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6364,7 +7904,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABCB</t>
+          <t>LION</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6381,7 +7921,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ARQQ</t>
+          <t>ABCB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6391,7 +7931,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-17 10:25 ET</t>
+          <t>2026-06-16 16:37 ET</t>
         </is>
       </c>
     </row>
@@ -6494,6 +8034,91 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>2026-06-17 10:25 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ACON</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
         </is>
       </c>
     </row>
@@ -6508,7 +8133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7340,7 +8965,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-16 16:48 ET</t>
+          <t>2026-06-17 15:59 ET</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7350,22 +8975,37 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>6.21</t>
+          <t>7.54</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>21.42%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>82092521</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>1547.67</t>
+          <t>63413054</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>69.17</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-1.44%</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1818.58%</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -7466,7 +9106,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-17 10:25 ET</t>
+          <t>2026-06-17 15:59 ET</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7476,22 +9116,37 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>22.84</t>
+          <t>22.62</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>14.54%</t>
+          <t>13.47%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1102792</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>397.47</t>
+          <t>2707064</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>73.24</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2.31</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>-63.51%</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>96.40%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -7754,6 +9409,291 @@
       <c r="N23" t="inlineStr">
         <is>
           <t>REIT - Specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>105.18</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>8.76%</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>66265805</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>69.40</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2.34</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>-31.64%</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>65.60%</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Capital Markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>9.62</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>7.61%</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>6882611</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>62.08</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>-41.48%</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>54.41%</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PDYN</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>6.95</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>16.33%</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>9552538</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>50.68</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>3.63</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>-46.58%</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>67.75%</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:59 ET</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>QURE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>48.15</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>78.40%</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>19093985</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>83.59</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>-32.66%</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>451.55%</t>
+